<commit_message>
Add NWC Year-1 memo and ~20-word justifications for all red assumptions
- Rename NWC line to (Increase)/decrease in net working capital with FY26 memo
- Scenarios col F, WACC col D, DCF col J, Comps, and 3-statement col L justifications
- Centralize assumption rationales in data.py JUST dict

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -151,6 +151,12 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
@@ -235,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -265,6 +271,9 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,16 +282,19 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -297,19 +309,19 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -319,13 +331,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -834,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -848,6 +860,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -954,767 +967,879 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="L3" s="17" t="inlineStr">
+        <is>
+          <t>Justification (~20 words)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>GROWTH &amp; MARGINS</t>
         </is>
       </c>
-      <c r="C4" s="18" t="n"/>
-      <c r="D4" s="18" t="n"/>
-      <c r="E4" s="18" t="n"/>
-      <c r="F4" s="18" t="n"/>
-      <c r="G4" s="18" t="n"/>
-      <c r="H4" s="18" t="n"/>
-      <c r="I4" s="18" t="n"/>
-      <c r="J4" s="18" t="n"/>
-      <c r="K4" s="18" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="21" t="n">
         <v>0.1860251096169196</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="21" t="n">
         <v>0.1007194095024595</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="21" t="n">
         <v>0.04858971266492285</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="22" t="n">
         <v>-0.061</v>
       </c>
-      <c r="H5" s="21" t="n">
+      <c r="H5" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="22" t="n">
         <v>0.04</v>
       </c>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="21" t="n">
         <v>0.5538906392908567</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.583141998806979</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="21" t="n">
         <v>0.5922493744407651</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="21" t="n">
         <v>0.566005440167168</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="22" t="n">
         <v>0.5649999999999999</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="22" t="n">
         <v>0.57</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="22" t="n">
         <v>0.575</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="22" t="n">
         <v>0.575</v>
       </c>
-      <c r="K6" s="21" t="n">
+      <c r="K6" s="22" t="n">
         <v>0.58</v>
       </c>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>SG&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>0.3399840799317627</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="21" t="n">
         <v>0.3531676701723352</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="21" t="n">
         <v>0.355339462337339</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="21" t="n">
         <v>0.3662706032821141</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="22" t="n">
         <v>0.425</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="22" t="n">
         <v>0.415</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="22" t="n">
         <v>0.405</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="22" t="n">
         <v>0.395</v>
       </c>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Amortization / other opex ($)</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="24" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="24" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="24" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="24" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="25" t="n">
         <v>7000</v>
       </c>
-      <c r="H8" s="23" t="n">
+      <c r="H8" s="25" t="n">
         <v>7000</v>
       </c>
-      <c r="I8" s="23" t="n">
+      <c r="I8" s="25" t="n">
         <v>7000</v>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="25" t="n">
         <v>7000</v>
       </c>
-      <c r="K8" s="23" t="n">
+      <c r="K8" s="25" t="n">
         <v>7000</v>
       </c>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Other income, net ($)</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="24" t="n">
         <v>4163</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="24" t="n">
         <v>43059</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="24" t="n">
         <v>70380</v>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="F9" s="24" t="n">
         <v>28352</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="25" t="n">
         <v>130000</v>
       </c>
-      <c r="H9" s="23" t="n">
+      <c r="H9" s="25" t="n">
         <v>60000</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="25" t="n">
         <v>75000</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="25" t="n">
         <v>95000</v>
       </c>
-      <c r="K9" s="23" t="n">
+      <c r="K9" s="25" t="n">
         <v>115000</v>
       </c>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Effective tax rate %</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <v>0.3585332413807594</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="21" t="n">
         <v>0.287509738088508</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="21" t="n">
         <v>0.2955893787336326</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="21" t="n">
         <v>0.2946823244826744</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="K10" s="22" t="n">
         <v>0.3</v>
       </c>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>CAPITAL &amp; NON-CASH ITEMS</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="18" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="19" t="n"/>
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="21" t="n">
         <v>0.03597686362326056</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="21" t="n">
         <v>0.03943996628437186</v>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="21" t="n">
         <v>0.04217214642137806</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="21" t="n">
         <v>0.04469475618323636</v>
       </c>
-      <c r="G12" s="21" t="n">
+      <c r="G12" s="22" t="n">
         <v>0.046</v>
       </c>
-      <c r="H12" s="21" t="n">
+      <c r="H12" s="22" t="n">
         <v>0.046</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="22" t="n">
         <v>0.045</v>
       </c>
-      <c r="J12" s="21" t="n">
+      <c r="J12" s="22" t="n">
         <v>0.045</v>
       </c>
-      <c r="K12" s="21" t="n">
+      <c r="K12" s="22" t="n">
         <v>0.045</v>
       </c>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Capex % of revenue</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="21" t="n">
         <v>0.07874429228811279</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="21" t="n">
         <v>0.06776652052264213</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="21" t="n">
         <v>0.0650948052563787</v>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="21" t="n">
         <v>0.06131915046925945</v>
       </c>
-      <c r="G13" s="21" t="n">
+      <c r="G13" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="H13" s="21" t="n">
+      <c r="H13" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="J13" s="21" t="n">
+      <c r="J13" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="K13" s="21" t="n">
+      <c r="K13" s="22" t="n">
         <v>0.05</v>
       </c>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Stock-based compensation ($)</t>
         </is>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <v>78075</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="24" t="n">
         <v>93560</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="24" t="n">
         <v>90011</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="24" t="n">
         <v>62203</v>
       </c>
-      <c r="G14" s="23" t="n">
+      <c r="G14" s="25" t="n">
         <v>70000</v>
       </c>
-      <c r="H14" s="23" t="n">
+      <c r="H14" s="25" t="n">
         <v>70000</v>
       </c>
-      <c r="I14" s="23" t="n">
+      <c r="I14" s="25" t="n">
         <v>70000</v>
       </c>
-      <c r="J14" s="23" t="n">
+      <c r="J14" s="25" t="n">
         <v>70000</v>
       </c>
-      <c r="K14" s="23" t="n">
+      <c r="K14" s="25" t="n">
         <v>70000</v>
       </c>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>WORKING CAPITAL &amp; BALANCE SHEET DRIVERS</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="19" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Inventories % of COGS</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="21" t="n">
         <v>0.4000264774148757</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="21" t="n">
         <v>0.330085765808543</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="21" t="n">
         <v>0.3340226506520835</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="21" t="n">
         <v>0.3529655068789499</v>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G16" s="22" t="n">
         <v>0.34</v>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="22" t="n">
         <v>0.335</v>
       </c>
-      <c r="I16" s="21" t="n">
+      <c r="I16" s="22" t="n">
         <v>0.33</v>
       </c>
-      <c r="J16" s="21" t="n">
+      <c r="J16" s="22" t="n">
         <v>0.33</v>
       </c>
-      <c r="K16" s="21" t="n">
+      <c r="K16" s="22" t="n">
         <v>0.33</v>
       </c>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Accounts payable % of COGS</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="21" t="n">
         <v>0.04774005037894764</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="21" t="n">
         <v>0.08689576951688993</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="21" t="n">
         <v>0.06286453501771355</v>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="21" t="n">
         <v>0.06878140521012073</v>
       </c>
-      <c r="G17" s="21" t="n">
+      <c r="G17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="H17" s="21" t="n">
+      <c r="H17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="I17" s="21" t="n">
+      <c r="I17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="J17" s="21" t="n">
+      <c r="J17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="K17" s="21" t="n">
+      <c r="K17" s="22" t="n">
         <v>0.068</v>
       </c>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Accrued liabilities % of revenue</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="21" t="n">
         <v>0.04922287331092786</v>
       </c>
-      <c r="D18" s="20" t="n">
+      <c r="D18" s="21" t="n">
         <v>0.03623504799424655</v>
       </c>
-      <c r="E18" s="20" t="n">
+      <c r="E18" s="21" t="n">
         <v>0.05283871763520759</v>
       </c>
-      <c r="F18" s="20" t="n">
+      <c r="F18" s="21" t="n">
         <v>0.05971412101669879</v>
       </c>
-      <c r="G18" s="21" t="n">
+      <c r="G18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="H18" s="21" t="n">
+      <c r="H18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="I18" s="21" t="n">
+      <c r="I18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="J18" s="21" t="n">
+      <c r="J18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="K18" s="21" t="n">
+      <c r="K18" s="22" t="n">
         <v>0.058</v>
       </c>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Other current assets % of revenue</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="21" t="n">
         <v>0.06870325668471483</v>
       </c>
-      <c r="D19" s="20" t="n">
+      <c r="D19" s="21" t="n">
         <v>0.05125166358639391</v>
       </c>
-      <c r="E19" s="20" t="n">
+      <c r="E19" s="21" t="n">
         <v>0.05231190108617899</v>
       </c>
-      <c r="F19" s="20" t="n">
+      <c r="F19" s="21" t="n">
         <v>0.06797921207645057</v>
       </c>
-      <c r="G19" s="21" t="n">
+      <c r="G19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="H19" s="21" t="n">
+      <c r="H19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="I19" s="21" t="n">
+      <c r="I19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="J19" s="21" t="n">
+      <c r="J19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="K19" s="21" t="n">
+      <c r="K19" s="22" t="n">
         <v>0.068</v>
       </c>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Operating lease ROU asset % of revenue</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="21" t="n">
         <v>0.1195261511040355</v>
       </c>
-      <c r="D20" s="20" t="n">
+      <c r="D20" s="21" t="n">
         <v>0.1315701656610818</v>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E20" s="21" t="n">
         <v>0.1337588918001165</v>
       </c>
-      <c r="F20" s="20" t="n">
+      <c r="F20" s="21" t="n">
         <v>0.1468287608307964</v>
       </c>
-      <c r="G20" s="21" t="n">
+      <c r="G20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="J20" s="21" t="n">
+      <c r="J20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="K20" s="21" t="n">
+      <c r="K20" s="22" t="n">
         <v>0.147</v>
       </c>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Other non-current assets % of revenue</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="21" t="n">
         <v>0.02002917692803345</v>
       </c>
-      <c r="D21" s="20" t="n">
+      <c r="D21" s="21" t="n">
         <v>0.02036119550760462</v>
       </c>
-      <c r="E21" s="20" t="n">
+      <c r="E21" s="21" t="n">
         <v>0.02407659296838742</v>
       </c>
-      <c r="F21" s="20" t="n">
+      <c r="F21" s="21" t="n">
         <v>0.03052861491902797</v>
       </c>
-      <c r="G21" s="21" t="n">
+      <c r="G21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="H21" s="21" t="n">
+      <c r="H21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="I21" s="21" t="n">
+      <c r="I21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="J21" s="21" t="n">
+      <c r="J21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="K21" s="21" t="n">
+      <c r="K21" s="22" t="n">
         <v>0.03</v>
       </c>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (current) % of revenue</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="21" t="n">
         <v>0.02564225860789656</v>
       </c>
-      <c r="D22" s="20" t="n">
+      <c r="D22" s="21" t="n">
         <v>0.02591358727754827</v>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E22" s="21" t="n">
         <v>0.02598703491061591</v>
       </c>
-      <c r="F22" s="20" t="n">
+      <c r="F22" s="21" t="n">
         <v>0.02690576981968188</v>
       </c>
-      <c r="G22" s="21" t="n">
+      <c r="G22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="H22" s="21" t="n">
+      <c r="H22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="I22" s="21" t="n">
+      <c r="I22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="J22" s="21" t="n">
+      <c r="J22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="K22" s="21" t="n">
+      <c r="K22" s="22" t="n">
         <v>0.027</v>
       </c>
+      <c r="L22" s="23" t="inlineStr">
+        <is>
+          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (non-current) % of revenue</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="21" t="n">
         <v>0.1063263776740277</v>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="21" t="n">
         <v>0.1199686712453887</v>
       </c>
-      <c r="E23" s="20" t="n">
+      <c r="E23" s="21" t="n">
         <v>0.1228392068624797</v>
       </c>
-      <c r="F23" s="20" t="n">
+      <c r="F23" s="21" t="n">
         <v>0.1350779997478068</v>
       </c>
-      <c r="G23" s="21" t="n">
+      <c r="G23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="H23" s="21" t="n">
+      <c r="H23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="I23" s="21" t="n">
+      <c r="I23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="J23" s="21" t="n">
+      <c r="J23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="K23" s="21" t="n">
+      <c r="K23" s="22" t="n">
         <v>0.135</v>
       </c>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Other current liabilities % of revenue</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="21" t="n">
         <v>0.08782065461170298</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="21" t="n">
         <v>0.0712106459549251</v>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="21" t="n">
         <v>0.06928582073919408</v>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="21" t="n">
         <v>0.05353890079801128</v>
       </c>
-      <c r="G24" s="21" t="n">
+      <c r="G24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="H24" s="21" t="n">
+      <c r="H24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="I24" s="21" t="n">
+      <c r="I24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="J24" s="21" t="n">
+      <c r="J24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="K24" s="21" t="n">
+      <c r="K24" s="22" t="n">
         <v>0.055</v>
       </c>
+      <c r="L24" s="23" t="inlineStr">
+        <is>
+          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Other non-current liab % of revenue</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="21" t="n">
         <v>0.005991602509235539</v>
       </c>
-      <c r="D25" s="20" t="n">
+      <c r="D25" s="21" t="n">
         <v>0.00468486304273564</v>
       </c>
-      <c r="E25" s="20" t="n">
+      <c r="E25" s="21" t="n">
         <v>0.003852428654513556</v>
       </c>
-      <c r="F25" s="20" t="n">
+      <c r="F25" s="21" t="n">
         <v>0.004986219444094176</v>
       </c>
-      <c r="G25" s="21" t="n">
+      <c r="G25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="H25" s="21" t="n">
+      <c r="H25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="I25" s="21" t="n">
+      <c r="I25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="J25" s="21" t="n">
+      <c r="J25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="K25" s="21" t="n">
+      <c r="K25" s="22" t="n">
         <v>0.005</v>
       </c>
+      <c r="L25" s="23" t="inlineStr">
+        <is>
+          <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>CAPITAL RETURN</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
-      <c r="I26" s="18" t="n"/>
-      <c r="J26" s="18" t="n"/>
-      <c r="K26" s="18" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Share repurchases ($)</t>
         </is>
       </c>
-      <c r="C27" s="22" t="n">
+      <c r="C27" s="24" t="n">
         <v>444001</v>
       </c>
-      <c r="D27" s="22" t="n">
+      <c r="D27" s="24" t="n">
         <v>558652</v>
       </c>
-      <c r="E27" s="22" t="n">
+      <c r="E27" s="24" t="n">
         <v>1636879</v>
       </c>
-      <c r="F27" s="22" t="n">
+      <c r="F27" s="24" t="n">
         <v>1178349</v>
       </c>
-      <c r="G27" s="23" t="n">
+      <c r="G27" s="25" t="n">
         <v>500000</v>
       </c>
-      <c r="H27" s="23" t="n">
+      <c r="H27" s="25" t="n">
         <v>500000</v>
       </c>
-      <c r="I27" s="23" t="n">
+      <c r="I27" s="25" t="n">
         <v>500000</v>
       </c>
-      <c r="J27" s="23" t="n">
+      <c r="J27" s="25" t="n">
         <v>500000</v>
       </c>
-      <c r="K27" s="23" t="n">
+      <c r="K27" s="25" t="n">
         <v>500000</v>
       </c>
+      <c r="L27" s="23" t="inlineStr">
+        <is>
+          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Avg repurchase price ($/sh)</t>
         </is>
       </c>
-      <c r="G28" s="24" t="n">
+      <c r="G28" s="26" t="n">
         <v>105</v>
       </c>
-      <c r="H28" s="24" t="n">
+      <c r="H28" s="26" t="n">
         <v>112</v>
       </c>
-      <c r="I28" s="24" t="n">
+      <c r="I28" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="J28" s="24" t="n">
+      <c r="J28" s="26" t="n">
         <v>128</v>
       </c>
-      <c r="K28" s="24" t="n">
+      <c r="K28" s="26" t="n">
         <v>135</v>
+      </c>
+      <c r="L28" s="23" t="inlineStr">
+        <is>
+          <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1755,6 +1880,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1815,701 +1941,701 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="26" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C4" s="27" t="n">
+      <c r="C4" s="29" t="n">
         <v>8110518</v>
       </c>
-      <c r="D4" s="27" t="n">
+      <c r="D4" s="29" t="n">
         <v>9619278</v>
       </c>
-      <c r="E4" s="27" t="n">
+      <c r="E4" s="29" t="n">
         <v>10588126</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="29" t="n">
         <v>11102600</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="24">
         <f>F4*(1+'Assumptions'!G5)</f>
         <v/>
       </c>
-      <c r="H4" s="22">
+      <c r="H4" s="24">
         <f>G4*(1+'Assumptions'!H5)</f>
         <v/>
       </c>
-      <c r="I4" s="22">
+      <c r="I4" s="24">
         <f>H4*(1+'Assumptions'!I5)</f>
         <v/>
       </c>
-      <c r="J4" s="22">
+      <c r="J4" s="24">
         <f>I4*(1+'Assumptions'!J5)</f>
         <v/>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="24">
         <f>J4*(1+'Assumptions'!K5)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Cost of goods sold</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="29" t="n">
         <v>3618178</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="29" t="n">
         <v>4009873</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="29" t="n">
         <v>4317315</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="29" t="n">
         <v>4818468</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="24">
         <f>G4*(1-'Assumptions'!G6)</f>
         <v/>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="24">
         <f>H4*(1-'Assumptions'!H6)</f>
         <v/>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="24">
         <f>I4*(1-'Assumptions'!I6)</f>
         <v/>
       </c>
-      <c r="J5" s="22">
+      <c r="J5" s="24">
         <f>J4*(1-'Assumptions'!J6)</f>
         <v/>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="24">
         <f>K4*(1-'Assumptions'!K6)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="31">
         <f>C4-C5</f>
         <v/>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="31">
         <f>D4-D5</f>
         <v/>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="31">
         <f>E4-E5</f>
         <v/>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="31">
         <f>F4-F5</f>
         <v/>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="31">
         <f>G4-G5</f>
         <v/>
       </c>
-      <c r="H6" s="29">
+      <c r="H6" s="31">
         <f>H4-H5</f>
         <v/>
       </c>
-      <c r="I6" s="29">
+      <c r="I6" s="31">
         <f>I4-I5</f>
         <v/>
       </c>
-      <c r="J6" s="29">
+      <c r="J6" s="31">
         <f>J4-J5</f>
         <v/>
       </c>
-      <c r="K6" s="29">
+      <c r="K6" s="31">
         <f>K4-K5</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Selling, general &amp; administrative</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="29" t="n">
         <v>2757447</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="29" t="n">
         <v>3397218</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="29" t="n">
         <v>3762379</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="29" t="n">
         <v>4066556</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="24">
         <f>G4*'Assumptions'!G7</f>
         <v/>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="24">
         <f>H4*'Assumptions'!H7</f>
         <v/>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="24">
         <f>I4*'Assumptions'!I7</f>
         <v/>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="24">
         <f>J4*'Assumptions'!J7</f>
         <v/>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="24">
         <f>K4*'Assumptions'!K7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Amortization of intangibles / other</t>
         </is>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="29" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="29" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="29" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="29" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="24">
         <f>'Assumptions'!G8</f>
         <v/>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="24">
         <f>'Assumptions'!H8</f>
         <v/>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="24">
         <f>'Assumptions'!I8</f>
         <v/>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="24">
         <f>'Assumptions'!J8</f>
         <v/>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="24">
         <f>'Assumptions'!K8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Operating income (EBIT)</t>
         </is>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="31">
         <f>C6-C7-C8</f>
         <v/>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="31">
         <f>D6-D7-D8</f>
         <v/>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="31">
         <f>E6-E7-E8</f>
         <v/>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="31">
         <f>F6-F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="31">
         <f>G6-G7-G8</f>
         <v/>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="31">
         <f>H6-H7-H8</f>
         <v/>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="31">
         <f>I6-I7-I8</f>
         <v/>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="31">
         <f>J6-J7-J8</f>
         <v/>
       </c>
-      <c r="K9" s="29">
+      <c r="K9" s="31">
         <f>K6-K7-K8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Other income, net</t>
         </is>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="29" t="n">
         <v>4163</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="29" t="n">
         <v>43059</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="29" t="n">
         <v>70380</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="29" t="n">
         <v>28352</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="24">
         <f>'Assumptions'!G9</f>
         <v/>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="24">
         <f>'Assumptions'!H9</f>
         <v/>
       </c>
-      <c r="I10" s="22">
+      <c r="I10" s="24">
         <f>'Assumptions'!I9</f>
         <v/>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="24">
         <f>'Assumptions'!J9</f>
         <v/>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="24">
         <f>'Assumptions'!K9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Pre-tax income</t>
         </is>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="31">
         <f>C9+C10</f>
         <v/>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="31">
         <f>D9+D10</f>
         <v/>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="31">
         <f>E9+E10</f>
         <v/>
       </c>
-      <c r="F11" s="29">
+      <c r="F11" s="31">
         <f>F9+F10</f>
         <v/>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="31">
         <f>G9+G10</f>
         <v/>
       </c>
-      <c r="H11" s="29">
+      <c r="H11" s="31">
         <f>H9+H10</f>
         <v/>
       </c>
-      <c r="I11" s="29">
+      <c r="I11" s="31">
         <f>I9+I10</f>
         <v/>
       </c>
-      <c r="J11" s="29">
+      <c r="J11" s="31">
         <f>J9+J10</f>
         <v/>
       </c>
-      <c r="K11" s="29">
+      <c r="K11" s="31">
         <f>K9+K10</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="29" t="n">
         <v>477771</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="29" t="n">
         <v>625545</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="29" t="n">
         <v>761461</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="29" t="n">
         <v>659784</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="24">
         <f>G11*'Assumptions'!G10</f>
         <v/>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="24">
         <f>H11*'Assumptions'!H10</f>
         <v/>
       </c>
-      <c r="I12" s="22">
+      <c r="I12" s="24">
         <f>I11*'Assumptions'!I10</f>
         <v/>
       </c>
-      <c r="J12" s="22">
+      <c r="J12" s="24">
         <f>J11*'Assumptions'!J10</f>
         <v/>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="24">
         <f>K11*'Assumptions'!K10</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="C13" s="30">
+      <c r="C13" s="32">
         <f>C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="30">
+      <c r="D13" s="32">
         <f>D11-D12</f>
         <v/>
       </c>
-      <c r="E13" s="30">
+      <c r="E13" s="32">
         <f>E11-E12</f>
         <v/>
       </c>
-      <c r="F13" s="30">
+      <c r="F13" s="32">
         <f>F11-F12</f>
         <v/>
       </c>
-      <c r="G13" s="30">
+      <c r="G13" s="32">
         <f>G11-G12</f>
         <v/>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="32">
         <f>H11-H12</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="32">
         <f>I11-I12</f>
         <v/>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="32">
         <f>J11-J12</f>
         <v/>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="32">
         <f>K11-K12</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Diluted weighted-avg shares (000)</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="29" t="n">
         <v>128017</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="29" t="n">
         <v>127060</v>
       </c>
-      <c r="E15" s="27" t="n">
+      <c r="E15" s="29" t="n">
         <v>123935</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="29" t="n">
         <v>119068</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="24">
         <f>F15-'Assumptions'!G27/'Assumptions'!G28</f>
         <v/>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="24">
         <f>G15-'Assumptions'!H27/'Assumptions'!H28</f>
         <v/>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="24">
         <f>H15-'Assumptions'!I27/'Assumptions'!I28</f>
         <v/>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="24">
         <f>I15-'Assumptions'!J27/'Assumptions'!J28</f>
         <v/>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="24">
         <f>J15-'Assumptions'!K27/'Assumptions'!K28</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>Diluted EPS ($)</t>
         </is>
       </c>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="33" t="n">
         <v>6.68</v>
       </c>
-      <c r="D16" s="31" t="n">
+      <c r="D16" s="33" t="n">
         <v>12.2</v>
       </c>
-      <c r="E16" s="31" t="n">
+      <c r="E16" s="33" t="n">
         <v>14.64</v>
       </c>
-      <c r="F16" s="31" t="n">
+      <c r="F16" s="33" t="n">
         <v>13.26</v>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="34">
         <f>G13/G15</f>
         <v/>
       </c>
-      <c r="H16" s="32">
+      <c r="H16" s="34">
         <f>H13/H15</f>
         <v/>
       </c>
-      <c r="I16" s="32">
+      <c r="I16" s="34">
         <f>I13/I15</f>
         <v/>
       </c>
-      <c r="J16" s="32">
+      <c r="J16" s="34">
         <f>J13/J15</f>
         <v/>
       </c>
-      <c r="K16" s="32">
+      <c r="K16" s="34">
         <f>K13/K15</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr">
         <is>
           <t>Margins &amp; growth</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
-      <c r="I18" s="18" t="n"/>
-      <c r="J18" s="18" t="n"/>
-      <c r="K18" s="18" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="36" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="37">
         <f>C6/C4</f>
         <v/>
       </c>
-      <c r="D19" s="35">
+      <c r="D19" s="37">
         <f>D6/D4</f>
         <v/>
       </c>
-      <c r="E19" s="35">
+      <c r="E19" s="37">
         <f>E6/E4</f>
         <v/>
       </c>
-      <c r="F19" s="35">
+      <c r="F19" s="37">
         <f>F6/F4</f>
         <v/>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="37">
         <f>G6/G4</f>
         <v/>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="37">
         <f>H6/H4</f>
         <v/>
       </c>
-      <c r="I19" s="35">
+      <c r="I19" s="37">
         <f>I6/I4</f>
         <v/>
       </c>
-      <c r="J19" s="35">
+      <c r="J19" s="37">
         <f>J6/J4</f>
         <v/>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="37">
         <f>K6/K4</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="34" t="inlineStr">
+      <c r="A20" s="36" t="inlineStr">
         <is>
           <t>Operating margin %</t>
         </is>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="37">
         <f>C9/C4</f>
         <v/>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="37">
         <f>D9/D4</f>
         <v/>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="37">
         <f>E9/E4</f>
         <v/>
       </c>
-      <c r="F20" s="35">
+      <c r="F20" s="37">
         <f>F9/F4</f>
         <v/>
       </c>
-      <c r="G20" s="35">
+      <c r="G20" s="37">
         <f>G9/G4</f>
         <v/>
       </c>
-      <c r="H20" s="35">
+      <c r="H20" s="37">
         <f>H9/H4</f>
         <v/>
       </c>
-      <c r="I20" s="35">
+      <c r="I20" s="37">
         <f>I9/I4</f>
         <v/>
       </c>
-      <c r="J20" s="35">
+      <c r="J20" s="37">
         <f>J9/J4</f>
         <v/>
       </c>
-      <c r="K20" s="35">
+      <c r="K20" s="37">
         <f>K9/K4</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="34" t="inlineStr">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>Net margin %</t>
         </is>
       </c>
-      <c r="C21" s="35">
+      <c r="C21" s="37">
         <f>C13/C4</f>
         <v/>
       </c>
-      <c r="D21" s="35">
+      <c r="D21" s="37">
         <f>D13/D4</f>
         <v/>
       </c>
-      <c r="E21" s="35">
+      <c r="E21" s="37">
         <f>E13/E4</f>
         <v/>
       </c>
-      <c r="F21" s="35">
+      <c r="F21" s="37">
         <f>F13/F4</f>
         <v/>
       </c>
-      <c r="G21" s="35">
+      <c r="G21" s="37">
         <f>G13/G4</f>
         <v/>
       </c>
-      <c r="H21" s="35">
+      <c r="H21" s="37">
         <f>H13/H4</f>
         <v/>
       </c>
-      <c r="I21" s="35">
+      <c r="I21" s="37">
         <f>I13/I4</f>
         <v/>
       </c>
-      <c r="J21" s="35">
+      <c r="J21" s="37">
         <f>J13/J4</f>
         <v/>
       </c>
-      <c r="K21" s="35">
+      <c r="K21" s="37">
         <f>K13/K4</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="C22" s="36" t="inlineStr">
+      <c r="C22" s="38" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="D22" s="35">
+      <c r="D22" s="37">
         <f>D4/C4-1</f>
         <v/>
       </c>
-      <c r="E22" s="35">
+      <c r="E22" s="37">
         <f>E4/D4-1</f>
         <v/>
       </c>
-      <c r="F22" s="35">
+      <c r="F22" s="37">
         <f>F4/E4-1</f>
         <v/>
       </c>
-      <c r="G22" s="35">
+      <c r="G22" s="37">
         <f>G4/F4-1</f>
         <v/>
       </c>
-      <c r="H22" s="35">
+      <c r="H22" s="37">
         <f>H4/G4-1</f>
         <v/>
       </c>
-      <c r="I22" s="35">
+      <c r="I22" s="37">
         <f>I4/H4-1</f>
         <v/>
       </c>
-      <c r="J22" s="35">
+      <c r="J22" s="37">
         <f>J4/I4-1</f>
         <v/>
       </c>
-      <c r="K22" s="35">
+      <c r="K22" s="37">
         <f>K4/J4-1</f>
         <v/>
       </c>
@@ -2577,6 +2703,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2637,1039 +2764,1039 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="26" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>ASSETS</t>
         </is>
       </c>
-      <c r="C4" s="18" t="n"/>
-      <c r="D4" s="18" t="n"/>
-      <c r="E4" s="18" t="n"/>
-      <c r="F4" s="18" t="n"/>
-      <c r="G4" s="18" t="n"/>
-      <c r="H4" s="18" t="n"/>
-      <c r="I4" s="18" t="n"/>
-      <c r="J4" s="18" t="n"/>
-      <c r="K4" s="18" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>Current assets:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Cash &amp; cash equivalents</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="29" t="n">
         <v>1154867</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="29" t="n">
         <v>2243971</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="29" t="n">
         <v>1984336</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="29" t="n">
         <v>1807202</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="24">
         <f>'Cash Flow'!G33</f>
         <v/>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="24">
         <f>'Cash Flow'!H33</f>
         <v/>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="24">
         <f>'Cash Flow'!I33</f>
         <v/>
       </c>
-      <c r="J6" s="22">
+      <c r="J6" s="24">
         <f>'Cash Flow'!J33</f>
         <v/>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="24">
         <f>'Cash Flow'!K33</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="29" t="n">
         <v>1447367</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="29" t="n">
         <v>1323602</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="29" t="n">
         <v>1442081</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="29" t="n">
         <v>1700753</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="24">
         <f>'Income Statement'!G5*'Assumptions'!G16</f>
         <v/>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="24">
         <f>'Income Statement'!H5*'Assumptions'!H16</f>
         <v/>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="24">
         <f>'Income Statement'!I5*'Assumptions'!I16</f>
         <v/>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="24">
         <f>'Income Statement'!J5*'Assumptions'!J16</f>
         <v/>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="24">
         <f>'Income Statement'!K5*'Assumptions'!K16</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Other current assets</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="24" t="n">
         <v>557219</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="24" t="n">
         <v>493004</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="24" t="n">
         <v>553885</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="24" t="n">
         <v>754746</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G19</f>
         <v/>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H19</f>
         <v/>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I19</f>
         <v/>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J19</f>
         <v/>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K19</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="40" t="n">
         <v>3159453</v>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="40" t="n">
         <v>4060577</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="40" t="n">
         <v>3980302</v>
       </c>
-      <c r="F9" s="38" t="n">
+      <c r="F9" s="40" t="n">
         <v>4262701</v>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="31">
         <f>G6+G7+G8</f>
         <v/>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="31">
         <f>H6+H7+H8</f>
         <v/>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="31">
         <f>I6+I7+I8</f>
         <v/>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="31">
         <f>J6+J7+J8</f>
         <v/>
       </c>
-      <c r="K9" s="29">
+      <c r="K9" s="31">
         <f>K6+K7+K8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="37" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Non-current assets:</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Property &amp; equipment, net</t>
         </is>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="29" t="n">
         <v>1269614</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="29" t="n">
         <v>1545811</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="29" t="n">
         <v>1780617</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="29" t="n">
         <v>2033720</v>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="24">
         <f>F11+'Income Statement'!G4*'Assumptions'!G13-'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="24">
         <f>G11+'Income Statement'!H4*'Assumptions'!H13-'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="24">
         <f>H11+'Income Statement'!I4*'Assumptions'!I13-'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J11" s="22">
+      <c r="J11" s="24">
         <f>I11+'Income Statement'!J4*'Assumptions'!J13-'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="24">
         <f>J11+'Income Statement'!K4*'Assumptions'!K13-'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Operating lease right-of-use assets</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="29" t="n">
         <v>969419</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="29" t="n">
         <v>1265610</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="29" t="n">
         <v>1416256</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="29" t="n">
         <v>1630181</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G20</f>
         <v/>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H20</f>
         <v/>
       </c>
-      <c r="I12" s="22">
+      <c r="I12" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I20</f>
         <v/>
       </c>
-      <c r="J12" s="22">
+      <c r="J12" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J20</f>
         <v/>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K20</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Goodwill &amp; intangible assets</t>
         </is>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="29" t="n">
         <v>46105</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="29" t="n">
         <v>24083</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="29" t="n">
         <v>171191</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="29" t="n">
         <v>191194</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="24">
         <f>F13</f>
         <v/>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="24">
         <f>G13</f>
         <v/>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="24">
         <f>H13</f>
         <v/>
       </c>
-      <c r="J13" s="22">
+      <c r="J13" s="24">
         <f>I13</f>
         <v/>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="24">
         <f>J13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="24" t="n">
         <v>162447</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="24" t="n">
         <v>195860</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="24" t="n">
         <v>254926</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="24" t="n">
         <v>338947</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G21</f>
         <v/>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H21</f>
         <v/>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I21</f>
         <v/>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J21</f>
         <v/>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K21</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="C15" s="39" t="n">
+      <c r="C15" s="41" t="n">
         <v>5607038</v>
       </c>
-      <c r="D15" s="39" t="n">
+      <c r="D15" s="41" t="n">
         <v>7091941</v>
       </c>
-      <c r="E15" s="39" t="n">
+      <c r="E15" s="41" t="n">
         <v>7603292</v>
       </c>
-      <c r="F15" s="39" t="n">
+      <c r="F15" s="41" t="n">
         <v>8456743</v>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="32">
         <f>G9+G11+G12+G13+G14</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="32">
         <f>H9+H11+H12+H13+H14</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="32">
         <f>I9+I11+I12+I13+I14</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="32">
         <f>J9+J11+J12+J13+J14</f>
         <v/>
       </c>
-      <c r="K15" s="30">
+      <c r="K15" s="32">
         <f>K9+K11+K12+K13+K14</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n"/>
-      <c r="J17" s="18" t="n"/>
-      <c r="K17" s="18" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="37" t="inlineStr">
+      <c r="A18" s="39" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Accounts payable</t>
         </is>
       </c>
-      <c r="C19" s="27" t="n">
+      <c r="C19" s="29" t="n">
         <v>172732</v>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D19" s="29" t="n">
         <v>348441</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="29" t="n">
         <v>271406</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="29" t="n">
         <v>331421</v>
       </c>
-      <c r="G19" s="22">
+      <c r="G19" s="24">
         <f>'Income Statement'!G5*'Assumptions'!G17</f>
         <v/>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="24">
         <f>'Income Statement'!H5*'Assumptions'!H17</f>
         <v/>
       </c>
-      <c r="I19" s="22">
+      <c r="I19" s="24">
         <f>'Income Statement'!I5*'Assumptions'!I17</f>
         <v/>
       </c>
-      <c r="J19" s="22">
+      <c r="J19" s="24">
         <f>'Income Statement'!J5*'Assumptions'!J17</f>
         <v/>
       </c>
-      <c r="K19" s="22">
+      <c r="K19" s="24">
         <f>'Income Statement'!K5*'Assumptions'!K17</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Accrued liabilities</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="29" t="n">
         <v>399223</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="29" t="n">
         <v>348555</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="29" t="n">
         <v>559463</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="29" t="n">
         <v>662982</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G18</f>
         <v/>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H18</f>
         <v/>
       </c>
-      <c r="I20" s="22">
+      <c r="I20" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I18</f>
         <v/>
       </c>
-      <c r="J20" s="22">
+      <c r="J20" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J18</f>
         <v/>
       </c>
-      <c r="K20" s="22">
+      <c r="K20" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K18</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Operating lease liabilities (current)</t>
         </is>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C21" s="29" t="n">
         <v>207972</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D21" s="29" t="n">
         <v>249270</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="29" t="n">
         <v>275154</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="29" t="n">
         <v>298724</v>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G22</f>
         <v/>
       </c>
-      <c r="H21" s="22">
+      <c r="H21" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H22</f>
         <v/>
       </c>
-      <c r="I21" s="22">
+      <c r="I21" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I22</f>
         <v/>
       </c>
-      <c r="J21" s="22">
+      <c r="J21" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J22</f>
         <v/>
       </c>
-      <c r="K21" s="22">
+      <c r="K21" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K22</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Other current liabilities</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="24" t="n">
         <v>712271</v>
       </c>
-      <c r="D22" s="22" t="n">
+      <c r="D22" s="24" t="n">
         <v>684995</v>
       </c>
-      <c r="E22" s="22" t="n">
+      <c r="E22" s="24" t="n">
         <v>733607</v>
       </c>
-      <c r="F22" s="22" t="n">
+      <c r="F22" s="24" t="n">
         <v>594421</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G24</f>
         <v/>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H24</f>
         <v/>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I24</f>
         <v/>
       </c>
-      <c r="J22" s="22">
+      <c r="J22" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J24</f>
         <v/>
       </c>
-      <c r="K22" s="22">
+      <c r="K22" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K24</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>Total current liabilities</t>
         </is>
       </c>
-      <c r="C23" s="38" t="n">
+      <c r="C23" s="40" t="n">
         <v>1492198</v>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D23" s="40" t="n">
         <v>1631261</v>
       </c>
-      <c r="E23" s="38" t="n">
+      <c r="E23" s="40" t="n">
         <v>1839630</v>
       </c>
-      <c r="F23" s="38" t="n">
+      <c r="F23" s="40" t="n">
         <v>1887548</v>
       </c>
-      <c r="G23" s="29">
+      <c r="G23" s="31">
         <f>G19+G20+G21+G22</f>
         <v/>
       </c>
-      <c r="H23" s="29">
+      <c r="H23" s="31">
         <f>H19+H20+H21+H22</f>
         <v/>
       </c>
-      <c r="I23" s="29">
+      <c r="I23" s="31">
         <f>I19+I20+I21+I22</f>
         <v/>
       </c>
-      <c r="J23" s="29">
+      <c r="J23" s="31">
         <f>J19+J20+J21+J22</f>
         <v/>
       </c>
-      <c r="K23" s="29">
+      <c r="K23" s="31">
         <f>K19+K20+K21+K22</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="37" t="inlineStr">
+      <c r="A24" s="39" t="inlineStr">
         <is>
           <t>Non-current liabilities:</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Operating lease liabilities (non-current)</t>
         </is>
       </c>
-      <c r="C25" s="27" t="n">
+      <c r="C25" s="29" t="n">
         <v>862362</v>
       </c>
-      <c r="D25" s="27" t="n">
+      <c r="D25" s="29" t="n">
         <v>1154012</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="29" t="n">
         <v>1300637</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="29" t="n">
         <v>1499717</v>
       </c>
-      <c r="G25" s="22">
+      <c r="G25" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G23</f>
         <v/>
       </c>
-      <c r="H25" s="22">
+      <c r="H25" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H23</f>
         <v/>
       </c>
-      <c r="I25" s="22">
+      <c r="I25" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I23</f>
         <v/>
       </c>
-      <c r="J25" s="22">
+      <c r="J25" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J23</f>
         <v/>
       </c>
-      <c r="K25" s="22">
+      <c r="K25" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K23</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Deferred income taxes</t>
         </is>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C26" s="29" t="n">
         <v>55084</v>
       </c>
-      <c r="D26" s="27" t="n">
+      <c r="D26" s="29" t="n">
         <v>29522</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="29" t="n">
         <v>98188</v>
       </c>
-      <c r="F26" s="27" t="n">
+      <c r="F26" s="29" t="n">
         <v>52278</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="24">
         <f>F26</f>
         <v/>
       </c>
-      <c r="H26" s="22">
+      <c r="H26" s="24">
         <f>G26</f>
         <v/>
       </c>
-      <c r="I26" s="22">
+      <c r="I26" s="24">
         <f>H26</f>
         <v/>
       </c>
-      <c r="J26" s="22">
+      <c r="J26" s="24">
         <f>I26</f>
         <v/>
       </c>
-      <c r="K26" s="22">
+      <c r="K26" s="24">
         <f>J26</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="C27" s="22" t="n">
+      <c r="C27" s="24" t="n">
         <v>48595</v>
       </c>
-      <c r="D27" s="22" t="n">
+      <c r="D27" s="24" t="n">
         <v>45065</v>
       </c>
-      <c r="E27" s="22" t="n">
+      <c r="E27" s="24" t="n">
         <v>40790</v>
       </c>
-      <c r="F27" s="22" t="n">
+      <c r="F27" s="24" t="n">
         <v>55360</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G25</f>
         <v/>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H25</f>
         <v/>
       </c>
-      <c r="I27" s="22">
+      <c r="I27" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I25</f>
         <v/>
       </c>
-      <c r="J27" s="22">
+      <c r="J27" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J25</f>
         <v/>
       </c>
-      <c r="K27" s="22">
+      <c r="K27" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="C28" s="38" t="n">
+      <c r="C28" s="40" t="n">
         <v>2458239</v>
       </c>
-      <c r="D28" s="38" t="n">
+      <c r="D28" s="40" t="n">
         <v>2859860</v>
       </c>
-      <c r="E28" s="38" t="n">
+      <c r="E28" s="40" t="n">
         <v>3279245</v>
       </c>
-      <c r="F28" s="38" t="n">
+      <c r="F28" s="40" t="n">
         <v>3494903</v>
       </c>
-      <c r="G28" s="29">
+      <c r="G28" s="31">
         <f>G23+G25+G26+G27</f>
         <v/>
       </c>
-      <c r="H28" s="29">
+      <c r="H28" s="31">
         <f>H23+H25+H26+H27</f>
         <v/>
       </c>
-      <c r="I28" s="29">
+      <c r="I28" s="31">
         <f>I23+I25+I26+I27</f>
         <v/>
       </c>
-      <c r="J28" s="29">
+      <c r="J28" s="31">
         <f>J23+J25+J26+J27</f>
         <v/>
       </c>
-      <c r="K28" s="29">
+      <c r="K28" s="31">
         <f>K23+K25+K26+K27</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="37" t="inlineStr">
+      <c r="A30" s="39" t="inlineStr">
         <is>
           <t>Shareholders' equity:</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>Common stock &amp; additional paid-in capital</t>
         </is>
       </c>
-      <c r="C31" s="27" t="n">
+      <c r="C31" s="29" t="n">
         <v>475256</v>
       </c>
-      <c r="D31" s="27" t="n">
+      <c r="D31" s="29" t="n">
         <v>575975</v>
       </c>
-      <c r="E31" s="27" t="n">
+      <c r="E31" s="29" t="n">
         <v>638771</v>
       </c>
-      <c r="F31" s="27" t="n">
+      <c r="F31" s="29" t="n">
         <v>669949</v>
       </c>
-      <c r="G31" s="22">
+      <c r="G31" s="24">
         <f>F31+'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="24">
         <f>G31+'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I31" s="22">
+      <c r="I31" s="24">
         <f>H31+'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J31" s="22">
+      <c r="J31" s="24">
         <f>I31+'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K31" s="22">
+      <c r="K31" s="24">
         <f>J31+'Assumptions'!K14</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="C32" s="27" t="n">
+      <c r="C32" s="29" t="n">
         <v>2926127</v>
       </c>
-      <c r="D32" s="27" t="n">
+      <c r="D32" s="29" t="n">
         <v>3920362</v>
       </c>
-      <c r="E32" s="27" t="n">
+      <c r="E32" s="29" t="n">
         <v>4109717</v>
       </c>
-      <c r="F32" s="27" t="n">
+      <c r="F32" s="29" t="n">
         <v>4522581</v>
       </c>
-      <c r="G32" s="22">
+      <c r="G32" s="24">
         <f>F32+'Income Statement'!G13-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H32" s="22">
+      <c r="H32" s="24">
         <f>G32+'Income Statement'!H13-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I32" s="22">
+      <c r="I32" s="24">
         <f>H32+'Income Statement'!I13-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J32" s="22">
+      <c r="J32" s="24">
         <f>I32+'Income Statement'!J13-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K32" s="22">
+      <c r="K32" s="24">
         <f>J32+'Income Statement'!K13-'Assumptions'!K27</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>Accumulated other comprehensive loss</t>
         </is>
       </c>
-      <c r="C33" s="27" t="n">
+      <c r="C33" s="29" t="n">
         <v>-252584</v>
       </c>
-      <c r="D33" s="27" t="n">
+      <c r="D33" s="29" t="n">
         <v>-264256</v>
       </c>
-      <c r="E33" s="27" t="n">
+      <c r="E33" s="29" t="n">
         <v>-424441</v>
       </c>
-      <c r="F33" s="27" t="n">
+      <c r="F33" s="29" t="n">
         <v>-230690</v>
       </c>
-      <c r="G33" s="22">
+      <c r="G33" s="24">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="22">
+      <c r="H33" s="24">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I33" s="22">
+      <c r="I33" s="24">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J33" s="22">
+      <c r="J33" s="24">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K33" s="22">
+      <c r="K33" s="24">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="30" t="inlineStr">
         <is>
           <t>TOTAL SHAREHOLDERS' EQUITY</t>
         </is>
       </c>
-      <c r="C34" s="38" t="n">
+      <c r="C34" s="40" t="n">
         <v>3148799</v>
       </c>
-      <c r="D34" s="38" t="n">
+      <c r="D34" s="40" t="n">
         <v>4232081</v>
       </c>
-      <c r="E34" s="38" t="n">
+      <c r="E34" s="40" t="n">
         <v>4324047</v>
       </c>
-      <c r="F34" s="38" t="n">
+      <c r="F34" s="40" t="n">
         <v>4961840</v>
       </c>
-      <c r="G34" s="29">
+      <c r="G34" s="31">
         <f>G31+G32+G33</f>
         <v/>
       </c>
-      <c r="H34" s="29">
+      <c r="H34" s="31">
         <f>H31+H32+H33</f>
         <v/>
       </c>
-      <c r="I34" s="29">
+      <c r="I34" s="31">
         <f>I31+I32+I33</f>
         <v/>
       </c>
-      <c r="J34" s="29">
+      <c r="J34" s="31">
         <f>J31+J32+J33</f>
         <v/>
       </c>
-      <c r="K34" s="29">
+      <c r="K34" s="31">
         <f>K31+K32+K33</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="28" t="inlineStr">
+      <c r="A35" s="30" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="32">
         <f>C28+C34</f>
         <v/>
       </c>
-      <c r="D35" s="30">
+      <c r="D35" s="32">
         <f>D28+D34</f>
         <v/>
       </c>
-      <c r="E35" s="30">
+      <c r="E35" s="32">
         <f>E28+E34</f>
         <v/>
       </c>
-      <c r="F35" s="30">
+      <c r="F35" s="32">
         <f>F28+F34</f>
         <v/>
       </c>
-      <c r="G35" s="30">
+      <c r="G35" s="32">
         <f>G28+G34</f>
         <v/>
       </c>
-      <c r="H35" s="30">
+      <c r="H35" s="32">
         <f>H28+H34</f>
         <v/>
       </c>
-      <c r="I35" s="30">
+      <c r="I35" s="32">
         <f>I28+I34</f>
         <v/>
       </c>
-      <c r="J35" s="30">
+      <c r="J35" s="32">
         <f>J28+J34</f>
         <v/>
       </c>
-      <c r="K35" s="30">
+      <c r="K35" s="32">
         <f>K28+K34</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="inlineStr">
+      <c r="A37" s="36" t="inlineStr">
         <is>
           <t>Balance check (Assets − L&amp;E)</t>
         </is>
       </c>
-      <c r="C37" s="40">
+      <c r="C37" s="42">
         <f>C15-C35</f>
         <v/>
       </c>
-      <c r="D37" s="40">
+      <c r="D37" s="42">
         <f>D15-D35</f>
         <v/>
       </c>
-      <c r="E37" s="40">
+      <c r="E37" s="42">
         <f>E15-E35</f>
         <v/>
       </c>
-      <c r="F37" s="40">
+      <c r="F37" s="42">
         <f>F15-F35</f>
         <v/>
       </c>
-      <c r="G37" s="40">
+      <c r="G37" s="42">
         <f>G15-G35</f>
         <v/>
       </c>
-      <c r="H37" s="40">
+      <c r="H37" s="42">
         <f>H15-H35</f>
         <v/>
       </c>
-      <c r="I37" s="40">
+      <c r="I37" s="42">
         <f>I15-I35</f>
         <v/>
       </c>
-      <c r="J37" s="40">
+      <c r="J37" s="42">
         <f>J15-J35</f>
         <v/>
       </c>
-      <c r="K37" s="40">
+      <c r="K37" s="42">
         <f>K15-K35</f>
         <v/>
       </c>
@@ -3777,6 +3904,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -3837,787 +3965,787 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="26" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>OPERATING ACTIVITIES</t>
         </is>
       </c>
-      <c r="C4" s="18" t="n"/>
-      <c r="D4" s="18" t="n"/>
-      <c r="E4" s="18" t="n"/>
-      <c r="F4" s="18" t="n"/>
-      <c r="G4" s="18" t="n"/>
-      <c r="H4" s="18" t="n"/>
-      <c r="I4" s="18" t="n"/>
-      <c r="J4" s="18" t="n"/>
-      <c r="K4" s="18" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="29" t="n">
         <v>854800</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="29" t="n">
         <v>1550190</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="29" t="n">
         <v>1814616</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="29" t="n">
         <v>1579183</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="24">
         <f>'Income Statement'!G13</f>
         <v/>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="24">
         <f>'Income Statement'!H13</f>
         <v/>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="24">
         <f>'Income Statement'!I13</f>
         <v/>
       </c>
-      <c r="J5" s="22">
+      <c r="J5" s="24">
         <f>'Income Statement'!J13</f>
         <v/>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="24">
         <f>'Income Statement'!K13</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="29" t="n">
         <v>291791</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="29" t="n">
         <v>379384</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="29" t="n">
         <v>446524</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="29" t="n">
         <v>496228</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="24">
         <f>'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="24">
         <f>'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="24">
         <f>'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J6" s="22">
+      <c r="J6" s="24">
         <f>'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="24">
         <f>'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Stock-based compensation</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="29" t="n">
         <v>78075</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="29" t="n">
         <v>93560</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="29" t="n">
         <v>90011</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="29" t="n">
         <v>62203</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="24">
         <f>'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="24">
         <f>'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="24">
         <f>'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="24">
         <f>'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="24">
         <f>'Assumptions'!K14</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
         </is>
       </c>
-      <c r="C8" s="41" t="inlineStr">
+      <c r="C8" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="41" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="41" t="inlineStr">
+      <c r="E8" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="41" t="inlineStr">
+      <c r="F8" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="24">
         <f>-('Balance Sheet'!G7-'Balance Sheet'!F7)</f>
         <v/>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="24">
         <f>-('Balance Sheet'!H7-'Balance Sheet'!G7)</f>
         <v/>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="24">
         <f>-('Balance Sheet'!I7-'Balance Sheet'!H7)</f>
         <v/>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="24">
         <f>-('Balance Sheet'!J7-'Balance Sheet'!I7)</f>
         <v/>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="24">
         <f>-('Balance Sheet'!K7-'Balance Sheet'!J7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
         </is>
       </c>
-      <c r="C9" s="41" t="inlineStr">
+      <c r="C9" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="41" t="inlineStr">
+      <c r="D9" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="41" t="inlineStr">
+      <c r="E9" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="41" t="inlineStr">
+      <c r="F9" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="24">
         <f>-('Balance Sheet'!G8-'Balance Sheet'!F8)</f>
         <v/>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="24">
         <f>-('Balance Sheet'!H8-'Balance Sheet'!G8)</f>
         <v/>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="24">
         <f>-('Balance Sheet'!I8-'Balance Sheet'!H8)</f>
         <v/>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="24">
         <f>-('Balance Sheet'!J8-'Balance Sheet'!I8)</f>
         <v/>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="24">
         <f>-('Balance Sheet'!K8-'Balance Sheet'!J8)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="41" t="inlineStr">
+      <c r="E10" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F10" s="41" t="inlineStr">
+      <c r="F10" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="24">
         <f>-('Balance Sheet'!G12-'Balance Sheet'!F12)</f>
         <v/>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="24">
         <f>-('Balance Sheet'!H12-'Balance Sheet'!G12)</f>
         <v/>
       </c>
-      <c r="I10" s="22">
+      <c r="I10" s="24">
         <f>-('Balance Sheet'!I12-'Balance Sheet'!H12)</f>
         <v/>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="24">
         <f>-('Balance Sheet'!J12-'Balance Sheet'!I12)</f>
         <v/>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="24">
         <f>-('Balance Sheet'!K12-'Balance Sheet'!J12)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
         </is>
       </c>
-      <c r="C11" s="41" t="inlineStr">
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="41" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="41" t="inlineStr">
+      <c r="E11" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="41" t="inlineStr">
+      <c r="F11" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="24">
         <f>-('Balance Sheet'!G14-'Balance Sheet'!F14)</f>
         <v/>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="24">
         <f>-('Balance Sheet'!H14-'Balance Sheet'!G14)</f>
         <v/>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="24">
         <f>-('Balance Sheet'!I14-'Balance Sheet'!H14)</f>
         <v/>
       </c>
-      <c r="J11" s="22">
+      <c r="J11" s="24">
         <f>-('Balance Sheet'!J14-'Balance Sheet'!I14)</f>
         <v/>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="24">
         <f>-('Balance Sheet'!K14-'Balance Sheet'!J14)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
         </is>
       </c>
-      <c r="C12" s="41" t="inlineStr">
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="41" t="inlineStr">
+      <c r="E12" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="41" t="inlineStr">
+      <c r="F12" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="24">
         <f>('Balance Sheet'!G19-'Balance Sheet'!F19)</f>
         <v/>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="24">
         <f>('Balance Sheet'!H19-'Balance Sheet'!G19)</f>
         <v/>
       </c>
-      <c r="I12" s="22">
+      <c r="I12" s="24">
         <f>('Balance Sheet'!I19-'Balance Sheet'!H19)</f>
         <v/>
       </c>
-      <c r="J12" s="22">
+      <c r="J12" s="24">
         <f>('Balance Sheet'!J19-'Balance Sheet'!I19)</f>
         <v/>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="24">
         <f>('Balance Sheet'!K19-'Balance Sheet'!J19)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
         </is>
       </c>
-      <c r="C13" s="41" t="inlineStr">
+      <c r="C13" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" s="41" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="41" t="inlineStr">
+      <c r="E13" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F13" s="41" t="inlineStr">
+      <c r="F13" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="24">
         <f>('Balance Sheet'!G20-'Balance Sheet'!F20)</f>
         <v/>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="24">
         <f>('Balance Sheet'!H20-'Balance Sheet'!G20)</f>
         <v/>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="24">
         <f>('Balance Sheet'!I20-'Balance Sheet'!H20)</f>
         <v/>
       </c>
-      <c r="J13" s="22">
+      <c r="J13" s="24">
         <f>('Balance Sheet'!J20-'Balance Sheet'!I20)</f>
         <v/>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="24">
         <f>('Balance Sheet'!K20-'Balance Sheet'!J20)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
         </is>
       </c>
-      <c r="C14" s="41" t="inlineStr">
+      <c r="C14" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="41" t="inlineStr">
+      <c r="E14" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="41" t="inlineStr">
+      <c r="F14" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="24">
         <f>('Balance Sheet'!G22-'Balance Sheet'!F22)</f>
         <v/>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="24">
         <f>('Balance Sheet'!H22-'Balance Sheet'!G22)</f>
         <v/>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="24">
         <f>('Balance Sheet'!I22-'Balance Sheet'!H22)</f>
         <v/>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="24">
         <f>('Balance Sheet'!J22-'Balance Sheet'!I22)</f>
         <v/>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="24">
         <f>('Balance Sheet'!K22-'Balance Sheet'!J22)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in operating lease liab.</t>
         </is>
       </c>
-      <c r="C15" s="41" t="inlineStr">
+      <c r="C15" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="41" t="inlineStr">
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="41" t="inlineStr">
+      <c r="E15" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="41" t="inlineStr">
+      <c r="F15" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="24">
         <f>('Balance Sheet'!G21-'Balance Sheet'!F21)+('Balance Sheet'!G25-'Balance Sheet'!F25)</f>
         <v/>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="24">
         <f>('Balance Sheet'!H21-'Balance Sheet'!G21)+('Balance Sheet'!H25-'Balance Sheet'!G25)</f>
         <v/>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="24">
         <f>('Balance Sheet'!I21-'Balance Sheet'!H21)+('Balance Sheet'!I25-'Balance Sheet'!H25)</f>
         <v/>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="24">
         <f>('Balance Sheet'!J21-'Balance Sheet'!I21)+('Balance Sheet'!J25-'Balance Sheet'!I25)</f>
         <v/>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="24">
         <f>('Balance Sheet'!K21-'Balance Sheet'!J21)+('Balance Sheet'!K25-'Balance Sheet'!J25)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in deferred income taxes</t>
         </is>
       </c>
-      <c r="C16" s="41" t="inlineStr">
+      <c r="C16" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="41" t="inlineStr">
+      <c r="E16" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="41" t="inlineStr">
+      <c r="F16" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="24">
         <f>('Balance Sheet'!G26-'Balance Sheet'!F26)</f>
         <v/>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="24">
         <f>('Balance Sheet'!H26-'Balance Sheet'!G26)</f>
         <v/>
       </c>
-      <c r="I16" s="22">
+      <c r="I16" s="24">
         <f>('Balance Sheet'!I26-'Balance Sheet'!H26)</f>
         <v/>
       </c>
-      <c r="J16" s="22">
+      <c r="J16" s="24">
         <f>('Balance Sheet'!J26-'Balance Sheet'!I26)</f>
         <v/>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="24">
         <f>('Balance Sheet'!K26-'Balance Sheet'!J26)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in other non-current liab.</t>
         </is>
       </c>
-      <c r="C17" s="41" t="inlineStr">
+      <c r="C17" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="41" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="41" t="inlineStr">
+      <c r="E17" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F17" s="41" t="inlineStr">
+      <c r="F17" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="24">
         <f>('Balance Sheet'!G27-'Balance Sheet'!F27)</f>
         <v/>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="24">
         <f>('Balance Sheet'!H27-'Balance Sheet'!G27)</f>
         <v/>
       </c>
-      <c r="I17" s="22">
+      <c r="I17" s="24">
         <f>('Balance Sheet'!I27-'Balance Sheet'!H27)</f>
         <v/>
       </c>
-      <c r="J17" s="22">
+      <c r="J17" s="24">
         <f>('Balance Sheet'!J27-'Balance Sheet'!I27)</f>
         <v/>
       </c>
-      <c r="K17" s="22">
+      <c r="K17" s="24">
         <f>('Balance Sheet'!K27-'Balance Sheet'!J27)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">  Working capital &amp; other (reported, net)</t>
         </is>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="24">
         <f>C19-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="24">
         <f>D19-D5-D6-D7</f>
         <v/>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="24">
         <f>E19-E5-E6-E7</f>
         <v/>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="24">
         <f>F19-F5-F6-F7</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="C19" s="38" t="n">
+      <c r="C19" s="40" t="n">
         <v>966463</v>
       </c>
-      <c r="D19" s="38" t="n">
+      <c r="D19" s="40" t="n">
         <v>2296164</v>
       </c>
-      <c r="E19" s="38" t="n">
+      <c r="E19" s="40" t="n">
         <v>2272713</v>
       </c>
-      <c r="F19" s="38" t="n">
+      <c r="F19" s="40" t="n">
         <v>1602477</v>
       </c>
-      <c r="G19" s="29">
+      <c r="G19" s="31">
         <f>G5+G6+G7+SUM(G8:G17)</f>
         <v/>
       </c>
-      <c r="H19" s="29">
+      <c r="H19" s="31">
         <f>H5+H6+H7+SUM(H8:H17)</f>
         <v/>
       </c>
-      <c r="I19" s="29">
+      <c r="I19" s="31">
         <f>I5+I6+I7+SUM(I8:I17)</f>
         <v/>
       </c>
-      <c r="J19" s="29">
+      <c r="J19" s="31">
         <f>J5+J6+J7+SUM(J8:J17)</f>
         <v/>
       </c>
-      <c r="K19" s="29">
+      <c r="K19" s="31">
         <f>K5+K6+K7+SUM(K8:K17)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>INVESTING ACTIVITIES</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="18" t="n"/>
-      <c r="I21" s="18" t="n"/>
-      <c r="J21" s="18" t="n"/>
-      <c r="K21" s="18" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="19" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Capital expenditures</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n">
+      <c r="C22" s="29" t="n">
         <v>-638657</v>
       </c>
-      <c r="D22" s="27" t="n">
+      <c r="D22" s="29" t="n">
         <v>-651865</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="29" t="n">
         <v>-689232</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="29" t="n">
         <v>-680802</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="24">
         <f>-'Income Statement'!G4*'Assumptions'!G13</f>
         <v/>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="24">
         <f>-'Income Statement'!H4*'Assumptions'!H13</f>
         <v/>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="24">
         <f>-'Income Statement'!I4*'Assumptions'!I13</f>
         <v/>
       </c>
-      <c r="J22" s="22">
+      <c r="J22" s="24">
         <f>-'Income Statement'!J4*'Assumptions'!J13</f>
         <v/>
       </c>
-      <c r="K22" s="22">
+      <c r="K22" s="24">
         <f>-'Income Statement'!K4*'Assumptions'!K13</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>Net cash from investing activities</t>
         </is>
       </c>
-      <c r="C23" s="38" t="n">
+      <c r="C23" s="40" t="n">
         <v>-569937</v>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D23" s="40" t="n">
         <v>-654132</v>
       </c>
-      <c r="E23" s="38" t="n">
+      <c r="E23" s="40" t="n">
         <v>-798174</v>
       </c>
-      <c r="F23" s="38" t="n">
+      <c r="F23" s="40" t="n">
         <v>-662118</v>
       </c>
-      <c r="G23" s="29">
+      <c r="G23" s="31">
         <f>G22</f>
         <v/>
       </c>
-      <c r="H23" s="29">
+      <c r="H23" s="31">
         <f>H22</f>
         <v/>
       </c>
-      <c r="I23" s="29">
+      <c r="I23" s="31">
         <f>I22</f>
         <v/>
       </c>
-      <c r="J23" s="29">
+      <c r="J23" s="31">
         <f>J22</f>
         <v/>
       </c>
-      <c r="K23" s="29">
+      <c r="K23" s="31">
         <f>K22</f>
         <v/>
       </c>
@@ -4630,95 +4758,95 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>FINANCING ACTIVITIES</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
-      <c r="I26" s="18" t="n"/>
-      <c r="J26" s="18" t="n"/>
-      <c r="K26" s="18" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Repurchase of common stock</t>
         </is>
       </c>
-      <c r="C27" s="27" t="n">
+      <c r="C27" s="29" t="n">
         <v>-444001</v>
       </c>
-      <c r="D27" s="27" t="n">
+      <c r="D27" s="29" t="n">
         <v>-558652</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="29" t="n">
         <v>-1636879</v>
       </c>
-      <c r="F27" s="27" t="n">
+      <c r="F27" s="29" t="n">
         <v>-1178349</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="24">
         <f>-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="24">
         <f>-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I27" s="22">
+      <c r="I27" s="24">
         <f>-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J27" s="22">
+      <c r="J27" s="24">
         <f>-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K27" s="22">
+      <c r="K27" s="24">
         <f>-'Assumptions'!K27</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="C28" s="38" t="n">
+      <c r="C28" s="40" t="n">
         <v>-467487</v>
       </c>
-      <c r="D28" s="38" t="n">
+      <c r="D28" s="40" t="n">
         <v>-548828</v>
       </c>
-      <c r="E28" s="38" t="n">
+      <c r="E28" s="40" t="n">
         <v>-1652508</v>
       </c>
-      <c r="F28" s="38" t="n">
+      <c r="F28" s="40" t="n">
         <v>-1208656</v>
       </c>
-      <c r="G28" s="29">
+      <c r="G28" s="31">
         <f>G27</f>
         <v/>
       </c>
-      <c r="H28" s="29">
+      <c r="H28" s="31">
         <f>H27</f>
         <v/>
       </c>
-      <c r="I28" s="29">
+      <c r="I28" s="31">
         <f>I27</f>
         <v/>
       </c>
-      <c r="J28" s="29">
+      <c r="J28" s="31">
         <f>J27</f>
         <v/>
       </c>
-      <c r="K28" s="29">
+      <c r="K28" s="31">
         <f>K27</f>
         <v/>
       </c>
@@ -4731,122 +4859,122 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="30" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="C31" s="29">
+      <c r="C31" s="31">
         <f>C19+C23+C28</f>
         <v/>
       </c>
-      <c r="D31" s="29">
+      <c r="D31" s="31">
         <f>D19+D23+D28</f>
         <v/>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="31">
         <f>E19+E23+E28</f>
         <v/>
       </c>
-      <c r="F31" s="29">
+      <c r="F31" s="31">
         <f>F19+F23+F28</f>
         <v/>
       </c>
-      <c r="G31" s="29">
+      <c r="G31" s="31">
         <f>G19+G23+G28</f>
         <v/>
       </c>
-      <c r="H31" s="29">
+      <c r="H31" s="31">
         <f>H19+H23+H28</f>
         <v/>
       </c>
-      <c r="I31" s="29">
+      <c r="I31" s="31">
         <f>I19+I23+I28</f>
         <v/>
       </c>
-      <c r="J31" s="29">
+      <c r="J31" s="31">
         <f>J19+J23+J28</f>
         <v/>
       </c>
-      <c r="K31" s="29">
+      <c r="K31" s="31">
         <f>K19+K23+K28</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Cash, beginning of year</t>
         </is>
       </c>
-      <c r="C32" s="27" t="n">
+      <c r="C32" s="29" t="n">
         <v>1150517</v>
       </c>
-      <c r="D32" s="27" t="n">
+      <c r="D32" s="29" t="n">
         <v>1154867</v>
       </c>
-      <c r="E32" s="27" t="n">
+      <c r="E32" s="29" t="n">
         <v>2243971</v>
       </c>
-      <c r="F32" s="27" t="n">
+      <c r="F32" s="29" t="n">
         <v>1984336</v>
       </c>
-      <c r="G32" s="22">
+      <c r="G32" s="24">
         <f>'Balance Sheet'!F6</f>
         <v/>
       </c>
-      <c r="H32" s="22">
+      <c r="H32" s="24">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I32" s="22">
+      <c r="I32" s="24">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J32" s="22">
+      <c r="J32" s="24">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K32" s="22">
+      <c r="K32" s="24">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="inlineStr">
+      <c r="A33" s="30" t="inlineStr">
         <is>
           <t>Cash, end of year</t>
         </is>
       </c>
-      <c r="C33" s="39" t="n">
+      <c r="C33" s="41" t="n">
         <v>1154867</v>
       </c>
-      <c r="D33" s="39" t="n">
+      <c r="D33" s="41" t="n">
         <v>2243971</v>
       </c>
-      <c r="E33" s="39" t="n">
+      <c r="E33" s="41" t="n">
         <v>1984336</v>
       </c>
-      <c r="F33" s="39" t="n">
+      <c r="F33" s="41" t="n">
         <v>1807202</v>
       </c>
-      <c r="G33" s="30">
+      <c r="G33" s="32">
         <f>G32+G31</f>
         <v/>
       </c>
-      <c r="H33" s="30">
+      <c r="H33" s="32">
         <f>H32+H31</f>
         <v/>
       </c>
-      <c r="I33" s="30">
+      <c r="I33" s="32">
         <f>I32+I31</f>
         <v/>
       </c>
-      <c r="J33" s="30">
+      <c r="J33" s="32">
         <f>J32+J31</f>
         <v/>
       </c>
-      <c r="K33" s="30">
+      <c r="K33" s="32">
         <f>K32+K31</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add clickable source links for red analyst assumptions
Each red input now has a ~20-word justification plus a hyperlink to the
dataset or filing that inspired it (Damodaran ERP, FRED Treasury, Yahoo
Finance betas/multiples, LULU 10-K and earnings release, etc.). Applied
across WACC, Scenarios, DCF, Comps, and 3-statement Assumptions tabs.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -162,6 +162,19 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="8"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
@@ -241,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -288,6 +301,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -309,19 +323,19 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -331,13 +345,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -777,7 +791,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions / inputs</t>
+          <t>Red font  =  analyst assumptions / inputs (justification + clickable source link)</t>
         </is>
       </c>
     </row>
@@ -846,7 +860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -861,6 +875,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -971,6 +986,11 @@
       <c r="L3" s="17" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
+        </is>
+      </c>
+      <c r="M3" s="17" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
@@ -1025,6 +1045,11 @@
           <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
         </is>
       </c>
+      <c r="M5" s="24" t="inlineStr">
+        <is>
+          <t>LULU Q2 FY2026 guidance</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -1064,6 +1089,11 @@
           <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
         </is>
       </c>
+      <c r="M6" s="24" t="inlineStr">
+        <is>
+          <t>LULU historical gross margin (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
@@ -1103,6 +1133,11 @@
           <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
         </is>
       </c>
+      <c r="M7" s="24" t="inlineStr">
+        <is>
+          <t>LULU historical SG&amp;A (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
@@ -1110,36 +1145,41 @@
           <t>Amortization / other opex ($)</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="25" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="25" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="25" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="25" t="n">
+      <c r="G8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="H8" s="25" t="n">
+      <c r="H8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="I8" s="25" t="n">
+      <c r="I8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="J8" s="25" t="n">
+      <c r="J8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="K8" s="25" t="n">
+      <c r="K8" s="26" t="n">
         <v>7000</v>
       </c>
       <c r="L8" s="23" t="inlineStr">
         <is>
           <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
+        </is>
+      </c>
+      <c r="M8" s="24" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1149,36 +1189,41 @@
           <t>Other income, net ($)</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="25" t="n">
         <v>4163</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="25" t="n">
         <v>43059</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="25" t="n">
         <v>70380</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="25" t="n">
         <v>28352</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="26" t="n">
         <v>130000</v>
       </c>
-      <c r="H9" s="25" t="n">
+      <c r="H9" s="26" t="n">
         <v>60000</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="I9" s="26" t="n">
         <v>75000</v>
       </c>
-      <c r="J9" s="25" t="n">
+      <c r="J9" s="26" t="n">
         <v>95000</v>
       </c>
-      <c r="K9" s="25" t="n">
+      <c r="K9" s="26" t="n">
         <v>115000</v>
       </c>
       <c r="L9" s="23" t="inlineStr">
         <is>
           <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+        </is>
+      </c>
+      <c r="M9" s="24" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1218,6 +1263,11 @@
       <c r="L10" s="23" t="inlineStr">
         <is>
           <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
+        </is>
+      </c>
+      <c r="M10" s="24" t="inlineStr">
+        <is>
+          <t>LULU effective tax history (10-K)</t>
         </is>
       </c>
     </row>
@@ -1275,6 +1325,11 @@
           <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
         </is>
       </c>
+      <c r="M12" s="24" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
@@ -1314,6 +1369,11 @@
           <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
         </is>
       </c>
+      <c r="M13" s="24" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -1321,36 +1381,41 @@
           <t>Stock-based compensation ($)</t>
         </is>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="25" t="n">
         <v>78075</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="25" t="n">
         <v>93560</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="25" t="n">
         <v>90011</v>
       </c>
-      <c r="F14" s="24" t="n">
+      <c r="F14" s="25" t="n">
         <v>62203</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="H14" s="25" t="n">
+      <c r="H14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="I14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="J14" s="25" t="n">
+      <c r="J14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="K14" s="25" t="n">
+      <c r="K14" s="26" t="n">
         <v>70000</v>
       </c>
       <c r="L14" s="23" t="inlineStr">
         <is>
           <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+        </is>
+      </c>
+      <c r="M14" s="24" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1408,6 +1473,11 @@
           <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
         </is>
       </c>
+      <c r="M16" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
@@ -1447,6 +1517,11 @@
           <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
         </is>
       </c>
+      <c r="M17" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
@@ -1486,6 +1561,11 @@
           <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
         </is>
       </c>
+      <c r="M18" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
@@ -1525,6 +1605,11 @@
           <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
         </is>
       </c>
+      <c r="M19" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
@@ -1564,6 +1649,11 @@
           <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
         </is>
       </c>
+      <c r="M20" s="24" t="inlineStr">
+        <is>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
@@ -1603,6 +1693,11 @@
           <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
         </is>
       </c>
+      <c r="M21" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
@@ -1642,6 +1737,11 @@
           <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
         </is>
       </c>
+      <c r="M22" s="24" t="inlineStr">
+        <is>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
@@ -1681,6 +1781,11 @@
           <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
         </is>
       </c>
+      <c r="M23" s="24" t="inlineStr">
+        <is>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
@@ -1720,6 +1825,11 @@
           <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
         </is>
       </c>
+      <c r="M24" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
@@ -1757,6 +1867,11 @@
       <c r="L25" s="23" t="inlineStr">
         <is>
           <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
+        </is>
+      </c>
+      <c r="M25" s="24" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1782,36 +1897,41 @@
           <t>Share repurchases ($)</t>
         </is>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C27" s="25" t="n">
         <v>444001</v>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="25" t="n">
         <v>558652</v>
       </c>
-      <c r="E27" s="24" t="n">
+      <c r="E27" s="25" t="n">
         <v>1636879</v>
       </c>
-      <c r="F27" s="24" t="n">
+      <c r="F27" s="25" t="n">
         <v>1178349</v>
       </c>
-      <c r="G27" s="25" t="n">
+      <c r="G27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="H27" s="25" t="n">
+      <c r="H27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="I27" s="25" t="n">
+      <c r="I27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="J27" s="25" t="n">
+      <c r="J27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="K27" s="25" t="n">
+      <c r="K27" s="26" t="n">
         <v>500000</v>
       </c>
       <c r="L27" s="23" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+        </is>
+      </c>
+      <c r="M27" s="24" t="inlineStr">
+        <is>
+          <t>LULU CF: share repurchases (10-K)</t>
         </is>
       </c>
     </row>
@@ -1821,24 +1941,29 @@
           <t>Avg repurchase price ($/sh)</t>
         </is>
       </c>
-      <c r="G28" s="26" t="n">
+      <c r="G28" s="27" t="n">
         <v>105</v>
       </c>
-      <c r="H28" s="26" t="n">
+      <c r="H28" s="27" t="n">
         <v>112</v>
       </c>
-      <c r="I28" s="26" t="n">
+      <c r="I28" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="J28" s="26" t="n">
+      <c r="J28" s="27" t="n">
         <v>128</v>
       </c>
-      <c r="K28" s="26" t="n">
+      <c r="K28" s="27" t="n">
         <v>135</v>
       </c>
       <c r="L28" s="23" t="inlineStr">
         <is>
           <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+        </is>
+      </c>
+      <c r="M28" s="24" t="inlineStr">
+        <is>
+          <t>LULU avg repurchase price (10-K/est.)</t>
         </is>
       </c>
     </row>
@@ -1855,6 +1980,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1881,6 +2027,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1941,27 +2088,27 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="27" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="27" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="G2" s="29" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -1973,35 +2120,35 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C4" s="29" t="n">
+      <c r="C4" s="30" t="n">
         <v>8110518</v>
       </c>
-      <c r="D4" s="29" t="n">
+      <c r="D4" s="30" t="n">
         <v>9619278</v>
       </c>
-      <c r="E4" s="29" t="n">
+      <c r="E4" s="30" t="n">
         <v>10588126</v>
       </c>
-      <c r="F4" s="29" t="n">
+      <c r="F4" s="30" t="n">
         <v>11102600</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="25">
         <f>F4*(1+'Assumptions'!G5)</f>
         <v/>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="25">
         <f>G4*(1+'Assumptions'!H5)</f>
         <v/>
       </c>
-      <c r="I4" s="24">
+      <c r="I4" s="25">
         <f>H4*(1+'Assumptions'!I5)</f>
         <v/>
       </c>
-      <c r="J4" s="24">
+      <c r="J4" s="25">
         <f>I4*(1+'Assumptions'!J5)</f>
         <v/>
       </c>
-      <c r="K4" s="24">
+      <c r="K4" s="25">
         <f>J4*(1+'Assumptions'!K5)</f>
         <v/>
       </c>
@@ -2012,78 +2159,78 @@
           <t>Cost of goods sold</t>
         </is>
       </c>
-      <c r="C5" s="29" t="n">
+      <c r="C5" s="30" t="n">
         <v>3618178</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="30" t="n">
         <v>4009873</v>
       </c>
-      <c r="E5" s="29" t="n">
+      <c r="E5" s="30" t="n">
         <v>4317315</v>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="30" t="n">
         <v>4818468</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="25">
         <f>G4*(1-'Assumptions'!G6)</f>
         <v/>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="25">
         <f>H4*(1-'Assumptions'!H6)</f>
         <v/>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="25">
         <f>I4*(1-'Assumptions'!I6)</f>
         <v/>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="25">
         <f>J4*(1-'Assumptions'!J6)</f>
         <v/>
       </c>
-      <c r="K5" s="24">
+      <c r="K5" s="25">
         <f>K4*(1-'Assumptions'!K6)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="32">
         <f>C4-C5</f>
         <v/>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="32">
         <f>D4-D5</f>
         <v/>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="32">
         <f>E4-E5</f>
         <v/>
       </c>
-      <c r="F6" s="31">
+      <c r="F6" s="32">
         <f>F4-F5</f>
         <v/>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>G4-G5</f>
         <v/>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f>H4-H5</f>
         <v/>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="32">
         <f>I4-I5</f>
         <v/>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>J4-J5</f>
         <v/>
       </c>
-      <c r="K6" s="31">
+      <c r="K6" s="32">
         <f>K4-K5</f>
         <v/>
       </c>
@@ -2094,35 +2241,35 @@
           <t>Selling, general &amp; administrative</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="30" t="n">
         <v>2757447</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <v>3397218</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="30" t="n">
         <v>3762379</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <v>4066556</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>G4*'Assumptions'!G7</f>
         <v/>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>H4*'Assumptions'!H7</f>
         <v/>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>I4*'Assumptions'!I7</f>
         <v/>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="25">
         <f>J4*'Assumptions'!J7</f>
         <v/>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="25">
         <f>K4*'Assumptions'!K7</f>
         <v/>
       </c>
@@ -2133,78 +2280,78 @@
           <t>Amortization of intangibles / other</t>
         </is>
       </c>
-      <c r="C8" s="29" t="n">
+      <c r="C8" s="30" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="30" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="29" t="n">
+      <c r="F8" s="30" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="25">
         <f>'Assumptions'!G8</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="25">
         <f>'Assumptions'!H8</f>
         <v/>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>'Assumptions'!I8</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="25">
         <f>'Assumptions'!J8</f>
         <v/>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="25">
         <f>'Assumptions'!K8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Operating income (EBIT)</t>
         </is>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="32">
         <f>C6-C7-C8</f>
         <v/>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="32">
         <f>D6-D7-D8</f>
         <v/>
       </c>
-      <c r="E9" s="31">
+      <c r="E9" s="32">
         <f>E6-E7-E8</f>
         <v/>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="32">
         <f>F6-F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="32">
         <f>G6-G7-G8</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>H6-H7-H8</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="32">
         <f>I6-I7-I8</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>J6-J7-J8</f>
         <v/>
       </c>
-      <c r="K9" s="31">
+      <c r="K9" s="32">
         <f>K6-K7-K8</f>
         <v/>
       </c>
@@ -2215,78 +2362,78 @@
           <t>Other income, net</t>
         </is>
       </c>
-      <c r="C10" s="29" t="n">
+      <c r="C10" s="30" t="n">
         <v>4163</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="30" t="n">
         <v>43059</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="30" t="n">
         <v>70380</v>
       </c>
-      <c r="F10" s="29" t="n">
+      <c r="F10" s="30" t="n">
         <v>28352</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="25">
         <f>'Assumptions'!G9</f>
         <v/>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="25">
         <f>'Assumptions'!H9</f>
         <v/>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="25">
         <f>'Assumptions'!I9</f>
         <v/>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="25">
         <f>'Assumptions'!J9</f>
         <v/>
       </c>
-      <c r="K10" s="24">
+      <c r="K10" s="25">
         <f>'Assumptions'!K9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Pre-tax income</t>
         </is>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="32">
         <f>C9+C10</f>
         <v/>
       </c>
-      <c r="D11" s="31">
+      <c r="D11" s="32">
         <f>D9+D10</f>
         <v/>
       </c>
-      <c r="E11" s="31">
+      <c r="E11" s="32">
         <f>E9+E10</f>
         <v/>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="32">
         <f>F9+F10</f>
         <v/>
       </c>
-      <c r="G11" s="31">
+      <c r="G11" s="32">
         <f>G9+G10</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="32">
         <f>H9+H10</f>
         <v/>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="32">
         <f>I9+I10</f>
         <v/>
       </c>
-      <c r="J11" s="31">
+      <c r="J11" s="32">
         <f>J9+J10</f>
         <v/>
       </c>
-      <c r="K11" s="31">
+      <c r="K11" s="32">
         <f>K9+K10</f>
         <v/>
       </c>
@@ -2297,78 +2444,78 @@
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="C12" s="29" t="n">
+      <c r="C12" s="30" t="n">
         <v>477771</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="30" t="n">
         <v>625545</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="30" t="n">
         <v>761461</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="30" t="n">
         <v>659784</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="25">
         <f>G11*'Assumptions'!G10</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>H11*'Assumptions'!H10</f>
         <v/>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="25">
         <f>I11*'Assumptions'!I10</f>
         <v/>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="25">
         <f>J11*'Assumptions'!J10</f>
         <v/>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="25">
         <f>K11*'Assumptions'!K10</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>D11-D12</f>
         <v/>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="33">
         <f>E11-E12</f>
         <v/>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>F11-F12</f>
         <v/>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="33">
         <f>G11-G12</f>
         <v/>
       </c>
-      <c r="H13" s="32">
+      <c r="H13" s="33">
         <f>H11-H12</f>
         <v/>
       </c>
-      <c r="I13" s="32">
+      <c r="I13" s="33">
         <f>I11-I12</f>
         <v/>
       </c>
-      <c r="J13" s="32">
+      <c r="J13" s="33">
         <f>J11-J12</f>
         <v/>
       </c>
-      <c r="K13" s="32">
+      <c r="K13" s="33">
         <f>K11-K12</f>
         <v/>
       </c>
@@ -2379,80 +2526,80 @@
           <t>Diluted weighted-avg shares (000)</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n">
+      <c r="C15" s="30" t="n">
         <v>128017</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="30" t="n">
         <v>127060</v>
       </c>
-      <c r="E15" s="29" t="n">
+      <c r="E15" s="30" t="n">
         <v>123935</v>
       </c>
-      <c r="F15" s="29" t="n">
+      <c r="F15" s="30" t="n">
         <v>119068</v>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="25">
         <f>F15-'Assumptions'!G27/'Assumptions'!G28</f>
         <v/>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="25">
         <f>G15-'Assumptions'!H27/'Assumptions'!H28</f>
         <v/>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="25">
         <f>H15-'Assumptions'!I27/'Assumptions'!I28</f>
         <v/>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="25">
         <f>I15-'Assumptions'!J27/'Assumptions'!J28</f>
         <v/>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="25">
         <f>J15-'Assumptions'!K27/'Assumptions'!K28</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Diluted EPS ($)</t>
         </is>
       </c>
-      <c r="C16" s="33" t="n">
+      <c r="C16" s="34" t="n">
         <v>6.68</v>
       </c>
-      <c r="D16" s="33" t="n">
+      <c r="D16" s="34" t="n">
         <v>12.2</v>
       </c>
-      <c r="E16" s="33" t="n">
+      <c r="E16" s="34" t="n">
         <v>14.64</v>
       </c>
-      <c r="F16" s="33" t="n">
+      <c r="F16" s="34" t="n">
         <v>13.26</v>
       </c>
-      <c r="G16" s="34">
+      <c r="G16" s="35">
         <f>G13/G15</f>
         <v/>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="35">
         <f>H13/H15</f>
         <v/>
       </c>
-      <c r="I16" s="34">
+      <c r="I16" s="35">
         <f>I13/I15</f>
         <v/>
       </c>
-      <c r="J16" s="34">
+      <c r="J16" s="35">
         <f>J13/J15</f>
         <v/>
       </c>
-      <c r="K16" s="34">
+      <c r="K16" s="35">
         <f>K13/K15</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="35" t="inlineStr">
+      <c r="A18" s="36" t="inlineStr">
         <is>
           <t>Margins &amp; growth</t>
         </is>
@@ -2468,174 +2615,174 @@
       <c r="K18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="C19" s="37">
+      <c r="C19" s="38">
         <f>C6/C4</f>
         <v/>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="38">
         <f>D6/D4</f>
         <v/>
       </c>
-      <c r="E19" s="37">
+      <c r="E19" s="38">
         <f>E6/E4</f>
         <v/>
       </c>
-      <c r="F19" s="37">
+      <c r="F19" s="38">
         <f>F6/F4</f>
         <v/>
       </c>
-      <c r="G19" s="37">
+      <c r="G19" s="38">
         <f>G6/G4</f>
         <v/>
       </c>
-      <c r="H19" s="37">
+      <c r="H19" s="38">
         <f>H6/H4</f>
         <v/>
       </c>
-      <c r="I19" s="37">
+      <c r="I19" s="38">
         <f>I6/I4</f>
         <v/>
       </c>
-      <c r="J19" s="37">
+      <c r="J19" s="38">
         <f>J6/J4</f>
         <v/>
       </c>
-      <c r="K19" s="37">
+      <c r="K19" s="38">
         <f>K6/K4</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>Operating margin %</t>
         </is>
       </c>
-      <c r="C20" s="37">
+      <c r="C20" s="38">
         <f>C9/C4</f>
         <v/>
       </c>
-      <c r="D20" s="37">
+      <c r="D20" s="38">
         <f>D9/D4</f>
         <v/>
       </c>
-      <c r="E20" s="37">
+      <c r="E20" s="38">
         <f>E9/E4</f>
         <v/>
       </c>
-      <c r="F20" s="37">
+      <c r="F20" s="38">
         <f>F9/F4</f>
         <v/>
       </c>
-      <c r="G20" s="37">
+      <c r="G20" s="38">
         <f>G9/G4</f>
         <v/>
       </c>
-      <c r="H20" s="37">
+      <c r="H20" s="38">
         <f>H9/H4</f>
         <v/>
       </c>
-      <c r="I20" s="37">
+      <c r="I20" s="38">
         <f>I9/I4</f>
         <v/>
       </c>
-      <c r="J20" s="37">
+      <c r="J20" s="38">
         <f>J9/J4</f>
         <v/>
       </c>
-      <c r="K20" s="37">
+      <c r="K20" s="38">
         <f>K9/K4</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="36" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>Net margin %</t>
         </is>
       </c>
-      <c r="C21" s="37">
+      <c r="C21" s="38">
         <f>C13/C4</f>
         <v/>
       </c>
-      <c r="D21" s="37">
+      <c r="D21" s="38">
         <f>D13/D4</f>
         <v/>
       </c>
-      <c r="E21" s="37">
+      <c r="E21" s="38">
         <f>E13/E4</f>
         <v/>
       </c>
-      <c r="F21" s="37">
+      <c r="F21" s="38">
         <f>F13/F4</f>
         <v/>
       </c>
-      <c r="G21" s="37">
+      <c r="G21" s="38">
         <f>G13/G4</f>
         <v/>
       </c>
-      <c r="H21" s="37">
+      <c r="H21" s="38">
         <f>H13/H4</f>
         <v/>
       </c>
-      <c r="I21" s="37">
+      <c r="I21" s="38">
         <f>I13/I4</f>
         <v/>
       </c>
-      <c r="J21" s="37">
+      <c r="J21" s="38">
         <f>J13/J4</f>
         <v/>
       </c>
-      <c r="K21" s="37">
+      <c r="K21" s="38">
         <f>K13/K4</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="36" t="inlineStr">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="C22" s="38" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="38">
         <f>D4/C4-1</f>
         <v/>
       </c>
-      <c r="E22" s="37">
+      <c r="E22" s="38">
         <f>E4/D4-1</f>
         <v/>
       </c>
-      <c r="F22" s="37">
+      <c r="F22" s="38">
         <f>F4/E4-1</f>
         <v/>
       </c>
-      <c r="G22" s="37">
+      <c r="G22" s="38">
         <f>G4/F4-1</f>
         <v/>
       </c>
-      <c r="H22" s="37">
+      <c r="H22" s="38">
         <f>H4/G4-1</f>
         <v/>
       </c>
-      <c r="I22" s="37">
+      <c r="I22" s="38">
         <f>I4/H4-1</f>
         <v/>
       </c>
-      <c r="J22" s="37">
+      <c r="J22" s="38">
         <f>J4/I4-1</f>
         <v/>
       </c>
-      <c r="K22" s="37">
+      <c r="K22" s="38">
         <f>K4/J4-1</f>
         <v/>
       </c>
@@ -2704,6 +2851,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2764,27 +2912,27 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="27" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="27" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="G2" s="29" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -2807,7 +2955,7 @@
       <c r="K4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>Current assets:</t>
         </is>
@@ -2819,35 +2967,35 @@
           <t>Cash &amp; cash equivalents</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="30" t="n">
         <v>1154867</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="30" t="n">
         <v>2243971</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="30" t="n">
         <v>1984336</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="30" t="n">
         <v>1807202</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="25">
         <f>'Cash Flow'!G33</f>
         <v/>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="25">
         <f>'Cash Flow'!H33</f>
         <v/>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="25">
         <f>'Cash Flow'!I33</f>
         <v/>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="25">
         <f>'Cash Flow'!J33</f>
         <v/>
       </c>
-      <c r="K6" s="24">
+      <c r="K6" s="25">
         <f>'Cash Flow'!K33</f>
         <v/>
       </c>
@@ -2858,35 +3006,35 @@
           <t>Inventories</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="30" t="n">
         <v>1447367</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <v>1323602</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="30" t="n">
         <v>1442081</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <v>1700753</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>'Income Statement'!G5*'Assumptions'!G16</f>
         <v/>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>'Income Statement'!H5*'Assumptions'!H16</f>
         <v/>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>'Income Statement'!I5*'Assumptions'!I16</f>
         <v/>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="25">
         <f>'Income Statement'!J5*'Assumptions'!J16</f>
         <v/>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="25">
         <f>'Income Statement'!K5*'Assumptions'!K16</f>
         <v/>
       </c>
@@ -2897,80 +3045,80 @@
           <t>Other current assets</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="25" t="n">
         <v>557219</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="25" t="n">
         <v>493004</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <v>553885</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="25" t="n">
         <v>754746</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G19</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H19</f>
         <v/>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I19</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J19</f>
         <v/>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K19</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="C9" s="40" t="n">
+      <c r="C9" s="41" t="n">
         <v>3159453</v>
       </c>
-      <c r="D9" s="40" t="n">
+      <c r="D9" s="41" t="n">
         <v>4060577</v>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="E9" s="41" t="n">
         <v>3980302</v>
       </c>
-      <c r="F9" s="40" t="n">
+      <c r="F9" s="41" t="n">
         <v>4262701</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="32">
         <f>G6+G7+G8</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>H6+H7+H8</f>
         <v/>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="32">
         <f>I6+I7+I8</f>
         <v/>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>J6+J7+J8</f>
         <v/>
       </c>
-      <c r="K9" s="31">
+      <c r="K9" s="32">
         <f>K6+K7+K8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="39" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>Non-current assets:</t>
         </is>
@@ -2982,35 +3130,35 @@
           <t>Property &amp; equipment, net</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n">
+      <c r="C11" s="30" t="n">
         <v>1269614</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="30" t="n">
         <v>1545811</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="30" t="n">
         <v>1780617</v>
       </c>
-      <c r="F11" s="29" t="n">
+      <c r="F11" s="30" t="n">
         <v>2033720</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="25">
         <f>F11+'Income Statement'!G4*'Assumptions'!G13-'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="25">
         <f>G11+'Income Statement'!H4*'Assumptions'!H13-'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="25">
         <f>H11+'Income Statement'!I4*'Assumptions'!I13-'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="25">
         <f>I11+'Income Statement'!J4*'Assumptions'!J13-'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K11" s="24">
+      <c r="K11" s="25">
         <f>J11+'Income Statement'!K4*'Assumptions'!K13-'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
@@ -3021,35 +3169,35 @@
           <t>Operating lease right-of-use assets</t>
         </is>
       </c>
-      <c r="C12" s="29" t="n">
+      <c r="C12" s="30" t="n">
         <v>969419</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="30" t="n">
         <v>1265610</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="30" t="n">
         <v>1416256</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="30" t="n">
         <v>1630181</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G20</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H20</f>
         <v/>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I20</f>
         <v/>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J20</f>
         <v/>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K20</f>
         <v/>
       </c>
@@ -3060,35 +3208,35 @@
           <t>Goodwill &amp; intangible assets</t>
         </is>
       </c>
-      <c r="C13" s="29" t="n">
+      <c r="C13" s="30" t="n">
         <v>46105</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="30" t="n">
         <v>24083</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="30" t="n">
         <v>171191</v>
       </c>
-      <c r="F13" s="29" t="n">
+      <c r="F13" s="30" t="n">
         <v>191194</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="25">
         <f>F13</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="25">
         <f>G13</f>
         <v/>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="25">
         <f>H13</f>
         <v/>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="25">
         <f>I13</f>
         <v/>
       </c>
-      <c r="K13" s="24">
+      <c r="K13" s="25">
         <f>J13</f>
         <v/>
       </c>
@@ -3099,74 +3247,74 @@
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="25" t="n">
         <v>162447</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="25" t="n">
         <v>195860</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="25" t="n">
         <v>254926</v>
       </c>
-      <c r="F14" s="24" t="n">
+      <c r="F14" s="25" t="n">
         <v>338947</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G21</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H21</f>
         <v/>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I21</f>
         <v/>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J21</f>
         <v/>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K21</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="C15" s="41" t="n">
+      <c r="C15" s="42" t="n">
         <v>5607038</v>
       </c>
-      <c r="D15" s="41" t="n">
+      <c r="D15" s="42" t="n">
         <v>7091941</v>
       </c>
-      <c r="E15" s="41" t="n">
+      <c r="E15" s="42" t="n">
         <v>7603292</v>
       </c>
-      <c r="F15" s="41" t="n">
+      <c r="F15" s="42" t="n">
         <v>8456743</v>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="33">
         <f>G9+G11+G12+G13+G14</f>
         <v/>
       </c>
-      <c r="H15" s="32">
+      <c r="H15" s="33">
         <f>H9+H11+H12+H13+H14</f>
         <v/>
       </c>
-      <c r="I15" s="32">
+      <c r="I15" s="33">
         <f>I9+I11+I12+I13+I14</f>
         <v/>
       </c>
-      <c r="J15" s="32">
+      <c r="J15" s="33">
         <f>J9+J11+J12+J13+J14</f>
         <v/>
       </c>
-      <c r="K15" s="32">
+      <c r="K15" s="33">
         <f>K9+K11+K12+K13+K14</f>
         <v/>
       </c>
@@ -3188,7 +3336,7 @@
       <c r="K17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="39" t="inlineStr">
+      <c r="A18" s="40" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
@@ -3200,35 +3348,35 @@
           <t>Accounts payable</t>
         </is>
       </c>
-      <c r="C19" s="29" t="n">
+      <c r="C19" s="30" t="n">
         <v>172732</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="30" t="n">
         <v>348441</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="30" t="n">
         <v>271406</v>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="30" t="n">
         <v>331421</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="25">
         <f>'Income Statement'!G5*'Assumptions'!G17</f>
         <v/>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="25">
         <f>'Income Statement'!H5*'Assumptions'!H17</f>
         <v/>
       </c>
-      <c r="I19" s="24">
+      <c r="I19" s="25">
         <f>'Income Statement'!I5*'Assumptions'!I17</f>
         <v/>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="25">
         <f>'Income Statement'!J5*'Assumptions'!J17</f>
         <v/>
       </c>
-      <c r="K19" s="24">
+      <c r="K19" s="25">
         <f>'Income Statement'!K5*'Assumptions'!K17</f>
         <v/>
       </c>
@@ -3239,35 +3387,35 @@
           <t>Accrued liabilities</t>
         </is>
       </c>
-      <c r="C20" s="29" t="n">
+      <c r="C20" s="30" t="n">
         <v>399223</v>
       </c>
-      <c r="D20" s="29" t="n">
+      <c r="D20" s="30" t="n">
         <v>348555</v>
       </c>
-      <c r="E20" s="29" t="n">
+      <c r="E20" s="30" t="n">
         <v>559463</v>
       </c>
-      <c r="F20" s="29" t="n">
+      <c r="F20" s="30" t="n">
         <v>662982</v>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G18</f>
         <v/>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H18</f>
         <v/>
       </c>
-      <c r="I20" s="24">
+      <c r="I20" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I18</f>
         <v/>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J18</f>
         <v/>
       </c>
-      <c r="K20" s="24">
+      <c r="K20" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K18</f>
         <v/>
       </c>
@@ -3278,35 +3426,35 @@
           <t>Operating lease liabilities (current)</t>
         </is>
       </c>
-      <c r="C21" s="29" t="n">
+      <c r="C21" s="30" t="n">
         <v>207972</v>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="30" t="n">
         <v>249270</v>
       </c>
-      <c r="E21" s="29" t="n">
+      <c r="E21" s="30" t="n">
         <v>275154</v>
       </c>
-      <c r="F21" s="29" t="n">
+      <c r="F21" s="30" t="n">
         <v>298724</v>
       </c>
-      <c r="G21" s="24">
+      <c r="G21" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G22</f>
         <v/>
       </c>
-      <c r="H21" s="24">
+      <c r="H21" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H22</f>
         <v/>
       </c>
-      <c r="I21" s="24">
+      <c r="I21" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I22</f>
         <v/>
       </c>
-      <c r="J21" s="24">
+      <c r="J21" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J22</f>
         <v/>
       </c>
-      <c r="K21" s="24">
+      <c r="K21" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K22</f>
         <v/>
       </c>
@@ -3317,80 +3465,80 @@
           <t>Other current liabilities</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n">
+      <c r="C22" s="25" t="n">
         <v>712271</v>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="25" t="n">
         <v>684995</v>
       </c>
-      <c r="E22" s="24" t="n">
+      <c r="E22" s="25" t="n">
         <v>733607</v>
       </c>
-      <c r="F22" s="24" t="n">
+      <c r="F22" s="25" t="n">
         <v>594421</v>
       </c>
-      <c r="G22" s="24">
+      <c r="G22" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G24</f>
         <v/>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H24</f>
         <v/>
       </c>
-      <c r="I22" s="24">
+      <c r="I22" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I24</f>
         <v/>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J24</f>
         <v/>
       </c>
-      <c r="K22" s="24">
+      <c r="K22" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K24</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Total current liabilities</t>
         </is>
       </c>
-      <c r="C23" s="40" t="n">
+      <c r="C23" s="41" t="n">
         <v>1492198</v>
       </c>
-      <c r="D23" s="40" t="n">
+      <c r="D23" s="41" t="n">
         <v>1631261</v>
       </c>
-      <c r="E23" s="40" t="n">
+      <c r="E23" s="41" t="n">
         <v>1839630</v>
       </c>
-      <c r="F23" s="40" t="n">
+      <c r="F23" s="41" t="n">
         <v>1887548</v>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="32">
         <f>G19+G20+G21+G22</f>
         <v/>
       </c>
-      <c r="H23" s="31">
+      <c r="H23" s="32">
         <f>H19+H20+H21+H22</f>
         <v/>
       </c>
-      <c r="I23" s="31">
+      <c r="I23" s="32">
         <f>I19+I20+I21+I22</f>
         <v/>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="32">
         <f>J19+J20+J21+J22</f>
         <v/>
       </c>
-      <c r="K23" s="31">
+      <c r="K23" s="32">
         <f>K19+K20+K21+K22</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="39" t="inlineStr">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>Non-current liabilities:</t>
         </is>
@@ -3402,35 +3550,35 @@
           <t>Operating lease liabilities (non-current)</t>
         </is>
       </c>
-      <c r="C25" s="29" t="n">
+      <c r="C25" s="30" t="n">
         <v>862362</v>
       </c>
-      <c r="D25" s="29" t="n">
+      <c r="D25" s="30" t="n">
         <v>1154012</v>
       </c>
-      <c r="E25" s="29" t="n">
+      <c r="E25" s="30" t="n">
         <v>1300637</v>
       </c>
-      <c r="F25" s="29" t="n">
+      <c r="F25" s="30" t="n">
         <v>1499717</v>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G23</f>
         <v/>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H23</f>
         <v/>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I23</f>
         <v/>
       </c>
-      <c r="J25" s="24">
+      <c r="J25" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J23</f>
         <v/>
       </c>
-      <c r="K25" s="24">
+      <c r="K25" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K23</f>
         <v/>
       </c>
@@ -3441,35 +3589,35 @@
           <t>Deferred income taxes</t>
         </is>
       </c>
-      <c r="C26" s="29" t="n">
+      <c r="C26" s="30" t="n">
         <v>55084</v>
       </c>
-      <c r="D26" s="29" t="n">
+      <c r="D26" s="30" t="n">
         <v>29522</v>
       </c>
-      <c r="E26" s="29" t="n">
+      <c r="E26" s="30" t="n">
         <v>98188</v>
       </c>
-      <c r="F26" s="29" t="n">
+      <c r="F26" s="30" t="n">
         <v>52278</v>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="25">
         <f>F26</f>
         <v/>
       </c>
-      <c r="H26" s="24">
+      <c r="H26" s="25">
         <f>G26</f>
         <v/>
       </c>
-      <c r="I26" s="24">
+      <c r="I26" s="25">
         <f>H26</f>
         <v/>
       </c>
-      <c r="J26" s="24">
+      <c r="J26" s="25">
         <f>I26</f>
         <v/>
       </c>
-      <c r="K26" s="24">
+      <c r="K26" s="25">
         <f>J26</f>
         <v/>
       </c>
@@ -3480,80 +3628,80 @@
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C27" s="25" t="n">
         <v>48595</v>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="25" t="n">
         <v>45065</v>
       </c>
-      <c r="E27" s="24" t="n">
+      <c r="E27" s="25" t="n">
         <v>40790</v>
       </c>
-      <c r="F27" s="24" t="n">
+      <c r="F27" s="25" t="n">
         <v>55360</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G25</f>
         <v/>
       </c>
-      <c r="H27" s="24">
+      <c r="H27" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H25</f>
         <v/>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I25</f>
         <v/>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J25</f>
         <v/>
       </c>
-      <c r="K27" s="24">
+      <c r="K27" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="C28" s="40" t="n">
+      <c r="C28" s="41" t="n">
         <v>2458239</v>
       </c>
-      <c r="D28" s="40" t="n">
+      <c r="D28" s="41" t="n">
         <v>2859860</v>
       </c>
-      <c r="E28" s="40" t="n">
+      <c r="E28" s="41" t="n">
         <v>3279245</v>
       </c>
-      <c r="F28" s="40" t="n">
+      <c r="F28" s="41" t="n">
         <v>3494903</v>
       </c>
-      <c r="G28" s="31">
+      <c r="G28" s="32">
         <f>G23+G25+G26+G27</f>
         <v/>
       </c>
-      <c r="H28" s="31">
+      <c r="H28" s="32">
         <f>H23+H25+H26+H27</f>
         <v/>
       </c>
-      <c r="I28" s="31">
+      <c r="I28" s="32">
         <f>I23+I25+I26+I27</f>
         <v/>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="32">
         <f>J23+J25+J26+J27</f>
         <v/>
       </c>
-      <c r="K28" s="31">
+      <c r="K28" s="32">
         <f>K23+K25+K26+K27</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="40" t="inlineStr">
         <is>
           <t>Shareholders' equity:</t>
         </is>
@@ -3565,35 +3713,35 @@
           <t>Common stock &amp; additional paid-in capital</t>
         </is>
       </c>
-      <c r="C31" s="29" t="n">
+      <c r="C31" s="30" t="n">
         <v>475256</v>
       </c>
-      <c r="D31" s="29" t="n">
+      <c r="D31" s="30" t="n">
         <v>575975</v>
       </c>
-      <c r="E31" s="29" t="n">
+      <c r="E31" s="30" t="n">
         <v>638771</v>
       </c>
-      <c r="F31" s="29" t="n">
+      <c r="F31" s="30" t="n">
         <v>669949</v>
       </c>
-      <c r="G31" s="24">
+      <c r="G31" s="25">
         <f>F31+'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H31" s="24">
+      <c r="H31" s="25">
         <f>G31+'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I31" s="24">
+      <c r="I31" s="25">
         <f>H31+'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J31" s="24">
+      <c r="J31" s="25">
         <f>I31+'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K31" s="24">
+      <c r="K31" s="25">
         <f>J31+'Assumptions'!K14</f>
         <v/>
       </c>
@@ -3604,35 +3752,35 @@
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="C32" s="29" t="n">
+      <c r="C32" s="30" t="n">
         <v>2926127</v>
       </c>
-      <c r="D32" s="29" t="n">
+      <c r="D32" s="30" t="n">
         <v>3920362</v>
       </c>
-      <c r="E32" s="29" t="n">
+      <c r="E32" s="30" t="n">
         <v>4109717</v>
       </c>
-      <c r="F32" s="29" t="n">
+      <c r="F32" s="30" t="n">
         <v>4522581</v>
       </c>
-      <c r="G32" s="24">
+      <c r="G32" s="25">
         <f>F32+'Income Statement'!G13-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H32" s="24">
+      <c r="H32" s="25">
         <f>G32+'Income Statement'!H13-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I32" s="24">
+      <c r="I32" s="25">
         <f>H32+'Income Statement'!I13-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J32" s="24">
+      <c r="J32" s="25">
         <f>I32+'Income Statement'!J13-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K32" s="24">
+      <c r="K32" s="25">
         <f>J32+'Income Statement'!K13-'Assumptions'!K27</f>
         <v/>
       </c>
@@ -3643,160 +3791,160 @@
           <t>Accumulated other comprehensive loss</t>
         </is>
       </c>
-      <c r="C33" s="29" t="n">
+      <c r="C33" s="30" t="n">
         <v>-252584</v>
       </c>
-      <c r="D33" s="29" t="n">
+      <c r="D33" s="30" t="n">
         <v>-264256</v>
       </c>
-      <c r="E33" s="29" t="n">
+      <c r="E33" s="30" t="n">
         <v>-424441</v>
       </c>
-      <c r="F33" s="29" t="n">
+      <c r="F33" s="30" t="n">
         <v>-230690</v>
       </c>
-      <c r="G33" s="24">
+      <c r="G33" s="25">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="24">
+      <c r="H33" s="25">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I33" s="24">
+      <c r="I33" s="25">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J33" s="24">
+      <c r="J33" s="25">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K33" s="24">
+      <c r="K33" s="25">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="30" t="inlineStr">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t>TOTAL SHAREHOLDERS' EQUITY</t>
         </is>
       </c>
-      <c r="C34" s="40" t="n">
+      <c r="C34" s="41" t="n">
         <v>3148799</v>
       </c>
-      <c r="D34" s="40" t="n">
+      <c r="D34" s="41" t="n">
         <v>4232081</v>
       </c>
-      <c r="E34" s="40" t="n">
+      <c r="E34" s="41" t="n">
         <v>4324047</v>
       </c>
-      <c r="F34" s="40" t="n">
+      <c r="F34" s="41" t="n">
         <v>4961840</v>
       </c>
-      <c r="G34" s="31">
+      <c r="G34" s="32">
         <f>G31+G32+G33</f>
         <v/>
       </c>
-      <c r="H34" s="31">
+      <c r="H34" s="32">
         <f>H31+H32+H33</f>
         <v/>
       </c>
-      <c r="I34" s="31">
+      <c r="I34" s="32">
         <f>I31+I32+I33</f>
         <v/>
       </c>
-      <c r="J34" s="31">
+      <c r="J34" s="32">
         <f>J31+J32+J33</f>
         <v/>
       </c>
-      <c r="K34" s="31">
+      <c r="K34" s="32">
         <f>K31+K32+K33</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="30" t="inlineStr">
+      <c r="A35" s="31" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="C35" s="32">
+      <c r="C35" s="33">
         <f>C28+C34</f>
         <v/>
       </c>
-      <c r="D35" s="32">
+      <c r="D35" s="33">
         <f>D28+D34</f>
         <v/>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="33">
         <f>E28+E34</f>
         <v/>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="33">
         <f>F28+F34</f>
         <v/>
       </c>
-      <c r="G35" s="32">
+      <c r="G35" s="33">
         <f>G28+G34</f>
         <v/>
       </c>
-      <c r="H35" s="32">
+      <c r="H35" s="33">
         <f>H28+H34</f>
         <v/>
       </c>
-      <c r="I35" s="32">
+      <c r="I35" s="33">
         <f>I28+I34</f>
         <v/>
       </c>
-      <c r="J35" s="32">
+      <c r="J35" s="33">
         <f>J28+J34</f>
         <v/>
       </c>
-      <c r="K35" s="32">
+      <c r="K35" s="33">
         <f>K28+K34</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="36" t="inlineStr">
+      <c r="A37" s="37" t="inlineStr">
         <is>
           <t>Balance check (Assets − L&amp;E)</t>
         </is>
       </c>
-      <c r="C37" s="42">
+      <c r="C37" s="43">
         <f>C15-C35</f>
         <v/>
       </c>
-      <c r="D37" s="42">
+      <c r="D37" s="43">
         <f>D15-D35</f>
         <v/>
       </c>
-      <c r="E37" s="42">
+      <c r="E37" s="43">
         <f>E15-E35</f>
         <v/>
       </c>
-      <c r="F37" s="42">
+      <c r="F37" s="43">
         <f>F15-F35</f>
         <v/>
       </c>
-      <c r="G37" s="42">
+      <c r="G37" s="43">
         <f>G15-G35</f>
         <v/>
       </c>
-      <c r="H37" s="42">
+      <c r="H37" s="43">
         <f>H15-H35</f>
         <v/>
       </c>
-      <c r="I37" s="42">
+      <c r="I37" s="43">
         <f>I15-I35</f>
         <v/>
       </c>
-      <c r="J37" s="42">
+      <c r="J37" s="43">
         <f>J15-J35</f>
         <v/>
       </c>
-      <c r="K37" s="42">
+      <c r="K37" s="43">
         <f>K15-K35</f>
         <v/>
       </c>
@@ -3905,6 +4053,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -3965,27 +4114,27 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="E2" s="27" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="F2" s="27" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="G2" s="29" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -4013,35 +4162,35 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="C5" s="29" t="n">
+      <c r="C5" s="30" t="n">
         <v>854800</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="30" t="n">
         <v>1550190</v>
       </c>
-      <c r="E5" s="29" t="n">
+      <c r="E5" s="30" t="n">
         <v>1814616</v>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="30" t="n">
         <v>1579183</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="25">
         <f>'Income Statement'!G13</f>
         <v/>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="25">
         <f>'Income Statement'!H13</f>
         <v/>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="25">
         <f>'Income Statement'!I13</f>
         <v/>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="25">
         <f>'Income Statement'!J13</f>
         <v/>
       </c>
-      <c r="K5" s="24">
+      <c r="K5" s="25">
         <f>'Income Statement'!K13</f>
         <v/>
       </c>
@@ -4052,35 +4201,35 @@
           <t>Depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="30" t="n">
         <v>291791</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="30" t="n">
         <v>379384</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="30" t="n">
         <v>446524</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="30" t="n">
         <v>496228</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="25">
         <f>'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="25">
         <f>'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="25">
         <f>'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="25">
         <f>'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K6" s="24">
+      <c r="K6" s="25">
         <f>'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
@@ -4091,35 +4240,35 @@
           <t>Stock-based compensation</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="30" t="n">
         <v>78075</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <v>93560</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="30" t="n">
         <v>90011</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <v>62203</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="25">
         <f>'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="25">
         <f>'Assumptions'!K14</f>
         <v/>
       </c>
@@ -4130,43 +4279,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
+      <c r="D8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="43" t="inlineStr">
+      <c r="F8" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="25">
         <f>-('Balance Sheet'!G7-'Balance Sheet'!F7)</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="25">
         <f>-('Balance Sheet'!H7-'Balance Sheet'!G7)</f>
         <v/>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>-('Balance Sheet'!I7-'Balance Sheet'!H7)</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="25">
         <f>-('Balance Sheet'!J7-'Balance Sheet'!I7)</f>
         <v/>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="25">
         <f>-('Balance Sheet'!K7-'Balance Sheet'!J7)</f>
         <v/>
       </c>
@@ -4177,43 +4326,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="43" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="43" t="inlineStr">
+      <c r="E9" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="43" t="inlineStr">
+      <c r="F9" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="25">
         <f>-('Balance Sheet'!G8-'Balance Sheet'!F8)</f>
         <v/>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="25">
         <f>-('Balance Sheet'!H8-'Balance Sheet'!G8)</f>
         <v/>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="25">
         <f>-('Balance Sheet'!I8-'Balance Sheet'!H8)</f>
         <v/>
       </c>
-      <c r="J9" s="24">
+      <c r="J9" s="25">
         <f>-('Balance Sheet'!J8-'Balance Sheet'!I8)</f>
         <v/>
       </c>
-      <c r="K9" s="24">
+      <c r="K9" s="25">
         <f>-('Balance Sheet'!K8-'Balance Sheet'!J8)</f>
         <v/>
       </c>
@@ -4224,43 +4373,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
+      <c r="D10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="43" t="inlineStr">
+      <c r="E10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F10" s="43" t="inlineStr">
+      <c r="F10" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="25">
         <f>-('Balance Sheet'!G12-'Balance Sheet'!F12)</f>
         <v/>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="25">
         <f>-('Balance Sheet'!H12-'Balance Sheet'!G12)</f>
         <v/>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="25">
         <f>-('Balance Sheet'!I12-'Balance Sheet'!H12)</f>
         <v/>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="25">
         <f>-('Balance Sheet'!J12-'Balance Sheet'!I12)</f>
         <v/>
       </c>
-      <c r="K10" s="24">
+      <c r="K10" s="25">
         <f>-('Balance Sheet'!K12-'Balance Sheet'!J12)</f>
         <v/>
       </c>
@@ -4271,43 +4420,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="25">
         <f>-('Balance Sheet'!G14-'Balance Sheet'!F14)</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="25">
         <f>-('Balance Sheet'!H14-'Balance Sheet'!G14)</f>
         <v/>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="25">
         <f>-('Balance Sheet'!I14-'Balance Sheet'!H14)</f>
         <v/>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="25">
         <f>-('Balance Sheet'!J14-'Balance Sheet'!I14)</f>
         <v/>
       </c>
-      <c r="K11" s="24">
+      <c r="K11" s="25">
         <f>-('Balance Sheet'!K14-'Balance Sheet'!J14)</f>
         <v/>
       </c>
@@ -4318,43 +4467,43 @@
           <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
         </is>
       </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="C12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
+      <c r="D12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="43" t="inlineStr">
+      <c r="E12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="43" t="inlineStr">
+      <c r="F12" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="25">
         <f>('Balance Sheet'!G19-'Balance Sheet'!F19)</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>('Balance Sheet'!H19-'Balance Sheet'!G19)</f>
         <v/>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="25">
         <f>('Balance Sheet'!I19-'Balance Sheet'!H19)</f>
         <v/>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="25">
         <f>('Balance Sheet'!J19-'Balance Sheet'!I19)</f>
         <v/>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="25">
         <f>('Balance Sheet'!K19-'Balance Sheet'!J19)</f>
         <v/>
       </c>
@@ -4365,43 +4514,43 @@
           <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="43" t="inlineStr">
+      <c r="E13" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F13" s="43" t="inlineStr">
+      <c r="F13" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="25">
         <f>('Balance Sheet'!G20-'Balance Sheet'!F20)</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="25">
         <f>('Balance Sheet'!H20-'Balance Sheet'!G20)</f>
         <v/>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="25">
         <f>('Balance Sheet'!I20-'Balance Sheet'!H20)</f>
         <v/>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="25">
         <f>('Balance Sheet'!J20-'Balance Sheet'!I20)</f>
         <v/>
       </c>
-      <c r="K13" s="24">
+      <c r="K13" s="25">
         <f>('Balance Sheet'!K20-'Balance Sheet'!J20)</f>
         <v/>
       </c>
@@ -4412,43 +4561,43 @@
           <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
         </is>
       </c>
-      <c r="C14" s="43" t="inlineStr">
+      <c r="C14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D14" s="43" t="inlineStr">
+      <c r="D14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="43" t="inlineStr">
+      <c r="E14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="43" t="inlineStr">
+      <c r="F14" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="25">
         <f>('Balance Sheet'!G22-'Balance Sheet'!F22)</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="25">
         <f>('Balance Sheet'!H22-'Balance Sheet'!G22)</f>
         <v/>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="25">
         <f>('Balance Sheet'!I22-'Balance Sheet'!H22)</f>
         <v/>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="25">
         <f>('Balance Sheet'!J22-'Balance Sheet'!I22)</f>
         <v/>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="25">
         <f>('Balance Sheet'!K22-'Balance Sheet'!J22)</f>
         <v/>
       </c>
@@ -4459,43 +4608,43 @@
           <t xml:space="preserve">  Incr./(decr.) in operating lease liab.</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="43" t="inlineStr">
+      <c r="E15" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="43" t="inlineStr">
+      <c r="F15" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="25">
         <f>('Balance Sheet'!G21-'Balance Sheet'!F21)+('Balance Sheet'!G25-'Balance Sheet'!F25)</f>
         <v/>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="25">
         <f>('Balance Sheet'!H21-'Balance Sheet'!G21)+('Balance Sheet'!H25-'Balance Sheet'!G25)</f>
         <v/>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="25">
         <f>('Balance Sheet'!I21-'Balance Sheet'!H21)+('Balance Sheet'!I25-'Balance Sheet'!H25)</f>
         <v/>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="25">
         <f>('Balance Sheet'!J21-'Balance Sheet'!I21)+('Balance Sheet'!J25-'Balance Sheet'!I25)</f>
         <v/>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="25">
         <f>('Balance Sheet'!K21-'Balance Sheet'!J21)+('Balance Sheet'!K25-'Balance Sheet'!J25)</f>
         <v/>
       </c>
@@ -4506,43 +4655,43 @@
           <t xml:space="preserve">  Incr./(decr.) in deferred income taxes</t>
         </is>
       </c>
-      <c r="C16" s="43" t="inlineStr">
+      <c r="C16" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="43" t="inlineStr">
+      <c r="D16" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="43" t="inlineStr">
+      <c r="E16" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="43" t="inlineStr">
+      <c r="F16" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="25">
         <f>('Balance Sheet'!G26-'Balance Sheet'!F26)</f>
         <v/>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="25">
         <f>('Balance Sheet'!H26-'Balance Sheet'!G26)</f>
         <v/>
       </c>
-      <c r="I16" s="24">
+      <c r="I16" s="25">
         <f>('Balance Sheet'!I26-'Balance Sheet'!H26)</f>
         <v/>
       </c>
-      <c r="J16" s="24">
+      <c r="J16" s="25">
         <f>('Balance Sheet'!J26-'Balance Sheet'!I26)</f>
         <v/>
       </c>
-      <c r="K16" s="24">
+      <c r="K16" s="25">
         <f>('Balance Sheet'!K26-'Balance Sheet'!J26)</f>
         <v/>
       </c>
@@ -4553,43 +4702,43 @@
           <t xml:space="preserve">  Incr./(decr.) in other non-current liab.</t>
         </is>
       </c>
-      <c r="C17" s="43" t="inlineStr">
+      <c r="C17" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="43" t="inlineStr">
+      <c r="E17" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F17" s="43" t="inlineStr">
+      <c r="F17" s="44" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="25">
         <f>('Balance Sheet'!G27-'Balance Sheet'!F27)</f>
         <v/>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="25">
         <f>('Balance Sheet'!H27-'Balance Sheet'!G27)</f>
         <v/>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="25">
         <f>('Balance Sheet'!I27-'Balance Sheet'!H27)</f>
         <v/>
       </c>
-      <c r="J17" s="24">
+      <c r="J17" s="25">
         <f>('Balance Sheet'!J27-'Balance Sheet'!I27)</f>
         <v/>
       </c>
-      <c r="K17" s="24">
+      <c r="K17" s="25">
         <f>('Balance Sheet'!K27-'Balance Sheet'!J27)</f>
         <v/>
       </c>
@@ -4600,58 +4749,58 @@
           <t xml:space="preserve">  Working capital &amp; other (reported, net)</t>
         </is>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="25">
         <f>C19-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="25">
         <f>D19-D5-D6-D7</f>
         <v/>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="25">
         <f>E19-E5-E6-E7</f>
         <v/>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="25">
         <f>F19-F5-F6-F7</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="C19" s="40" t="n">
+      <c r="C19" s="41" t="n">
         <v>966463</v>
       </c>
-      <c r="D19" s="40" t="n">
+      <c r="D19" s="41" t="n">
         <v>2296164</v>
       </c>
-      <c r="E19" s="40" t="n">
+      <c r="E19" s="41" t="n">
         <v>2272713</v>
       </c>
-      <c r="F19" s="40" t="n">
+      <c r="F19" s="41" t="n">
         <v>1602477</v>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="32">
         <f>G5+G6+G7+SUM(G8:G17)</f>
         <v/>
       </c>
-      <c r="H19" s="31">
+      <c r="H19" s="32">
         <f>H5+H6+H7+SUM(H8:H17)</f>
         <v/>
       </c>
-      <c r="I19" s="31">
+      <c r="I19" s="32">
         <f>I5+I6+I7+SUM(I8:I17)</f>
         <v/>
       </c>
-      <c r="J19" s="31">
+      <c r="J19" s="32">
         <f>J5+J6+J7+SUM(J8:J17)</f>
         <v/>
       </c>
-      <c r="K19" s="31">
+      <c r="K19" s="32">
         <f>K5+K6+K7+SUM(K8:K17)</f>
         <v/>
       </c>
@@ -4678,74 +4827,74 @@
           <t>Capital expenditures</t>
         </is>
       </c>
-      <c r="C22" s="29" t="n">
+      <c r="C22" s="30" t="n">
         <v>-638657</v>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="30" t="n">
         <v>-651865</v>
       </c>
-      <c r="E22" s="29" t="n">
+      <c r="E22" s="30" t="n">
         <v>-689232</v>
       </c>
-      <c r="F22" s="29" t="n">
+      <c r="F22" s="30" t="n">
         <v>-680802</v>
       </c>
-      <c r="G22" s="24">
+      <c r="G22" s="25">
         <f>-'Income Statement'!G4*'Assumptions'!G13</f>
         <v/>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="25">
         <f>-'Income Statement'!H4*'Assumptions'!H13</f>
         <v/>
       </c>
-      <c r="I22" s="24">
+      <c r="I22" s="25">
         <f>-'Income Statement'!I4*'Assumptions'!I13</f>
         <v/>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="25">
         <f>-'Income Statement'!J4*'Assumptions'!J13</f>
         <v/>
       </c>
-      <c r="K22" s="24">
+      <c r="K22" s="25">
         <f>-'Income Statement'!K4*'Assumptions'!K13</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Net cash from investing activities</t>
         </is>
       </c>
-      <c r="C23" s="40" t="n">
+      <c r="C23" s="41" t="n">
         <v>-569937</v>
       </c>
-      <c r="D23" s="40" t="n">
+      <c r="D23" s="41" t="n">
         <v>-654132</v>
       </c>
-      <c r="E23" s="40" t="n">
+      <c r="E23" s="41" t="n">
         <v>-798174</v>
       </c>
-      <c r="F23" s="40" t="n">
+      <c r="F23" s="41" t="n">
         <v>-662118</v>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="32">
         <f>G22</f>
         <v/>
       </c>
-      <c r="H23" s="31">
+      <c r="H23" s="32">
         <f>H22</f>
         <v/>
       </c>
-      <c r="I23" s="31">
+      <c r="I23" s="32">
         <f>I22</f>
         <v/>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="32">
         <f>J22</f>
         <v/>
       </c>
-      <c r="K23" s="31">
+      <c r="K23" s="32">
         <f>K22</f>
         <v/>
       </c>
@@ -4779,74 +4928,74 @@
           <t>Repurchase of common stock</t>
         </is>
       </c>
-      <c r="C27" s="29" t="n">
+      <c r="C27" s="30" t="n">
         <v>-444001</v>
       </c>
-      <c r="D27" s="29" t="n">
+      <c r="D27" s="30" t="n">
         <v>-558652</v>
       </c>
-      <c r="E27" s="29" t="n">
+      <c r="E27" s="30" t="n">
         <v>-1636879</v>
       </c>
-      <c r="F27" s="29" t="n">
+      <c r="F27" s="30" t="n">
         <v>-1178349</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="25">
         <f>-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H27" s="24">
+      <c r="H27" s="25">
         <f>-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="25">
         <f>-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="25">
         <f>-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K27" s="24">
+      <c r="K27" s="25">
         <f>-'Assumptions'!K27</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="C28" s="40" t="n">
+      <c r="C28" s="41" t="n">
         <v>-467487</v>
       </c>
-      <c r="D28" s="40" t="n">
+      <c r="D28" s="41" t="n">
         <v>-548828</v>
       </c>
-      <c r="E28" s="40" t="n">
+      <c r="E28" s="41" t="n">
         <v>-1652508</v>
       </c>
-      <c r="F28" s="40" t="n">
+      <c r="F28" s="41" t="n">
         <v>-1208656</v>
       </c>
-      <c r="G28" s="31">
+      <c r="G28" s="32">
         <f>G27</f>
         <v/>
       </c>
-      <c r="H28" s="31">
+      <c r="H28" s="32">
         <f>H27</f>
         <v/>
       </c>
-      <c r="I28" s="31">
+      <c r="I28" s="32">
         <f>I27</f>
         <v/>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="32">
         <f>J27</f>
         <v/>
       </c>
-      <c r="K28" s="31">
+      <c r="K28" s="32">
         <f>K27</f>
         <v/>
       </c>
@@ -4859,44 +5008,44 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="inlineStr">
+      <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="32">
         <f>C19+C23+C28</f>
         <v/>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="32">
         <f>D19+D23+D28</f>
         <v/>
       </c>
-      <c r="E31" s="31">
+      <c r="E31" s="32">
         <f>E19+E23+E28</f>
         <v/>
       </c>
-      <c r="F31" s="31">
+      <c r="F31" s="32">
         <f>F19+F23+F28</f>
         <v/>
       </c>
-      <c r="G31" s="31">
+      <c r="G31" s="32">
         <f>G19+G23+G28</f>
         <v/>
       </c>
-      <c r="H31" s="31">
+      <c r="H31" s="32">
         <f>H19+H23+H28</f>
         <v/>
       </c>
-      <c r="I31" s="31">
+      <c r="I31" s="32">
         <f>I19+I23+I28</f>
         <v/>
       </c>
-      <c r="J31" s="31">
+      <c r="J31" s="32">
         <f>J19+J23+J28</f>
         <v/>
       </c>
-      <c r="K31" s="31">
+      <c r="K31" s="32">
         <f>K19+K23+K28</f>
         <v/>
       </c>
@@ -4907,74 +5056,74 @@
           <t>Cash, beginning of year</t>
         </is>
       </c>
-      <c r="C32" s="29" t="n">
+      <c r="C32" s="30" t="n">
         <v>1150517</v>
       </c>
-      <c r="D32" s="29" t="n">
+      <c r="D32" s="30" t="n">
         <v>1154867</v>
       </c>
-      <c r="E32" s="29" t="n">
+      <c r="E32" s="30" t="n">
         <v>2243971</v>
       </c>
-      <c r="F32" s="29" t="n">
+      <c r="F32" s="30" t="n">
         <v>1984336</v>
       </c>
-      <c r="G32" s="24">
+      <c r="G32" s="25">
         <f>'Balance Sheet'!F6</f>
         <v/>
       </c>
-      <c r="H32" s="24">
+      <c r="H32" s="25">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I32" s="24">
+      <c r="I32" s="25">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J32" s="24">
+      <c r="J32" s="25">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K32" s="24">
+      <c r="K32" s="25">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="30" t="inlineStr">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t>Cash, end of year</t>
         </is>
       </c>
-      <c r="C33" s="41" t="n">
+      <c r="C33" s="42" t="n">
         <v>1154867</v>
       </c>
-      <c r="D33" s="41" t="n">
+      <c r="D33" s="42" t="n">
         <v>2243971</v>
       </c>
-      <c r="E33" s="41" t="n">
+      <c r="E33" s="42" t="n">
         <v>1984336</v>
       </c>
-      <c r="F33" s="41" t="n">
+      <c r="F33" s="42" t="n">
         <v>1807202</v>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="33">
         <f>G32+G31</f>
         <v/>
       </c>
-      <c r="H33" s="32">
+      <c r="H33" s="33">
         <f>H32+H31</f>
         <v/>
       </c>
-      <c r="I33" s="32">
+      <c r="I33" s="33">
         <f>I32+I31</f>
         <v/>
       </c>
-      <c r="J33" s="32">
+      <c r="J33" s="33">
         <f>J32+J31</f>
         <v/>
       </c>
-      <c r="K33" s="32">
+      <c r="K33" s="33">
         <f>K32+K31</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Place source links immediately left of every justification
Standardize all tabs: source column directly left of justification column
(WACC D|E, Scenarios F|G, DCF J|K, 3-statement L|M, Comps peers D|E).
Uses Excel HYPERLINK formulas for visible blue clickable links.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -165,12 +165,6 @@
       <i val="1"/>
       <color rgb="000000CC"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <i val="1"/>
-      <color rgb="000000CC"/>
-      <sz val="8"/>
       <u val="single"/>
     </font>
     <font>
@@ -298,10 +292,12 @@
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -323,19 +319,19 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -345,13 +341,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -791,7 +787,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions / inputs (justification + clickable source link)</t>
+          <t>Red font  =  analyst assumptions — source link in col L, justification in col M</t>
         </is>
       </c>
     </row>
@@ -863,19 +859,18 @@
   <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -985,12 +980,12 @@
     <row r="3">
       <c r="L3" s="17" t="inlineStr">
         <is>
+          <t>Source (click link)</t>
+        </is>
+      </c>
+      <c r="M3" s="17" t="inlineStr">
+        <is>
           <t>Justification (~20 words)</t>
-        </is>
-      </c>
-      <c r="M3" s="17" t="inlineStr">
-        <is>
-          <t>Source</t>
         </is>
       </c>
     </row>
@@ -1040,14 +1035,13 @@
       <c r="K5" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="L5" s="23">
+        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 guidance")</f>
+        <v/>
+      </c>
+      <c r="M5" s="24" t="inlineStr">
         <is>
           <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
-        </is>
-      </c>
-      <c r="M5" s="24" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 guidance</t>
         </is>
       </c>
     </row>
@@ -1084,14 +1078,13 @@
       <c r="K6" s="22" t="n">
         <v>0.58</v>
       </c>
-      <c r="L6" s="23" t="inlineStr">
+      <c r="L6" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical gross margin (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M6" s="24" t="inlineStr">
         <is>
           <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
-        </is>
-      </c>
-      <c r="M6" s="24" t="inlineStr">
-        <is>
-          <t>LULU historical gross margin (10-K)</t>
         </is>
       </c>
     </row>
@@ -1128,14 +1121,13 @@
       <c r="K7" s="22" t="n">
         <v>0.395</v>
       </c>
-      <c r="L7" s="23" t="inlineStr">
+      <c r="L7" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical SG&amp;A (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M7" s="24" t="inlineStr">
         <is>
           <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
-        </is>
-      </c>
-      <c r="M7" s="24" t="inlineStr">
-        <is>
-          <t>LULU historical SG&amp;A (10-K)</t>
         </is>
       </c>
     </row>
@@ -1172,14 +1164,13 @@
       <c r="K8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="L8" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K")</f>
+        <v/>
+      </c>
+      <c r="M8" s="24" t="inlineStr">
         <is>
           <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
-        </is>
-      </c>
-      <c r="M8" s="24" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1216,14 +1207,13 @@
       <c r="K9" s="26" t="n">
         <v>115000</v>
       </c>
-      <c r="L9" s="23" t="inlineStr">
+      <c r="L9" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K")</f>
+        <v/>
+      </c>
+      <c r="M9" s="24" t="inlineStr">
         <is>
           <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
-        </is>
-      </c>
-      <c r="M9" s="24" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1260,14 +1250,13 @@
       <c r="K10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="L10" s="23" t="inlineStr">
+      <c r="L10" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU effective tax history (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M10" s="24" t="inlineStr">
         <is>
           <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
-        </is>
-      </c>
-      <c r="M10" s="24" t="inlineStr">
-        <is>
-          <t>LULU effective tax history (10-K)</t>
         </is>
       </c>
     </row>
@@ -1320,14 +1309,13 @@
       <c r="K12" s="22" t="n">
         <v>0.045</v>
       </c>
-      <c r="L12" s="23" t="inlineStr">
+      <c r="L12" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M12" s="24" t="inlineStr">
         <is>
           <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
-        </is>
-      </c>
-      <c r="M12" s="24" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1364,14 +1352,13 @@
       <c r="K13" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="L13" s="23" t="inlineStr">
+      <c r="L13" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M13" s="24" t="inlineStr">
         <is>
           <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
-        </is>
-      </c>
-      <c r="M13" s="24" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1408,14 +1395,13 @@
       <c r="K14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="L14" s="23" t="inlineStr">
+      <c r="L14" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M14" s="24" t="inlineStr">
         <is>
           <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
-        </is>
-      </c>
-      <c r="M14" s="24" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1468,14 +1454,13 @@
       <c r="K16" s="22" t="n">
         <v>0.33</v>
       </c>
-      <c r="L16" s="23" t="inlineStr">
+      <c r="L16" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M16" s="24" t="inlineStr">
         <is>
           <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
-        </is>
-      </c>
-      <c r="M16" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1512,14 +1497,13 @@
       <c r="K17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="L17" s="23" t="inlineStr">
+      <c r="L17" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M17" s="24" t="inlineStr">
         <is>
           <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
-        </is>
-      </c>
-      <c r="M17" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1556,14 +1540,13 @@
       <c r="K18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="L18" s="23" t="inlineStr">
+      <c r="L18" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M18" s="24" t="inlineStr">
         <is>
           <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
-        </is>
-      </c>
-      <c r="M18" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1600,14 +1583,13 @@
       <c r="K19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="L19" s="23" t="inlineStr">
+      <c r="L19" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M19" s="24" t="inlineStr">
         <is>
           <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
-        </is>
-      </c>
-      <c r="M19" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1644,14 +1626,13 @@
       <c r="K20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="L20" s="23" t="inlineStr">
+      <c r="L20" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M20" s="24" t="inlineStr">
         <is>
           <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
-        </is>
-      </c>
-      <c r="M20" s="24" t="inlineStr">
-        <is>
-          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1688,14 +1669,13 @@
       <c r="K21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="L21" s="23" t="inlineStr">
+      <c r="L21" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M21" s="24" t="inlineStr">
         <is>
           <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
-        </is>
-      </c>
-      <c r="M21" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1732,14 +1712,13 @@
       <c r="K22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="L22" s="23" t="inlineStr">
+      <c r="L22" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M22" s="24" t="inlineStr">
         <is>
           <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
-        </is>
-      </c>
-      <c r="M22" s="24" t="inlineStr">
-        <is>
-          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1776,14 +1755,13 @@
       <c r="K23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="L23" s="23" t="inlineStr">
+      <c r="L23" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M23" s="24" t="inlineStr">
         <is>
           <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
-        </is>
-      </c>
-      <c r="M23" s="24" t="inlineStr">
-        <is>
-          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1820,14 +1798,13 @@
       <c r="K24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="L24" s="23" t="inlineStr">
+      <c r="L24" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M24" s="24" t="inlineStr">
         <is>
           <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
-        </is>
-      </c>
-      <c r="M24" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1864,14 +1841,13 @@
       <c r="K25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="L25" s="23" t="inlineStr">
+      <c r="L25" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M25" s="24" t="inlineStr">
         <is>
           <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
-        </is>
-      </c>
-      <c r="M25" s="24" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1924,14 +1900,13 @@
       <c r="K27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="L27" s="23" t="inlineStr">
+      <c r="L27" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF: share repurchases (10-K)")</f>
+        <v/>
+      </c>
+      <c r="M27" s="24" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
-        </is>
-      </c>
-      <c r="M27" s="24" t="inlineStr">
-        <is>
-          <t>LULU CF: share repurchases (10-K)</t>
         </is>
       </c>
     </row>
@@ -1956,14 +1931,13 @@
       <c r="K28" s="27" t="n">
         <v>135</v>
       </c>
-      <c r="L28" s="23" t="inlineStr">
+      <c r="L28" s="23">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU avg repurchase price (10-K/est.)")</f>
+        <v/>
+      </c>
+      <c r="M28" s="24" t="inlineStr">
         <is>
           <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
-        </is>
-      </c>
-      <c r="M28" s="24" t="inlineStr">
-        <is>
-          <t>LULU avg repurchase price (10-K/est.)</t>
         </is>
       </c>
     </row>
@@ -1980,27 +1954,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2015,19 +1968,18 @@
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2839,19 +2791,18 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -4041,19 +3992,18 @@
   <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Fix assumption source links: native Excel hyperlinks beside justification
Replace HYPERLINK() formulas with openpyxl hyperlink objects (same method
as blue 10-K links). Source column sits immediately RIGHT of justification
on every tab. Re-upload-ready xlsx.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -164,7 +164,13 @@
       <name val="Garamond"/>
       <i val="1"/>
       <color rgb="000000CC"/>
-      <sz val="8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="9"/>
       <u val="single"/>
     </font>
     <font>
@@ -292,10 +298,10 @@
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -319,19 +325,19 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -341,13 +347,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -859,7 +865,7 @@
   <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -869,8 +875,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -980,12 +986,12 @@
     <row r="3">
       <c r="L3" s="17" t="inlineStr">
         <is>
-          <t>Source (click link)</t>
+          <t>Justification (~20 words)</t>
         </is>
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Source (click)</t>
         </is>
       </c>
     </row>
@@ -1035,13 +1041,14 @@
       <c r="K5" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="L5" s="23">
-        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 guidance")</f>
-        <v/>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
+        </is>
       </c>
       <c r="M5" s="24" t="inlineStr">
         <is>
-          <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
+          <t>LULU Q2 FY2026 guidance</t>
         </is>
       </c>
     </row>
@@ -1078,13 +1085,14 @@
       <c r="K6" s="22" t="n">
         <v>0.58</v>
       </c>
-      <c r="L6" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical gross margin (10-K)")</f>
-        <v/>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
+        </is>
       </c>
       <c r="M6" s="24" t="inlineStr">
         <is>
-          <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
+          <t>LULU historical gross margin (10-K)</t>
         </is>
       </c>
     </row>
@@ -1121,13 +1129,14 @@
       <c r="K7" s="22" t="n">
         <v>0.395</v>
       </c>
-      <c r="L7" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical SG&amp;A (10-K)")</f>
-        <v/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
+        </is>
       </c>
       <c r="M7" s="24" t="inlineStr">
         <is>
-          <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
+          <t>LULU historical SG&amp;A (10-K)</t>
         </is>
       </c>
     </row>
@@ -1164,13 +1173,14 @@
       <c r="K8" s="26" t="n">
         <v>7000</v>
       </c>
-      <c r="L8" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K")</f>
-        <v/>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
+        </is>
       </c>
       <c r="M8" s="24" t="inlineStr">
         <is>
-          <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
+          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1207,13 +1217,14 @@
       <c r="K9" s="26" t="n">
         <v>115000</v>
       </c>
-      <c r="L9" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K")</f>
-        <v/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+        </is>
       </c>
       <c r="M9" s="24" t="inlineStr">
         <is>
-          <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+          <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
@@ -1250,13 +1261,14 @@
       <c r="K10" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="L10" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU effective tax history (10-K)")</f>
-        <v/>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
+        </is>
       </c>
       <c r="M10" s="24" t="inlineStr">
         <is>
-          <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
+          <t>LULU effective tax history (10-K)</t>
         </is>
       </c>
     </row>
@@ -1309,13 +1321,14 @@
       <c r="K12" s="22" t="n">
         <v>0.045</v>
       </c>
-      <c r="L12" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
-        <v/>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
+        </is>
       </c>
       <c r="M12" s="24" t="inlineStr">
         <is>
-          <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
+          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1352,13 +1365,14 @@
       <c r="K13" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="L13" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
-        <v/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+        </is>
       </c>
       <c r="M13" s="24" t="inlineStr">
         <is>
-          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1395,13 +1409,14 @@
       <c r="K14" s="26" t="n">
         <v>70000</v>
       </c>
-      <c r="L14" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
-        <v/>
+      <c r="L14" s="23" t="inlineStr">
+        <is>
+          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+        </is>
       </c>
       <c r="M14" s="24" t="inlineStr">
         <is>
-          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+          <t>LULU CF statement (10-K)</t>
         </is>
       </c>
     </row>
@@ -1454,13 +1469,14 @@
       <c r="K16" s="22" t="n">
         <v>0.33</v>
       </c>
-      <c r="L16" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+        </is>
       </c>
       <c r="M16" s="24" t="inlineStr">
         <is>
-          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1497,13 +1513,14 @@
       <c r="K17" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="L17" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+        </is>
       </c>
       <c r="M17" s="24" t="inlineStr">
         <is>
-          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1540,13 +1557,14 @@
       <c r="K18" s="22" t="n">
         <v>0.058</v>
       </c>
-      <c r="L18" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+        </is>
       </c>
       <c r="M18" s="24" t="inlineStr">
         <is>
-          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1601,14 @@
       <c r="K19" s="22" t="n">
         <v>0.068</v>
       </c>
-      <c r="L19" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+        </is>
       </c>
       <c r="M19" s="24" t="inlineStr">
         <is>
-          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1626,13 +1645,14 @@
       <c r="K20" s="22" t="n">
         <v>0.147</v>
       </c>
-      <c r="L20" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
-        <v/>
+      <c r="L20" s="23" t="inlineStr">
+        <is>
+          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+        </is>
       </c>
       <c r="M20" s="24" t="inlineStr">
         <is>
-          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1669,13 +1689,14 @@
       <c r="K21" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="L21" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+        </is>
       </c>
       <c r="M21" s="24" t="inlineStr">
         <is>
-          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1712,13 +1733,14 @@
       <c r="K22" s="22" t="n">
         <v>0.027</v>
       </c>
-      <c r="L22" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
-        <v/>
+      <c r="L22" s="23" t="inlineStr">
+        <is>
+          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+        </is>
       </c>
       <c r="M22" s="24" t="inlineStr">
         <is>
-          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1755,13 +1777,14 @@
       <c r="K23" s="22" t="n">
         <v>0.135</v>
       </c>
-      <c r="L23" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU lease disclosures (10-K)")</f>
-        <v/>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+        </is>
       </c>
       <c r="M23" s="24" t="inlineStr">
         <is>
-          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
     </row>
@@ -1798,13 +1821,14 @@
       <c r="K24" s="22" t="n">
         <v>0.055</v>
       </c>
-      <c r="L24" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L24" s="23" t="inlineStr">
+        <is>
+          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+        </is>
       </c>
       <c r="M24" s="24" t="inlineStr">
         <is>
-          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1841,13 +1865,14 @@
       <c r="K25" s="22" t="n">
         <v>0.005</v>
       </c>
-      <c r="L25" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU balance sheet (10-K)")</f>
-        <v/>
+      <c r="L25" s="23" t="inlineStr">
+        <is>
+          <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
+        </is>
       </c>
       <c r="M25" s="24" t="inlineStr">
         <is>
-          <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
     </row>
@@ -1900,13 +1925,14 @@
       <c r="K27" s="26" t="n">
         <v>500000</v>
       </c>
-      <c r="L27" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF: share repurchases (10-K)")</f>
-        <v/>
+      <c r="L27" s="23" t="inlineStr">
+        <is>
+          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+        </is>
       </c>
       <c r="M27" s="24" t="inlineStr">
         <is>
-          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+          <t>LULU CF: share repurchases (10-K)</t>
         </is>
       </c>
     </row>
@@ -1931,13 +1957,14 @@
       <c r="K28" s="27" t="n">
         <v>135</v>
       </c>
-      <c r="L28" s="23">
-        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU avg repurchase price (10-K/est.)")</f>
-        <v/>
+      <c r="L28" s="23" t="inlineStr">
+        <is>
+          <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+        </is>
       </c>
       <c r="M28" s="24" t="inlineStr">
         <is>
-          <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+          <t>LULU avg repurchase price (10-K/est.)</t>
         </is>
       </c>
     </row>
@@ -1954,6 +1981,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1968,7 +2016,7 @@
   <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -1978,8 +2026,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2791,7 +2839,7 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -2801,8 +2849,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -3992,7 +4040,7 @@
   <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -4002,8 +4050,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Add 'where to find' hints to every source link
Each red-assumption source cell now shows a Find: line explaining what
to search for in the linked page (e.g. DGS10 latest yield for 4.3% RFR).
Cover-tab and reported-figure links include the same guidance.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -266,7 +266,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -302,7 +304,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -314,7 +316,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -793,7 +795,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions — source link in col L, justification in col M</t>
+          <t>Red font  =  analyst assumptions — justification in col L, source &amp; where to find in col M</t>
         </is>
       </c>
     </row>
@@ -804,24 +806,27 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="42" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>SEC EDGAR XBRL company facts, CIK 0001397187 (Forms 10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>SEC EDGAR filings, CIK 0001397187 (Forms 10-K)
+Find: Filter by Form 10-K; open FY2025 filing (accession 0001397187-26-000020).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>FY2025 Form 10-K (ended Feb 1, 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>FY2025 Form 10-K (ended Feb 1, 2026)
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Q2 FY2026 results &amp; FY2026 guidance (Sep 3, 2026 earnings release)</t>
+          <t>Q2 FY2026 results &amp; FY2026 guidance (Sep 3, 2026 earnings release)
+Find: Search 'outlook', 'guidance', or 'full year 2026' for revenue and diluted EPS ranges.</t>
         </is>
       </c>
     </row>
@@ -876,7 +881,7 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -931,10 +936,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Source &amp; find</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
@@ -991,7 +996,7 @@
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t>Source (click)</t>
+          <t>Source &amp; where to find</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1016,7 @@
       <c r="J4" s="19" t="n"/>
       <c r="K4" s="19" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
@@ -1048,11 +1053,12 @@
       </c>
       <c r="M5" s="24" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>LULU Q2 FY2026 guidance
+Find: Release → FY2026 revenue guidance (−5% to −7%); FY27–30 recovery path is analyst projection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Gross margin %</t>
@@ -1092,11 +1098,12 @@
       </c>
       <c r="M6" s="24" t="inlineStr">
         <is>
-          <t>LULU historical gross margin (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>LULU historical gross margin (10-K)
+Find: Income Statement → gross profit ÷ net revenue; FY22–25 history vs 56.5–58.0% forecast recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
           <t>SG&amp;A % of revenue</t>
@@ -1136,11 +1143,12 @@
       </c>
       <c r="M7" s="24" t="inlineStr">
         <is>
-          <t>LULU historical SG&amp;A (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>LULU historical SG&amp;A (10-K)
+Find: Income Statement → SG&amp;A ÷ net revenue; ratio declines toward 39.5% on cost discipline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Amortization / other opex ($)</t>
@@ -1180,11 +1188,12 @@
       </c>
       <c r="M8" s="24" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>LULU FY2025 10-K
+Find: Income Statement / footnotes → amortization of intangibles (~$7M run-rate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Other income, net ($)</t>
@@ -1224,11 +1233,12 @@
       </c>
       <c r="M9" s="24" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>LULU FY2025 10-K
+Find: Income Statement → 'Other income (expense), net' / interest income on cash balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Effective tax rate %</t>
@@ -1268,7 +1278,8 @@
       </c>
       <c r="M10" s="24" t="inlineStr">
         <is>
-          <t>LULU effective tax history (10-K)</t>
+          <t>LULU effective tax history (10-K)
+Find: Income Statement → provision for income taxes ÷ pretax income (effective rate history).</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1299,7 @@
       <c r="J11" s="19" t="n"/>
       <c r="K11" s="19" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>D&amp;A % of revenue</t>
@@ -1328,11 +1339,12 @@
       </c>
       <c r="M12" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+          <t>LULU CF statement (10-K)
+Find: Cash Flow Statement → depreciation &amp; amortization as % of revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Capex % of revenue</t>
@@ -1372,11 +1384,12 @@
       </c>
       <c r="M13" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>LULU CF statement (10-K)
+Find: Cash Flow Statement → capital expenditures as % of revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Stock-based compensation ($)</t>
@@ -1416,7 +1429,8 @@
       </c>
       <c r="M14" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)</t>
+          <t>LULU CF statement (10-K)
+Find: Cash Flow Statement → 'Stock-based compensation' (operating add-back).</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1450,7 @@
       <c r="J15" s="19" t="n"/>
       <c r="K15" s="19" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Inventories % of COGS</t>
@@ -1476,11 +1490,12 @@
       </c>
       <c r="M16" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → 'Inventories' ÷ COGS (or revenue) for turnover / build assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Accounts payable % of COGS</t>
@@ -1520,11 +1535,12 @@
       </c>
       <c r="M17" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → 'Accounts payable' ÷ COGS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Accrued liabilities % of revenue</t>
@@ -1564,11 +1580,12 @@
       </c>
       <c r="M18" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → 'Accrued liabilities' ÷ net revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Other current assets % of revenue</t>
@@ -1608,11 +1625,12 @@
       </c>
       <c r="M19" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → prepaid expenses &amp; other current assets ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Operating lease ROU asset % of revenue</t>
@@ -1652,11 +1670,12 @@
       </c>
       <c r="M20" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
+          <t>LULU lease disclosures (10-K)
+Find: Balance Sheet / Note → 'Operating lease right-of-use assets' ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Other non-current assets % of revenue</t>
@@ -1696,11 +1715,12 @@
       </c>
       <c r="M21" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → other non-current assets ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (current) % of revenue</t>
@@ -1740,11 +1760,12 @@
       </c>
       <c r="M22" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+          <t>LULU lease disclosures (10-K)
+Find: Balance Sheet → current portion of operating lease liabilities ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (non-current) % of revenue</t>
@@ -1784,11 +1805,12 @@
       </c>
       <c r="M23" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
+          <t>LULU lease disclosures (10-K)
+Find: Balance Sheet → non-current operating lease liabilities ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Other current liabilities % of revenue</t>
@@ -1828,11 +1850,12 @@
       </c>
       <c r="M24" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → other current liabilities (gift cards, deferred revenue) ÷ revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Other non-current liab % of revenue</t>
@@ -1872,7 +1895,8 @@
       </c>
       <c r="M25" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU balance sheet (10-K)
+Find: Balance Sheet → other non-current liabilities ÷ revenue.</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1916,7 @@
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="19" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Share repurchases ($)</t>
@@ -1932,11 +1956,12 @@
       </c>
       <c r="M27" s="24" t="inlineStr">
         <is>
-          <t>LULU CF: share repurchases (10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+          <t>LULU CF: share repurchases (10-K)
+Find: Cash Flow Statement → 'Repurchase of common stock' (FY24–25 peak vs $500M forecast).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Avg repurchase price ($/sh)</t>
@@ -1964,7 +1989,8 @@
       </c>
       <c r="M28" s="24" t="inlineStr">
         <is>
-          <t>LULU avg repurchase price (10-K/est.)</t>
+          <t>LULU avg repurchase price (10-K/est.)
+Find: Cash Flow / equity footnote → average price paid per share in buyback programs.</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2053,7 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2082,30 +2108,34 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Source &amp; find</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">
@@ -2850,7 +2880,7 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2905,30 +2935,34 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Source &amp; find</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">
@@ -4051,7 +4085,7 @@
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -4106,30 +4140,34 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Source &amp; find</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>10-K
+Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Show exact Ctrl+F search strings in every source cell
Replace generic find hints with quoted line items, table fields, and
expected values (e.g. DGS10 latest yield for 4.3% RFR, 10-K line names).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -795,7 +795,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions — justification in col L, source &amp; where to find in col M</t>
+          <t>Red font  =  analyst assumptions — justification in col L, source &amp; Ctrl+F lines in col M</t>
         </is>
       </c>
     </row>
@@ -806,27 +806,27 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
           <t>SEC EDGAR filings, CIK 0001397187 (Forms 10-K)
-Find: Filter by Form 10-K; open FY2025 filing (accession 0001397187-26-000020).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
+Ctrl+F: "10-K" → FY2025 accession 0001397187-26-000020</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
       <c r="B17" s="9" t="inlineStr">
         <is>
           <t>FY2025 Form 10-K (ended Feb 1, 2026)
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Q2 FY2026 results &amp; FY2026 guidance (Sep 3, 2026 earnings release)
-Find: Search 'outlook', 'guidance', or 'full year 2026' for revenue and diluted EPS ranges.</t>
+Ctrl+F: "full year 2026" | "net revenue" | "diluted earnings per share"</t>
         </is>
       </c>
     </row>
@@ -936,10 +936,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source &amp; find</t>
+          <t>Ctrl+F lines</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t>Source &amp; where to find</t>
+          <t>Source &amp; Ctrl+F lines</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       <c r="J4" s="19" t="n"/>
       <c r="K4" s="19" t="n"/>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
@@ -1054,11 +1054,11 @@
       <c r="M5" s="24" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 guidance
-Find: Release → FY2026 revenue guidance (−5% to −7%); FY27–30 recovery path is analyst projection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+Ctrl+F: "full year 2026" → "net revenue" → "5% to 7%" decrease; FY27–30 = projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Gross margin %</t>
@@ -1099,11 +1099,11 @@
       <c r="M6" s="24" t="inlineStr">
         <is>
           <t>LULU historical gross margin (10-K)
-Find: Income Statement → gross profit ÷ net revenue; FY22–25 history vs 56.5–58.0% forecast recovery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+Ctrl+F: "Gross profit" $6,284,132 ÷ "Net revenue" $11,102,600 = 56.6% FY25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
           <t>SG&amp;A % of revenue</t>
@@ -1144,11 +1144,11 @@
       <c r="M7" s="24" t="inlineStr">
         <is>
           <t>LULU historical SG&amp;A (10-K)
-Find: Income Statement → SG&amp;A ÷ net revenue; ratio declines toward 39.5% on cost discipline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
+Ctrl+F: "Selling, general and administrative expenses" $4,066,556 ÷ revenue = 36.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Amortization / other opex ($)</t>
@@ -1189,11 +1189,11 @@
       <c r="M8" s="24" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K
-Find: Income Statement / footnotes → amortization of intangibles (~$7M run-rate).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+Ctrl+F: "Amortization of intangible assets" → FY25 $6,961 (≈$7M run-rate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Other income, net ($)</t>
@@ -1234,11 +1234,11 @@
       <c r="M9" s="24" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K
-Find: Income Statement → 'Other income (expense), net' / interest income on cash balances.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+Ctrl+F: "Other income (expense), net" → FY25 $28,352 (interest income on cash)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Effective tax rate %</t>
@@ -1279,7 +1279,7 @@
       <c r="M10" s="24" t="inlineStr">
         <is>
           <t>LULU effective tax history (10-K)
-Find: Income Statement → provision for income taxes ÷ pretax income (effective rate history).</t>
+Ctrl+F: "Provision for income taxes" $659,784 ÷ "Income before income taxes" $2,238,967 = 29.5%</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       <c r="J11" s="19" t="n"/>
       <c r="K11" s="19" t="n"/>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>D&amp;A % of revenue</t>
@@ -1340,11 +1340,11 @@
       <c r="M12" s="24" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)
-Find: Cash Flow Statement → depreciation &amp; amortization as % of revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+Ctrl+F: "Depreciation and amortization" $496,228 ÷ "Net revenue" $11,102,600 = 4.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Capex % of revenue</t>
@@ -1385,11 +1385,11 @@
       <c r="M13" s="24" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)
-Find: Cash Flow Statement → capital expenditures as % of revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+Ctrl+F: "Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Stock-based compensation ($)</t>
@@ -1430,7 +1430,7 @@
       <c r="M14" s="24" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)
-Find: Cash Flow Statement → 'Stock-based compensation' (operating add-back).</t>
+Ctrl+F: "Stock-based compensation" → FY25 $62,203; model $70,000</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       <c r="J15" s="19" t="n"/>
       <c r="K15" s="19" t="n"/>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Inventories % of COGS</t>
@@ -1491,11 +1491,11 @@
       <c r="M16" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → 'Inventories' ÷ COGS (or revenue) for turnover / build assumptions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
+Ctrl+F: "Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Accounts payable % of COGS</t>
@@ -1536,11 +1536,11 @@
       <c r="M17" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → 'Accounts payable' ÷ COGS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
+Ctrl+F: "Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Accrued liabilities % of revenue</t>
@@ -1581,11 +1581,11 @@
       <c r="M18" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → 'Accrued liabilities' ÷ net revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
+Ctrl+F: "Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Other current assets % of revenue</t>
@@ -1626,11 +1626,11 @@
       <c r="M19" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → prepaid expenses &amp; other current assets ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="42" customHeight="1">
+Ctrl+F: "Other current assets" → derive from current assets less cash, A/R, inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Operating lease ROU asset % of revenue</t>
@@ -1671,11 +1671,11 @@
       <c r="M20" s="24" t="inlineStr">
         <is>
           <t>LULU lease disclosures (10-K)
-Find: Balance Sheet / Note → 'Operating lease right-of-use assets' ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="42" customHeight="1">
+Ctrl+F: "Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Other non-current assets % of revenue</t>
@@ -1716,11 +1716,11 @@
       <c r="M21" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → other non-current assets ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="42" customHeight="1">
+Ctrl+F: "Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (current) % of revenue</t>
@@ -1761,11 +1761,11 @@
       <c r="M22" s="24" t="inlineStr">
         <is>
           <t>LULU lease disclosures (10-K)
-Find: Balance Sheet → current portion of operating lease liabilities ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
+Ctrl+F: "Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Op lease liab (non-current) % of revenue</t>
@@ -1806,11 +1806,11 @@
       <c r="M23" s="24" t="inlineStr">
         <is>
           <t>LULU lease disclosures (10-K)
-Find: Balance Sheet → non-current operating lease liabilities ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
+Ctrl+F: "Operating lease liabilities" $1,499,717 (non-current) ÷ revenue = 13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Other current liabilities % of revenue</t>
@@ -1851,11 +1851,11 @@
       <c r="M24" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → other current liabilities (gift cards, deferred revenue) ÷ revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="42" customHeight="1">
+Ctrl+F: "Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Other non-current liab % of revenue</t>
@@ -1896,7 +1896,7 @@
       <c r="M25" s="24" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)
-Find: Balance Sheet → other non-current liabilities ÷ revenue.</t>
+Ctrl+F: "Other non-current liabilities" → minor long-term accruals ÷ revenue</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="19" t="n"/>
     </row>
-    <row r="27" ht="42" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Share repurchases ($)</t>
@@ -1957,11 +1957,11 @@
       <c r="M27" s="24" t="inlineStr">
         <is>
           <t>LULU CF: share repurchases (10-K)
-Find: Cash Flow Statement → 'Repurchase of common stock' (FY24–25 peak vs $500M forecast).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="42" customHeight="1">
+Ctrl+F: "Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Avg repurchase price ($/sh)</t>
@@ -1990,7 +1990,7 @@
       <c r="M28" s="24" t="inlineStr">
         <is>
           <t>LULU avg repurchase price (10-K/est.)
-Find: Cash Flow / equity footnote → average price paid per share in buyback programs.</t>
+Ctrl+F: "Repurchase of common stock" footnote → avg price paid per share</t>
         </is>
       </c>
     </row>
@@ -2108,34 +2108,34 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source &amp; find</t>
+          <t>Ctrl+F lines</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">
@@ -2935,34 +2935,34 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source &amp; find</t>
+          <t>Ctrl+F lines</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">
@@ -4140,34 +4140,34 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Source &amp; find</t>
+          <t>Ctrl+F lines</t>
         </is>
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
           <t>10-K
-Find: Interactive 10-K viewer → table of contents or Ctrl+F for financial statements.</t>
+Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
       <c r="G2" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Add dedicated Ctrl+F column beside every assumption source
Split source links from proof strings: Justification | Source (click) |
Ctrl+F (prove number) on WACC, Scenarios, DCF, Comps, and 3-statement tabs.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -254,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -304,6 +304,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -795,7 +798,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Red font  =  analyst assumptions — justification in col L, source &amp; Ctrl+F lines in col M</t>
+          <t>Red font  =  analyst assumptions — Justification (L) | Source (M) | Ctrl+F (N)</t>
         </is>
       </c>
     </row>
@@ -867,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -880,8 +883,9 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -996,7 +1000,12 @@
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t>Source &amp; Ctrl+F lines</t>
+          <t>Source (click)</t>
+        </is>
+      </c>
+      <c r="N3" s="17" t="inlineStr">
+        <is>
+          <t>Ctrl+F (prove number)</t>
         </is>
       </c>
     </row>
@@ -1053,8 +1062,12 @@
       </c>
       <c r="M5" s="24" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance
-Ctrl+F: "full year 2026" → "net revenue" → "5% to 7%" decrease; FY27–30 = projection</t>
+          <t>LULU Q2 FY2026 guidance</t>
+        </is>
+      </c>
+      <c r="N5" s="25" t="inlineStr">
+        <is>
+          <t>"full year 2026" → "net revenue" → "5% to 7%" decrease; FY27–30 = projection</t>
         </is>
       </c>
     </row>
@@ -1098,8 +1111,12 @@
       </c>
       <c r="M6" s="24" t="inlineStr">
         <is>
-          <t>LULU historical gross margin (10-K)
-Ctrl+F: "Gross profit" $6,284,132 ÷ "Net revenue" $11,102,600 = 56.6% FY25</t>
+          <t>LULU historical gross margin (10-K)</t>
+        </is>
+      </c>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>"Gross profit" $6,284,132 ÷ "Net revenue" $11,102,600 = 56.6% FY25</t>
         </is>
       </c>
     </row>
@@ -1143,8 +1160,12 @@
       </c>
       <c r="M7" s="24" t="inlineStr">
         <is>
-          <t>LULU historical SG&amp;A (10-K)
-Ctrl+F: "Selling, general and administrative expenses" $4,066,556 ÷ revenue = 36.7%</t>
+          <t>LULU historical SG&amp;A (10-K)</t>
+        </is>
+      </c>
+      <c r="N7" s="25" t="inlineStr">
+        <is>
+          <t>"Selling, general and administrative expenses" $4,066,556 ÷ revenue = 36.7%</t>
         </is>
       </c>
     </row>
@@ -1154,31 +1175,31 @@
           <t>Amortization / other opex ($)</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="26" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="26" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="26" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="26" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="27" t="n">
         <v>7000</v>
       </c>
-      <c r="H8" s="26" t="n">
+      <c r="H8" s="27" t="n">
         <v>7000</v>
       </c>
-      <c r="I8" s="26" t="n">
+      <c r="I8" s="27" t="n">
         <v>7000</v>
       </c>
-      <c r="J8" s="26" t="n">
+      <c r="J8" s="27" t="n">
         <v>7000</v>
       </c>
-      <c r="K8" s="26" t="n">
+      <c r="K8" s="27" t="n">
         <v>7000</v>
       </c>
       <c r="L8" s="23" t="inlineStr">
@@ -1188,8 +1209,12 @@
       </c>
       <c r="M8" s="24" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K
-Ctrl+F: "Amortization of intangible assets" → FY25 $6,961 (≈$7M run-rate)</t>
+          <t>LULU FY2025 10-K</t>
+        </is>
+      </c>
+      <c r="N8" s="25" t="inlineStr">
+        <is>
+          <t>"Amortization of intangible assets" → FY25 $6,961 (≈$7M run-rate)</t>
         </is>
       </c>
     </row>
@@ -1199,31 +1224,31 @@
           <t>Other income, net ($)</t>
         </is>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="26" t="n">
         <v>4163</v>
       </c>
-      <c r="D9" s="25" t="n">
+      <c r="D9" s="26" t="n">
         <v>43059</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="26" t="n">
         <v>70380</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="26" t="n">
         <v>28352</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="27" t="n">
         <v>130000</v>
       </c>
-      <c r="H9" s="26" t="n">
+      <c r="H9" s="27" t="n">
         <v>60000</v>
       </c>
-      <c r="I9" s="26" t="n">
+      <c r="I9" s="27" t="n">
         <v>75000</v>
       </c>
-      <c r="J9" s="26" t="n">
+      <c r="J9" s="27" t="n">
         <v>95000</v>
       </c>
-      <c r="K9" s="26" t="n">
+      <c r="K9" s="27" t="n">
         <v>115000</v>
       </c>
       <c r="L9" s="23" t="inlineStr">
@@ -1233,8 +1258,12 @@
       </c>
       <c r="M9" s="24" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K
-Ctrl+F: "Other income (expense), net" → FY25 $28,352 (interest income on cash)</t>
+          <t>LULU FY2025 10-K</t>
+        </is>
+      </c>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>"Other income (expense), net" → FY25 $28,352 (interest income on cash)</t>
         </is>
       </c>
     </row>
@@ -1278,8 +1307,12 @@
       </c>
       <c r="M10" s="24" t="inlineStr">
         <is>
-          <t>LULU effective tax history (10-K)
-Ctrl+F: "Provision for income taxes" $659,784 ÷ "Income before income taxes" $2,238,967 = 29.5%</t>
+          <t>LULU effective tax history (10-K)</t>
+        </is>
+      </c>
+      <c r="N10" s="25" t="inlineStr">
+        <is>
+          <t>"Provision for income taxes" $659,784 ÷ "Income before income taxes" $2,238,967 = 29.5%</t>
         </is>
       </c>
     </row>
@@ -1339,8 +1372,12 @@
       </c>
       <c r="M12" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)
-Ctrl+F: "Depreciation and amortization" $496,228 ÷ "Net revenue" $11,102,600 = 4.5%</t>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t>"Depreciation and amortization" $496,228 ÷ "Net revenue" $11,102,600 = 4.5%</t>
         </is>
       </c>
     </row>
@@ -1384,8 +1421,12 @@
       </c>
       <c r="M13" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)
-Ctrl+F: "Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
+      <c r="N13" s="25" t="inlineStr">
+        <is>
+          <t>"Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
         </is>
       </c>
     </row>
@@ -1395,31 +1436,31 @@
           <t>Stock-based compensation ($)</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="26" t="n">
         <v>78075</v>
       </c>
-      <c r="D14" s="25" t="n">
+      <c r="D14" s="26" t="n">
         <v>93560</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="26" t="n">
         <v>90011</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F14" s="26" t="n">
         <v>62203</v>
       </c>
-      <c r="G14" s="26" t="n">
+      <c r="G14" s="27" t="n">
         <v>70000</v>
       </c>
-      <c r="H14" s="26" t="n">
+      <c r="H14" s="27" t="n">
         <v>70000</v>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I14" s="27" t="n">
         <v>70000</v>
       </c>
-      <c r="J14" s="26" t="n">
+      <c r="J14" s="27" t="n">
         <v>70000</v>
       </c>
-      <c r="K14" s="26" t="n">
+      <c r="K14" s="27" t="n">
         <v>70000</v>
       </c>
       <c r="L14" s="23" t="inlineStr">
@@ -1429,8 +1470,12 @@
       </c>
       <c r="M14" s="24" t="inlineStr">
         <is>
-          <t>LULU CF statement (10-K)
-Ctrl+F: "Stock-based compensation" → FY25 $62,203; model $70,000</t>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
+      <c r="N14" s="25" t="inlineStr">
+        <is>
+          <t>"Stock-based compensation" → FY25 $62,203; model $70,000</t>
         </is>
       </c>
     </row>
@@ -1490,8 +1535,12 @@
       </c>
       <c r="M16" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>"Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
         </is>
       </c>
     </row>
@@ -1535,8 +1584,12 @@
       </c>
       <c r="M17" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N17" s="25" t="inlineStr">
+        <is>
+          <t>"Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
         </is>
       </c>
     </row>
@@ -1580,8 +1633,12 @@
       </c>
       <c r="M18" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N18" s="25" t="inlineStr">
+        <is>
+          <t>"Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
         </is>
       </c>
     </row>
@@ -1625,8 +1682,12 @@
       </c>
       <c r="M19" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Other current assets" → derive from current assets less cash, A/R, inventory</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N19" s="25" t="inlineStr">
+        <is>
+          <t>"Other current assets" → derive from current assets less cash, A/R, inventory</t>
         </is>
       </c>
     </row>
@@ -1670,8 +1731,12 @@
       </c>
       <c r="M20" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)
-Ctrl+F: "Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
+      <c r="N20" s="25" t="inlineStr">
+        <is>
+          <t>"Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
         </is>
       </c>
     </row>
@@ -1715,8 +1780,12 @@
       </c>
       <c r="M21" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N21" s="25" t="inlineStr">
+        <is>
+          <t>"Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
         </is>
       </c>
     </row>
@@ -1760,8 +1829,12 @@
       </c>
       <c r="M22" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)
-Ctrl+F: "Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
+      <c r="N22" s="25" t="inlineStr">
+        <is>
+          <t>"Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
         </is>
       </c>
     </row>
@@ -1805,8 +1878,12 @@
       </c>
       <c r="M23" s="24" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)
-Ctrl+F: "Operating lease liabilities" $1,499,717 (non-current) ÷ revenue = 13.5%</t>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
+      <c r="N23" s="25" t="inlineStr">
+        <is>
+          <t>"Operating lease liabilities" $1,499,717 (non-current) ÷ revenue = 13.5%</t>
         </is>
       </c>
     </row>
@@ -1850,8 +1927,12 @@
       </c>
       <c r="M24" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N24" s="25" t="inlineStr">
+        <is>
+          <t>"Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
         </is>
       </c>
     </row>
@@ -1895,8 +1976,12 @@
       </c>
       <c r="M25" s="24" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)
-Ctrl+F: "Other non-current liabilities" → minor long-term accruals ÷ revenue</t>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="N25" s="25" t="inlineStr">
+        <is>
+          <t>"Other non-current liabilities" → minor long-term accruals ÷ revenue</t>
         </is>
       </c>
     </row>
@@ -1922,31 +2007,31 @@
           <t>Share repurchases ($)</t>
         </is>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C27" s="26" t="n">
         <v>444001</v>
       </c>
-      <c r="D27" s="25" t="n">
+      <c r="D27" s="26" t="n">
         <v>558652</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="26" t="n">
         <v>1636879</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F27" s="26" t="n">
         <v>1178349</v>
       </c>
-      <c r="G27" s="26" t="n">
+      <c r="G27" s="27" t="n">
         <v>500000</v>
       </c>
-      <c r="H27" s="26" t="n">
+      <c r="H27" s="27" t="n">
         <v>500000</v>
       </c>
-      <c r="I27" s="26" t="n">
+      <c r="I27" s="27" t="n">
         <v>500000</v>
       </c>
-      <c r="J27" s="26" t="n">
+      <c r="J27" s="27" t="n">
         <v>500000</v>
       </c>
-      <c r="K27" s="26" t="n">
+      <c r="K27" s="27" t="n">
         <v>500000</v>
       </c>
       <c r="L27" s="23" t="inlineStr">
@@ -1956,8 +2041,12 @@
       </c>
       <c r="M27" s="24" t="inlineStr">
         <is>
-          <t>LULU CF: share repurchases (10-K)
-Ctrl+F: "Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
+          <t>LULU CF: share repurchases (10-K)</t>
+        </is>
+      </c>
+      <c r="N27" s="25" t="inlineStr">
+        <is>
+          <t>"Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
         </is>
       </c>
     </row>
@@ -1967,19 +2056,19 @@
           <t>Avg repurchase price ($/sh)</t>
         </is>
       </c>
-      <c r="G28" s="27" t="n">
+      <c r="G28" s="28" t="n">
         <v>105</v>
       </c>
-      <c r="H28" s="27" t="n">
+      <c r="H28" s="28" t="n">
         <v>112</v>
       </c>
-      <c r="I28" s="27" t="n">
+      <c r="I28" s="28" t="n">
         <v>120</v>
       </c>
-      <c r="J28" s="27" t="n">
+      <c r="J28" s="28" t="n">
         <v>128</v>
       </c>
-      <c r="K28" s="27" t="n">
+      <c r="K28" s="28" t="n">
         <v>135</v>
       </c>
       <c r="L28" s="23" t="inlineStr">
@@ -1989,8 +2078,12 @@
       </c>
       <c r="M28" s="24" t="inlineStr">
         <is>
-          <t>LULU avg repurchase price (10-K/est.)
-Ctrl+F: "Repurchase of common stock" footnote → avg price paid per share</t>
+          <t>LULU avg repurchase price (10-K/est.)</t>
+        </is>
+      </c>
+      <c r="N28" s="25" t="inlineStr">
+        <is>
+          <t>"Repurchase of common stock" footnote → avg price paid per share</t>
         </is>
       </c>
     </row>
@@ -2052,8 +2145,9 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2114,31 +2208,31 @@
           <t>Ctrl+F lines</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
+      <c r="C2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="D2" s="28" t="inlineStr">
+      <c r="D2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="E2" s="28" t="inlineStr">
+      <c r="E2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="F2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="30" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -2150,35 +2244,35 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="31" t="n">
         <v>8110518</v>
       </c>
-      <c r="D4" s="30" t="n">
+      <c r="D4" s="31" t="n">
         <v>9619278</v>
       </c>
-      <c r="E4" s="30" t="n">
+      <c r="E4" s="31" t="n">
         <v>10588126</v>
       </c>
-      <c r="F4" s="30" t="n">
+      <c r="F4" s="31" t="n">
         <v>11102600</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="26">
         <f>F4*(1+'Assumptions'!G5)</f>
         <v/>
       </c>
-      <c r="H4" s="25">
+      <c r="H4" s="26">
         <f>G4*(1+'Assumptions'!H5)</f>
         <v/>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="26">
         <f>H4*(1+'Assumptions'!I5)</f>
         <v/>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="26">
         <f>I4*(1+'Assumptions'!J5)</f>
         <v/>
       </c>
-      <c r="K4" s="25">
+      <c r="K4" s="26">
         <f>J4*(1+'Assumptions'!K5)</f>
         <v/>
       </c>
@@ -2189,78 +2283,78 @@
           <t>Cost of goods sold</t>
         </is>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="31" t="n">
         <v>3618178</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>4009873</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="31" t="n">
         <v>4317315</v>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="31" t="n">
         <v>4818468</v>
       </c>
-      <c r="G5" s="25">
+      <c r="G5" s="26">
         <f>G4*(1-'Assumptions'!G6)</f>
         <v/>
       </c>
-      <c r="H5" s="25">
+      <c r="H5" s="26">
         <f>H4*(1-'Assumptions'!H6)</f>
         <v/>
       </c>
-      <c r="I5" s="25">
+      <c r="I5" s="26">
         <f>I4*(1-'Assumptions'!I6)</f>
         <v/>
       </c>
-      <c r="J5" s="25">
+      <c r="J5" s="26">
         <f>J4*(1-'Assumptions'!J6)</f>
         <v/>
       </c>
-      <c r="K5" s="25">
+      <c r="K5" s="26">
         <f>K4*(1-'Assumptions'!K6)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="33">
         <f>C4-C5</f>
         <v/>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="33">
         <f>D4-D5</f>
         <v/>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="33">
         <f>E4-E5</f>
         <v/>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="33">
         <f>F4-F5</f>
         <v/>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="33">
         <f>G4-G5</f>
         <v/>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="33">
         <f>H4-H5</f>
         <v/>
       </c>
-      <c r="I6" s="32">
+      <c r="I6" s="33">
         <f>I4-I5</f>
         <v/>
       </c>
-      <c r="J6" s="32">
+      <c r="J6" s="33">
         <f>J4-J5</f>
         <v/>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="33">
         <f>K4-K5</f>
         <v/>
       </c>
@@ -2271,35 +2365,35 @@
           <t>Selling, general &amp; administrative</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="31" t="n">
         <v>2757447</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>3397218</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <v>3762379</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>4066556</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="26">
         <f>G4*'Assumptions'!G7</f>
         <v/>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="26">
         <f>H4*'Assumptions'!H7</f>
         <v/>
       </c>
-      <c r="I7" s="25">
+      <c r="I7" s="26">
         <f>I4*'Assumptions'!I7</f>
         <v/>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="26">
         <f>J4*'Assumptions'!J7</f>
         <v/>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="26">
         <f>K4*'Assumptions'!K7</f>
         <v/>
       </c>
@@ -2310,78 +2404,78 @@
           <t>Amortization of intangibles / other</t>
         </is>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="31" t="n">
         <v>406485</v>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="31" t="n">
         <v>79511</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="31" t="n">
         <v>2735</v>
       </c>
-      <c r="F8" s="30" t="n">
+      <c r="F8" s="31" t="n">
         <v>6961</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="26">
         <f>'Assumptions'!G8</f>
         <v/>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="26">
         <f>'Assumptions'!H8</f>
         <v/>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="26">
         <f>'Assumptions'!I8</f>
         <v/>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="26">
         <f>'Assumptions'!J8</f>
         <v/>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="26">
         <f>'Assumptions'!K8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Operating income (EBIT)</t>
         </is>
       </c>
-      <c r="C9" s="32">
+      <c r="C9" s="33">
         <f>C6-C7-C8</f>
         <v/>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="33">
         <f>D6-D7-D8</f>
         <v/>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="33">
         <f>E6-E7-E8</f>
         <v/>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="33">
         <f>F6-F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="33">
         <f>G6-G7-G8</f>
         <v/>
       </c>
-      <c r="H9" s="32">
+      <c r="H9" s="33">
         <f>H6-H7-H8</f>
         <v/>
       </c>
-      <c r="I9" s="32">
+      <c r="I9" s="33">
         <f>I6-I7-I8</f>
         <v/>
       </c>
-      <c r="J9" s="32">
+      <c r="J9" s="33">
         <f>J6-J7-J8</f>
         <v/>
       </c>
-      <c r="K9" s="32">
+      <c r="K9" s="33">
         <f>K6-K7-K8</f>
         <v/>
       </c>
@@ -2392,78 +2486,78 @@
           <t>Other income, net</t>
         </is>
       </c>
-      <c r="C10" s="30" t="n">
+      <c r="C10" s="31" t="n">
         <v>4163</v>
       </c>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="31" t="n">
         <v>43059</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="31" t="n">
         <v>70380</v>
       </c>
-      <c r="F10" s="30" t="n">
+      <c r="F10" s="31" t="n">
         <v>28352</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="26">
         <f>'Assumptions'!G9</f>
         <v/>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="26">
         <f>'Assumptions'!H9</f>
         <v/>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="26">
         <f>'Assumptions'!I9</f>
         <v/>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="26">
         <f>'Assumptions'!J9</f>
         <v/>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="26">
         <f>'Assumptions'!K9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Pre-tax income</t>
         </is>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="33">
         <f>C9+C10</f>
         <v/>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="33">
         <f>D9+D10</f>
         <v/>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="33">
         <f>E9+E10</f>
         <v/>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="33">
         <f>F9+F10</f>
         <v/>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="33">
         <f>G9+G10</f>
         <v/>
       </c>
-      <c r="H11" s="32">
+      <c r="H11" s="33">
         <f>H9+H10</f>
         <v/>
       </c>
-      <c r="I11" s="32">
+      <c r="I11" s="33">
         <f>I9+I10</f>
         <v/>
       </c>
-      <c r="J11" s="32">
+      <c r="J11" s="33">
         <f>J9+J10</f>
         <v/>
       </c>
-      <c r="K11" s="32">
+      <c r="K11" s="33">
         <f>K9+K10</f>
         <v/>
       </c>
@@ -2474,78 +2568,78 @@
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="C12" s="30" t="n">
+      <c r="C12" s="31" t="n">
         <v>477771</v>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <v>625545</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="31" t="n">
         <v>761461</v>
       </c>
-      <c r="F12" s="30" t="n">
+      <c r="F12" s="31" t="n">
         <v>659784</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="26">
         <f>G11*'Assumptions'!G10</f>
         <v/>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="26">
         <f>H11*'Assumptions'!H10</f>
         <v/>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="26">
         <f>I11*'Assumptions'!I10</f>
         <v/>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="26">
         <f>J11*'Assumptions'!J10</f>
         <v/>
       </c>
-      <c r="K12" s="25">
+      <c r="K12" s="26">
         <f>K11*'Assumptions'!K10</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="34">
         <f>C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="34">
         <f>D11-D12</f>
         <v/>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="34">
         <f>E11-E12</f>
         <v/>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="34">
         <f>F11-F12</f>
         <v/>
       </c>
-      <c r="G13" s="33">
+      <c r="G13" s="34">
         <f>G11-G12</f>
         <v/>
       </c>
-      <c r="H13" s="33">
+      <c r="H13" s="34">
         <f>H11-H12</f>
         <v/>
       </c>
-      <c r="I13" s="33">
+      <c r="I13" s="34">
         <f>I11-I12</f>
         <v/>
       </c>
-      <c r="J13" s="33">
+      <c r="J13" s="34">
         <f>J11-J12</f>
         <v/>
       </c>
-      <c r="K13" s="33">
+      <c r="K13" s="34">
         <f>K11-K12</f>
         <v/>
       </c>
@@ -2556,80 +2650,80 @@
           <t>Diluted weighted-avg shares (000)</t>
         </is>
       </c>
-      <c r="C15" s="30" t="n">
+      <c r="C15" s="31" t="n">
         <v>128017</v>
       </c>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="31" t="n">
         <v>127060</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="31" t="n">
         <v>123935</v>
       </c>
-      <c r="F15" s="30" t="n">
+      <c r="F15" s="31" t="n">
         <v>119068</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="26">
         <f>F15-'Assumptions'!G27/'Assumptions'!G28</f>
         <v/>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="26">
         <f>G15-'Assumptions'!H27/'Assumptions'!H28</f>
         <v/>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="26">
         <f>H15-'Assumptions'!I27/'Assumptions'!I28</f>
         <v/>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="26">
         <f>I15-'Assumptions'!J27/'Assumptions'!J28</f>
         <v/>
       </c>
-      <c r="K15" s="25">
+      <c r="K15" s="26">
         <f>J15-'Assumptions'!K27/'Assumptions'!K28</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Diluted EPS ($)</t>
         </is>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="35" t="n">
         <v>6.68</v>
       </c>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="35" t="n">
         <v>12.2</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="35" t="n">
         <v>14.64</v>
       </c>
-      <c r="F16" s="34" t="n">
+      <c r="F16" s="35" t="n">
         <v>13.26</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16" s="36">
         <f>G13/G15</f>
         <v/>
       </c>
-      <c r="H16" s="35">
+      <c r="H16" s="36">
         <f>H13/H15</f>
         <v/>
       </c>
-      <c r="I16" s="35">
+      <c r="I16" s="36">
         <f>I13/I15</f>
         <v/>
       </c>
-      <c r="J16" s="35">
+      <c r="J16" s="36">
         <f>J13/J15</f>
         <v/>
       </c>
-      <c r="K16" s="35">
+      <c r="K16" s="36">
         <f>K13/K15</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="36" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>Margins &amp; growth</t>
         </is>
@@ -2645,174 +2739,174 @@
       <c r="K18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="C19" s="38">
+      <c r="C19" s="39">
         <f>C6/C4</f>
         <v/>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="39">
         <f>D6/D4</f>
         <v/>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="39">
         <f>E6/E4</f>
         <v/>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="39">
         <f>F6/F4</f>
         <v/>
       </c>
-      <c r="G19" s="38">
+      <c r="G19" s="39">
         <f>G6/G4</f>
         <v/>
       </c>
-      <c r="H19" s="38">
+      <c r="H19" s="39">
         <f>H6/H4</f>
         <v/>
       </c>
-      <c r="I19" s="38">
+      <c r="I19" s="39">
         <f>I6/I4</f>
         <v/>
       </c>
-      <c r="J19" s="38">
+      <c r="J19" s="39">
         <f>J6/J4</f>
         <v/>
       </c>
-      <c r="K19" s="38">
+      <c r="K19" s="39">
         <f>K6/K4</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="37" t="inlineStr">
+      <c r="A20" s="38" t="inlineStr">
         <is>
           <t>Operating margin %</t>
         </is>
       </c>
-      <c r="C20" s="38">
+      <c r="C20" s="39">
         <f>C9/C4</f>
         <v/>
       </c>
-      <c r="D20" s="38">
+      <c r="D20" s="39">
         <f>D9/D4</f>
         <v/>
       </c>
-      <c r="E20" s="38">
+      <c r="E20" s="39">
         <f>E9/E4</f>
         <v/>
       </c>
-      <c r="F20" s="38">
+      <c r="F20" s="39">
         <f>F9/F4</f>
         <v/>
       </c>
-      <c r="G20" s="38">
+      <c r="G20" s="39">
         <f>G9/G4</f>
         <v/>
       </c>
-      <c r="H20" s="38">
+      <c r="H20" s="39">
         <f>H9/H4</f>
         <v/>
       </c>
-      <c r="I20" s="38">
+      <c r="I20" s="39">
         <f>I9/I4</f>
         <v/>
       </c>
-      <c r="J20" s="38">
+      <c r="J20" s="39">
         <f>J9/J4</f>
         <v/>
       </c>
-      <c r="K20" s="38">
+      <c r="K20" s="39">
         <f>K9/K4</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>Net margin %</t>
         </is>
       </c>
-      <c r="C21" s="38">
+      <c r="C21" s="39">
         <f>C13/C4</f>
         <v/>
       </c>
-      <c r="D21" s="38">
+      <c r="D21" s="39">
         <f>D13/D4</f>
         <v/>
       </c>
-      <c r="E21" s="38">
+      <c r="E21" s="39">
         <f>E13/E4</f>
         <v/>
       </c>
-      <c r="F21" s="38">
+      <c r="F21" s="39">
         <f>F13/F4</f>
         <v/>
       </c>
-      <c r="G21" s="38">
+      <c r="G21" s="39">
         <f>G13/G4</f>
         <v/>
       </c>
-      <c r="H21" s="38">
+      <c r="H21" s="39">
         <f>H13/H4</f>
         <v/>
       </c>
-      <c r="I21" s="38">
+      <c r="I21" s="39">
         <f>I13/I4</f>
         <v/>
       </c>
-      <c r="J21" s="38">
+      <c r="J21" s="39">
         <f>J13/J4</f>
         <v/>
       </c>
-      <c r="K21" s="38">
+      <c r="K21" s="39">
         <f>K13/K4</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="37" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="C22" s="39" t="inlineStr">
+      <c r="C22" s="40" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="D22" s="38">
+      <c r="D22" s="39">
         <f>D4/C4-1</f>
         <v/>
       </c>
-      <c r="E22" s="38">
+      <c r="E22" s="39">
         <f>E4/D4-1</f>
         <v/>
       </c>
-      <c r="F22" s="38">
+      <c r="F22" s="39">
         <f>F4/E4-1</f>
         <v/>
       </c>
-      <c r="G22" s="38">
+      <c r="G22" s="39">
         <f>G4/F4-1</f>
         <v/>
       </c>
-      <c r="H22" s="38">
+      <c r="H22" s="39">
         <f>H4/G4-1</f>
         <v/>
       </c>
-      <c r="I22" s="38">
+      <c r="I22" s="39">
         <f>I4/H4-1</f>
         <v/>
       </c>
-      <c r="J22" s="38">
+      <c r="J22" s="39">
         <f>J4/I4-1</f>
         <v/>
       </c>
-      <c r="K22" s="38">
+      <c r="K22" s="39">
         <f>K4/J4-1</f>
         <v/>
       </c>
@@ -2879,8 +2973,9 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2941,31 +3036,31 @@
           <t>Ctrl+F lines</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
+      <c r="C2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="D2" s="28" t="inlineStr">
+      <c r="D2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="E2" s="28" t="inlineStr">
+      <c r="E2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="F2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="30" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -2988,7 +3083,7 @@
       <c r="K4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="40" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>Current assets:</t>
         </is>
@@ -3000,35 +3095,35 @@
           <t>Cash &amp; cash equivalents</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="31" t="n">
         <v>1154867</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <v>2243971</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="31" t="n">
         <v>1984336</v>
       </c>
-      <c r="F6" s="30" t="n">
+      <c r="F6" s="31" t="n">
         <v>1807202</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="26">
         <f>'Cash Flow'!G33</f>
         <v/>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="26">
         <f>'Cash Flow'!H33</f>
         <v/>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="26">
         <f>'Cash Flow'!I33</f>
         <v/>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="26">
         <f>'Cash Flow'!J33</f>
         <v/>
       </c>
-      <c r="K6" s="25">
+      <c r="K6" s="26">
         <f>'Cash Flow'!K33</f>
         <v/>
       </c>
@@ -3039,35 +3134,35 @@
           <t>Inventories</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="31" t="n">
         <v>1447367</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>1323602</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <v>1442081</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>1700753</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="26">
         <f>'Income Statement'!G5*'Assumptions'!G16</f>
         <v/>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="26">
         <f>'Income Statement'!H5*'Assumptions'!H16</f>
         <v/>
       </c>
-      <c r="I7" s="25">
+      <c r="I7" s="26">
         <f>'Income Statement'!I5*'Assumptions'!I16</f>
         <v/>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="26">
         <f>'Income Statement'!J5*'Assumptions'!J16</f>
         <v/>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="26">
         <f>'Income Statement'!K5*'Assumptions'!K16</f>
         <v/>
       </c>
@@ -3078,80 +3173,80 @@
           <t>Other current assets</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="26" t="n">
         <v>557219</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="26" t="n">
         <v>493004</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="26" t="n">
         <v>553885</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="26" t="n">
         <v>754746</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G19</f>
         <v/>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H19</f>
         <v/>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I19</f>
         <v/>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J19</f>
         <v/>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K19</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="C9" s="41" t="n">
+      <c r="C9" s="42" t="n">
         <v>3159453</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="42" t="n">
         <v>4060577</v>
       </c>
-      <c r="E9" s="41" t="n">
+      <c r="E9" s="42" t="n">
         <v>3980302</v>
       </c>
-      <c r="F9" s="41" t="n">
+      <c r="F9" s="42" t="n">
         <v>4262701</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="33">
         <f>G6+G7+G8</f>
         <v/>
       </c>
-      <c r="H9" s="32">
+      <c r="H9" s="33">
         <f>H6+H7+H8</f>
         <v/>
       </c>
-      <c r="I9" s="32">
+      <c r="I9" s="33">
         <f>I6+I7+I8</f>
         <v/>
       </c>
-      <c r="J9" s="32">
+      <c r="J9" s="33">
         <f>J6+J7+J8</f>
         <v/>
       </c>
-      <c r="K9" s="32">
+      <c r="K9" s="33">
         <f>K6+K7+K8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
         <is>
           <t>Non-current assets:</t>
         </is>
@@ -3163,35 +3258,35 @@
           <t>Property &amp; equipment, net</t>
         </is>
       </c>
-      <c r="C11" s="30" t="n">
+      <c r="C11" s="31" t="n">
         <v>1269614</v>
       </c>
-      <c r="D11" s="30" t="n">
+      <c r="D11" s="31" t="n">
         <v>1545811</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="31" t="n">
         <v>1780617</v>
       </c>
-      <c r="F11" s="30" t="n">
+      <c r="F11" s="31" t="n">
         <v>2033720</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="26">
         <f>F11+'Income Statement'!G4*'Assumptions'!G13-'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="26">
         <f>G11+'Income Statement'!H4*'Assumptions'!H13-'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="26">
         <f>H11+'Income Statement'!I4*'Assumptions'!I13-'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J11" s="25">
+      <c r="J11" s="26">
         <f>I11+'Income Statement'!J4*'Assumptions'!J13-'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K11" s="25">
+      <c r="K11" s="26">
         <f>J11+'Income Statement'!K4*'Assumptions'!K13-'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
@@ -3202,35 +3297,35 @@
           <t>Operating lease right-of-use assets</t>
         </is>
       </c>
-      <c r="C12" s="30" t="n">
+      <c r="C12" s="31" t="n">
         <v>969419</v>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <v>1265610</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="31" t="n">
         <v>1416256</v>
       </c>
-      <c r="F12" s="30" t="n">
+      <c r="F12" s="31" t="n">
         <v>1630181</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G20</f>
         <v/>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H20</f>
         <v/>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I20</f>
         <v/>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J20</f>
         <v/>
       </c>
-      <c r="K12" s="25">
+      <c r="K12" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K20</f>
         <v/>
       </c>
@@ -3241,35 +3336,35 @@
           <t>Goodwill &amp; intangible assets</t>
         </is>
       </c>
-      <c r="C13" s="30" t="n">
+      <c r="C13" s="31" t="n">
         <v>46105</v>
       </c>
-      <c r="D13" s="30" t="n">
+      <c r="D13" s="31" t="n">
         <v>24083</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="31" t="n">
         <v>171191</v>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="31" t="n">
         <v>191194</v>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="26">
         <f>F13</f>
         <v/>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="26">
         <f>G13</f>
         <v/>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="26">
         <f>H13</f>
         <v/>
       </c>
-      <c r="J13" s="25">
+      <c r="J13" s="26">
         <f>I13</f>
         <v/>
       </c>
-      <c r="K13" s="25">
+      <c r="K13" s="26">
         <f>J13</f>
         <v/>
       </c>
@@ -3280,74 +3375,74 @@
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="26" t="n">
         <v>162447</v>
       </c>
-      <c r="D14" s="25" t="n">
+      <c r="D14" s="26" t="n">
         <v>195860</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="26" t="n">
         <v>254926</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F14" s="26" t="n">
         <v>338947</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G21</f>
         <v/>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H21</f>
         <v/>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I21</f>
         <v/>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J21</f>
         <v/>
       </c>
-      <c r="K14" s="25">
+      <c r="K14" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K21</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="C15" s="42" t="n">
+      <c r="C15" s="43" t="n">
         <v>5607038</v>
       </c>
-      <c r="D15" s="42" t="n">
+      <c r="D15" s="43" t="n">
         <v>7091941</v>
       </c>
-      <c r="E15" s="42" t="n">
+      <c r="E15" s="43" t="n">
         <v>7603292</v>
       </c>
-      <c r="F15" s="42" t="n">
+      <c r="F15" s="43" t="n">
         <v>8456743</v>
       </c>
-      <c r="G15" s="33">
+      <c r="G15" s="34">
         <f>G9+G11+G12+G13+G14</f>
         <v/>
       </c>
-      <c r="H15" s="33">
+      <c r="H15" s="34">
         <f>H9+H11+H12+H13+H14</f>
         <v/>
       </c>
-      <c r="I15" s="33">
+      <c r="I15" s="34">
         <f>I9+I11+I12+I13+I14</f>
         <v/>
       </c>
-      <c r="J15" s="33">
+      <c r="J15" s="34">
         <f>J9+J11+J12+J13+J14</f>
         <v/>
       </c>
-      <c r="K15" s="33">
+      <c r="K15" s="34">
         <f>K9+K11+K12+K13+K14</f>
         <v/>
       </c>
@@ -3369,7 +3464,7 @@
       <c r="K17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="40" t="inlineStr">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
@@ -3381,35 +3476,35 @@
           <t>Accounts payable</t>
         </is>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="31" t="n">
         <v>172732</v>
       </c>
-      <c r="D19" s="30" t="n">
+      <c r="D19" s="31" t="n">
         <v>348441</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="31" t="n">
         <v>271406</v>
       </c>
-      <c r="F19" s="30" t="n">
+      <c r="F19" s="31" t="n">
         <v>331421</v>
       </c>
-      <c r="G19" s="25">
+      <c r="G19" s="26">
         <f>'Income Statement'!G5*'Assumptions'!G17</f>
         <v/>
       </c>
-      <c r="H19" s="25">
+      <c r="H19" s="26">
         <f>'Income Statement'!H5*'Assumptions'!H17</f>
         <v/>
       </c>
-      <c r="I19" s="25">
+      <c r="I19" s="26">
         <f>'Income Statement'!I5*'Assumptions'!I17</f>
         <v/>
       </c>
-      <c r="J19" s="25">
+      <c r="J19" s="26">
         <f>'Income Statement'!J5*'Assumptions'!J17</f>
         <v/>
       </c>
-      <c r="K19" s="25">
+      <c r="K19" s="26">
         <f>'Income Statement'!K5*'Assumptions'!K17</f>
         <v/>
       </c>
@@ -3420,35 +3515,35 @@
           <t>Accrued liabilities</t>
         </is>
       </c>
-      <c r="C20" s="30" t="n">
+      <c r="C20" s="31" t="n">
         <v>399223</v>
       </c>
-      <c r="D20" s="30" t="n">
+      <c r="D20" s="31" t="n">
         <v>348555</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="31" t="n">
         <v>559463</v>
       </c>
-      <c r="F20" s="30" t="n">
+      <c r="F20" s="31" t="n">
         <v>662982</v>
       </c>
-      <c r="G20" s="25">
+      <c r="G20" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G18</f>
         <v/>
       </c>
-      <c r="H20" s="25">
+      <c r="H20" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H18</f>
         <v/>
       </c>
-      <c r="I20" s="25">
+      <c r="I20" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I18</f>
         <v/>
       </c>
-      <c r="J20" s="25">
+      <c r="J20" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J18</f>
         <v/>
       </c>
-      <c r="K20" s="25">
+      <c r="K20" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K18</f>
         <v/>
       </c>
@@ -3459,35 +3554,35 @@
           <t>Operating lease liabilities (current)</t>
         </is>
       </c>
-      <c r="C21" s="30" t="n">
+      <c r="C21" s="31" t="n">
         <v>207972</v>
       </c>
-      <c r="D21" s="30" t="n">
+      <c r="D21" s="31" t="n">
         <v>249270</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="E21" s="31" t="n">
         <v>275154</v>
       </c>
-      <c r="F21" s="30" t="n">
+      <c r="F21" s="31" t="n">
         <v>298724</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G22</f>
         <v/>
       </c>
-      <c r="H21" s="25">
+      <c r="H21" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H22</f>
         <v/>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I22</f>
         <v/>
       </c>
-      <c r="J21" s="25">
+      <c r="J21" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J22</f>
         <v/>
       </c>
-      <c r="K21" s="25">
+      <c r="K21" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K22</f>
         <v/>
       </c>
@@ -3498,80 +3593,80 @@
           <t>Other current liabilities</t>
         </is>
       </c>
-      <c r="C22" s="25" t="n">
+      <c r="C22" s="26" t="n">
         <v>712271</v>
       </c>
-      <c r="D22" s="25" t="n">
+      <c r="D22" s="26" t="n">
         <v>684995</v>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E22" s="26" t="n">
         <v>733607</v>
       </c>
-      <c r="F22" s="25" t="n">
+      <c r="F22" s="26" t="n">
         <v>594421</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G24</f>
         <v/>
       </c>
-      <c r="H22" s="25">
+      <c r="H22" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H24</f>
         <v/>
       </c>
-      <c r="I22" s="25">
+      <c r="I22" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I24</f>
         <v/>
       </c>
-      <c r="J22" s="25">
+      <c r="J22" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J24</f>
         <v/>
       </c>
-      <c r="K22" s="25">
+      <c r="K22" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K24</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Total current liabilities</t>
         </is>
       </c>
-      <c r="C23" s="41" t="n">
+      <c r="C23" s="42" t="n">
         <v>1492198</v>
       </c>
-      <c r="D23" s="41" t="n">
+      <c r="D23" s="42" t="n">
         <v>1631261</v>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E23" s="42" t="n">
         <v>1839630</v>
       </c>
-      <c r="F23" s="41" t="n">
+      <c r="F23" s="42" t="n">
         <v>1887548</v>
       </c>
-      <c r="G23" s="32">
+      <c r="G23" s="33">
         <f>G19+G20+G21+G22</f>
         <v/>
       </c>
-      <c r="H23" s="32">
+      <c r="H23" s="33">
         <f>H19+H20+H21+H22</f>
         <v/>
       </c>
-      <c r="I23" s="32">
+      <c r="I23" s="33">
         <f>I19+I20+I21+I22</f>
         <v/>
       </c>
-      <c r="J23" s="32">
+      <c r="J23" s="33">
         <f>J19+J20+J21+J22</f>
         <v/>
       </c>
-      <c r="K23" s="32">
+      <c r="K23" s="33">
         <f>K19+K20+K21+K22</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="40" t="inlineStr">
+      <c r="A24" s="41" t="inlineStr">
         <is>
           <t>Non-current liabilities:</t>
         </is>
@@ -3583,35 +3678,35 @@
           <t>Operating lease liabilities (non-current)</t>
         </is>
       </c>
-      <c r="C25" s="30" t="n">
+      <c r="C25" s="31" t="n">
         <v>862362</v>
       </c>
-      <c r="D25" s="30" t="n">
+      <c r="D25" s="31" t="n">
         <v>1154012</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="E25" s="31" t="n">
         <v>1300637</v>
       </c>
-      <c r="F25" s="30" t="n">
+      <c r="F25" s="31" t="n">
         <v>1499717</v>
       </c>
-      <c r="G25" s="25">
+      <c r="G25" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G23</f>
         <v/>
       </c>
-      <c r="H25" s="25">
+      <c r="H25" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H23</f>
         <v/>
       </c>
-      <c r="I25" s="25">
+      <c r="I25" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I23</f>
         <v/>
       </c>
-      <c r="J25" s="25">
+      <c r="J25" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J23</f>
         <v/>
       </c>
-      <c r="K25" s="25">
+      <c r="K25" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K23</f>
         <v/>
       </c>
@@ -3622,35 +3717,35 @@
           <t>Deferred income taxes</t>
         </is>
       </c>
-      <c r="C26" s="30" t="n">
+      <c r="C26" s="31" t="n">
         <v>55084</v>
       </c>
-      <c r="D26" s="30" t="n">
+      <c r="D26" s="31" t="n">
         <v>29522</v>
       </c>
-      <c r="E26" s="30" t="n">
+      <c r="E26" s="31" t="n">
         <v>98188</v>
       </c>
-      <c r="F26" s="30" t="n">
+      <c r="F26" s="31" t="n">
         <v>52278</v>
       </c>
-      <c r="G26" s="25">
+      <c r="G26" s="26">
         <f>F26</f>
         <v/>
       </c>
-      <c r="H26" s="25">
+      <c r="H26" s="26">
         <f>G26</f>
         <v/>
       </c>
-      <c r="I26" s="25">
+      <c r="I26" s="26">
         <f>H26</f>
         <v/>
       </c>
-      <c r="J26" s="25">
+      <c r="J26" s="26">
         <f>I26</f>
         <v/>
       </c>
-      <c r="K26" s="25">
+      <c r="K26" s="26">
         <f>J26</f>
         <v/>
       </c>
@@ -3661,80 +3756,80 @@
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C27" s="26" t="n">
         <v>48595</v>
       </c>
-      <c r="D27" s="25" t="n">
+      <c r="D27" s="26" t="n">
         <v>45065</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="26" t="n">
         <v>40790</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F27" s="26" t="n">
         <v>55360</v>
       </c>
-      <c r="G27" s="25">
+      <c r="G27" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G25</f>
         <v/>
       </c>
-      <c r="H27" s="25">
+      <c r="H27" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H25</f>
         <v/>
       </c>
-      <c r="I27" s="25">
+      <c r="I27" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I25</f>
         <v/>
       </c>
-      <c r="J27" s="25">
+      <c r="J27" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J25</f>
         <v/>
       </c>
-      <c r="K27" s="25">
+      <c r="K27" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="32" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>2458239</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>2859860</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="42" t="n">
         <v>3279245</v>
       </c>
-      <c r="F28" s="41" t="n">
+      <c r="F28" s="42" t="n">
         <v>3494903</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="33">
         <f>G23+G25+G26+G27</f>
         <v/>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="33">
         <f>H23+H25+H26+H27</f>
         <v/>
       </c>
-      <c r="I28" s="32">
+      <c r="I28" s="33">
         <f>I23+I25+I26+I27</f>
         <v/>
       </c>
-      <c r="J28" s="32">
+      <c r="J28" s="33">
         <f>J23+J25+J26+J27</f>
         <v/>
       </c>
-      <c r="K28" s="32">
+      <c r="K28" s="33">
         <f>K23+K25+K26+K27</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="40" t="inlineStr">
+      <c r="A30" s="41" t="inlineStr">
         <is>
           <t>Shareholders' equity:</t>
         </is>
@@ -3746,35 +3841,35 @@
           <t>Common stock &amp; additional paid-in capital</t>
         </is>
       </c>
-      <c r="C31" s="30" t="n">
+      <c r="C31" s="31" t="n">
         <v>475256</v>
       </c>
-      <c r="D31" s="30" t="n">
+      <c r="D31" s="31" t="n">
         <v>575975</v>
       </c>
-      <c r="E31" s="30" t="n">
+      <c r="E31" s="31" t="n">
         <v>638771</v>
       </c>
-      <c r="F31" s="30" t="n">
+      <c r="F31" s="31" t="n">
         <v>669949</v>
       </c>
-      <c r="G31" s="25">
+      <c r="G31" s="26">
         <f>F31+'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H31" s="25">
+      <c r="H31" s="26">
         <f>G31+'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I31" s="25">
+      <c r="I31" s="26">
         <f>H31+'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J31" s="25">
+      <c r="J31" s="26">
         <f>I31+'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K31" s="25">
+      <c r="K31" s="26">
         <f>J31+'Assumptions'!K14</f>
         <v/>
       </c>
@@ -3785,35 +3880,35 @@
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="C32" s="30" t="n">
+      <c r="C32" s="31" t="n">
         <v>2926127</v>
       </c>
-      <c r="D32" s="30" t="n">
+      <c r="D32" s="31" t="n">
         <v>3920362</v>
       </c>
-      <c r="E32" s="30" t="n">
+      <c r="E32" s="31" t="n">
         <v>4109717</v>
       </c>
-      <c r="F32" s="30" t="n">
+      <c r="F32" s="31" t="n">
         <v>4522581</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="26">
         <f>F32+'Income Statement'!G13-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="26">
         <f>G32+'Income Statement'!H13-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I32" s="25">
+      <c r="I32" s="26">
         <f>H32+'Income Statement'!I13-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J32" s="25">
+      <c r="J32" s="26">
         <f>I32+'Income Statement'!J13-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K32" s="25">
+      <c r="K32" s="26">
         <f>J32+'Income Statement'!K13-'Assumptions'!K27</f>
         <v/>
       </c>
@@ -3824,160 +3919,160 @@
           <t>Accumulated other comprehensive loss</t>
         </is>
       </c>
-      <c r="C33" s="30" t="n">
+      <c r="C33" s="31" t="n">
         <v>-252584</v>
       </c>
-      <c r="D33" s="30" t="n">
+      <c r="D33" s="31" t="n">
         <v>-264256</v>
       </c>
-      <c r="E33" s="30" t="n">
+      <c r="E33" s="31" t="n">
         <v>-424441</v>
       </c>
-      <c r="F33" s="30" t="n">
+      <c r="F33" s="31" t="n">
         <v>-230690</v>
       </c>
-      <c r="G33" s="25">
+      <c r="G33" s="26">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="25">
+      <c r="H33" s="26">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I33" s="25">
+      <c r="I33" s="26">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J33" s="25">
+      <c r="J33" s="26">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K33" s="25">
+      <c r="K33" s="26">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="32" t="inlineStr">
         <is>
           <t>TOTAL SHAREHOLDERS' EQUITY</t>
         </is>
       </c>
-      <c r="C34" s="41" t="n">
+      <c r="C34" s="42" t="n">
         <v>3148799</v>
       </c>
-      <c r="D34" s="41" t="n">
+      <c r="D34" s="42" t="n">
         <v>4232081</v>
       </c>
-      <c r="E34" s="41" t="n">
+      <c r="E34" s="42" t="n">
         <v>4324047</v>
       </c>
-      <c r="F34" s="41" t="n">
+      <c r="F34" s="42" t="n">
         <v>4961840</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="33">
         <f>G31+G32+G33</f>
         <v/>
       </c>
-      <c r="H34" s="32">
+      <c r="H34" s="33">
         <f>H31+H32+H33</f>
         <v/>
       </c>
-      <c r="I34" s="32">
+      <c r="I34" s="33">
         <f>I31+I32+I33</f>
         <v/>
       </c>
-      <c r="J34" s="32">
+      <c r="J34" s="33">
         <f>J31+J32+J33</f>
         <v/>
       </c>
-      <c r="K34" s="32">
+      <c r="K34" s="33">
         <f>K31+K32+K33</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="31" t="inlineStr">
+      <c r="A35" s="32" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="C35" s="33">
+      <c r="C35" s="34">
         <f>C28+C34</f>
         <v/>
       </c>
-      <c r="D35" s="33">
+      <c r="D35" s="34">
         <f>D28+D34</f>
         <v/>
       </c>
-      <c r="E35" s="33">
+      <c r="E35" s="34">
         <f>E28+E34</f>
         <v/>
       </c>
-      <c r="F35" s="33">
+      <c r="F35" s="34">
         <f>F28+F34</f>
         <v/>
       </c>
-      <c r="G35" s="33">
+      <c r="G35" s="34">
         <f>G28+G34</f>
         <v/>
       </c>
-      <c r="H35" s="33">
+      <c r="H35" s="34">
         <f>H28+H34</f>
         <v/>
       </c>
-      <c r="I35" s="33">
+      <c r="I35" s="34">
         <f>I28+I34</f>
         <v/>
       </c>
-      <c r="J35" s="33">
+      <c r="J35" s="34">
         <f>J28+J34</f>
         <v/>
       </c>
-      <c r="K35" s="33">
+      <c r="K35" s="34">
         <f>K28+K34</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="37" t="inlineStr">
+      <c r="A37" s="38" t="inlineStr">
         <is>
           <t>Balance check (Assets − L&amp;E)</t>
         </is>
       </c>
-      <c r="C37" s="43">
+      <c r="C37" s="44">
         <f>C15-C35</f>
         <v/>
       </c>
-      <c r="D37" s="43">
+      <c r="D37" s="44">
         <f>D15-D35</f>
         <v/>
       </c>
-      <c r="E37" s="43">
+      <c r="E37" s="44">
         <f>E15-E35</f>
         <v/>
       </c>
-      <c r="F37" s="43">
+      <c r="F37" s="44">
         <f>F15-F35</f>
         <v/>
       </c>
-      <c r="G37" s="43">
+      <c r="G37" s="44">
         <f>G15-G35</f>
         <v/>
       </c>
-      <c r="H37" s="43">
+      <c r="H37" s="44">
         <f>H15-H35</f>
         <v/>
       </c>
-      <c r="I37" s="43">
+      <c r="I37" s="44">
         <f>I15-I35</f>
         <v/>
       </c>
-      <c r="J37" s="43">
+      <c r="J37" s="44">
         <f>J15-J35</f>
         <v/>
       </c>
-      <c r="K37" s="43">
+      <c r="K37" s="44">
         <f>K15-K35</f>
         <v/>
       </c>
@@ -4084,8 +4179,9 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -4146,31 +4242,31 @@
           <t>Ctrl+F lines</t>
         </is>
       </c>
-      <c r="C2" s="28" t="inlineStr">
+      <c r="C2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="D2" s="28" t="inlineStr">
+      <c r="D2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="E2" s="28" t="inlineStr">
+      <c r="E2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="F2" s="29" t="inlineStr">
         <is>
           <t>10-K
 Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="30" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
@@ -4198,35 +4294,35 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="31" t="n">
         <v>854800</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>1550190</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="31" t="n">
         <v>1814616</v>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="31" t="n">
         <v>1579183</v>
       </c>
-      <c r="G5" s="25">
+      <c r="G5" s="26">
         <f>'Income Statement'!G13</f>
         <v/>
       </c>
-      <c r="H5" s="25">
+      <c r="H5" s="26">
         <f>'Income Statement'!H13</f>
         <v/>
       </c>
-      <c r="I5" s="25">
+      <c r="I5" s="26">
         <f>'Income Statement'!I13</f>
         <v/>
       </c>
-      <c r="J5" s="25">
+      <c r="J5" s="26">
         <f>'Income Statement'!J13</f>
         <v/>
       </c>
-      <c r="K5" s="25">
+      <c r="K5" s="26">
         <f>'Income Statement'!K13</f>
         <v/>
       </c>
@@ -4237,35 +4333,35 @@
           <t>Depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="31" t="n">
         <v>291791</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <v>379384</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="31" t="n">
         <v>446524</v>
       </c>
-      <c r="F6" s="30" t="n">
+      <c r="F6" s="31" t="n">
         <v>496228</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="26">
         <f>'Income Statement'!G4*'Assumptions'!G12</f>
         <v/>
       </c>
-      <c r="H6" s="25">
+      <c r="H6" s="26">
         <f>'Income Statement'!H4*'Assumptions'!H12</f>
         <v/>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I12</f>
         <v/>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J12</f>
         <v/>
       </c>
-      <c r="K6" s="25">
+      <c r="K6" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K12</f>
         <v/>
       </c>
@@ -4276,35 +4372,35 @@
           <t>Stock-based compensation</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="31" t="n">
         <v>78075</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>93560</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <v>90011</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>62203</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="26">
         <f>'Assumptions'!G14</f>
         <v/>
       </c>
-      <c r="H7" s="25">
+      <c r="H7" s="26">
         <f>'Assumptions'!H14</f>
         <v/>
       </c>
-      <c r="I7" s="25">
+      <c r="I7" s="26">
         <f>'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="26">
         <f>'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K7" s="25">
+      <c r="K7" s="26">
         <f>'Assumptions'!K14</f>
         <v/>
       </c>
@@ -4315,43 +4411,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="44" t="inlineStr">
+      <c r="E8" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="44" t="inlineStr">
+      <c r="F8" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="26">
         <f>-('Balance Sheet'!G7-'Balance Sheet'!F7)</f>
         <v/>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="26">
         <f>-('Balance Sheet'!H7-'Balance Sheet'!G7)</f>
         <v/>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="26">
         <f>-('Balance Sheet'!I7-'Balance Sheet'!H7)</f>
         <v/>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="26">
         <f>-('Balance Sheet'!J7-'Balance Sheet'!I7)</f>
         <v/>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="26">
         <f>-('Balance Sheet'!K7-'Balance Sheet'!J7)</f>
         <v/>
       </c>
@@ -4362,43 +4458,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
         </is>
       </c>
-      <c r="C9" s="44" t="inlineStr">
+      <c r="C9" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="44" t="inlineStr">
+      <c r="D9" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="44" t="inlineStr">
+      <c r="E9" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="44" t="inlineStr">
+      <c r="F9" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="26">
         <f>-('Balance Sheet'!G8-'Balance Sheet'!F8)</f>
         <v/>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="26">
         <f>-('Balance Sheet'!H8-'Balance Sheet'!G8)</f>
         <v/>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="26">
         <f>-('Balance Sheet'!I8-'Balance Sheet'!H8)</f>
         <v/>
       </c>
-      <c r="J9" s="25">
+      <c r="J9" s="26">
         <f>-('Balance Sheet'!J8-'Balance Sheet'!I8)</f>
         <v/>
       </c>
-      <c r="K9" s="25">
+      <c r="K9" s="26">
         <f>-('Balance Sheet'!K8-'Balance Sheet'!J8)</f>
         <v/>
       </c>
@@ -4409,43 +4505,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
         </is>
       </c>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
+      <c r="D10" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="44" t="inlineStr">
+      <c r="E10" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F10" s="44" t="inlineStr">
+      <c r="F10" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="26">
         <f>-('Balance Sheet'!G12-'Balance Sheet'!F12)</f>
         <v/>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="26">
         <f>-('Balance Sheet'!H12-'Balance Sheet'!G12)</f>
         <v/>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="26">
         <f>-('Balance Sheet'!I12-'Balance Sheet'!H12)</f>
         <v/>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="26">
         <f>-('Balance Sheet'!J12-'Balance Sheet'!I12)</f>
         <v/>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="26">
         <f>-('Balance Sheet'!K12-'Balance Sheet'!J12)</f>
         <v/>
       </c>
@@ -4456,43 +4552,43 @@
           <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
         </is>
       </c>
-      <c r="C11" s="44" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="44" t="inlineStr">
+      <c r="D11" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="44" t="inlineStr">
+      <c r="E11" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="44" t="inlineStr">
+      <c r="F11" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="26">
         <f>-('Balance Sheet'!G14-'Balance Sheet'!F14)</f>
         <v/>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="26">
         <f>-('Balance Sheet'!H14-'Balance Sheet'!G14)</f>
         <v/>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="26">
         <f>-('Balance Sheet'!I14-'Balance Sheet'!H14)</f>
         <v/>
       </c>
-      <c r="J11" s="25">
+      <c r="J11" s="26">
         <f>-('Balance Sheet'!J14-'Balance Sheet'!I14)</f>
         <v/>
       </c>
-      <c r="K11" s="25">
+      <c r="K11" s="26">
         <f>-('Balance Sheet'!K14-'Balance Sheet'!J14)</f>
         <v/>
       </c>
@@ -4503,43 +4599,43 @@
           <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
         </is>
       </c>
-      <c r="C12" s="44" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="44" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="44" t="inlineStr">
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="44" t="inlineStr">
+      <c r="F12" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="26">
         <f>('Balance Sheet'!G19-'Balance Sheet'!F19)</f>
         <v/>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="26">
         <f>('Balance Sheet'!H19-'Balance Sheet'!G19)</f>
         <v/>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="26">
         <f>('Balance Sheet'!I19-'Balance Sheet'!H19)</f>
         <v/>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="26">
         <f>('Balance Sheet'!J19-'Balance Sheet'!I19)</f>
         <v/>
       </c>
-      <c r="K12" s="25">
+      <c r="K12" s="26">
         <f>('Balance Sheet'!K19-'Balance Sheet'!J19)</f>
         <v/>
       </c>
@@ -4550,43 +4646,43 @@
           <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
         </is>
       </c>
-      <c r="C13" s="44" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" s="44" t="inlineStr">
+      <c r="D13" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="44" t="inlineStr">
+      <c r="E13" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F13" s="44" t="inlineStr">
+      <c r="F13" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="26">
         <f>('Balance Sheet'!G20-'Balance Sheet'!F20)</f>
         <v/>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="26">
         <f>('Balance Sheet'!H20-'Balance Sheet'!G20)</f>
         <v/>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="26">
         <f>('Balance Sheet'!I20-'Balance Sheet'!H20)</f>
         <v/>
       </c>
-      <c r="J13" s="25">
+      <c r="J13" s="26">
         <f>('Balance Sheet'!J20-'Balance Sheet'!I20)</f>
         <v/>
       </c>
-      <c r="K13" s="25">
+      <c r="K13" s="26">
         <f>('Balance Sheet'!K20-'Balance Sheet'!J20)</f>
         <v/>
       </c>
@@ -4597,43 +4693,43 @@
           <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
         </is>
       </c>
-      <c r="C14" s="44" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D14" s="44" t="inlineStr">
+      <c r="D14" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="44" t="inlineStr">
+      <c r="E14" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="44" t="inlineStr">
+      <c r="F14" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="26">
         <f>('Balance Sheet'!G22-'Balance Sheet'!F22)</f>
         <v/>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="26">
         <f>('Balance Sheet'!H22-'Balance Sheet'!G22)</f>
         <v/>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="26">
         <f>('Balance Sheet'!I22-'Balance Sheet'!H22)</f>
         <v/>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="26">
         <f>('Balance Sheet'!J22-'Balance Sheet'!I22)</f>
         <v/>
       </c>
-      <c r="K14" s="25">
+      <c r="K14" s="26">
         <f>('Balance Sheet'!K22-'Balance Sheet'!J22)</f>
         <v/>
       </c>
@@ -4644,43 +4740,43 @@
           <t xml:space="preserve">  Incr./(decr.) in operating lease liab.</t>
         </is>
       </c>
-      <c r="C15" s="44" t="inlineStr">
+      <c r="C15" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="44" t="inlineStr">
+      <c r="D15" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="44" t="inlineStr">
+      <c r="E15" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="44" t="inlineStr">
+      <c r="F15" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="26">
         <f>('Balance Sheet'!G21-'Balance Sheet'!F21)+('Balance Sheet'!G25-'Balance Sheet'!F25)</f>
         <v/>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="26">
         <f>('Balance Sheet'!H21-'Balance Sheet'!G21)+('Balance Sheet'!H25-'Balance Sheet'!G25)</f>
         <v/>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="26">
         <f>('Balance Sheet'!I21-'Balance Sheet'!H21)+('Balance Sheet'!I25-'Balance Sheet'!H25)</f>
         <v/>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="26">
         <f>('Balance Sheet'!J21-'Balance Sheet'!I21)+('Balance Sheet'!J25-'Balance Sheet'!I25)</f>
         <v/>
       </c>
-      <c r="K15" s="25">
+      <c r="K15" s="26">
         <f>('Balance Sheet'!K21-'Balance Sheet'!J21)+('Balance Sheet'!K25-'Balance Sheet'!J25)</f>
         <v/>
       </c>
@@ -4691,43 +4787,43 @@
           <t xml:space="preserve">  Incr./(decr.) in deferred income taxes</t>
         </is>
       </c>
-      <c r="C16" s="44" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="44" t="inlineStr">
+      <c r="D16" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="44" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="44" t="inlineStr">
+      <c r="F16" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="26">
         <f>('Balance Sheet'!G26-'Balance Sheet'!F26)</f>
         <v/>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="26">
         <f>('Balance Sheet'!H26-'Balance Sheet'!G26)</f>
         <v/>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="26">
         <f>('Balance Sheet'!I26-'Balance Sheet'!H26)</f>
         <v/>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="26">
         <f>('Balance Sheet'!J26-'Balance Sheet'!I26)</f>
         <v/>
       </c>
-      <c r="K16" s="25">
+      <c r="K16" s="26">
         <f>('Balance Sheet'!K26-'Balance Sheet'!J26)</f>
         <v/>
       </c>
@@ -4738,43 +4834,43 @@
           <t xml:space="preserve">  Incr./(decr.) in other non-current liab.</t>
         </is>
       </c>
-      <c r="C17" s="44" t="inlineStr">
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="44" t="inlineStr">
+      <c r="D17" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="44" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F17" s="44" t="inlineStr">
+      <c r="F17" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="25">
+      <c r="G17" s="26">
         <f>('Balance Sheet'!G27-'Balance Sheet'!F27)</f>
         <v/>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="26">
         <f>('Balance Sheet'!H27-'Balance Sheet'!G27)</f>
         <v/>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="26">
         <f>('Balance Sheet'!I27-'Balance Sheet'!H27)</f>
         <v/>
       </c>
-      <c r="J17" s="25">
+      <c r="J17" s="26">
         <f>('Balance Sheet'!J27-'Balance Sheet'!I27)</f>
         <v/>
       </c>
-      <c r="K17" s="25">
+      <c r="K17" s="26">
         <f>('Balance Sheet'!K27-'Balance Sheet'!J27)</f>
         <v/>
       </c>
@@ -4785,58 +4881,58 @@
           <t xml:space="preserve">  Working capital &amp; other (reported, net)</t>
         </is>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="26">
         <f>C19-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="26">
         <f>D19-D5-D6-D7</f>
         <v/>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="26">
         <f>E19-E5-E6-E7</f>
         <v/>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="26">
         <f>F19-F5-F6-F7</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="C19" s="41" t="n">
+      <c r="C19" s="42" t="n">
         <v>966463</v>
       </c>
-      <c r="D19" s="41" t="n">
+      <c r="D19" s="42" t="n">
         <v>2296164</v>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="E19" s="42" t="n">
         <v>2272713</v>
       </c>
-      <c r="F19" s="41" t="n">
+      <c r="F19" s="42" t="n">
         <v>1602477</v>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="33">
         <f>G5+G6+G7+SUM(G8:G17)</f>
         <v/>
       </c>
-      <c r="H19" s="32">
+      <c r="H19" s="33">
         <f>H5+H6+H7+SUM(H8:H17)</f>
         <v/>
       </c>
-      <c r="I19" s="32">
+      <c r="I19" s="33">
         <f>I5+I6+I7+SUM(I8:I17)</f>
         <v/>
       </c>
-      <c r="J19" s="32">
+      <c r="J19" s="33">
         <f>J5+J6+J7+SUM(J8:J17)</f>
         <v/>
       </c>
-      <c r="K19" s="32">
+      <c r="K19" s="33">
         <f>K5+K6+K7+SUM(K8:K17)</f>
         <v/>
       </c>
@@ -4863,74 +4959,74 @@
           <t>Capital expenditures</t>
         </is>
       </c>
-      <c r="C22" s="30" t="n">
+      <c r="C22" s="31" t="n">
         <v>-638657</v>
       </c>
-      <c r="D22" s="30" t="n">
+      <c r="D22" s="31" t="n">
         <v>-651865</v>
       </c>
-      <c r="E22" s="30" t="n">
+      <c r="E22" s="31" t="n">
         <v>-689232</v>
       </c>
-      <c r="F22" s="30" t="n">
+      <c r="F22" s="31" t="n">
         <v>-680802</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="26">
         <f>-'Income Statement'!G4*'Assumptions'!G13</f>
         <v/>
       </c>
-      <c r="H22" s="25">
+      <c r="H22" s="26">
         <f>-'Income Statement'!H4*'Assumptions'!H13</f>
         <v/>
       </c>
-      <c r="I22" s="25">
+      <c r="I22" s="26">
         <f>-'Income Statement'!I4*'Assumptions'!I13</f>
         <v/>
       </c>
-      <c r="J22" s="25">
+      <c r="J22" s="26">
         <f>-'Income Statement'!J4*'Assumptions'!J13</f>
         <v/>
       </c>
-      <c r="K22" s="25">
+      <c r="K22" s="26">
         <f>-'Income Statement'!K4*'Assumptions'!K13</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Net cash from investing activities</t>
         </is>
       </c>
-      <c r="C23" s="41" t="n">
+      <c r="C23" s="42" t="n">
         <v>-569937</v>
       </c>
-      <c r="D23" s="41" t="n">
+      <c r="D23" s="42" t="n">
         <v>-654132</v>
       </c>
-      <c r="E23" s="41" t="n">
+      <c r="E23" s="42" t="n">
         <v>-798174</v>
       </c>
-      <c r="F23" s="41" t="n">
+      <c r="F23" s="42" t="n">
         <v>-662118</v>
       </c>
-      <c r="G23" s="32">
+      <c r="G23" s="33">
         <f>G22</f>
         <v/>
       </c>
-      <c r="H23" s="32">
+      <c r="H23" s="33">
         <f>H22</f>
         <v/>
       </c>
-      <c r="I23" s="32">
+      <c r="I23" s="33">
         <f>I22</f>
         <v/>
       </c>
-      <c r="J23" s="32">
+      <c r="J23" s="33">
         <f>J22</f>
         <v/>
       </c>
-      <c r="K23" s="32">
+      <c r="K23" s="33">
         <f>K22</f>
         <v/>
       </c>
@@ -4964,74 +5060,74 @@
           <t>Repurchase of common stock</t>
         </is>
       </c>
-      <c r="C27" s="30" t="n">
+      <c r="C27" s="31" t="n">
         <v>-444001</v>
       </c>
-      <c r="D27" s="30" t="n">
+      <c r="D27" s="31" t="n">
         <v>-558652</v>
       </c>
-      <c r="E27" s="30" t="n">
+      <c r="E27" s="31" t="n">
         <v>-1636879</v>
       </c>
-      <c r="F27" s="30" t="n">
+      <c r="F27" s="31" t="n">
         <v>-1178349</v>
       </c>
-      <c r="G27" s="25">
+      <c r="G27" s="26">
         <f>-'Assumptions'!G27</f>
         <v/>
       </c>
-      <c r="H27" s="25">
+      <c r="H27" s="26">
         <f>-'Assumptions'!H27</f>
         <v/>
       </c>
-      <c r="I27" s="25">
+      <c r="I27" s="26">
         <f>-'Assumptions'!I27</f>
         <v/>
       </c>
-      <c r="J27" s="25">
+      <c r="J27" s="26">
         <f>-'Assumptions'!J27</f>
         <v/>
       </c>
-      <c r="K27" s="25">
+      <c r="K27" s="26">
         <f>-'Assumptions'!K27</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="32" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>-467487</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>-548828</v>
       </c>
-      <c r="E28" s="41" t="n">
+      <c r="E28" s="42" t="n">
         <v>-1652508</v>
       </c>
-      <c r="F28" s="41" t="n">
+      <c r="F28" s="42" t="n">
         <v>-1208656</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="33">
         <f>G27</f>
         <v/>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="33">
         <f>H27</f>
         <v/>
       </c>
-      <c r="I28" s="32">
+      <c r="I28" s="33">
         <f>I27</f>
         <v/>
       </c>
-      <c r="J28" s="32">
+      <c r="J28" s="33">
         <f>J27</f>
         <v/>
       </c>
-      <c r="K28" s="32">
+      <c r="K28" s="33">
         <f>K27</f>
         <v/>
       </c>
@@ -5044,44 +5140,44 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="inlineStr">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="33">
         <f>C19+C23+C28</f>
         <v/>
       </c>
-      <c r="D31" s="32">
+      <c r="D31" s="33">
         <f>D19+D23+D28</f>
         <v/>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="33">
         <f>E19+E23+E28</f>
         <v/>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="33">
         <f>F19+F23+F28</f>
         <v/>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="33">
         <f>G19+G23+G28</f>
         <v/>
       </c>
-      <c r="H31" s="32">
+      <c r="H31" s="33">
         <f>H19+H23+H28</f>
         <v/>
       </c>
-      <c r="I31" s="32">
+      <c r="I31" s="33">
         <f>I19+I23+I28</f>
         <v/>
       </c>
-      <c r="J31" s="32">
+      <c r="J31" s="33">
         <f>J19+J23+J28</f>
         <v/>
       </c>
-      <c r="K31" s="32">
+      <c r="K31" s="33">
         <f>K19+K23+K28</f>
         <v/>
       </c>
@@ -5092,74 +5188,74 @@
           <t>Cash, beginning of year</t>
         </is>
       </c>
-      <c r="C32" s="30" t="n">
+      <c r="C32" s="31" t="n">
         <v>1150517</v>
       </c>
-      <c r="D32" s="30" t="n">
+      <c r="D32" s="31" t="n">
         <v>1154867</v>
       </c>
-      <c r="E32" s="30" t="n">
+      <c r="E32" s="31" t="n">
         <v>2243971</v>
       </c>
-      <c r="F32" s="30" t="n">
+      <c r="F32" s="31" t="n">
         <v>1984336</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="26">
         <f>'Balance Sheet'!F6</f>
         <v/>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="26">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I32" s="25">
+      <c r="I32" s="26">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J32" s="25">
+      <c r="J32" s="26">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K32" s="25">
+      <c r="K32" s="26">
         <f>J33</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="31" t="inlineStr">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>Cash, end of year</t>
         </is>
       </c>
-      <c r="C33" s="42" t="n">
+      <c r="C33" s="43" t="n">
         <v>1154867</v>
       </c>
-      <c r="D33" s="42" t="n">
+      <c r="D33" s="43" t="n">
         <v>2243971</v>
       </c>
-      <c r="E33" s="42" t="n">
+      <c r="E33" s="43" t="n">
         <v>1984336</v>
       </c>
-      <c r="F33" s="42" t="n">
+      <c r="F33" s="43" t="n">
         <v>1807202</v>
       </c>
-      <c r="G33" s="33">
+      <c r="G33" s="34">
         <f>G32+G31</f>
         <v/>
       </c>
-      <c r="H33" s="33">
+      <c r="H33" s="34">
         <f>H32+H31</f>
         <v/>
       </c>
-      <c r="I33" s="33">
+      <c r="I33" s="34">
         <f>I32+I31</f>
         <v/>
       </c>
-      <c r="J33" s="33">
+      <c r="J33" s="34">
         <f>J32+J31</f>
         <v/>
       </c>
-      <c r="K33" s="33">
+      <c r="K33" s="34">
         <f>K32+K31</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Make every Ctrl+F string match verbatim text in linked sources
- Rewrite all SOURCE_HINT/REPORTED_HINTS with exact 10-K line labels
  (e.g. Accrued liabilities and other, Right-of-use lease assets,
  Income tax expense, Stock-based compensation expense)
- Anchor earnings guidance to exact release quotes (decline of 5% to 7%,
  $10.350B–$10.500B, $9.48–$9.73)
- Switch peer/beta sources to StockAnalysis for reliable Ctrl+F labels
- Add verify_ctrl_f.py to check quoted phrases against live sources

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -816,7 +816,7 @@
       <c r="B16" s="9" t="inlineStr">
         <is>
           <t>SEC EDGAR filings, CIK 0001397187 (Forms 10-K)
-Ctrl+F: "10-K" → FY2025 accession 0001397187-26-000020</t>
+Ctrl+F: Ctrl+F "10-K" → FY2025 accession 0001397187-26-000020</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       <c r="B17" s="9" t="inlineStr">
         <is>
           <t>FY2025 Form 10-K (ended Feb 1, 2026)
-Ctrl+F: "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
+Ctrl+F: Ctrl+F "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Q2 FY2026 results &amp; FY2026 guidance (Sep 3, 2026 earnings release)
-Ctrl+F: "full year 2026" | "net revenue" | "diluted earnings per share"</t>
+Ctrl+F: Ctrl+F "decline of 5% to 7%" | "$10.350 billion to $10.500 billion" | "$9.48 to $9.73"</t>
         </is>
       </c>
     </row>
@@ -1005,23 +1005,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>Justification (~20 words)</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>Source (click)</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -1056,7 +1039,7 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>"full year 2026" → "net revenue" → "5% to 7%" decrease; FY27–30 = projection</t>
+          <t>Ctrl+F "decline of 5% to 7%" → FY2026 guide; FY27–30 = model projection</t>
         </is>
       </c>
       <c r="F5" s="23" t="n">
@@ -1102,7 +1085,7 @@
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>"Gross profit" $6,284,132 ÷ "Net revenue" $11,102,600 = 56.6% FY25</t>
+          <t>Ctrl+F "Gross profit" → 6,284,132 ÷ "Net revenue" 11,102,600 = 56.6% FY25 anchor</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
@@ -1151,7 +1134,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>"Selling, general and administrative expenses" $4,066,556 ÷ revenue = 36.7%</t>
+          <t>Ctrl+F "Selling, general and administrative expenses" → 4,066,556 ÷ revenue 11,102,600</t>
         </is>
       </c>
       <c r="E7" s="23" t="n">
@@ -1200,7 +1183,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>"Amortization of intangible assets" → FY25 $6,961 (≈$7M run-rate)</t>
+          <t>Ctrl+F "Amortization of intangible assets" → 6,961 ($000); model $7,000/yr</t>
         </is>
       </c>
       <c r="E8" s="25" t="n">
@@ -1249,7 +1232,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>"Other income (expense), net" → FY25 $28,352 (interest income on cash)</t>
+          <t>Ctrl+F "Other income (expense), net" → 28,352 ($000) FY25; model steps down</t>
         </is>
       </c>
       <c r="E9" s="25" t="n">
@@ -1298,7 +1281,7 @@
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>"Provision for income taxes" $659,784 ÷ "Income before income taxes" $2,238,967 = 29.5%</t>
+          <t>Ctrl+F "Income tax expense" → 659,784 ÷ "Income before income tax expense" 2,238,967 = 29.5%</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
@@ -1363,7 +1346,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>"Depreciation and amortization" $496,228 ÷ "Net revenue" $11,102,600 = 4.5%</t>
+          <t>Ctrl+F "Depreciation and amortization" → 496,228 ÷ "Net revenue" 11,102,600 = 4.5%</t>
         </is>
       </c>
       <c r="E12" s="23" t="n">
@@ -1412,7 +1395,7 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>"Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
@@ -1461,7 +1444,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>"Stock-based compensation" → FY25 $62,203; model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
         </is>
       </c>
       <c r="E14" s="25" t="n">
@@ -1526,7 +1509,7 @@
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
-          <t>"Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
         </is>
       </c>
       <c r="E16" s="23" t="n">
@@ -1575,7 +1558,7 @@
       </c>
       <c r="D17" s="22" t="inlineStr">
         <is>
-          <t>"Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E17" s="23" t="n">
@@ -1624,7 +1607,7 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>"Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
@@ -1673,7 +1656,7 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>"Other current assets" → derive from current assets less cash, A/R, inventory</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
@@ -1722,7 +1705,7 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>"Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
@@ -1771,7 +1754,7 @@
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>"Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
+          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
@@ -1820,7 +1803,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>"Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
       <c r="E22" s="23" t="n">
@@ -1869,7 +1852,7 @@
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>"Operating lease liabilities" $1,499,717 (non-current) ÷ revenue = 13.5%</t>
+          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
         </is>
       </c>
       <c r="E23" s="23" t="n">
@@ -1918,7 +1901,7 @@
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>"Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
+          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
@@ -1967,7 +1950,7 @@
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>"Other non-current liabilities" → minor long-term accruals ÷ revenue</t>
+          <t>Ctrl+F "Other non-current liabilities" → 55,360 ÷ "Net revenue" 11,102,600 = 0.5%</t>
         </is>
       </c>
       <c r="E25" s="23" t="n">
@@ -2032,7 +2015,7 @@
       </c>
       <c r="D27" s="22" t="inlineStr">
         <is>
-          <t>"Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
         </is>
       </c>
       <c r="E27" s="25" t="n">
@@ -2081,7 +2064,7 @@
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
-          <t>"Repurchase of common stock" footnote → avg price paid per share</t>
+          <t>Ctrl+F "Average Price Paid per Share" → repurchase table in Note 15 / equity</t>
         </is>
       </c>
       <c r="I28" s="27" t="n">
@@ -2275,7 +2258,7 @@
       </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>"full year 2026" → "net revenue" → "5% to 7%" decrease; FY27–30 = projection</t>
+          <t>Ctrl+F "decline of 5% to 7%" → FY2026 guide; FY27–30 = model projection</t>
         </is>
       </c>
       <c r="E4" s="31" t="n">
@@ -2329,7 +2312,7 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>"Gross profit" $6,284,132 ÷ "Net revenue" $11,102,600 = 56.6% FY25</t>
+          <t>Ctrl+F "Gross profit" → 6,284,132 ÷ "Net revenue" 11,102,600 = 56.6% FY25 anchor</t>
         </is>
       </c>
       <c r="E5" s="31" t="n">
@@ -2426,7 +2409,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>"Selling, general and administrative expenses" $4,066,556 ÷ revenue = 36.7%</t>
+          <t>Ctrl+F "Selling, general and administrative expenses" → 4,066,556 ÷ revenue 11,102,600</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -2480,7 +2463,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>"Amortization of intangible assets" → FY25 $6,961 (≈$7M run-rate)</t>
+          <t>Ctrl+F "Amortization of intangible assets" → 6,961 ($000); model $7,000/yr</t>
         </is>
       </c>
       <c r="E8" s="31" t="n">
@@ -2577,7 +2560,7 @@
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>"Other income (expense), net" → FY25 $28,352 (interest income on cash)</t>
+          <t>Ctrl+F "Other income (expense), net" → 28,352 ($000) FY25; model steps down</t>
         </is>
       </c>
       <c r="E10" s="31" t="n">
@@ -2674,7 +2657,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>"Provision for income taxes" $659,784 ÷ "Income before income taxes" $2,238,967 = 29.5%</t>
+          <t>Ctrl+F "Income tax expense" → 659,784 ÷ "Income before income tax expense" 2,238,967 = 29.5%</t>
         </is>
       </c>
       <c r="E12" s="31" t="n">
@@ -2773,8 +2756,8 @@
       </c>
       <c r="D15" s="22" t="inlineStr">
         <is>
-          <t>"Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr
-Also: "Repurchase of common stock" footnote → avg price paid per share</t>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr
+Also: Ctrl+F "Average Price Paid per Share" → repurchase table in Note 15 / equity</t>
         </is>
       </c>
       <c r="E15" s="31" t="n">
@@ -3286,7 +3269,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>"Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -3340,7 +3323,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>"Other current assets" → derive from current assets less cash, A/R, inventory</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
         </is>
       </c>
       <c r="E8" s="25" t="n">
@@ -3440,7 +3423,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>"Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
         </is>
       </c>
       <c r="E11" s="31" t="n">
@@ -3494,7 +3477,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>"Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E12" s="31" t="n">
@@ -3587,7 +3570,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>"Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
+          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
         </is>
       </c>
       <c r="E14" s="25" t="n">
@@ -3703,7 +3686,7 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>"Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E19" s="31" t="n">
@@ -3757,7 +3740,7 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>"Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E20" s="31" t="n">
@@ -3811,7 +3794,7 @@
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>"Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
       <c r="E21" s="31" t="n">
@@ -3865,7 +3848,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>"Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
+          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
         </is>
       </c>
       <c r="E22" s="25" t="n">
@@ -3965,7 +3948,7 @@
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>"Operating lease liabilities" $1,499,717 (non-current) ÷ revenue = 13.5%</t>
+          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
         </is>
       </c>
       <c r="E25" s="31" t="n">
@@ -4058,7 +4041,7 @@
       </c>
       <c r="D27" s="22" t="inlineStr">
         <is>
-          <t>"Other non-current liabilities" → minor long-term accruals ÷ revenue</t>
+          <t>Ctrl+F "Other non-current liabilities" → 55,360 ÷ "Net revenue" 11,102,600 = 0.5%</t>
         </is>
       </c>
       <c r="E27" s="25" t="n">
@@ -4158,7 +4141,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>"Stock-based compensation" → FY25 $62,203; model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
         </is>
       </c>
       <c r="E31" s="31" t="n">
@@ -4212,7 +4195,7 @@
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
-          <t>"Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
         </is>
       </c>
       <c r="E32" s="31" t="n">
@@ -4699,7 +4682,7 @@
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>"Depreciation and amortization" $496,228 ÷ "Net revenue" $11,102,600 = 4.5%</t>
+          <t>Ctrl+F "Depreciation and amortization" → 496,228 ÷ "Net revenue" 11,102,600 = 4.5%</t>
         </is>
       </c>
       <c r="E6" s="31" t="n">
@@ -4753,7 +4736,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>"Stock-based compensation" → FY25 $62,203; model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -4807,7 +4790,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>"Inventories" $1,700,753 ÷ "Cost of goods sold" $4,818,468 = 35.3%</t>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
         </is>
       </c>
       <c r="E8" s="46" t="inlineStr">
@@ -4869,7 +4852,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>"Other current assets" → derive from current assets less cash, A/R, inventory</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
         </is>
       </c>
       <c r="E9" s="46" t="inlineStr">
@@ -4931,7 +4914,7 @@
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>"Operating lease right-of-use assets" $1,630,181 ÷ revenue = 14.7%</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E10" s="46" t="inlineStr">
@@ -4993,7 +4976,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>"Other non-current assets" → total non-current assets less PP&amp;E, ROU, goodwill</t>
+          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
         </is>
       </c>
       <c r="E11" s="46" t="inlineStr">
@@ -5055,7 +5038,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>"Accounts payable" $331,421 ÷ "Cost of goods sold" $4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E12" s="46" t="inlineStr">
@@ -5117,7 +5100,7 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>"Accrued liabilities" $662,982 ÷ "Net revenue" $11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E13" s="46" t="inlineStr">
@@ -5179,7 +5162,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>"Other current liabilities" → gift cards, deferred revenue (ex-lease) ÷ revenue</t>
+          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
         </is>
       </c>
       <c r="E14" s="46" t="inlineStr">
@@ -5241,7 +5224,7 @@
       </c>
       <c r="D15" s="22" t="inlineStr">
         <is>
-          <t>"Current portion of operating lease liabilities" $298,724 ÷ revenue = 2.7%</t>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
       <c r="E15" s="46" t="inlineStr">
@@ -5475,7 +5458,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>"Capital expenditures" $(680,802) ÷ "Net revenue" = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
         </is>
       </c>
       <c r="E22" s="31" t="n">
@@ -5591,7 +5574,7 @@
       </c>
       <c r="D27" s="22" t="inlineStr">
         <is>
-          <t>"Repurchase of common stock" → FY25 $(1,178,349); model $(500,000)/yr</t>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
         </is>
       </c>
       <c r="E27" s="31" t="n">

</xml_diff>

<commit_message>
Fix source misreads: 13% is YoY EBIT decline, not the margin
- Q2 release: income from operations decreased 13% to $453.7M; operating margin is 18.8% (560bps from tariffs)
- FY26 13.9% EBIT margin is now labeled a model assumption (near 13.2% Q2 ex-tariff)
- Correct other source mismatches: SG&A YTD 42.3% vs FY25 36.7%, OCA residual 6.8%, SBC is above FY25, other income $130M is model-only, capex below 2026 guide
- Pitch: share count −7% (128.0M→119.1M WAS), not −13%; FY25 19.9% OM is not the trough

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1124,17 +1124,17 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
+          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>LULU historical SG&amp;A (10-K)</t>
+          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Selling, general and administrative expenses" → 4,066,556 ÷ revenue 11,102,600</t>
+          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
         </is>
       </c>
       <c r="E7" s="23" t="n">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+          <t>FY26 $130M other income is a model assumption (FY25 10-K is $28.4M; YTD FY26 $22.8M); steps down as cash is used.</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other income (expense), net" → 28,352 ($000) FY25; model steps down</t>
+          <t>Ctrl+F "Other income (expense), net" → FY25 28,352 ($000). Model FY26 $130,000 is an assumption, not a reported figure</t>
         </is>
       </c>
       <c r="E9" s="25" t="n">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>LULU effective tax history (10-K)</t>
+          <t>LULU Q2 FY2026 outlook (≈30% tax)</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Income tax expense" → 659,784 ÷ "Income before income tax expense" 2,238,967 = 29.5%</t>
+          <t>Ctrl+F "a tax rate of approximately 30%" on the earnings outlook; FY25 10-K 29.5%. 3-statement model 30%</t>
         </is>
       </c>
       <c r="E10" s="23" t="n">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
         </is>
       </c>
       <c r="E14" s="25" t="n">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
+          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
@@ -2399,17 +2399,17 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>SG&amp;A leverage improves slowly as revenue stabilizes; ratio declines toward 39.5% by FY2030 from cost discipline.</t>
+          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>LULU historical SG&amp;A (10-K)</t>
+          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Selling, general and administrative expenses" → 4,066,556 ÷ revenue 11,102,600</t>
+          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Interest income declines as cash is deployed; $130M FY26 stepping down with lower cash balances.</t>
+          <t>FY26 $130M other income is a model assumption (FY25 10-K is $28.4M; YTD FY26 $22.8M); steps down as cash is used.</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other income (expense), net" → 28,352 ($000) FY25; model steps down</t>
+          <t>Ctrl+F "Other income (expense), net" → FY25 28,352 ($000). Model FY26 $130,000 is an assumption, not a reported figure</t>
         </is>
       </c>
       <c r="E10" s="31" t="n">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>LULU effective tax history (10-K)</t>
+          <t>LULU Q2 FY2026 outlook (≈30% tax)</t>
         </is>
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Income tax expense" → 659,784 ÷ "Income before income tax expense" 2,238,967 = 29.5%</t>
+          <t>Ctrl+F "a tax rate of approximately 30%" on the earnings outlook; FY25 10-K 29.5%. 3-statement model 30%</t>
         </is>
       </c>
       <c r="E12" s="31" t="n">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
+          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
         </is>
       </c>
       <c r="E8" s="25" t="n">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
         </is>
       </c>
       <c r="E11" s="31" t="n">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E14" s="25" t="n">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
         </is>
       </c>
       <c r="E22" s="25" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
         </is>
       </c>
       <c r="E31" s="31" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC; modest decline from FY25 as headcount growth slows in restructuring period.</t>
+          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000); model $70,000</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Other current assets 6.8% of revenue; prepaid and receivable balance consistent with recent history.</t>
+          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets" → 211,620 ÷ revenue = 1.9% FY25</t>
+          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
         </is>
       </c>
       <c r="E9" s="46" t="inlineStr">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>Other non-current assets 3.0% of revenue; deferred costs and long-term deposits at normalized level.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Deferred income tax assets" → in non-current assets; model 3.0% of revenue</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E11" s="46" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Other current liabilities 5.5% of revenue; gift cards, deferred revenue, and other short-term obligations.</t>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other current liabilities" → 45,954 | "Unredeemed gift card liability" → 316,632</t>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
         </is>
       </c>
       <c r="E14" s="46" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Capex fades from 5.5% to 5.0%; reflects completion of major supply-chain projects and normalized store growth.</t>
+          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → capex ($000); ÷ revenue 11,102,600 = 6.1%; model fades to 5.0%</t>
+          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
         </is>
       </c>
       <c r="E22" s="31" t="n">

</xml_diff>

<commit_message>
Source-true assumptions: direct 10-K HTML, fix rf/tax/capex/comps
- Link 10-K sources to lulu-20260201.htm so Ctrl+F finds D&A 496,228 (not the EDGAR viewer TOC)
- rf 4.8% from FRED DGS10 4.77% on 2026-09-03 (was stale 4.3%)
- cash tax 30% from FY26 guide; WACC 10.5%
- capex FY26 7.0% from 10-K $725-745M guide; DCF uses 5.5% 5-year blend
- other income $45M from YTD $22,829; SBC $62M from 10-K 62,203
- peer EV/EBITDA set to live StockAnalysis prints (NKE 12.0, DECK 8.0, ONON 14.0, ADS 9.3, VFC 10.7)

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -824,7 +824,7 @@
       <c r="B17" s="9" t="inlineStr">
         <is>
           <t>FY2025 Form 10-K (ended Feb 1, 2026)
-Ctrl+F: Ctrl+F "CONSOLIDATED STATEMENTS OF OPERATIONS" or "CONSOLIDATED BALANCE SHEETS"</t>
+Ctrl+F: Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
     </row>
@@ -1222,17 +1222,17 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>FY26 $130M other income is a model assumption (FY25 10-K is $28.4M; YTD FY26 $22.8M); steps down as cash is used.</t>
+          <t>FY26 $45M other income annualizes YTD $22,829; then steps down as cash is deployed (FY25 was only $28,352).</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K</t>
+          <t>Q2 FY2026 YTD other income (earnings)</t>
         </is>
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other income (expense), net" → FY25 28,352 ($000). Model FY26 $130,000 is an assumption, not a reported figure</t>
+          <t>Ctrl+F "22,829" → YTD other income ($000) on the earnings P&amp;L. FY26 model $45,000 annualizes that run-rate.</t>
         </is>
       </c>
       <c r="E9" s="25" t="n">
@@ -1248,19 +1248,19 @@
         <v>28352</v>
       </c>
       <c r="I9" s="26" t="n">
-        <v>130000</v>
+        <v>45000</v>
       </c>
       <c r="J9" s="26" t="n">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="K9" s="26" t="n">
-        <v>75000</v>
+        <v>35000</v>
       </c>
       <c r="L9" s="26" t="n">
-        <v>95000</v>
+        <v>30000</v>
       </c>
       <c r="M9" s="26" t="n">
-        <v>115000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
+          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
+          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
@@ -1411,13 +1411,13 @@
         <v>0.06131915046925945</v>
       </c>
       <c r="I13" s="24" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J13" s="24" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K13" s="24" t="n">
         <v>0.055</v>
-      </c>
-      <c r="J13" s="24" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="K13" s="24" t="n">
-        <v>0.05</v>
       </c>
       <c r="L13" s="24" t="n">
         <v>0.05</v>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
+          <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
         </is>
       </c>
       <c r="E14" s="25" t="n">
@@ -1460,19 +1460,19 @@
         <v>62203</v>
       </c>
       <c r="I14" s="26" t="n">
-        <v>70000</v>
+        <v>62000</v>
       </c>
       <c r="J14" s="26" t="n">
-        <v>70000</v>
+        <v>62000</v>
       </c>
       <c r="K14" s="26" t="n">
-        <v>70000</v>
+        <v>62000</v>
       </c>
       <c r="L14" s="26" t="n">
-        <v>70000</v>
+        <v>62000</v>
       </c>
       <c r="M14" s="26" t="n">
-        <v>70000</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="15">
@@ -2054,33 +2054,33 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+          <t>FY26 repurchase price $100 matches the current quote; path $100→$130 is a recovery assumption (FY25 10-K paid $168–$199).</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>LULU avg repurchase price (10-K/est.)</t>
+          <t>NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Average Price Paid per Share" → repurchase table in Note 15 / equity</t>
+          <t>Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
         </is>
       </c>
       <c r="I28" s="27" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="J28" s="27" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="K28" s="27" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="L28" s="27" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="M28" s="27" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30">
@@ -2550,17 +2550,17 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>FY26 $130M other income is a model assumption (FY25 10-K is $28.4M; YTD FY26 $22.8M); steps down as cash is used.</t>
+          <t>FY26 $45M other income annualizes YTD $22,829; then steps down as cash is deployed (FY25 was only $28,352).</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K</t>
+          <t>Q2 FY2026 YTD other income (earnings)</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Other income (expense), net" → FY25 28,352 ($000). Model FY26 $130,000 is an assumption, not a reported figure</t>
+          <t>Ctrl+F "22,829" → YTD other income ($000) on the earnings P&amp;L. FY26 model $45,000 annualizes that run-rate.</t>
         </is>
       </c>
       <c r="E10" s="31" t="n">
@@ -2745,19 +2745,19 @@
       <c r="B15" s="22" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.
-Also: Repurchase price rises with recovery thesis; $105 to $135 reflects assumed gradual share-price normalization.</t>
+Also: FY26 repurchase price $100 matches the current quote; path $100→$130 is a recovery assumption (FY25 10-K paid $168–$199).</t>
         </is>
       </c>
       <c r="C15" s="35" t="inlineStr">
         <is>
           <t>LULU CF: share repurchases (10-K)
-Also: LULU avg repurchase price (10-K/est.)</t>
+Also: NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
       <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr
-Also: Ctrl+F "Average Price Paid per Share" → repurchase table in Note 15 / equity</t>
+Also: Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
         </is>
       </c>
       <c r="E15" s="31" t="n">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
+          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
+          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
         </is>
       </c>
       <c r="E11" s="31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
+          <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
         </is>
       </c>
       <c r="E31" s="31" t="n">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>$70M annual SBC is a model assumption, modestly above FY25 $62.2M (not a decline); near-term run-rate as growth slows.</t>
+          <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 ($000) FY25. Model $70,000 is above FY25, not a decline</t>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
         </is>
       </c>
       <c r="E7" s="31" t="n">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Model 5.5%→5.0% is below FY25 6.1% and below 2026 10-K guide $725–745M; assumes capex discipline after the reset.</t>
+          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex ($000) = 6.1% of revenue. Also Ctrl+F "725.0 million" (2026 guide $725–745M). Model 5.5%→5.0% is below both</t>
+          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
         </is>
       </c>
       <c r="E22" s="31" t="n">

</xml_diff>

<commit_message>
Source FY27-30 growth from Street 3Y forecast 2.26%, not Net revenue
Ctrl+F 'Revenue Growth Forecast (3Y)' on StockAnalysis is unique.
Model out-year growth set to 2.3% (was 2.8%/3-4%).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1029,17 +1029,17 @@
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
+          <t>FY26 −6.1% is guidance midpoint. FY27 +2.6% then +2.3% tracks StockAnalysis next-year +2.64% and 3Y forecast 2.26%.</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance</t>
+          <t>StockAnalysis: LULU revenue forecast (FY27–30)</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 guide; FY27–30 = model projection</t>
+          <t>FY26: earnings release Ctrl+F "decline of 5% to 7%". FY27–30: this page Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. Model 2.3%.</t>
         </is>
       </c>
       <c r="F5" s="23" t="n">
@@ -1055,16 +1055,16 @@
         <v>-0.061</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>0.01</v>
+        <v>0.026</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>0.03</v>
+        <v>0.023</v>
       </c>
       <c r="L5" s="24" t="n">
-        <v>0.04</v>
+        <v>0.023</v>
       </c>
       <c r="M5" s="24" t="n">
-        <v>0.04</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>FY26 −6.1% matches guidance; FY27–30 step up to low-single-digit then mid-single-digit recovery path.</t>
+          <t>FY26 −6.1% is guidance midpoint. FY27 +2.6% then +2.3% tracks StockAnalysis next-year +2.64% and 3Y forecast 2.26%.</t>
         </is>
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance</t>
+          <t>StockAnalysis: LULU revenue forecast (FY27–30)</t>
         </is>
       </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 guide; FY27–30 = model projection</t>
+          <t>FY26: earnings release Ctrl+F "decline of 5% to 7%". FY27–30: this page Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. Model 2.3%.</t>
         </is>
       </c>
       <c r="E4" s="31" t="n">

</xml_diff>

<commit_message>
Rebuild models with FY26 tariff add-back and fix opening cash
Excel now interpolates clean 13.2% OM and adds $134.5M in FY26 only.
3-statement FY26 opening cash rolls from FY25 ending cash so the
balance sheet ties in the forecast years.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -873,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1070,12 +1070,12 @@
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Gross margin %</t>
+          <t>Gross margin % (clean, ex-refunds)</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
+          <t>Clean GM 56.5%→58.0% (ex-refunds), still below peak ~58–59%. FY26 COGS is then reduced by the $134.5M IEEPA refund.</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -1119,273 +1119,273 @@
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>SG&amp;A % of revenue</t>
+          <t>IEEPA tariff refunds ($k, FY26 only)</t>
         </is>
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
+          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
+          <t>Q2 FY2026 release: $134.5M IEEPA tariff refunds</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="n">
-        <v>0.3399840799317627</v>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>0.3531676701723352</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <v>0.355339462337339</v>
-      </c>
-      <c r="H7" s="23" t="n">
-        <v>0.3662706032821141</v>
-      </c>
-      <c r="I7" s="24" t="n">
-        <v>0.425</v>
-      </c>
-      <c r="J7" s="24" t="n">
-        <v>0.415</v>
-      </c>
-      <c r="K7" s="24" t="n">
-        <v>0.405</v>
-      </c>
-      <c r="L7" s="24" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M7" s="24" t="n">
-        <v>0.395</v>
+          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="26" t="n">
+        <v>134500</v>
+      </c>
+      <c r="J7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>Amortization / other opex ($)</t>
+          <t>SG&amp;A % of revenue</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
+          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K</t>
+          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Amortization of intangible assets" → 6,961 ($000); model $7,000/yr</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>406485</v>
-      </c>
-      <c r="F8" s="25" t="n">
-        <v>79511</v>
-      </c>
-      <c r="G8" s="25" t="n">
-        <v>2735</v>
-      </c>
-      <c r="H8" s="25" t="n">
-        <v>6961</v>
-      </c>
-      <c r="I8" s="26" t="n">
-        <v>7000</v>
-      </c>
-      <c r="J8" s="26" t="n">
-        <v>7000</v>
-      </c>
-      <c r="K8" s="26" t="n">
-        <v>7000</v>
-      </c>
-      <c r="L8" s="26" t="n">
-        <v>7000</v>
-      </c>
-      <c r="M8" s="26" t="n">
-        <v>7000</v>
+          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>0.3399840799317627</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>0.3531676701723352</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0.355339462337339</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>0.3662706032821141</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="J8" s="24" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="K8" s="24" t="n">
+        <v>0.405</v>
+      </c>
+      <c r="L8" s="24" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M8" s="24" t="n">
+        <v>0.395</v>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Other income, net ($)</t>
+          <t>Amortization / other opex ($)</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>FY26 $45M other income annualizes YTD $22,829; then steps down as cash is deployed (FY25 was only $28,352).</t>
+          <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>Q2 FY2026 YTD other income (earnings)</t>
+          <t>LULU FY2025 10-K</t>
         </is>
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "22,829" → YTD other income ($000) on the earnings P&amp;L. FY26 model $45,000 annualizes that run-rate.</t>
+          <t>Ctrl+F "Amortization of intangible assets" → 6,961 ($000); model $7,000/yr</t>
         </is>
       </c>
       <c r="E9" s="25" t="n">
-        <v>4163</v>
+        <v>406485</v>
       </c>
       <c r="F9" s="25" t="n">
-        <v>43059</v>
+        <v>79511</v>
       </c>
       <c r="G9" s="25" t="n">
-        <v>70380</v>
+        <v>2735</v>
       </c>
       <c r="H9" s="25" t="n">
-        <v>28352</v>
+        <v>6961</v>
       </c>
       <c r="I9" s="26" t="n">
-        <v>45000</v>
+        <v>7000</v>
       </c>
       <c r="J9" s="26" t="n">
-        <v>40000</v>
+        <v>7000</v>
       </c>
       <c r="K9" s="26" t="n">
-        <v>35000</v>
+        <v>7000</v>
       </c>
       <c r="L9" s="26" t="n">
-        <v>30000</v>
+        <v>7000</v>
       </c>
       <c r="M9" s="26" t="n">
-        <v>25000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
+          <t>Other income, net ($)</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>FY26 $45M other income annualizes YTD $22,829; then steps down as cash is deployed (FY25 was only $28,352).</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 YTD other income (earnings)</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "22,829" → YTD other income ($000) on the earnings P&amp;L. FY26 model $45,000 annualizes that run-rate.</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>4163</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>43059</v>
+      </c>
+      <c r="G10" s="25" t="n">
+        <v>70380</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <v>28352</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>45000</v>
+      </c>
+      <c r="J10" s="26" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K10" s="26" t="n">
+        <v>35000</v>
+      </c>
+      <c r="L10" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M10" s="26" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
           <t>Effective tax rate %</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 outlook (≈30% tax)</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "a tax rate of approximately 30%" on the earnings outlook; FY25 10-K 29.5%. 3-statement model 30%</t>
         </is>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E11" s="23" t="n">
         <v>0.3585332413807594</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F11" s="23" t="n">
         <v>0.287509738088508</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G11" s="23" t="n">
         <v>0.2955893787336326</v>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H11" s="23" t="n">
         <v>0.2946823244826744</v>
       </c>
-      <c r="I10" s="24" t="n">
+      <c r="I11" s="24" t="n">
         <v>0.3</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J11" s="24" t="n">
         <v>0.3</v>
       </c>
-      <c r="K10" s="24" t="n">
+      <c r="K11" s="24" t="n">
         <v>0.3</v>
       </c>
-      <c r="L10" s="24" t="n">
+      <c r="L11" s="24" t="n">
         <v>0.3</v>
       </c>
-      <c r="M10" s="24" t="n">
+      <c r="M11" s="24" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>CAPITAL &amp; NON-CASH ITEMS</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="18" t="n"/>
-      <c r="L11" s="18" t="n"/>
-      <c r="M11" s="18" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>D&amp;A % of revenue</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
-      </c>
-      <c r="D12" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Depreciation and amortization" → 496,228 ÷ "Net revenue" 11,102,600 = 4.5%</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="n">
-        <v>0.03597686362326056</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>0.03943996628437186</v>
-      </c>
-      <c r="G12" s="23" t="n">
-        <v>0.04217214642137806</v>
-      </c>
-      <c r="H12" s="23" t="n">
-        <v>0.04469475618323636</v>
-      </c>
-      <c r="I12" s="24" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="J12" s="24" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="K12" s="24" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="L12" s="24" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="M12" s="24" t="n">
-        <v>0.045</v>
-      </c>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="18" t="n"/>
+      <c r="M12" s="18" t="n"/>
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>Capex % of revenue</t>
+          <t>D&amp;A % of revenue</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
+          <t>D&amp;A 4.5–4.6% of revenue; tracks recent depreciation intensity on PPE and lease-related amortization.</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -1395,160 +1395,160 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
+          <t>Ctrl+F "Depreciation and amortization" → 496,228 ÷ "Net revenue" 11,102,600 = 4.5%</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
-        <v>0.07874429228811279</v>
+        <v>0.03597686362326056</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>0.06776652052264213</v>
+        <v>0.03943996628437186</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>0.0650948052563787</v>
+        <v>0.04217214642137806</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>0.06131915046925945</v>
+        <v>0.04469475618323636</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.046</v>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.06</v>
+        <v>0.046</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.055</v>
+        <v>0.045</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0.05</v>
+        <v>0.045</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>0.05</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
+          <t>Capex % of revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="n">
+        <v>0.07874429228811279</v>
+      </c>
+      <c r="F14" s="23" t="n">
+        <v>0.06776652052264213</v>
+      </c>
+      <c r="G14" s="23" t="n">
+        <v>0.0650948052563787</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <v>0.06131915046925945</v>
+      </c>
+      <c r="I14" s="24" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J14" s="24" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="L14" s="24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="24" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
           <t>Stock-based compensation ($)</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
         </is>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E15" s="25" t="n">
         <v>78075</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F15" s="25" t="n">
         <v>93560</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G15" s="25" t="n">
         <v>90011</v>
       </c>
-      <c r="H14" s="25" t="n">
+      <c r="H15" s="25" t="n">
         <v>62203</v>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I15" s="26" t="n">
         <v>62000</v>
       </c>
-      <c r="J14" s="26" t="n">
+      <c r="J15" s="26" t="n">
         <v>62000</v>
       </c>
-      <c r="K14" s="26" t="n">
+      <c r="K15" s="26" t="n">
         <v>62000</v>
       </c>
-      <c r="L14" s="26" t="n">
+      <c r="L15" s="26" t="n">
         <v>62000</v>
       </c>
-      <c r="M14" s="26" t="n">
+      <c r="M15" s="26" t="n">
         <v>62000</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>WORKING CAPITAL &amp; BALANCE SHEET DRIVERS</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="18" t="n"/>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Inventories % of COGS</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
-        </is>
-      </c>
-      <c r="E16" s="23" t="n">
-        <v>0.4000264774148757</v>
-      </c>
-      <c r="F16" s="23" t="n">
-        <v>0.330085765808543</v>
-      </c>
-      <c r="G16" s="23" t="n">
-        <v>0.3340226506520835</v>
-      </c>
-      <c r="H16" s="23" t="n">
-        <v>0.3529655068789499</v>
-      </c>
-      <c r="I16" s="24" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="J16" s="24" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="K16" s="24" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L16" s="24" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="M16" s="24" t="n">
-        <v>0.33</v>
-      </c>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="18" t="n"/>
+      <c r="L16" s="18" t="n"/>
+      <c r="M16" s="18" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Accounts payable % of COGS</t>
+          <t>Inventories % of COGS</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
         </is>
       </c>
       <c r="C17" s="21" t="inlineStr">
@@ -1558,46 +1558,46 @@
       </c>
       <c r="D17" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
         </is>
       </c>
       <c r="E17" s="23" t="n">
-        <v>0.04774005037894764</v>
+        <v>0.4000264774148757</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>0.08689576951688993</v>
+        <v>0.330085765808543</v>
       </c>
       <c r="G17" s="23" t="n">
-        <v>0.06286453501771355</v>
+        <v>0.3340226506520835</v>
       </c>
       <c r="H17" s="23" t="n">
-        <v>0.06878140521012073</v>
+        <v>0.3529655068789499</v>
       </c>
       <c r="I17" s="24" t="n">
-        <v>0.068</v>
+        <v>0.34</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.068</v>
+        <v>0.335</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.068</v>
+        <v>0.33</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>0.068</v>
+        <v>0.33</v>
       </c>
       <c r="M17" s="24" t="n">
-        <v>0.068</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Accrued liabilities % of revenue</t>
+          <t>Accounts payable % of COGS</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
@@ -1607,46 +1607,46 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
-        <v>0.04922287331092786</v>
+        <v>0.04774005037894764</v>
       </c>
       <c r="F18" s="23" t="n">
-        <v>0.03623504799424655</v>
+        <v>0.08689576951688993</v>
       </c>
       <c r="G18" s="23" t="n">
-        <v>0.05283871763520759</v>
+        <v>0.06286453501771355</v>
       </c>
       <c r="H18" s="23" t="n">
-        <v>0.05971412101669879</v>
+        <v>0.06878140521012073</v>
       </c>
       <c r="I18" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="M18" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Other current assets % of revenue</t>
+          <t>Accrued liabilities % of revenue</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -1656,193 +1656,193 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
-        <v>0.06870325668471483</v>
+        <v>0.04922287331092786</v>
       </c>
       <c r="F19" s="23" t="n">
-        <v>0.05125166358639391</v>
+        <v>0.03623504799424655</v>
       </c>
       <c r="G19" s="23" t="n">
-        <v>0.05231190108617899</v>
+        <v>0.05283871763520759</v>
       </c>
       <c r="H19" s="23" t="n">
-        <v>0.06797921207645057</v>
+        <v>0.05971412101669879</v>
       </c>
       <c r="I19" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="M19" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Operating lease ROU asset % of revenue</t>
+          <t>Other current assets % of revenue</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
+          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
-        <v>0.1195261511040355</v>
+        <v>0.06870325668471483</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>0.1315701656610818</v>
+        <v>0.05125166358639391</v>
       </c>
       <c r="G20" s="23" t="n">
-        <v>0.1337588918001165</v>
+        <v>0.05231190108617899</v>
       </c>
       <c r="H20" s="23" t="n">
-        <v>0.1468287608307964</v>
+        <v>0.06797921207645057</v>
       </c>
       <c r="I20" s="24" t="n">
-        <v>0.147</v>
+        <v>0.068</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.147</v>
+        <v>0.068</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.147</v>
+        <v>0.068</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>0.147</v>
+        <v>0.068</v>
       </c>
       <c r="M20" s="24" t="n">
-        <v>0.147</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Other non-current assets % of revenue</t>
+          <t>Operating lease ROU asset % of revenue</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
+          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
-        <v>0.02002917692803345</v>
+        <v>0.1195261511040355</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>0.02036119550760462</v>
+        <v>0.1315701656610818</v>
       </c>
       <c r="G21" s="23" t="n">
-        <v>0.02407659296838742</v>
+        <v>0.1337588918001165</v>
       </c>
       <c r="H21" s="23" t="n">
-        <v>0.03052861491902797</v>
+        <v>0.1468287608307964</v>
       </c>
       <c r="I21" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="M21" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>Op lease liab (current) % of revenue</t>
+          <t>Other non-current assets % of revenue</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E22" s="23" t="n">
-        <v>0.02564225860789656</v>
+        <v>0.02002917692803345</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>0.02591358727754827</v>
+        <v>0.02036119550760462</v>
       </c>
       <c r="G22" s="23" t="n">
-        <v>0.02598703491061591</v>
+        <v>0.02407659296838742</v>
       </c>
       <c r="H22" s="23" t="n">
-        <v>0.02690576981968188</v>
+        <v>0.03052861491902797</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="K22" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Op lease liab (non-current) % of revenue</t>
+          <t>Op lease liab (current) % of revenue</t>
         </is>
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
         </is>
       </c>
       <c r="C23" s="21" t="inlineStr">
@@ -1852,239 +1852,288 @@
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
       <c r="E23" s="23" t="n">
-        <v>0.1063263776740277</v>
+        <v>0.02564225860789656</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>0.1199686712453887</v>
+        <v>0.02591358727754827</v>
       </c>
       <c r="G23" s="23" t="n">
-        <v>0.1228392068624797</v>
+        <v>0.02598703491061591</v>
       </c>
       <c r="H23" s="23" t="n">
-        <v>0.1350779997478068</v>
+        <v>0.02690576981968188</v>
       </c>
       <c r="I23" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="J23" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="M23" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Other current liabilities % of revenue</t>
+          <t>Op lease liab (non-current) % of revenue</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
-        <v>0.08782065461170298</v>
+        <v>0.1063263776740277</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>0.0712106459549251</v>
+        <v>0.1199686712453887</v>
       </c>
       <c r="G24" s="23" t="n">
-        <v>0.06928582073919408</v>
+        <v>0.1228392068624797</v>
       </c>
       <c r="H24" s="23" t="n">
-        <v>0.05353890079801128</v>
+        <v>0.1350779997478068</v>
       </c>
       <c r="I24" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="J24" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="K24" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="L24" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="M24" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
+          <t>Other current liabilities % of revenue</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="n">
+        <v>0.08782065461170298</v>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>0.0712106459549251</v>
+      </c>
+      <c r="G25" s="23" t="n">
+        <v>0.06928582073919408</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <v>0.05353890079801128</v>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="J25" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="K25" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="L25" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M25" s="24" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
           <t>Other non-current liab % of revenue</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
         </is>
       </c>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Other non-current liabilities" → 55,360 ÷ "Net revenue" 11,102,600 = 0.5%</t>
         </is>
       </c>
-      <c r="E25" s="23" t="n">
+      <c r="E26" s="23" t="n">
         <v>0.005991602509235539</v>
       </c>
-      <c r="F25" s="23" t="n">
+      <c r="F26" s="23" t="n">
         <v>0.00468486304273564</v>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G26" s="23" t="n">
         <v>0.003852428654513556</v>
       </c>
-      <c r="H25" s="23" t="n">
+      <c r="H26" s="23" t="n">
         <v>0.004986219444094176</v>
       </c>
-      <c r="I25" s="24" t="n">
+      <c r="I26" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="J25" s="24" t="n">
+      <c r="J26" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="K25" s="24" t="n">
+      <c r="K26" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="L25" s="24" t="n">
+      <c r="L26" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="M25" s="24" t="n">
+      <c r="M26" s="24" t="n">
         <v>0.005</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>CAPITAL RETURN</t>
         </is>
       </c>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
-      <c r="I26" s="18" t="n"/>
-      <c r="J26" s="18" t="n"/>
-      <c r="K26" s="18" t="n"/>
-      <c r="L26" s="18" t="n"/>
-      <c r="M26" s="18" t="n"/>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>Share repurchases ($)</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="inlineStr">
-        <is>
-          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>LULU CF: share repurchases (10-K)</t>
-        </is>
-      </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
-        </is>
-      </c>
-      <c r="E27" s="25" t="n">
-        <v>444001</v>
-      </c>
-      <c r="F27" s="25" t="n">
-        <v>558652</v>
-      </c>
-      <c r="G27" s="25" t="n">
-        <v>1636879</v>
-      </c>
-      <c r="H27" s="25" t="n">
-        <v>1178349</v>
-      </c>
-      <c r="I27" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="J27" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="K27" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="L27" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M27" s="26" t="n">
-        <v>500000</v>
-      </c>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
         <is>
+          <t>Share repurchases ($)</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>LULU CF: share repurchases (10-K)</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>444001</v>
+      </c>
+      <c r="F28" s="25" t="n">
+        <v>558652</v>
+      </c>
+      <c r="G28" s="25" t="n">
+        <v>1636879</v>
+      </c>
+      <c r="H28" s="25" t="n">
+        <v>1178349</v>
+      </c>
+      <c r="I28" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J28" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="K28" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="L28" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M28" s="26" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
           <t>Avg repurchase price ($/sh)</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>FY26 repurchase price $100 matches the current quote; path $100→$130 is a recovery assumption (FY25 10-K paid $168–$199).</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
         </is>
       </c>
-      <c r="I28" s="27" t="n">
+      <c r="I29" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="J28" s="27" t="n">
+      <c r="J29" s="27" t="n">
         <v>108</v>
       </c>
-      <c r="K28" s="27" t="n">
+      <c r="K29" s="27" t="n">
         <v>115</v>
       </c>
-      <c r="L28" s="27" t="n">
+      <c r="L29" s="27" t="n">
         <v>122</v>
       </c>
-      <c r="M28" s="27" t="n">
+      <c r="M29" s="27" t="n">
         <v>130</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="28" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
         <is>
           <t>Historical columns = derived ratios (black); projection columns = analyst inputs (red).</t>
         </is>
@@ -2102,10 +2151,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId17"/>
@@ -2115,8 +2164,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2128,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2297,12 +2347,12 @@
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Cost of goods sold</t>
+          <t>Cost of goods sold (ex-refunds)</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>Gross margin recovers gradually from promo pressure; 56.5% to 58.0% still below peak ~58–59% historical.</t>
+          <t>Clean GM 56.5%→58.0% (ex-refunds), still below peak ~58–59%. FY26 COGS is then reduced by the $134.5M IEEPA refund.</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
@@ -2348,675 +2398,772 @@
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Less: IEEPA tariff refunds (FY26 only)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 release: $134.5M IEEPA tariff refunds</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
+        </is>
+      </c>
+      <c r="E6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="26">
+        <f>-'Assumptions'!I7</f>
+        <v/>
+      </c>
+      <c r="J6" s="26">
+        <f>-'Assumptions'!J7</f>
+        <v/>
+      </c>
+      <c r="K6" s="26">
+        <f>-'Assumptions'!K7</f>
+        <v/>
+      </c>
+      <c r="L6" s="26">
+        <f>-'Assumptions'!L7</f>
+        <v/>
+      </c>
+      <c r="M6" s="26">
+        <f>-'Assumptions'!M7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="E6" s="33">
-        <f>E4-E5</f>
-        <v/>
-      </c>
-      <c r="F6" s="33">
-        <f>F4-F5</f>
-        <v/>
-      </c>
-      <c r="G6" s="33">
-        <f>G4-G5</f>
-        <v/>
-      </c>
-      <c r="H6" s="33">
-        <f>H4-H5</f>
-        <v/>
-      </c>
-      <c r="I6" s="33">
-        <f>I4-I5</f>
-        <v/>
-      </c>
-      <c r="J6" s="33">
-        <f>J4-J5</f>
-        <v/>
-      </c>
-      <c r="K6" s="33">
-        <f>K4-K5</f>
-        <v/>
-      </c>
-      <c r="L6" s="33">
-        <f>L4-L5</f>
-        <v/>
-      </c>
-      <c r="M6" s="33">
-        <f>M4-M5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>Selling, general &amp; administrative</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
-        </is>
-      </c>
-      <c r="E7" s="31" t="n">
-        <v>2757447</v>
-      </c>
-      <c r="F7" s="31" t="n">
-        <v>3397218</v>
-      </c>
-      <c r="G7" s="31" t="n">
-        <v>3762379</v>
-      </c>
-      <c r="H7" s="31" t="n">
-        <v>4066556</v>
-      </c>
-      <c r="I7" s="26">
-        <f>I4*'Assumptions'!I7</f>
-        <v/>
-      </c>
-      <c r="J7" s="26">
-        <f>J4*'Assumptions'!J7</f>
-        <v/>
-      </c>
-      <c r="K7" s="26">
-        <f>K4*'Assumptions'!K7</f>
-        <v/>
-      </c>
-      <c r="L7" s="26">
-        <f>L4*'Assumptions'!L7</f>
-        <v/>
-      </c>
-      <c r="M7" s="26">
-        <f>M4*'Assumptions'!M7</f>
+      <c r="E7" s="33">
+        <f>E4-E5-E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="33">
+        <f>F4-F5-F6</f>
+        <v/>
+      </c>
+      <c r="G7" s="33">
+        <f>G4-G5-G6</f>
+        <v/>
+      </c>
+      <c r="H7" s="33">
+        <f>H4-H5-H6</f>
+        <v/>
+      </c>
+      <c r="I7" s="33">
+        <f>I4-I5-I6</f>
+        <v/>
+      </c>
+      <c r="J7" s="33">
+        <f>J4-J5-J6</f>
+        <v/>
+      </c>
+      <c r="K7" s="33">
+        <f>K4-K5-K6</f>
+        <v/>
+      </c>
+      <c r="L7" s="33">
+        <f>L4-L5-L6</f>
+        <v/>
+      </c>
+      <c r="M7" s="33">
+        <f>M4-M5-M6</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
+          <t>Selling, general &amp; administrative</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>FY26 SG&amp;A 42.5% matches YTD 42.3% (earnings), vs FY25 36.7% 10-K; then fades to 39.5% as volume stabilizes.</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>LULU Q2 FY2026 earnings release (YTD SG&amp;A %)</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "41.7%" (Q2 SG&amp;A % of net revenue) and "42.3%" (first two quarters). FY25 10-K is 36.7%. Model FY26 42.5%</t>
+        </is>
+      </c>
+      <c r="E8" s="31" t="n">
+        <v>2757447</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>3397218</v>
+      </c>
+      <c r="G8" s="31" t="n">
+        <v>3762379</v>
+      </c>
+      <c r="H8" s="31" t="n">
+        <v>4066556</v>
+      </c>
+      <c r="I8" s="26">
+        <f>I4*'Assumptions'!I8</f>
+        <v/>
+      </c>
+      <c r="J8" s="26">
+        <f>J4*'Assumptions'!J8</f>
+        <v/>
+      </c>
+      <c r="K8" s="26">
+        <f>K4*'Assumptions'!K8</f>
+        <v/>
+      </c>
+      <c r="L8" s="26">
+        <f>L4*'Assumptions'!L8</f>
+        <v/>
+      </c>
+      <c r="M8" s="26">
+        <f>M4*'Assumptions'!M8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
           <t>Amortization of intangibles / other</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>$7M annual amortization run-rate; stable intangible amortization per recent 10-K disclosure levels.</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Amortization of intangible assets" → 6,961 ($000); model $7,000/yr</t>
         </is>
       </c>
-      <c r="E8" s="31" t="n">
+      <c r="E9" s="31" t="n">
         <v>406485</v>
       </c>
-      <c r="F8" s="31" t="n">
+      <c r="F9" s="31" t="n">
         <v>79511</v>
       </c>
-      <c r="G8" s="31" t="n">
+      <c r="G9" s="31" t="n">
         <v>2735</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H9" s="31" t="n">
         <v>6961</v>
       </c>
-      <c r="I8" s="26">
-        <f>'Assumptions'!I8</f>
-        <v/>
-      </c>
-      <c r="J8" s="26">
-        <f>'Assumptions'!J8</f>
-        <v/>
-      </c>
-      <c r="K8" s="26">
-        <f>'Assumptions'!K8</f>
-        <v/>
-      </c>
-      <c r="L8" s="26">
-        <f>'Assumptions'!L8</f>
-        <v/>
-      </c>
-      <c r="M8" s="26">
-        <f>'Assumptions'!M8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="I9" s="26">
+        <f>'Assumptions'!I9</f>
+        <v/>
+      </c>
+      <c r="J9" s="26">
+        <f>'Assumptions'!J9</f>
+        <v/>
+      </c>
+      <c r="K9" s="26">
+        <f>'Assumptions'!K9</f>
+        <v/>
+      </c>
+      <c r="L9" s="26">
+        <f>'Assumptions'!L9</f>
+        <v/>
+      </c>
+      <c r="M9" s="26">
+        <f>'Assumptions'!M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Operating income (EBIT)</t>
         </is>
       </c>
-      <c r="E9" s="33">
-        <f>E6-E7-E8</f>
-        <v/>
-      </c>
-      <c r="F9" s="33">
-        <f>F6-F7-F8</f>
-        <v/>
-      </c>
-      <c r="G9" s="33">
-        <f>G6-G7-G8</f>
-        <v/>
-      </c>
-      <c r="H9" s="33">
-        <f>H6-H7-H8</f>
-        <v/>
-      </c>
-      <c r="I9" s="33">
-        <f>I6-I7-I8</f>
-        <v/>
-      </c>
-      <c r="J9" s="33">
-        <f>J6-J7-J8</f>
-        <v/>
-      </c>
-      <c r="K9" s="33">
-        <f>K6-K7-K8</f>
-        <v/>
-      </c>
-      <c r="L9" s="33">
-        <f>L6-L7-L8</f>
-        <v/>
-      </c>
-      <c r="M9" s="33">
-        <f>M6-M7-M8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="E10" s="33">
+        <f>E7-E8-E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="33">
+        <f>F7-F8-F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="33">
+        <f>G7-G8-G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="33">
+        <f>H7-H8-H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="33">
+        <f>I7-I8-I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="33">
+        <f>J7-J8-J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="33">
+        <f>K7-K8-K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="33">
+        <f>L7-L8-L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="33">
+        <f>M7-M8-M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Other income, net</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>FY26 $45M other income annualizes YTD $22,829; then steps down as cash is deployed (FY25 was only $28,352).</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>Q2 FY2026 YTD other income (earnings)</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "22,829" → YTD other income ($000) on the earnings P&amp;L. FY26 model $45,000 annualizes that run-rate.</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
+      <c r="E11" s="31" t="n">
         <v>4163</v>
       </c>
-      <c r="F10" s="31" t="n">
+      <c r="F11" s="31" t="n">
         <v>43059</v>
       </c>
-      <c r="G10" s="31" t="n">
+      <c r="G11" s="31" t="n">
         <v>70380</v>
       </c>
-      <c r="H10" s="31" t="n">
+      <c r="H11" s="31" t="n">
         <v>28352</v>
       </c>
-      <c r="I10" s="26">
-        <f>'Assumptions'!I9</f>
-        <v/>
-      </c>
-      <c r="J10" s="26">
-        <f>'Assumptions'!J9</f>
-        <v/>
-      </c>
-      <c r="K10" s="26">
-        <f>'Assumptions'!K9</f>
-        <v/>
-      </c>
-      <c r="L10" s="26">
-        <f>'Assumptions'!L9</f>
-        <v/>
-      </c>
-      <c r="M10" s="26">
-        <f>'Assumptions'!M9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="I11" s="26">
+        <f>'Assumptions'!I10</f>
+        <v/>
+      </c>
+      <c r="J11" s="26">
+        <f>'Assumptions'!J10</f>
+        <v/>
+      </c>
+      <c r="K11" s="26">
+        <f>'Assumptions'!K10</f>
+        <v/>
+      </c>
+      <c r="L11" s="26">
+        <f>'Assumptions'!L10</f>
+        <v/>
+      </c>
+      <c r="M11" s="26">
+        <f>'Assumptions'!M10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Pre-tax income</t>
         </is>
       </c>
-      <c r="E11" s="33">
-        <f>E9+E10</f>
-        <v/>
-      </c>
-      <c r="F11" s="33">
-        <f>F9+F10</f>
-        <v/>
-      </c>
-      <c r="G11" s="33">
-        <f>G9+G10</f>
-        <v/>
-      </c>
-      <c r="H11" s="33">
-        <f>H9+H10</f>
-        <v/>
-      </c>
-      <c r="I11" s="33">
-        <f>I9+I10</f>
-        <v/>
-      </c>
-      <c r="J11" s="33">
-        <f>J9+J10</f>
-        <v/>
-      </c>
-      <c r="K11" s="33">
-        <f>K9+K10</f>
-        <v/>
-      </c>
-      <c r="L11" s="33">
-        <f>L9+L10</f>
-        <v/>
-      </c>
-      <c r="M11" s="33">
-        <f>M9+M10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="E12" s="33">
+        <f>E10+E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="33">
+        <f>F10+F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="33">
+        <f>G10+G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="33">
+        <f>H10+H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="33">
+        <f>I10+I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="33">
+        <f>J10+J11</f>
+        <v/>
+      </c>
+      <c r="K12" s="33">
+        <f>K10+K11</f>
+        <v/>
+      </c>
+      <c r="L12" s="33">
+        <f>L10+L11</f>
+        <v/>
+      </c>
+      <c r="M12" s="33">
+        <f>M10+M11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Income tax expense</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>30% effective tax rate on projections; conservative vs recent ~29% effective, allows for jurisdictional mix.</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 outlook (≈30% tax)</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "a tax rate of approximately 30%" on the earnings outlook; FY25 10-K 29.5%. 3-statement model 30%</t>
         </is>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E13" s="31" t="n">
         <v>477771</v>
       </c>
-      <c r="F12" s="31" t="n">
+      <c r="F13" s="31" t="n">
         <v>625545</v>
       </c>
-      <c r="G12" s="31" t="n">
+      <c r="G13" s="31" t="n">
         <v>761461</v>
       </c>
-      <c r="H12" s="31" t="n">
+      <c r="H13" s="31" t="n">
         <v>659784</v>
       </c>
-      <c r="I12" s="26">
-        <f>I11*'Assumptions'!I10</f>
-        <v/>
-      </c>
-      <c r="J12" s="26">
-        <f>J11*'Assumptions'!J10</f>
-        <v/>
-      </c>
-      <c r="K12" s="26">
-        <f>K11*'Assumptions'!K10</f>
-        <v/>
-      </c>
-      <c r="L12" s="26">
-        <f>L11*'Assumptions'!L10</f>
-        <v/>
-      </c>
-      <c r="M12" s="26">
-        <f>M11*'Assumptions'!M10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="I13" s="26">
+        <f>I12*'Assumptions'!I11</f>
+        <v/>
+      </c>
+      <c r="J13" s="26">
+        <f>J12*'Assumptions'!J11</f>
+        <v/>
+      </c>
+      <c r="K13" s="26">
+        <f>K12*'Assumptions'!K11</f>
+        <v/>
+      </c>
+      <c r="L13" s="26">
+        <f>L12*'Assumptions'!L11</f>
+        <v/>
+      </c>
+      <c r="M13" s="26">
+        <f>M12*'Assumptions'!M11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="E13" s="34">
-        <f>E11-E12</f>
-        <v/>
-      </c>
-      <c r="F13" s="34">
-        <f>F11-F12</f>
-        <v/>
-      </c>
-      <c r="G13" s="34">
-        <f>G11-G12</f>
-        <v/>
-      </c>
-      <c r="H13" s="34">
-        <f>H11-H12</f>
-        <v/>
-      </c>
-      <c r="I13" s="34">
-        <f>I11-I12</f>
-        <v/>
-      </c>
-      <c r="J13" s="34">
-        <f>J11-J12</f>
-        <v/>
-      </c>
-      <c r="K13" s="34">
-        <f>K11-K12</f>
-        <v/>
-      </c>
-      <c r="L13" s="34">
-        <f>L11-L12</f>
-        <v/>
-      </c>
-      <c r="M13" s="34">
-        <f>M11-M12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="E14" s="34">
+        <f>E12-E13</f>
+        <v/>
+      </c>
+      <c r="F14" s="34">
+        <f>F12-F13</f>
+        <v/>
+      </c>
+      <c r="G14" s="34">
+        <f>G12-G13</f>
+        <v/>
+      </c>
+      <c r="H14" s="34">
+        <f>H12-H13</f>
+        <v/>
+      </c>
+      <c r="I14" s="34">
+        <f>I12-I13</f>
+        <v/>
+      </c>
+      <c r="J14" s="34">
+        <f>J12-J13</f>
+        <v/>
+      </c>
+      <c r="K14" s="34">
+        <f>K12-K13</f>
+        <v/>
+      </c>
+      <c r="L14" s="34">
+        <f>L12-L13</f>
+        <v/>
+      </c>
+      <c r="M14" s="34">
+        <f>M12-M13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Diluted weighted-avg shares (000)</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.
 Also: FY26 repurchase price $100 matches the current quote; path $100→$130 is a recovery assumption (FY25 10-K paid $168–$199).</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C16" s="35" t="inlineStr">
         <is>
           <t>LULU CF: share repurchases (10-K)
 Also: NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr
 Also: Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
         </is>
       </c>
-      <c r="E15" s="31" t="n">
+      <c r="E16" s="31" t="n">
         <v>128017</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="F16" s="31" t="n">
         <v>127060</v>
       </c>
-      <c r="G15" s="31" t="n">
+      <c r="G16" s="31" t="n">
         <v>123935</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H16" s="31" t="n">
         <v>119068</v>
       </c>
-      <c r="I15" s="26">
-        <f>H15-'Assumptions'!I27/'Assumptions'!I28</f>
-        <v/>
-      </c>
-      <c r="J15" s="26">
-        <f>I15-'Assumptions'!J27/'Assumptions'!J28</f>
-        <v/>
-      </c>
-      <c r="K15" s="26">
-        <f>J15-'Assumptions'!K27/'Assumptions'!K28</f>
-        <v/>
-      </c>
-      <c r="L15" s="26">
-        <f>K15-'Assumptions'!L27/'Assumptions'!L28</f>
-        <v/>
-      </c>
-      <c r="M15" s="26">
-        <f>L15-'Assumptions'!M27/'Assumptions'!M28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="I16" s="26">
+        <f>H16-'Assumptions'!I28/'Assumptions'!I29</f>
+        <v/>
+      </c>
+      <c r="J16" s="26">
+        <f>I16-'Assumptions'!J28/'Assumptions'!J29</f>
+        <v/>
+      </c>
+      <c r="K16" s="26">
+        <f>J16-'Assumptions'!K28/'Assumptions'!K29</f>
+        <v/>
+      </c>
+      <c r="L16" s="26">
+        <f>K16-'Assumptions'!L28/'Assumptions'!L29</f>
+        <v/>
+      </c>
+      <c r="M16" s="26">
+        <f>L16-'Assumptions'!M28/'Assumptions'!M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>Diluted EPS ($)</t>
         </is>
       </c>
-      <c r="E16" s="36" t="n">
+      <c r="E17" s="36" t="n">
         <v>6.68</v>
       </c>
-      <c r="F16" s="36" t="n">
+      <c r="F17" s="36" t="n">
         <v>12.2</v>
       </c>
-      <c r="G16" s="36" t="n">
+      <c r="G17" s="36" t="n">
         <v>14.64</v>
       </c>
-      <c r="H16" s="36" t="n">
+      <c r="H17" s="36" t="n">
         <v>13.26</v>
       </c>
-      <c r="I16" s="37">
-        <f>I13/I15</f>
-        <v/>
-      </c>
-      <c r="J16" s="37">
-        <f>J13/J15</f>
-        <v/>
-      </c>
-      <c r="K16" s="37">
-        <f>K13/K15</f>
-        <v/>
-      </c>
-      <c r="L16" s="37">
-        <f>L13/L15</f>
-        <v/>
-      </c>
-      <c r="M16" s="37">
-        <f>M13/M15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="I17" s="37">
+        <f>I14/I16</f>
+        <v/>
+      </c>
+      <c r="J17" s="37">
+        <f>J14/J16</f>
+        <v/>
+      </c>
+      <c r="K17" s="37">
+        <f>K14/K16</f>
+        <v/>
+      </c>
+      <c r="L17" s="37">
+        <f>L14/L16</f>
+        <v/>
+      </c>
+      <c r="M17" s="37">
+        <f>M14/M16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>Margins &amp; growth</t>
         </is>
       </c>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
-      <c r="I18" s="18" t="n"/>
-      <c r="J18" s="18" t="n"/>
-      <c r="K18" s="18" t="n"/>
-      <c r="L18" s="18" t="n"/>
-      <c r="M18" s="18" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="39" t="inlineStr">
-        <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="E19" s="40">
-        <f>E6/E4</f>
-        <v/>
-      </c>
-      <c r="F19" s="40">
-        <f>F6/F4</f>
-        <v/>
-      </c>
-      <c r="G19" s="40">
-        <f>G6/G4</f>
-        <v/>
-      </c>
-      <c r="H19" s="40">
-        <f>H6/H4</f>
-        <v/>
-      </c>
-      <c r="I19" s="40">
-        <f>I6/I4</f>
-        <v/>
-      </c>
-      <c r="J19" s="40">
-        <f>J6/J4</f>
-        <v/>
-      </c>
-      <c r="K19" s="40">
-        <f>K6/K4</f>
-        <v/>
-      </c>
-      <c r="L19" s="40">
-        <f>L6/L4</f>
-        <v/>
-      </c>
-      <c r="M19" s="40">
-        <f>M6/M4</f>
-        <v/>
-      </c>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="18" t="n"/>
+      <c r="M19" s="18" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="inlineStr">
         <is>
-          <t>Operating margin %</t>
+          <t>Gross margin %</t>
         </is>
       </c>
       <c r="E20" s="40">
-        <f>E9/E4</f>
+        <f>E7/E4</f>
         <v/>
       </c>
       <c r="F20" s="40">
-        <f>F9/F4</f>
+        <f>F7/F4</f>
         <v/>
       </c>
       <c r="G20" s="40">
-        <f>G9/G4</f>
+        <f>G7/G4</f>
         <v/>
       </c>
       <c r="H20" s="40">
-        <f>H9/H4</f>
+        <f>H7/H4</f>
         <v/>
       </c>
       <c r="I20" s="40">
-        <f>I9/I4</f>
+        <f>I7/I4</f>
         <v/>
       </c>
       <c r="J20" s="40">
-        <f>J9/J4</f>
+        <f>J7/J4</f>
         <v/>
       </c>
       <c r="K20" s="40">
-        <f>K9/K4</f>
+        <f>K7/K4</f>
         <v/>
       </c>
       <c r="L20" s="40">
-        <f>L9/L4</f>
+        <f>L7/L4</f>
         <v/>
       </c>
       <c r="M20" s="40">
-        <f>M9/M4</f>
+        <f>M7/M4</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="39" t="inlineStr">
         <is>
-          <t>Net margin %</t>
+          <t>Clean operating margin % (ex-refunds)</t>
         </is>
       </c>
       <c r="E21" s="40">
-        <f>E13/E4</f>
+        <f>(E10+E6)/E4</f>
         <v/>
       </c>
       <c r="F21" s="40">
-        <f>F13/F4</f>
+        <f>(F10+F6)/F4</f>
         <v/>
       </c>
       <c r="G21" s="40">
-        <f>G13/G4</f>
+        <f>(G10+G6)/G4</f>
         <v/>
       </c>
       <c r="H21" s="40">
-        <f>H13/H4</f>
+        <f>(H10+H6)/H4</f>
         <v/>
       </c>
       <c r="I21" s="40">
-        <f>I13/I4</f>
+        <f>(I10+I6)/I4</f>
         <v/>
       </c>
       <c r="J21" s="40">
-        <f>J13/J4</f>
+        <f>(J10+J6)/J4</f>
         <v/>
       </c>
       <c r="K21" s="40">
-        <f>K13/K4</f>
+        <f>(K10+K6)/K4</f>
         <v/>
       </c>
       <c r="L21" s="40">
-        <f>L13/L4</f>
+        <f>(L10+L6)/L4</f>
         <v/>
       </c>
       <c r="M21" s="40">
-        <f>M13/M4</f>
+        <f>(M10+M6)/M4</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="inlineStr">
         <is>
+          <t>Operating margin % (reported, incl. FY26 refund)</t>
+        </is>
+      </c>
+      <c r="E22" s="40">
+        <f>E10/E4</f>
+        <v/>
+      </c>
+      <c r="F22" s="40">
+        <f>F10/F4</f>
+        <v/>
+      </c>
+      <c r="G22" s="40">
+        <f>G10/G4</f>
+        <v/>
+      </c>
+      <c r="H22" s="40">
+        <f>H10/H4</f>
+        <v/>
+      </c>
+      <c r="I22" s="40">
+        <f>I10/I4</f>
+        <v/>
+      </c>
+      <c r="J22" s="40">
+        <f>J10/J4</f>
+        <v/>
+      </c>
+      <c r="K22" s="40">
+        <f>K10/K4</f>
+        <v/>
+      </c>
+      <c r="L22" s="40">
+        <f>L10/L4</f>
+        <v/>
+      </c>
+      <c r="M22" s="40">
+        <f>M10/M4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>Net margin %</t>
+        </is>
+      </c>
+      <c r="E23" s="40">
+        <f>E14/E4</f>
+        <v/>
+      </c>
+      <c r="F23" s="40">
+        <f>F14/F4</f>
+        <v/>
+      </c>
+      <c r="G23" s="40">
+        <f>G14/G4</f>
+        <v/>
+      </c>
+      <c r="H23" s="40">
+        <f>H14/H4</f>
+        <v/>
+      </c>
+      <c r="I23" s="40">
+        <f>I14/I4</f>
+        <v/>
+      </c>
+      <c r="J23" s="40">
+        <f>J14/J4</f>
+        <v/>
+      </c>
+      <c r="K23" s="40">
+        <f>K14/K4</f>
+        <v/>
+      </c>
+      <c r="L23" s="40">
+        <f>L14/L4</f>
+        <v/>
+      </c>
+      <c r="M23" s="40">
+        <f>M14/M4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="E22" s="41" t="inlineStr">
+      <c r="E24" s="41" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="F22" s="40">
+      <c r="F24" s="40">
         <f>F4/E4-1</f>
         <v/>
       </c>
-      <c r="G22" s="40">
+      <c r="G24" s="40">
         <f>G4/F4-1</f>
         <v/>
       </c>
-      <c r="H22" s="40">
+      <c r="H24" s="40">
         <f>H4/G4-1</f>
         <v/>
       </c>
-      <c r="I22" s="40">
+      <c r="I24" s="40">
         <f>I4/H4-1</f>
         <v/>
       </c>
-      <c r="J22" s="40">
+      <c r="J24" s="40">
         <f>J4/I4-1</f>
         <v/>
       </c>
-      <c r="K22" s="40">
+      <c r="K24" s="40">
         <f>K4/J4-1</f>
         <v/>
       </c>
-      <c r="L22" s="40">
+      <c r="L24" s="40">
         <f>L4/K4-1</f>
         <v/>
       </c>
-      <c r="M22" s="40">
+      <c r="M24" s="40">
         <f>M4/L4-1</f>
         <v/>
       </c>
@@ -3037,35 +3184,40 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3285,23 +3437,23 @@
         <v>1700753</v>
       </c>
       <c r="I7" s="26">
-        <f>'Income Statement'!I5*'Assumptions'!I16</f>
+        <f>'Income Statement'!I5*'Assumptions'!I17</f>
         <v/>
       </c>
       <c r="J7" s="26">
-        <f>'Income Statement'!J5*'Assumptions'!J16</f>
+        <f>'Income Statement'!J5*'Assumptions'!J17</f>
         <v/>
       </c>
       <c r="K7" s="26">
-        <f>'Income Statement'!K5*'Assumptions'!K16</f>
+        <f>'Income Statement'!K5*'Assumptions'!K17</f>
         <v/>
       </c>
       <c r="L7" s="26">
-        <f>'Income Statement'!L5*'Assumptions'!L16</f>
+        <f>'Income Statement'!L5*'Assumptions'!L17</f>
         <v/>
       </c>
       <c r="M7" s="26">
-        <f>'Income Statement'!M5*'Assumptions'!M16</f>
+        <f>'Income Statement'!M5*'Assumptions'!M17</f>
         <v/>
       </c>
     </row>
@@ -3339,23 +3491,23 @@
         <v>754746</v>
       </c>
       <c r="I8" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I19</f>
+        <f>'Income Statement'!I4*'Assumptions'!I20</f>
         <v/>
       </c>
       <c r="J8" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J19</f>
+        <f>'Income Statement'!J4*'Assumptions'!J20</f>
         <v/>
       </c>
       <c r="K8" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K19</f>
+        <f>'Income Statement'!K4*'Assumptions'!K20</f>
         <v/>
       </c>
       <c r="L8" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L19</f>
+        <f>'Income Statement'!L4*'Assumptions'!L20</f>
         <v/>
       </c>
       <c r="M8" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M19</f>
+        <f>'Income Statement'!M4*'Assumptions'!M20</f>
         <v/>
       </c>
     </row>
@@ -3439,23 +3591,23 @@
         <v>2033720</v>
       </c>
       <c r="I11" s="26">
-        <f>H11+'Income Statement'!I4*'Assumptions'!I13-'Income Statement'!I4*'Assumptions'!I12</f>
+        <f>H11+'Income Statement'!I4*'Assumptions'!I14-'Income Statement'!I4*'Assumptions'!I13</f>
         <v/>
       </c>
       <c r="J11" s="26">
-        <f>I11+'Income Statement'!J4*'Assumptions'!J13-'Income Statement'!J4*'Assumptions'!J12</f>
+        <f>I11+'Income Statement'!J4*'Assumptions'!J14-'Income Statement'!J4*'Assumptions'!J13</f>
         <v/>
       </c>
       <c r="K11" s="26">
-        <f>J11+'Income Statement'!K4*'Assumptions'!K13-'Income Statement'!K4*'Assumptions'!K12</f>
+        <f>J11+'Income Statement'!K4*'Assumptions'!K14-'Income Statement'!K4*'Assumptions'!K13</f>
         <v/>
       </c>
       <c r="L11" s="26">
-        <f>K11+'Income Statement'!L4*'Assumptions'!L13-'Income Statement'!L4*'Assumptions'!L12</f>
+        <f>K11+'Income Statement'!L4*'Assumptions'!L14-'Income Statement'!L4*'Assumptions'!L13</f>
         <v/>
       </c>
       <c r="M11" s="26">
-        <f>L11+'Income Statement'!M4*'Assumptions'!M13-'Income Statement'!M4*'Assumptions'!M12</f>
+        <f>L11+'Income Statement'!M4*'Assumptions'!M14-'Income Statement'!M4*'Assumptions'!M13</f>
         <v/>
       </c>
     </row>
@@ -3493,23 +3645,23 @@
         <v>1630181</v>
       </c>
       <c r="I12" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I20</f>
+        <f>'Income Statement'!I4*'Assumptions'!I21</f>
         <v/>
       </c>
       <c r="J12" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J20</f>
+        <f>'Income Statement'!J4*'Assumptions'!J21</f>
         <v/>
       </c>
       <c r="K12" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K20</f>
+        <f>'Income Statement'!K4*'Assumptions'!K21</f>
         <v/>
       </c>
       <c r="L12" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L20</f>
+        <f>'Income Statement'!L4*'Assumptions'!L21</f>
         <v/>
       </c>
       <c r="M12" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M20</f>
+        <f>'Income Statement'!M4*'Assumptions'!M21</f>
         <v/>
       </c>
     </row>
@@ -3586,23 +3738,23 @@
         <v>338947</v>
       </c>
       <c r="I14" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I21</f>
+        <f>'Income Statement'!I4*'Assumptions'!I22</f>
         <v/>
       </c>
       <c r="J14" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J21</f>
+        <f>'Income Statement'!J4*'Assumptions'!J22</f>
         <v/>
       </c>
       <c r="K14" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K21</f>
+        <f>'Income Statement'!K4*'Assumptions'!K22</f>
         <v/>
       </c>
       <c r="L14" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L21</f>
+        <f>'Income Statement'!L4*'Assumptions'!L22</f>
         <v/>
       </c>
       <c r="M14" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M21</f>
+        <f>'Income Statement'!M4*'Assumptions'!M22</f>
         <v/>
       </c>
     </row>
@@ -3702,23 +3854,23 @@
         <v>331421</v>
       </c>
       <c r="I19" s="26">
-        <f>'Income Statement'!I5*'Assumptions'!I17</f>
+        <f>'Income Statement'!I5*'Assumptions'!I18</f>
         <v/>
       </c>
       <c r="J19" s="26">
-        <f>'Income Statement'!J5*'Assumptions'!J17</f>
+        <f>'Income Statement'!J5*'Assumptions'!J18</f>
         <v/>
       </c>
       <c r="K19" s="26">
-        <f>'Income Statement'!K5*'Assumptions'!K17</f>
+        <f>'Income Statement'!K5*'Assumptions'!K18</f>
         <v/>
       </c>
       <c r="L19" s="26">
-        <f>'Income Statement'!L5*'Assumptions'!L17</f>
+        <f>'Income Statement'!L5*'Assumptions'!L18</f>
         <v/>
       </c>
       <c r="M19" s="26">
-        <f>'Income Statement'!M5*'Assumptions'!M17</f>
+        <f>'Income Statement'!M5*'Assumptions'!M18</f>
         <v/>
       </c>
     </row>
@@ -3756,23 +3908,23 @@
         <v>662982</v>
       </c>
       <c r="I20" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I18</f>
+        <f>'Income Statement'!I4*'Assumptions'!I19</f>
         <v/>
       </c>
       <c r="J20" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J18</f>
+        <f>'Income Statement'!J4*'Assumptions'!J19</f>
         <v/>
       </c>
       <c r="K20" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K18</f>
+        <f>'Income Statement'!K4*'Assumptions'!K19</f>
         <v/>
       </c>
       <c r="L20" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L18</f>
+        <f>'Income Statement'!L4*'Assumptions'!L19</f>
         <v/>
       </c>
       <c r="M20" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M18</f>
+        <f>'Income Statement'!M4*'Assumptions'!M19</f>
         <v/>
       </c>
     </row>
@@ -3810,23 +3962,23 @@
         <v>298724</v>
       </c>
       <c r="I21" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I22</f>
+        <f>'Income Statement'!I4*'Assumptions'!I23</f>
         <v/>
       </c>
       <c r="J21" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J22</f>
+        <f>'Income Statement'!J4*'Assumptions'!J23</f>
         <v/>
       </c>
       <c r="K21" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K22</f>
+        <f>'Income Statement'!K4*'Assumptions'!K23</f>
         <v/>
       </c>
       <c r="L21" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L22</f>
+        <f>'Income Statement'!L4*'Assumptions'!L23</f>
         <v/>
       </c>
       <c r="M21" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M22</f>
+        <f>'Income Statement'!M4*'Assumptions'!M23</f>
         <v/>
       </c>
     </row>
@@ -3864,23 +4016,23 @@
         <v>594421</v>
       </c>
       <c r="I22" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I24</f>
+        <f>'Income Statement'!I4*'Assumptions'!I25</f>
         <v/>
       </c>
       <c r="J22" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J24</f>
+        <f>'Income Statement'!J4*'Assumptions'!J25</f>
         <v/>
       </c>
       <c r="K22" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K24</f>
+        <f>'Income Statement'!K4*'Assumptions'!K25</f>
         <v/>
       </c>
       <c r="L22" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L24</f>
+        <f>'Income Statement'!L4*'Assumptions'!L25</f>
         <v/>
       </c>
       <c r="M22" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M24</f>
+        <f>'Income Statement'!M4*'Assumptions'!M25</f>
         <v/>
       </c>
     </row>
@@ -3964,23 +4116,23 @@
         <v>1499717</v>
       </c>
       <c r="I25" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I23</f>
+        <f>'Income Statement'!I4*'Assumptions'!I24</f>
         <v/>
       </c>
       <c r="J25" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J23</f>
+        <f>'Income Statement'!J4*'Assumptions'!J24</f>
         <v/>
       </c>
       <c r="K25" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K23</f>
+        <f>'Income Statement'!K4*'Assumptions'!K24</f>
         <v/>
       </c>
       <c r="L25" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L23</f>
+        <f>'Income Statement'!L4*'Assumptions'!L24</f>
         <v/>
       </c>
       <c r="M25" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M23</f>
+        <f>'Income Statement'!M4*'Assumptions'!M24</f>
         <v/>
       </c>
     </row>
@@ -4057,23 +4209,23 @@
         <v>55360</v>
       </c>
       <c r="I27" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I25</f>
+        <f>'Income Statement'!I4*'Assumptions'!I26</f>
         <v/>
       </c>
       <c r="J27" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J25</f>
+        <f>'Income Statement'!J4*'Assumptions'!J26</f>
         <v/>
       </c>
       <c r="K27" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K25</f>
+        <f>'Income Statement'!K4*'Assumptions'!K26</f>
         <v/>
       </c>
       <c r="L27" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L25</f>
+        <f>'Income Statement'!L4*'Assumptions'!L26</f>
         <v/>
       </c>
       <c r="M27" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M25</f>
+        <f>'Income Statement'!M4*'Assumptions'!M26</f>
         <v/>
       </c>
     </row>
@@ -4157,23 +4309,23 @@
         <v>669949</v>
       </c>
       <c r="I31" s="26">
-        <f>H31+'Assumptions'!I14</f>
+        <f>H31+'Assumptions'!I15</f>
         <v/>
       </c>
       <c r="J31" s="26">
-        <f>I31+'Assumptions'!J14</f>
+        <f>I31+'Assumptions'!J15</f>
         <v/>
       </c>
       <c r="K31" s="26">
-        <f>J31+'Assumptions'!K14</f>
+        <f>J31+'Assumptions'!K15</f>
         <v/>
       </c>
       <c r="L31" s="26">
-        <f>K31+'Assumptions'!L14</f>
+        <f>K31+'Assumptions'!L15</f>
         <v/>
       </c>
       <c r="M31" s="26">
-        <f>L31+'Assumptions'!M14</f>
+        <f>L31+'Assumptions'!M15</f>
         <v/>
       </c>
     </row>
@@ -4211,23 +4363,23 @@
         <v>4522581</v>
       </c>
       <c r="I32" s="26">
-        <f>H32+'Income Statement'!I13-'Assumptions'!I27</f>
+        <f>H32+'Income Statement'!I14-'Assumptions'!I28</f>
         <v/>
       </c>
       <c r="J32" s="26">
-        <f>I32+'Income Statement'!J13-'Assumptions'!J27</f>
+        <f>I32+'Income Statement'!J14-'Assumptions'!J28</f>
         <v/>
       </c>
       <c r="K32" s="26">
-        <f>J32+'Income Statement'!K13-'Assumptions'!K27</f>
+        <f>J32+'Income Statement'!K14-'Assumptions'!K28</f>
         <v/>
       </c>
       <c r="L32" s="26">
-        <f>K32+'Income Statement'!L13-'Assumptions'!L27</f>
+        <f>K32+'Income Statement'!L14-'Assumptions'!L28</f>
         <v/>
       </c>
       <c r="M32" s="26">
-        <f>L32+'Income Statement'!M13-'Assumptions'!M27</f>
+        <f>L32+'Income Statement'!M14-'Assumptions'!M28</f>
         <v/>
       </c>
     </row>
@@ -4644,23 +4796,23 @@
         <v>1579183</v>
       </c>
       <c r="I5" s="25">
-        <f>'Income Statement'!I13</f>
+        <f>'Income Statement'!I14</f>
         <v/>
       </c>
       <c r="J5" s="25">
-        <f>'Income Statement'!J13</f>
+        <f>'Income Statement'!J14</f>
         <v/>
       </c>
       <c r="K5" s="25">
-        <f>'Income Statement'!K13</f>
+        <f>'Income Statement'!K14</f>
         <v/>
       </c>
       <c r="L5" s="25">
-        <f>'Income Statement'!L13</f>
+        <f>'Income Statement'!L14</f>
         <v/>
       </c>
       <c r="M5" s="25">
-        <f>'Income Statement'!M13</f>
+        <f>'Income Statement'!M14</f>
         <v/>
       </c>
     </row>
@@ -4698,23 +4850,23 @@
         <v>496228</v>
       </c>
       <c r="I6" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I12</f>
+        <f>'Income Statement'!I4*'Assumptions'!I13</f>
         <v/>
       </c>
       <c r="J6" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J12</f>
+        <f>'Income Statement'!J4*'Assumptions'!J13</f>
         <v/>
       </c>
       <c r="K6" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K12</f>
+        <f>'Income Statement'!K4*'Assumptions'!K13</f>
         <v/>
       </c>
       <c r="L6" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L12</f>
+        <f>'Income Statement'!L4*'Assumptions'!L13</f>
         <v/>
       </c>
       <c r="M6" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M12</f>
+        <f>'Income Statement'!M4*'Assumptions'!M13</f>
         <v/>
       </c>
     </row>
@@ -4752,23 +4904,23 @@
         <v>62203</v>
       </c>
       <c r="I7" s="26">
-        <f>'Assumptions'!I14</f>
+        <f>'Assumptions'!I15</f>
         <v/>
       </c>
       <c r="J7" s="26">
-        <f>'Assumptions'!J14</f>
+        <f>'Assumptions'!J15</f>
         <v/>
       </c>
       <c r="K7" s="26">
-        <f>'Assumptions'!K14</f>
+        <f>'Assumptions'!K15</f>
         <v/>
       </c>
       <c r="L7" s="26">
-        <f>'Assumptions'!L14</f>
+        <f>'Assumptions'!L15</f>
         <v/>
       </c>
       <c r="M7" s="26">
-        <f>'Assumptions'!M14</f>
+        <f>'Assumptions'!M15</f>
         <v/>
       </c>
     </row>
@@ -5474,23 +5626,23 @@
         <v>-680802</v>
       </c>
       <c r="I22" s="26">
-        <f>-'Income Statement'!I4*'Assumptions'!I13</f>
+        <f>-'Income Statement'!I4*'Assumptions'!I14</f>
         <v/>
       </c>
       <c r="J22" s="26">
-        <f>-'Income Statement'!J4*'Assumptions'!J13</f>
+        <f>-'Income Statement'!J4*'Assumptions'!J14</f>
         <v/>
       </c>
       <c r="K22" s="26">
-        <f>-'Income Statement'!K4*'Assumptions'!K13</f>
+        <f>-'Income Statement'!K4*'Assumptions'!K14</f>
         <v/>
       </c>
       <c r="L22" s="26">
-        <f>-'Income Statement'!L4*'Assumptions'!L13</f>
+        <f>-'Income Statement'!L4*'Assumptions'!L14</f>
         <v/>
       </c>
       <c r="M22" s="26">
-        <f>-'Income Statement'!M4*'Assumptions'!M13</f>
+        <f>-'Income Statement'!M4*'Assumptions'!M14</f>
         <v/>
       </c>
     </row>
@@ -5590,23 +5742,23 @@
         <v>-1178349</v>
       </c>
       <c r="I27" s="26">
-        <f>-'Assumptions'!I27</f>
+        <f>-'Assumptions'!I28</f>
         <v/>
       </c>
       <c r="J27" s="26">
-        <f>-'Assumptions'!J27</f>
+        <f>-'Assumptions'!J28</f>
         <v/>
       </c>
       <c r="K27" s="26">
-        <f>-'Assumptions'!K27</f>
+        <f>-'Assumptions'!K28</f>
         <v/>
       </c>
       <c r="L27" s="26">
-        <f>-'Assumptions'!L27</f>
+        <f>-'Assumptions'!L28</f>
         <v/>
       </c>
       <c r="M27" s="26">
-        <f>-'Assumptions'!M27</f>
+        <f>-'Assumptions'!M28</f>
         <v/>
       </c>
     </row>
@@ -5711,12 +5863,15 @@
       <c r="F32" s="31" t="n">
         <v>1154867</v>
       </c>
-      <c r="G32" s="25">
-        <f>'Balance Sheet'!F6</f>
-        <v/>
+      <c r="G32" s="31" t="n">
+        <v>2243971</v>
       </c>
       <c r="H32" s="31" t="n">
         <v>1984336</v>
+      </c>
+      <c r="I32" s="25">
+        <f>H33</f>
+        <v/>
       </c>
       <c r="J32" s="25">
         <f>I33</f>

</xml_diff>

<commit_message>
Rebuild models with unique 19.9% OM and capex-blend Ctrl+F
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
+          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
+          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
+          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
+          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E11" s="31" t="n">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>FY26 capex 7.0% matches 10-K guide midpoint ~$735M on $10.425B sales; fades 6.0%→5.0% after the build year.</t>
+          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "725.0 million" and "745.0 million" on this 10-K HTML. Midpoint $735M / FY26 sales $10.425B ≈ 7.0% (FY26 model).</t>
+          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E22" s="31" t="n">

</xml_diff>

<commit_message>
Rebuild models with FY26-vs-FY25 capex comparison in Ctrl+F
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
+          <t>FY26 7.0% is up vs FY25 6.1% ($735M vs $681M). Then 6.0 / 5.5 / 5.0 / 5.0 returns toward the FY25 run-rate and the 4.5% D&amp;A floor.</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
+          <t>Ctrl+F "680,802" → FY25 $680.8M / 6.1% of sales. Ctrl+F "$725.0 million and $745.0 million" → FY26 mid $735M / 7.0%. FY26 is up vs FY25, not down. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0: FY27 6.0% returns to the FY25 6.1% run-rate, then fades toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
+          <t>FY26 7.0% is up vs FY25 6.1% ($735M vs $681M). Then 6.0 / 5.5 / 5.0 / 5.0 returns toward the FY25 run-rate and the 4.5% D&amp;A floor.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
+          <t>Ctrl+F "680,802" → FY25 $680.8M / 6.1% of sales. Ctrl+F "$725.0 million and $745.0 million" → FY26 mid $735M / 7.0%. FY26 is up vs FY25, not down. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0: FY27 6.0% returns to the FY25 6.1% run-rate, then fades toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E11" s="31" t="n">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M guide mid / $10.425B sales. Then 6.0 / 5.5 / 5.0 / 5.0 (step off FY25 actual 6.1% toward D&amp;A 4.5%).</t>
+          <t>FY26 7.0% is up vs FY25 6.1% ($735M vs $681M). Then 6.0 / 5.5 / 5.0 / 5.0 returns toward the FY25 run-rate and the 4.5% D&amp;A floor.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "$725.0 million and $745.0 million" → 2026 guide. Mid $735M ÷ $10,425M sales = 7.0% (FY26). Ctrl+F "680,802" → FY25 actual 6.1%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0 steps off that 6.1% toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
+          <t>Ctrl+F "680,802" → FY25 $680.8M / 6.1% of sales. Ctrl+F "$725.0 million and $745.0 million" → FY26 mid $735M / 7.0%. FY26 is up vs FY25, not down. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0: FY27 6.0% returns to the FY25 6.1% run-rate, then fades toward D&amp;A 4.5% (Ctrl+F "496,228").</t>
         </is>
       </c>
       <c r="E22" s="31" t="n">

</xml_diff>

<commit_message>
Put the 5.5% capex blend in a 20-word Excel justification
FY26 7% is $735M on guided $10.4B sales, not FY25 $11.1B.
5.5% = (7+6+5.5+5+4)/5, with the 10-K and earnings links.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1434,8 +1434,8 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M ÷ ~$10.4B guided sales (the $10B year), not ÷ FY25 $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 back toward FY25 6.1%.
-Also: FY26 sales are the guided $10.35–$10.50B year (~$10.4B). FY25 was $11.1B. Same capex math must use the $10B denominator.</t>
+          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.
+Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
       <c r="C14" s="27" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M ÷ ~$10.4B guided sales (the $10B year), not ÷ FY25 $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 back toward FY25 6.1%.</t>
+          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>FY26 7.0% = $735M ÷ ~$10.4B guided sales (the $10B year), not ÷ FY25 $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 back toward FY25 6.1%.</t>
+          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">

</xml_diff>

<commit_message>
State the capex fade as 7.0% toward FY25 6.1% with the 5.5% equation
Since FY26 7.0% steps toward the FY25 6.1% run-rate, we assume
a fade: DCF 5.5% = (7.0+6.0+5.5+5.0+4.0)/5.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.
+          <t>FY26 7.0% is $735M / $10.4B, not / FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 $680.8M on $11.1B sales = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M. Divide by the $10B year ($10.425B guide), not by $11.1B: 735 / 10,425 = 7.0%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0.
+          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.
 Also: Ctrl+F "$10.350 billion to $10.500 billion" → FY26 net revenue guide (one hit). Mid $10.425B. That is the $10B year vs FY25 $11.1B. 7.0% capex uses this $10.4B denominator.</t>
         </is>
       </c>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.</t>
+          <t>FY26 7.0% is $735M / $10.4B, not / FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 $680.8M on $11.1B sales = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M. Divide by the $10B year ($10.425B guide), not by $11.1B: 735 / 10,425 = 7.0%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
+          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
       <c r="E11" s="32" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>FY26 7% is $735M / $10.4B sales, not / $11.1B. Then 6.0 / 5.5 / 5.0 / 5.0 after the spike.</t>
+          <t>FY26 7.0% is $735M / $10.4B, not / FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 $680.8M on $11.1B sales = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M. Divide by the $10B year ($10.425B guide), not by $11.1B: 735 / 10,425 = 7.0%. Path 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
+          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
       <c r="E22" s="32" t="n">

</xml_diff>

<commit_message>
Write the capex Ctrl+F cell as the FY25 6.1% / FY26 7.0% / fade block
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1446,8 +1446,8 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.
-Also: Ctrl+F "$10.350 billion to $10.500 billion" → FY26 net revenue guide (one hit). Mid $10.425B. That is the $10B year vs FY25 $11.1B. 7.0% capex uses this $10.4B denominator.</t>
+          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.
+Also: Ctrl+F "$10.350 billion to $10.500 billion" → FY26 net revenue guide (one hit). Mid $10.425B. That is the $10B year vs FY25 $11.1B. 7.0% capex uses this $10.4B denominator. FY26 is a $10B sales year: $735M / $10.425B = 7.0%. Then fade 6.0 / 5.5 / 5.0 / 4.0. DCF 5.5% = (7.0+6.0+5.5+5.0+4.0)/5.</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
+          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.</t>
         </is>
       </c>
       <c r="E11" s="32" t="n">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 $735M / $10.4B = 7.0%. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
+          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.</t>
         </is>
       </c>
       <c r="E22" s="32" t="n">

</xml_diff>

<commit_message>
Organize the capex Ctrl+F cell into FY25 / FY26 / blend blocks
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1021,7 +1021,7 @@
       <c r="L4" s="18" t="n"/>
       <c r="M4" s="18" t="n"/>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
@@ -1067,7 +1067,7 @@
         <v>0.023</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Gross margin % (clean, ex-refunds)</t>
@@ -1116,7 +1116,7 @@
         <v>0.58</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
           <t>IEEPA tariff refunds ($k, FY26 only)</t>
@@ -1165,7 +1165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
           <t>SG&amp;A % of revenue</t>
@@ -1214,7 +1214,7 @@
         <v>0.395</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Amortization / other opex ($)</t>
@@ -1263,7 +1263,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Other income, net ($)</t>
@@ -1312,7 +1312,7 @@
         <v>25000</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Effective tax rate %</t>
@@ -1377,7 +1377,7 @@
       <c r="L12" s="18" t="n"/>
       <c r="M12" s="18" t="n"/>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
           <t>D&amp;A % of revenue</t>
@@ -1426,7 +1426,7 @@
         <v>0.045</v>
       </c>
     </row>
-    <row r="14" ht="54" customHeight="1">
+    <row r="14" ht="150" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Capex % of revenue</t>
@@ -1446,8 +1446,18 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.
-Also: Ctrl+F "$10.350 billion to $10.500 billion" → FY26 net revenue guide (one hit). Mid $10.425B. That is the $10B year vs FY25 $11.1B. 7.0% capex uses this $10.4B denominator. FY26 is a $10B sales year: $735M / $10.425B = 7.0%. Then fade 6.0 / 5.5 / 5.0 / 4.0. DCF 5.5% = (7.0+6.0+5.5+5.0+4.0)/5.</t>
+          <t>FY25 actual (10-K)
+  Ctrl+F "680,802"  →  capex $680.8M
+  Ctrl+F "11,102,600"  →  sales $11.1B
+  680.8 / 11,102.6 = 6.1%
+FY26 capex (10-K)
+  Ctrl+F "$725.0 million and $745.0 million"  →  mid $735M
+FY26 sales (earnings)
+  Ctrl+F "$10.350 billion to $10.500 billion"  →  $10.35–$10.50B (mid $10.425B)
+  7.0% = $735M / $10.425B    ($10B year, not FY25 $11.1B)
+DCF blend
+  Fade  7.0 / 6.0 / 5.5 / 5.0 / 4.0
+  5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
@@ -1478,7 +1488,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Stock-based compensation ($)</t>
@@ -1543,7 +1553,7 @@
       <c r="L16" s="18" t="n"/>
       <c r="M16" s="18" t="n"/>
     </row>
-    <row r="17" ht="36" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Inventories % of COGS</t>
@@ -1592,7 +1602,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Accounts payable % of COGS</t>
@@ -1641,7 +1651,7 @@
         <v>0.068</v>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Accrued liabilities % of revenue</t>
@@ -1690,7 +1700,7 @@
         <v>0.058</v>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Other current assets % of revenue</t>
@@ -1739,7 +1749,7 @@
         <v>0.068</v>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Operating lease ROU asset % of revenue</t>
@@ -1788,7 +1798,7 @@
         <v>0.147</v>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Other non-current assets % of revenue</t>
@@ -1837,7 +1847,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Op lease liab (current) % of revenue</t>
@@ -1886,7 +1896,7 @@
         <v>0.027</v>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Op lease liab (non-current) % of revenue</t>
@@ -1935,7 +1945,7 @@
         <v>0.135</v>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Other current liabilities % of revenue</t>
@@ -1984,7 +1994,7 @@
         <v>0.055</v>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Other non-current liab % of revenue</t>
@@ -2049,7 +2059,7 @@
       <c r="L27" s="18" t="n"/>
       <c r="M27" s="18" t="n"/>
     </row>
-    <row r="28" ht="36" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Share repurchases ($)</t>
@@ -2098,7 +2108,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Avg repurchase price ($/sh)</t>
@@ -2293,7 +2303,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Net revenue</t>
@@ -2347,7 +2357,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Cost of goods sold (ex-refunds)</t>
@@ -2401,7 +2411,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: IEEPA tariff refunds (FY26 only)</t>
@@ -2498,7 +2508,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Selling, general &amp; administrative</t>
@@ -2552,7 +2562,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Amortization of intangibles / other</t>
@@ -2649,7 +2659,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Other income, net</t>
@@ -2746,7 +2756,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Income tax expense</t>
@@ -2843,7 +2853,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="54" customHeight="1">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Diluted weighted-avg shares (000)</t>
@@ -3406,7 +3416,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Inventories</t>
@@ -3460,7 +3470,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Other current assets</t>
@@ -3560,7 +3570,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="150" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Property &amp; equipment, net</t>
@@ -3578,7 +3588,18 @@
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.</t>
+          <t>FY25 actual (10-K)
+  Ctrl+F "680,802"  →  capex $680.8M
+  Ctrl+F "11,102,600"  →  sales $11.1B
+  680.8 / 11,102.6 = 6.1%
+FY26 capex (10-K)
+  Ctrl+F "$725.0 million and $745.0 million"  →  mid $735M
+FY26 sales (earnings)
+  Ctrl+F "$10.350 billion to $10.500 billion"  →  $10.35–$10.50B (mid $10.425B)
+  7.0% = $735M / $10.425B    ($10B year, not FY25 $11.1B)
+DCF blend
+  Fade  7.0 / 6.0 / 5.5 / 5.0 / 4.0
+  5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="E11" s="32" t="n">
@@ -3614,7 +3635,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Operating lease right-of-use assets</t>
@@ -3707,7 +3728,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
@@ -3823,7 +3844,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Accounts payable</t>
@@ -3877,7 +3898,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Accrued liabilities</t>
@@ -3931,7 +3952,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Operating lease liabilities (current)</t>
@@ -3985,7 +4006,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Other current liabilities</t>
@@ -4085,7 +4106,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Operating lease liabilities (non-current)</t>
@@ -4178,7 +4199,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
@@ -4278,7 +4299,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1">
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
         <is>
           <t>Common stock &amp; additional paid-in capital</t>
@@ -4332,7 +4353,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Retained earnings</t>
@@ -4819,7 +4840,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Depreciation &amp; amortization</t>
@@ -4873,7 +4894,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Stock-based compensation</t>
@@ -4927,7 +4948,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
@@ -4989,7 +5010,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
@@ -5051,7 +5072,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
@@ -5113,7 +5134,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
@@ -5175,7 +5196,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
@@ -5237,7 +5258,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
@@ -5299,7 +5320,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
@@ -5361,7 +5382,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Incr./(decr.) in operating lease liab.</t>
@@ -5595,7 +5616,7 @@
       <c r="L21" s="18" t="n"/>
       <c r="M21" s="18" t="n"/>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22" ht="150" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Capital expenditures</t>
@@ -5613,7 +5634,18 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "680,802" → FY25 capex $680.8M. Ctrl+F "11,102,600" → FY25 sales $11.1B. 680.8 / 11,102.6 = 6.1%. Ctrl+F "$725.0 million and $745.0 million" → FY26 capex mid $735M.</t>
+          <t>FY25 actual (10-K)
+  Ctrl+F "680,802"  →  capex $680.8M
+  Ctrl+F "11,102,600"  →  sales $11.1B
+  680.8 / 11,102.6 = 6.1%
+FY26 capex (10-K)
+  Ctrl+F "$725.0 million and $745.0 million"  →  mid $735M
+FY26 sales (earnings)
+  Ctrl+F "$10.350 billion to $10.500 billion"  →  $10.35–$10.50B (mid $10.425B)
+  7.0% = $735M / $10.425B    ($10B year, not FY25 $11.1B)
+DCF blend
+  Fade  7.0 / 6.0 / 5.5 / 5.0 / 4.0
+  5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="E22" s="32" t="n">
@@ -5711,7 +5743,7 @@
       <c r="L26" s="18" t="n"/>
       <c r="M26" s="18" t="n"/>
     </row>
-    <row r="27" ht="36" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Repurchase of common stock</t>

</xml_diff>

<commit_message>
Split accounts receivable out of other current assets in NWC
AR is a 10-K line (FY25 $190.7M). It was buried in OCA; NWC now
shows AR + inventory − AP, with OCA as the prepaid residual only.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -873,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1605,61 +1605,61 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Accounts payable % of COGS</t>
+          <t>Accounts receivable % of revenue</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Wholesale and marketplace receivables; hold the FY25 mix.</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657 ($000). 190,657 / 11,102,600 = 1.7% of sales. Model holds 1.7%.</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
-        <v>0.04774005037894764</v>
+        <v>0.0163868694946488</v>
       </c>
       <c r="F18" s="23" t="n">
-        <v>0.08689576951688993</v>
+        <v>0.01297072399820444</v>
       </c>
       <c r="G18" s="23" t="n">
-        <v>0.06286453501771355</v>
+        <v>0.01134978937727035</v>
       </c>
       <c r="H18" s="23" t="n">
-        <v>0.06878140521012073</v>
+        <v>0.01717228396952065</v>
       </c>
       <c r="I18" s="24" t="n">
-        <v>0.068</v>
+        <v>0.017</v>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.068</v>
+        <v>0.017</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.068</v>
+        <v>0.017</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.068</v>
+        <v>0.017</v>
       </c>
       <c r="M18" s="24" t="n">
-        <v>0.068</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Accrued liabilities % of revenue</t>
+          <t>Accounts payable % of COGS</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -1669,46 +1669,46 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
-        <v>0.04922287331092786</v>
+        <v>0.04774005037894764</v>
       </c>
       <c r="F19" s="23" t="n">
-        <v>0.03623504799424655</v>
+        <v>0.08689576951688993</v>
       </c>
       <c r="G19" s="23" t="n">
-        <v>0.05283871763520759</v>
+        <v>0.06286453501771355</v>
       </c>
       <c r="H19" s="23" t="n">
-        <v>0.05971412101669879</v>
+        <v>0.06878140521012073</v>
       </c>
       <c r="I19" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
       <c r="M19" s="24" t="n">
-        <v>0.058</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Other current assets % of revenue</t>
+          <t>Accrued liabilities % of revenue</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -1718,193 +1718,193 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
-        <v>0.06870325668471483</v>
+        <v>0.04922287331092786</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>0.05125166358639391</v>
+        <v>0.03623504799424655</v>
       </c>
       <c r="G20" s="23" t="n">
-        <v>0.05231190108617899</v>
+        <v>0.05283871763520759</v>
       </c>
       <c r="H20" s="23" t="n">
-        <v>0.06797921207645057</v>
+        <v>0.05971412101669879</v>
       </c>
       <c r="I20" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
       <c r="M20" s="24" t="n">
-        <v>0.068</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Operating lease ROU asset % of revenue</t>
+          <t>Other current assets % of revenue</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+          <t>OCA 5.1% is current assets minus cash, AR, and inventory (prepaids / tax receivables). AR is its own line, not inside OCA.</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
+          <t>OCA = "Total current assets" 4,262,701 − cash 1,807,202 − "Accounts receivable, net" 190,657 − "Inventories" 1,700,753 = 564,089 (5.1% of sales). AR is not inside this residual.</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
-        <v>0.1195261511040355</v>
+        <v>0.05231638719006604</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>0.1315701656610818</v>
+        <v>0.03828093958818947</v>
       </c>
       <c r="G21" s="23" t="n">
-        <v>0.1337588918001165</v>
+        <v>0.04096211170890864</v>
       </c>
       <c r="H21" s="23" t="n">
-        <v>0.1468287608307964</v>
+        <v>0.05080692810692991</v>
       </c>
       <c r="I21" s="24" t="n">
-        <v>0.147</v>
+        <v>0.051</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>0.147</v>
+        <v>0.051</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>0.147</v>
+        <v>0.051</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0.147</v>
+        <v>0.051</v>
       </c>
       <c r="M21" s="24" t="n">
-        <v>0.147</v>
+        <v>0.051</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>Other non-current assets % of revenue</t>
+          <t>Operating lease ROU asset % of revenue</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
+          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E22" s="23" t="n">
-        <v>0.02002917692803345</v>
+        <v>0.1195261511040355</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>0.02036119550760462</v>
+        <v>0.1315701656610818</v>
       </c>
       <c r="G22" s="23" t="n">
-        <v>0.02407659296838742</v>
+        <v>0.1337588918001165</v>
       </c>
       <c r="H22" s="23" t="n">
-        <v>0.03052861491902797</v>
+        <v>0.1468287608307964</v>
       </c>
       <c r="I22" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="J22" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="K22" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0.03</v>
+        <v>0.147</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Op lease liab (current) % of revenue</t>
+          <t>Other non-current assets % of revenue</t>
         </is>
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C23" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E23" s="23" t="n">
-        <v>0.02564225860789656</v>
+        <v>0.02002917692803345</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>0.02591358727754827</v>
+        <v>0.02036119550760462</v>
       </c>
       <c r="G23" s="23" t="n">
-        <v>0.02598703491061591</v>
+        <v>0.02407659296838742</v>
       </c>
       <c r="H23" s="23" t="n">
-        <v>0.02690576981968188</v>
+        <v>0.03052861491902797</v>
       </c>
       <c r="I23" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="J23" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
       <c r="M23" s="24" t="n">
-        <v>0.027</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Op lease liab (non-current) % of revenue</t>
+          <t>Op lease liab (current) % of revenue</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -1914,239 +1914,288 @@
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
-        <v>0.1063263776740277</v>
+        <v>0.02564225860789656</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>0.1199686712453887</v>
+        <v>0.02591358727754827</v>
       </c>
       <c r="G24" s="23" t="n">
-        <v>0.1228392068624797</v>
+        <v>0.02598703491061591</v>
       </c>
       <c r="H24" s="23" t="n">
-        <v>0.1350779997478068</v>
+        <v>0.02690576981968188</v>
       </c>
       <c r="I24" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="J24" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="K24" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="L24" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
       <c r="M24" s="24" t="n">
-        <v>0.135</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Other current liabilities % of revenue</t>
+          <t>Op lease liab (non-current) % of revenue</t>
         </is>
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
         </is>
       </c>
       <c r="E25" s="23" t="n">
-        <v>0.08782065461170298</v>
+        <v>0.1063263776740277</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>0.0712106459549251</v>
+        <v>0.1199686712453887</v>
       </c>
       <c r="G25" s="23" t="n">
-        <v>0.06928582073919408</v>
+        <v>0.1228392068624797</v>
       </c>
       <c r="H25" s="23" t="n">
-        <v>0.05353890079801128</v>
+        <v>0.1350779997478068</v>
       </c>
       <c r="I25" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="J25" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="K25" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="L25" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
       <c r="M25" s="24" t="n">
-        <v>0.055</v>
+        <v>0.135</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
         <is>
+          <t>Other current liabilities % of revenue</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+        </is>
+      </c>
+      <c r="E26" s="23" t="n">
+        <v>0.08782065461170298</v>
+      </c>
+      <c r="F26" s="23" t="n">
+        <v>0.0712106459549251</v>
+      </c>
+      <c r="G26" s="23" t="n">
+        <v>0.06928582073919408</v>
+      </c>
+      <c r="H26" s="23" t="n">
+        <v>0.05353890079801128</v>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="J26" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="K26" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="L26" s="24" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M26" s="24" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
           <t>Other non-current liab % of revenue</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Other non-current liabilities" → 55,360 ÷ "Net revenue" 11,102,600 = 0.5%</t>
         </is>
       </c>
-      <c r="E26" s="23" t="n">
+      <c r="E27" s="23" t="n">
         <v>0.005991602509235539</v>
       </c>
-      <c r="F26" s="23" t="n">
+      <c r="F27" s="23" t="n">
         <v>0.00468486304273564</v>
       </c>
-      <c r="G26" s="23" t="n">
+      <c r="G27" s="23" t="n">
         <v>0.003852428654513556</v>
       </c>
-      <c r="H26" s="23" t="n">
+      <c r="H27" s="23" t="n">
         <v>0.004986219444094176</v>
       </c>
-      <c r="I26" s="24" t="n">
+      <c r="I27" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="J26" s="24" t="n">
+      <c r="J27" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="K26" s="24" t="n">
+      <c r="K27" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="L26" s="24" t="n">
+      <c r="L27" s="24" t="n">
         <v>0.005</v>
       </c>
-      <c r="M26" s="24" t="n">
+      <c r="M27" s="24" t="n">
         <v>0.005</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>CAPITAL RETURN</t>
         </is>
       </c>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="M27" s="18" t="n"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>Share repurchases ($)</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
-        </is>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>LULU CF: share repurchases (10-K)</t>
-        </is>
-      </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
-        </is>
-      </c>
-      <c r="E28" s="25" t="n">
-        <v>444001</v>
-      </c>
-      <c r="F28" s="25" t="n">
-        <v>558652</v>
-      </c>
-      <c r="G28" s="25" t="n">
-        <v>1636879</v>
-      </c>
-      <c r="H28" s="25" t="n">
-        <v>1178349</v>
-      </c>
-      <c r="I28" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="J28" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="K28" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="L28" s="26" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M28" s="26" t="n">
-        <v>500000</v>
-      </c>
+      <c r="E28" s="18" t="n"/>
+      <c r="F28" s="18" t="n"/>
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="18" t="n"/>
+      <c r="J28" s="18" t="n"/>
+      <c r="K28" s="18" t="n"/>
+      <c r="L28" s="18" t="n"/>
+      <c r="M28" s="18" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="19" t="inlineStr">
         <is>
+          <t>Share repurchases ($)</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="inlineStr">
+        <is>
+          <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>LULU CF: share repurchases (10-K)</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>444001</v>
+      </c>
+      <c r="F29" s="25" t="n">
+        <v>558652</v>
+      </c>
+      <c r="G29" s="25" t="n">
+        <v>1636879</v>
+      </c>
+      <c r="H29" s="25" t="n">
+        <v>1178349</v>
+      </c>
+      <c r="I29" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J29" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="K29" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="L29" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M29" s="26" t="n">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
           <t>Avg repurchase price ($/sh)</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>FY26 repurchase price $100 matches the current quote; path $100→$130 is a recovery assumption (FY25 10-K paid $168–$199).</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
         </is>
       </c>
-      <c r="I29" s="28" t="n">
+      <c r="I30" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="J29" s="28" t="n">
+      <c r="J30" s="28" t="n">
         <v>108</v>
       </c>
-      <c r="K29" s="28" t="n">
+      <c r="K30" s="28" t="n">
         <v>115</v>
       </c>
-      <c r="L29" s="28" t="n">
+      <c r="L30" s="28" t="n">
         <v>122</v>
       </c>
-      <c r="M29" s="28" t="n">
+      <c r="M30" s="28" t="n">
         <v>130</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="29" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>Historical columns = derived ratios (black); projection columns = analyst inputs (red).</t>
         </is>
@@ -2178,8 +2227,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2890,23 +2940,23 @@
         <v>119068</v>
       </c>
       <c r="I16" s="26">
-        <f>H16-'Assumptions'!I28/'Assumptions'!I29</f>
+        <f>H16-'Assumptions'!I29/'Assumptions'!I30</f>
         <v/>
       </c>
       <c r="J16" s="26">
-        <f>I16-'Assumptions'!J28/'Assumptions'!J29</f>
+        <f>I16-'Assumptions'!J29/'Assumptions'!J30</f>
         <v/>
       </c>
       <c r="K16" s="26">
-        <f>J16-'Assumptions'!K28/'Assumptions'!K29</f>
+        <f>J16-'Assumptions'!K29/'Assumptions'!K30</f>
         <v/>
       </c>
       <c r="L16" s="26">
-        <f>K16-'Assumptions'!L28/'Assumptions'!L29</f>
+        <f>K16-'Assumptions'!L29/'Assumptions'!L30</f>
         <v/>
       </c>
       <c r="M16" s="26">
-        <f>L16-'Assumptions'!M28/'Assumptions'!M29</f>
+        <f>L16-'Assumptions'!M29/'Assumptions'!M30</f>
         <v/>
       </c>
     </row>
@@ -3242,7 +3292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3396,197 +3446,251 @@
         <v>1807202</v>
       </c>
       <c r="I6" s="25">
-        <f>'Cash Flow'!I33</f>
+        <f>'Cash Flow'!I34</f>
         <v/>
       </c>
       <c r="J6" s="25">
-        <f>'Cash Flow'!J33</f>
+        <f>'Cash Flow'!J34</f>
         <v/>
       </c>
       <c r="K6" s="25">
-        <f>'Cash Flow'!K33</f>
+        <f>'Cash Flow'!K34</f>
         <v/>
       </c>
       <c r="L6" s="25">
-        <f>'Cash Flow'!L33</f>
+        <f>'Cash Flow'!L34</f>
         <v/>
       </c>
       <c r="M6" s="25">
-        <f>'Cash Flow'!M33</f>
+        <f>'Cash Flow'!M34</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Accounts receivable, net</t>
         </is>
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Wholesale and marketplace receivables; hold the FY25 mix.</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657 ($000). 190,657 / 11,102,600 = 1.7% of sales. Model holds 1.7%.</t>
         </is>
       </c>
       <c r="E7" s="32" t="n">
-        <v>1447367</v>
+        <v>132906</v>
       </c>
       <c r="F7" s="32" t="n">
-        <v>1323602</v>
+        <v>124769</v>
       </c>
       <c r="G7" s="32" t="n">
-        <v>1442081</v>
+        <v>120173</v>
       </c>
       <c r="H7" s="32" t="n">
-        <v>1700753</v>
+        <v>190657</v>
       </c>
       <c r="I7" s="26">
-        <f>'Income Statement'!I5*'Assumptions'!I17</f>
+        <f>'Income Statement'!I4*'Assumptions'!I18</f>
         <v/>
       </c>
       <c r="J7" s="26">
-        <f>'Income Statement'!J5*'Assumptions'!J17</f>
+        <f>'Income Statement'!J4*'Assumptions'!J18</f>
         <v/>
       </c>
       <c r="K7" s="26">
-        <f>'Income Statement'!K5*'Assumptions'!K17</f>
+        <f>'Income Statement'!K4*'Assumptions'!K18</f>
         <v/>
       </c>
       <c r="L7" s="26">
-        <f>'Income Statement'!L5*'Assumptions'!L17</f>
+        <f>'Income Statement'!L4*'Assumptions'!L18</f>
         <v/>
       </c>
       <c r="M7" s="26">
-        <f>'Income Statement'!M5*'Assumptions'!M17</f>
+        <f>'Income Statement'!M4*'Assumptions'!M18</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>1447367</v>
+      </c>
+      <c r="F8" s="32" t="n">
+        <v>1323602</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>1442081</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>1700753</v>
+      </c>
+      <c r="I8" s="26">
+        <f>'Income Statement'!I5*'Assumptions'!I17</f>
+        <v/>
+      </c>
+      <c r="J8" s="26">
+        <f>'Income Statement'!J5*'Assumptions'!J17</f>
+        <v/>
+      </c>
+      <c r="K8" s="26">
+        <f>'Income Statement'!K5*'Assumptions'!K17</f>
+        <v/>
+      </c>
+      <c r="L8" s="26">
+        <f>'Income Statement'!L5*'Assumptions'!L17</f>
+        <v/>
+      </c>
+      <c r="M8" s="26">
+        <f>'Income Statement'!M5*'Assumptions'!M17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
           <t>Other current assets</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>OCA 5.1% is current assets minus cash, AR, and inventory (prepaids / tax receivables). AR is its own line, not inside OCA.</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>557219</v>
-      </c>
-      <c r="F8" s="25" t="n">
-        <v>493004</v>
-      </c>
-      <c r="G8" s="25" t="n">
-        <v>553885</v>
-      </c>
-      <c r="H8" s="25" t="n">
-        <v>754746</v>
-      </c>
-      <c r="I8" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I20</f>
-        <v/>
-      </c>
-      <c r="J8" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J20</f>
-        <v/>
-      </c>
-      <c r="K8" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K20</f>
-        <v/>
-      </c>
-      <c r="L8" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L20</f>
-        <v/>
-      </c>
-      <c r="M8" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>OCA = "Total current assets" 4,262,701 − cash 1,807,202 − "Accounts receivable, net" 190,657 − "Inventories" 1,700,753 = 564,089 (5.1% of sales). AR is not inside this residual.</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>424313</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>368235</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>433712</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>564089</v>
+      </c>
+      <c r="I9" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I21</f>
+        <v/>
+      </c>
+      <c r="J9" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J21</f>
+        <v/>
+      </c>
+      <c r="K9" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K21</f>
+        <v/>
+      </c>
+      <c r="L9" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L21</f>
+        <v/>
+      </c>
+      <c r="M9" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="E9" s="43" t="n">
+      <c r="E10" s="43" t="n">
         <v>3159453</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F10" s="43" t="n">
         <v>4060577</v>
       </c>
-      <c r="G9" s="43" t="n">
+      <c r="G10" s="43" t="n">
         <v>3980302</v>
       </c>
-      <c r="H9" s="43" t="n">
+      <c r="H10" s="43" t="n">
         <v>4262701</v>
       </c>
-      <c r="I9" s="34">
-        <f>I6+I7+I8</f>
-        <v/>
-      </c>
-      <c r="J9" s="34">
-        <f>J6+J7+J8</f>
-        <v/>
-      </c>
-      <c r="K9" s="34">
-        <f>K6+K7+K8</f>
-        <v/>
-      </c>
-      <c r="L9" s="34">
-        <f>L6+L7+L8</f>
-        <v/>
-      </c>
-      <c r="M9" s="34">
-        <f>M6+M7+M8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="I10" s="34">
+        <f>I6+I7+I8+I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="34">
+        <f>J6+J7+J8+J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="34">
+        <f>K6+K7+K8+K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="34">
+        <f>L6+L7+L8+L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="34">
+        <f>M6+M7+M8+M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Non-current assets:</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Property &amp; equipment, net</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>FY26 7.0% is $735M / $10.4B, not / FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>FY25 actual (10-K)
   Ctrl+F "680,802"  →  capex $680.8M
@@ -3602,311 +3706,257 @@
   5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
-      <c r="E11" s="32" t="n">
+      <c r="E12" s="32" t="n">
         <v>1269614</v>
       </c>
-      <c r="F11" s="32" t="n">
+      <c r="F12" s="32" t="n">
         <v>1545811</v>
       </c>
-      <c r="G11" s="32" t="n">
+      <c r="G12" s="32" t="n">
         <v>1780617</v>
       </c>
-      <c r="H11" s="32" t="n">
+      <c r="H12" s="32" t="n">
         <v>2033720</v>
       </c>
-      <c r="I11" s="26">
-        <f>H11+'Income Statement'!I4*'Assumptions'!I14-'Income Statement'!I4*'Assumptions'!I13</f>
-        <v/>
-      </c>
-      <c r="J11" s="26">
-        <f>I11+'Income Statement'!J4*'Assumptions'!J14-'Income Statement'!J4*'Assumptions'!J13</f>
-        <v/>
-      </c>
-      <c r="K11" s="26">
-        <f>J11+'Income Statement'!K4*'Assumptions'!K14-'Income Statement'!K4*'Assumptions'!K13</f>
-        <v/>
-      </c>
-      <c r="L11" s="26">
-        <f>K11+'Income Statement'!L4*'Assumptions'!L14-'Income Statement'!L4*'Assumptions'!L13</f>
-        <v/>
-      </c>
-      <c r="M11" s="26">
-        <f>L11+'Income Statement'!M4*'Assumptions'!M14-'Income Statement'!M4*'Assumptions'!M13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="I12" s="26">
+        <f>H12+'Income Statement'!I4*'Assumptions'!I14-'Income Statement'!I4*'Assumptions'!I13</f>
+        <v/>
+      </c>
+      <c r="J12" s="26">
+        <f>I12+'Income Statement'!J4*'Assumptions'!J14-'Income Statement'!J4*'Assumptions'!J13</f>
+        <v/>
+      </c>
+      <c r="K12" s="26">
+        <f>J12+'Income Statement'!K4*'Assumptions'!K14-'Income Statement'!K4*'Assumptions'!K13</f>
+        <v/>
+      </c>
+      <c r="L12" s="26">
+        <f>K12+'Income Statement'!L4*'Assumptions'!L14-'Income Statement'!L4*'Assumptions'!L13</f>
+        <v/>
+      </c>
+      <c r="M12" s="26">
+        <f>L12+'Income Statement'!M4*'Assumptions'!M14-'Income Statement'!M4*'Assumptions'!M13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Operating lease right-of-use assets</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
-      <c r="E12" s="32" t="n">
+      <c r="E13" s="32" t="n">
         <v>969419</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F13" s="32" t="n">
         <v>1265610</v>
       </c>
-      <c r="G12" s="32" t="n">
+      <c r="G13" s="32" t="n">
         <v>1416256</v>
       </c>
-      <c r="H12" s="32" t="n">
+      <c r="H13" s="32" t="n">
         <v>1630181</v>
       </c>
-      <c r="I12" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I21</f>
-        <v/>
-      </c>
-      <c r="J12" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J21</f>
-        <v/>
-      </c>
-      <c r="K12" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K21</f>
-        <v/>
-      </c>
-      <c r="L12" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L21</f>
-        <v/>
-      </c>
-      <c r="M12" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="I13" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I22</f>
+        <v/>
+      </c>
+      <c r="J13" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J22</f>
+        <v/>
+      </c>
+      <c r="K13" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K22</f>
+        <v/>
+      </c>
+      <c r="L13" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L22</f>
+        <v/>
+      </c>
+      <c r="M13" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Goodwill &amp; intangible assets</t>
         </is>
       </c>
-      <c r="E13" s="32" t="n">
+      <c r="E14" s="32" t="n">
         <v>46105</v>
       </c>
-      <c r="F13" s="32" t="n">
+      <c r="F14" s="32" t="n">
         <v>24083</v>
       </c>
-      <c r="G13" s="32" t="n">
+      <c r="G14" s="32" t="n">
         <v>171191</v>
       </c>
-      <c r="H13" s="32" t="n">
+      <c r="H14" s="32" t="n">
         <v>191194</v>
       </c>
-      <c r="I13" s="25">
-        <f>H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="25">
-        <f>I13</f>
-        <v/>
-      </c>
-      <c r="K13" s="25">
-        <f>J13</f>
-        <v/>
-      </c>
-      <c r="L13" s="25">
-        <f>K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="25">
-        <f>L13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="I14" s="25">
+        <f>H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="25">
+        <f>I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="25">
+        <f>J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="25">
+        <f>K14</f>
+        <v/>
+      </c>
+      <c r="M14" s="25">
+        <f>L14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Other non-current assets</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E15" s="25" t="n">
         <v>162447</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F15" s="25" t="n">
         <v>195860</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G15" s="25" t="n">
         <v>254926</v>
       </c>
-      <c r="H14" s="25" t="n">
+      <c r="H15" s="25" t="n">
         <v>338947</v>
       </c>
-      <c r="I14" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I22</f>
-        <v/>
-      </c>
-      <c r="J14" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J22</f>
-        <v/>
-      </c>
-      <c r="K14" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K22</f>
-        <v/>
-      </c>
-      <c r="L14" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L22</f>
-        <v/>
-      </c>
-      <c r="M14" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="I15" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I23</f>
+        <v/>
+      </c>
+      <c r="J15" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J23</f>
+        <v/>
+      </c>
+      <c r="K15" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K23</f>
+        <v/>
+      </c>
+      <c r="L15" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L23</f>
+        <v/>
+      </c>
+      <c r="M15" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="E15" s="44" t="n">
+      <c r="E16" s="44" t="n">
         <v>5607038</v>
       </c>
-      <c r="F15" s="44" t="n">
+      <c r="F16" s="44" t="n">
         <v>7091941</v>
       </c>
-      <c r="G15" s="44" t="n">
+      <c r="G16" s="44" t="n">
         <v>7603292</v>
       </c>
-      <c r="H15" s="44" t="n">
+      <c r="H16" s="44" t="n">
         <v>8456743</v>
       </c>
-      <c r="I15" s="35">
-        <f>I9+I11+I12+I13+I14</f>
-        <v/>
-      </c>
-      <c r="J15" s="35">
-        <f>J9+J11+J12+J13+J14</f>
-        <v/>
-      </c>
-      <c r="K15" s="35">
-        <f>K9+K11+K12+K13+K14</f>
-        <v/>
-      </c>
-      <c r="L15" s="35">
-        <f>L9+L11+L12+L13+L14</f>
-        <v/>
-      </c>
-      <c r="M15" s="35">
-        <f>M9+M11+M12+M13+M14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="I16" s="35">
+        <f>I10+I12+I13+I14+I15</f>
+        <v/>
+      </c>
+      <c r="J16" s="35">
+        <f>J10+J12+J13+J14+J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="35">
+        <f>K10+K12+K13+K14+K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="35">
+        <f>L10+L12+L13+L14+L15</f>
+        <v/>
+      </c>
+      <c r="M16" s="35">
+        <f>M10+M12+M13+M14+M15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n"/>
-      <c r="J17" s="18" t="n"/>
-      <c r="K17" s="18" t="n"/>
-      <c r="L17" s="18" t="n"/>
-      <c r="M17" s="18" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="42" t="inlineStr">
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="18" t="n"/>
+      <c r="H18" s="18" t="n"/>
+      <c r="I18" s="18" t="n"/>
+      <c r="J18" s="18" t="n"/>
+      <c r="K18" s="18" t="n"/>
+      <c r="L18" s="18" t="n"/>
+      <c r="M18" s="18" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Accounts payable</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="inlineStr">
-        <is>
-          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>LULU balance sheet (10-K)</t>
-        </is>
-      </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
-        </is>
-      </c>
-      <c r="E19" s="32" t="n">
-        <v>172732</v>
-      </c>
-      <c r="F19" s="32" t="n">
-        <v>348441</v>
-      </c>
-      <c r="G19" s="32" t="n">
-        <v>271406</v>
-      </c>
-      <c r="H19" s="32" t="n">
-        <v>331421</v>
-      </c>
-      <c r="I19" s="26">
-        <f>'Income Statement'!I5*'Assumptions'!I18</f>
-        <v/>
-      </c>
-      <c r="J19" s="26">
-        <f>'Income Statement'!J5*'Assumptions'!J18</f>
-        <v/>
-      </c>
-      <c r="K19" s="26">
-        <f>'Income Statement'!K5*'Assumptions'!K18</f>
-        <v/>
-      </c>
-      <c r="L19" s="26">
-        <f>'Income Statement'!L5*'Assumptions'!L18</f>
-        <v/>
-      </c>
-      <c r="M19" s="26">
-        <f>'Income Statement'!M5*'Assumptions'!M18</f>
-        <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Accrued liabilities</t>
+          <t>Accounts payable</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -3916,658 +3966,712 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E20" s="32" t="n">
-        <v>399223</v>
+        <v>172732</v>
       </c>
       <c r="F20" s="32" t="n">
-        <v>348555</v>
+        <v>348441</v>
       </c>
       <c r="G20" s="32" t="n">
-        <v>559463</v>
+        <v>271406</v>
       </c>
       <c r="H20" s="32" t="n">
-        <v>662982</v>
+        <v>331421</v>
       </c>
       <c r="I20" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I19</f>
+        <f>'Income Statement'!I5*'Assumptions'!I19</f>
         <v/>
       </c>
       <c r="J20" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J19</f>
+        <f>'Income Statement'!J5*'Assumptions'!J19</f>
         <v/>
       </c>
       <c r="K20" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K19</f>
+        <f>'Income Statement'!K5*'Assumptions'!K19</f>
         <v/>
       </c>
       <c r="L20" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L19</f>
+        <f>'Income Statement'!L5*'Assumptions'!L19</f>
         <v/>
       </c>
       <c r="M20" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M19</f>
+        <f>'Income Statement'!M5*'Assumptions'!M19</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Operating lease liabilities (current)</t>
+          <t>Accrued liabilities</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E21" s="32" t="n">
-        <v>207972</v>
+        <v>399223</v>
       </c>
       <c r="F21" s="32" t="n">
-        <v>249270</v>
+        <v>348555</v>
       </c>
       <c r="G21" s="32" t="n">
-        <v>275154</v>
+        <v>559463</v>
       </c>
       <c r="H21" s="32" t="n">
-        <v>298724</v>
+        <v>662982</v>
       </c>
       <c r="I21" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I23</f>
+        <f>'Income Statement'!I4*'Assumptions'!I20</f>
         <v/>
       </c>
       <c r="J21" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J23</f>
+        <f>'Income Statement'!J4*'Assumptions'!J20</f>
         <v/>
       </c>
       <c r="K21" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K23</f>
+        <f>'Income Statement'!K4*'Assumptions'!K20</f>
         <v/>
       </c>
       <c r="L21" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L23</f>
+        <f>'Income Statement'!L4*'Assumptions'!L20</f>
         <v/>
       </c>
       <c r="M21" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M23</f>
+        <f>'Income Statement'!M4*'Assumptions'!M20</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
         <is>
+          <t>Operating lease liabilities (current)</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
+        </is>
+      </c>
+      <c r="E22" s="32" t="n">
+        <v>207972</v>
+      </c>
+      <c r="F22" s="32" t="n">
+        <v>249270</v>
+      </c>
+      <c r="G22" s="32" t="n">
+        <v>275154</v>
+      </c>
+      <c r="H22" s="32" t="n">
+        <v>298724</v>
+      </c>
+      <c r="I22" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I24</f>
+        <v/>
+      </c>
+      <c r="J22" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J24</f>
+        <v/>
+      </c>
+      <c r="K22" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K24</f>
+        <v/>
+      </c>
+      <c r="L22" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L24</f>
+        <v/>
+      </c>
+      <c r="M22" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
           <t>Other current liabilities</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
         </is>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E23" s="25" t="n">
         <v>712271</v>
       </c>
-      <c r="F22" s="25" t="n">
+      <c r="F23" s="25" t="n">
         <v>684995</v>
       </c>
-      <c r="G22" s="25" t="n">
+      <c r="G23" s="25" t="n">
         <v>733607</v>
       </c>
-      <c r="H22" s="25" t="n">
+      <c r="H23" s="25" t="n">
         <v>594421</v>
       </c>
-      <c r="I22" s="26">
+      <c r="I23" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I26</f>
+        <v/>
+      </c>
+      <c r="J23" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J26</f>
+        <v/>
+      </c>
+      <c r="K23" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K26</f>
+        <v/>
+      </c>
+      <c r="L23" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L26</f>
+        <v/>
+      </c>
+      <c r="M23" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Total current liabilities</t>
+        </is>
+      </c>
+      <c r="E24" s="43" t="n">
+        <v>1492198</v>
+      </c>
+      <c r="F24" s="43" t="n">
+        <v>1631261</v>
+      </c>
+      <c r="G24" s="43" t="n">
+        <v>1839630</v>
+      </c>
+      <c r="H24" s="43" t="n">
+        <v>1887548</v>
+      </c>
+      <c r="I24" s="34">
+        <f>I20+I21+I22+I23</f>
+        <v/>
+      </c>
+      <c r="J24" s="34">
+        <f>J20+J21+J22+J23</f>
+        <v/>
+      </c>
+      <c r="K24" s="34">
+        <f>K20+K21+K22+K23</f>
+        <v/>
+      </c>
+      <c r="L24" s="34">
+        <f>L20+L21+L22+L23</f>
+        <v/>
+      </c>
+      <c r="M24" s="34">
+        <f>M20+M21+M22+M23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="inlineStr">
+        <is>
+          <t>Non-current liabilities:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Operating lease liabilities (non-current)</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>LULU lease disclosures (10-K)</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
+        </is>
+      </c>
+      <c r="E26" s="32" t="n">
+        <v>862362</v>
+      </c>
+      <c r="F26" s="32" t="n">
+        <v>1154012</v>
+      </c>
+      <c r="G26" s="32" t="n">
+        <v>1300637</v>
+      </c>
+      <c r="H26" s="32" t="n">
+        <v>1499717</v>
+      </c>
+      <c r="I26" s="26">
         <f>'Income Statement'!I4*'Assumptions'!I25</f>
         <v/>
       </c>
-      <c r="J22" s="26">
+      <c r="J26" s="26">
         <f>'Income Statement'!J4*'Assumptions'!J25</f>
         <v/>
       </c>
-      <c r="K22" s="26">
+      <c r="K26" s="26">
         <f>'Income Statement'!K4*'Assumptions'!K25</f>
         <v/>
       </c>
-      <c r="L22" s="26">
+      <c r="L26" s="26">
         <f>'Income Statement'!L4*'Assumptions'!L25</f>
         <v/>
       </c>
-      <c r="M22" s="26">
+      <c r="M26" s="26">
         <f>'Income Statement'!M4*'Assumptions'!M25</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Total current liabilities</t>
-        </is>
-      </c>
-      <c r="E23" s="43" t="n">
-        <v>1492198</v>
-      </c>
-      <c r="F23" s="43" t="n">
-        <v>1631261</v>
-      </c>
-      <c r="G23" s="43" t="n">
-        <v>1839630</v>
-      </c>
-      <c r="H23" s="43" t="n">
-        <v>1887548</v>
-      </c>
-      <c r="I23" s="34">
-        <f>I19+I20+I21+I22</f>
-        <v/>
-      </c>
-      <c r="J23" s="34">
-        <f>J19+J20+J21+J22</f>
-        <v/>
-      </c>
-      <c r="K23" s="34">
-        <f>K19+K20+K21+K22</f>
-        <v/>
-      </c>
-      <c r="L23" s="34">
-        <f>L19+L20+L21+L22</f>
-        <v/>
-      </c>
-      <c r="M23" s="34">
-        <f>M19+M20+M21+M22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="42" t="inlineStr">
-        <is>
-          <t>Non-current liabilities:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Operating lease liabilities (non-current)</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>Non-current lease liabilities 13.5% of revenue; long-term store lease commitments per 10-K.</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>LULU lease disclosures (10-K)</t>
-        </is>
-      </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Non-current lease liabilities" → 1,499,717 ÷ "Net revenue" 11,102,600 = 13.5%</t>
-        </is>
-      </c>
-      <c r="E25" s="32" t="n">
-        <v>862362</v>
-      </c>
-      <c r="F25" s="32" t="n">
-        <v>1154012</v>
-      </c>
-      <c r="G25" s="32" t="n">
-        <v>1300637</v>
-      </c>
-      <c r="H25" s="32" t="n">
-        <v>1499717</v>
-      </c>
-      <c r="I25" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I24</f>
-        <v/>
-      </c>
-      <c r="J25" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J24</f>
-        <v/>
-      </c>
-      <c r="K25" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K24</f>
-        <v/>
-      </c>
-      <c r="L25" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L24</f>
-        <v/>
-      </c>
-      <c r="M25" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Deferred income taxes</t>
         </is>
       </c>
-      <c r="E26" s="32" t="n">
+      <c r="E27" s="32" t="n">
         <v>55084</v>
       </c>
-      <c r="F26" s="32" t="n">
+      <c r="F27" s="32" t="n">
         <v>29522</v>
       </c>
-      <c r="G26" s="32" t="n">
+      <c r="G27" s="32" t="n">
         <v>98188</v>
       </c>
-      <c r="H26" s="32" t="n">
+      <c r="H27" s="32" t="n">
         <v>52278</v>
       </c>
-      <c r="I26" s="25">
-        <f>H26</f>
-        <v/>
-      </c>
-      <c r="J26" s="25">
-        <f>I26</f>
-        <v/>
-      </c>
-      <c r="K26" s="25">
-        <f>J26</f>
-        <v/>
-      </c>
-      <c r="L26" s="25">
-        <f>K26</f>
-        <v/>
-      </c>
-      <c r="M26" s="25">
-        <f>L26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="I27" s="25">
+        <f>H27</f>
+        <v/>
+      </c>
+      <c r="J27" s="25">
+        <f>I27</f>
+        <v/>
+      </c>
+      <c r="K27" s="25">
+        <f>J27</f>
+        <v/>
+      </c>
+      <c r="L27" s="25">
+        <f>K27</f>
+        <v/>
+      </c>
+      <c r="M27" s="25">
+        <f>L27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Other non-current liabilities</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>Other non-current liabilities 0.5% of revenue; minor long-term accruals and provisions.</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Other non-current liabilities" → 55,360 ÷ "Net revenue" 11,102,600 = 0.5%</t>
         </is>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E28" s="25" t="n">
         <v>48595</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="F28" s="25" t="n">
         <v>45065</v>
       </c>
-      <c r="G27" s="25" t="n">
+      <c r="G28" s="25" t="n">
         <v>40790</v>
       </c>
-      <c r="H27" s="25" t="n">
+      <c r="H28" s="25" t="n">
         <v>55360</v>
       </c>
-      <c r="I27" s="26">
-        <f>'Income Statement'!I4*'Assumptions'!I26</f>
-        <v/>
-      </c>
-      <c r="J27" s="26">
-        <f>'Income Statement'!J4*'Assumptions'!J26</f>
-        <v/>
-      </c>
-      <c r="K27" s="26">
-        <f>'Income Statement'!K4*'Assumptions'!K26</f>
-        <v/>
-      </c>
-      <c r="L27" s="26">
-        <f>'Income Statement'!L4*'Assumptions'!L26</f>
-        <v/>
-      </c>
-      <c r="M27" s="26">
-        <f>'Income Statement'!M4*'Assumptions'!M26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="33" t="inlineStr">
+      <c r="I28" s="26">
+        <f>'Income Statement'!I4*'Assumptions'!I27</f>
+        <v/>
+      </c>
+      <c r="J28" s="26">
+        <f>'Income Statement'!J4*'Assumptions'!J27</f>
+        <v/>
+      </c>
+      <c r="K28" s="26">
+        <f>'Income Statement'!K4*'Assumptions'!K27</f>
+        <v/>
+      </c>
+      <c r="L28" s="26">
+        <f>'Income Statement'!L4*'Assumptions'!L27</f>
+        <v/>
+      </c>
+      <c r="M28" s="26">
+        <f>'Income Statement'!M4*'Assumptions'!M27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="E28" s="43" t="n">
+      <c r="E29" s="43" t="n">
         <v>2458239</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F29" s="43" t="n">
         <v>2859860</v>
       </c>
-      <c r="G28" s="43" t="n">
+      <c r="G29" s="43" t="n">
         <v>3279245</v>
       </c>
-      <c r="H28" s="43" t="n">
+      <c r="H29" s="43" t="n">
         <v>3494903</v>
       </c>
-      <c r="I28" s="34">
-        <f>I23+I25+I26+I27</f>
-        <v/>
-      </c>
-      <c r="J28" s="34">
-        <f>J23+J25+J26+J27</f>
-        <v/>
-      </c>
-      <c r="K28" s="34">
-        <f>K23+K25+K26+K27</f>
-        <v/>
-      </c>
-      <c r="L28" s="34">
-        <f>L23+L25+L26+L27</f>
-        <v/>
-      </c>
-      <c r="M28" s="34">
-        <f>M23+M25+M26+M27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="42" t="inlineStr">
+      <c r="I29" s="34">
+        <f>I24+I26+I27+I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="34">
+        <f>J24+J26+J27+J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="34">
+        <f>K24+K26+K27+K28</f>
+        <v/>
+      </c>
+      <c r="L29" s="34">
+        <f>L24+L26+L27+L28</f>
+        <v/>
+      </c>
+      <c r="M29" s="34">
+        <f>M24+M26+M27+M28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
         <is>
           <t>Shareholders' equity:</t>
         </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Common stock &amp; additional paid-in capital</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="inlineStr">
-        <is>
-          <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
-      </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
-        </is>
-      </c>
-      <c r="E31" s="32" t="n">
-        <v>475256</v>
-      </c>
-      <c r="F31" s="32" t="n">
-        <v>575975</v>
-      </c>
-      <c r="G31" s="32" t="n">
-        <v>638771</v>
-      </c>
-      <c r="H31" s="32" t="n">
-        <v>669949</v>
-      </c>
-      <c r="I31" s="26">
-        <f>H31+'Assumptions'!I15</f>
-        <v/>
-      </c>
-      <c r="J31" s="26">
-        <f>I31+'Assumptions'!J15</f>
-        <v/>
-      </c>
-      <c r="K31" s="26">
-        <f>J31+'Assumptions'!K15</f>
-        <v/>
-      </c>
-      <c r="L31" s="26">
-        <f>K31+'Assumptions'!L15</f>
-        <v/>
-      </c>
-      <c r="M31" s="26">
-        <f>L31+'Assumptions'!M15</f>
-        <v/>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
         <is>
+          <t>Common stock &amp; additional paid-in capital</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>$62M SBC holds the FY25 10-K run-rate (Stock-based compensation expense 62,203).</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K)</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Stock-based compensation expense" → 62,203 on this 10-K HTML. Model $62,000.</t>
+        </is>
+      </c>
+      <c r="E32" s="32" t="n">
+        <v>475256</v>
+      </c>
+      <c r="F32" s="32" t="n">
+        <v>575975</v>
+      </c>
+      <c r="G32" s="32" t="n">
+        <v>638771</v>
+      </c>
+      <c r="H32" s="32" t="n">
+        <v>669949</v>
+      </c>
+      <c r="I32" s="26">
+        <f>H32+'Assumptions'!I15</f>
+        <v/>
+      </c>
+      <c r="J32" s="26">
+        <f>I32+'Assumptions'!J15</f>
+        <v/>
+      </c>
+      <c r="K32" s="26">
+        <f>J32+'Assumptions'!K15</f>
+        <v/>
+      </c>
+      <c r="L32" s="26">
+        <f>K32+'Assumptions'!L15</f>
+        <v/>
+      </c>
+      <c r="M32" s="26">
+        <f>L32+'Assumptions'!M15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>LULU CF: share repurchases (10-K)</t>
         </is>
       </c>
-      <c r="D32" s="22" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
         </is>
       </c>
-      <c r="E32" s="32" t="n">
+      <c r="E33" s="32" t="n">
         <v>2926127</v>
       </c>
-      <c r="F32" s="32" t="n">
+      <c r="F33" s="32" t="n">
         <v>3920362</v>
       </c>
-      <c r="G32" s="32" t="n">
+      <c r="G33" s="32" t="n">
         <v>4109717</v>
       </c>
-      <c r="H32" s="32" t="n">
+      <c r="H33" s="32" t="n">
         <v>4522581</v>
       </c>
-      <c r="I32" s="26">
-        <f>H32+'Income Statement'!I14-'Assumptions'!I28</f>
-        <v/>
-      </c>
-      <c r="J32" s="26">
-        <f>I32+'Income Statement'!J14-'Assumptions'!J28</f>
-        <v/>
-      </c>
-      <c r="K32" s="26">
-        <f>J32+'Income Statement'!K14-'Assumptions'!K28</f>
-        <v/>
-      </c>
-      <c r="L32" s="26">
-        <f>K32+'Income Statement'!L14-'Assumptions'!L28</f>
-        <v/>
-      </c>
-      <c r="M32" s="26">
-        <f>L32+'Income Statement'!M14-'Assumptions'!M28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="I33" s="26">
+        <f>H33+'Income Statement'!I14-'Assumptions'!I29</f>
+        <v/>
+      </c>
+      <c r="J33" s="26">
+        <f>I33+'Income Statement'!J14-'Assumptions'!J29</f>
+        <v/>
+      </c>
+      <c r="K33" s="26">
+        <f>J33+'Income Statement'!K14-'Assumptions'!K29</f>
+        <v/>
+      </c>
+      <c r="L33" s="26">
+        <f>K33+'Income Statement'!L14-'Assumptions'!L29</f>
+        <v/>
+      </c>
+      <c r="M33" s="26">
+        <f>L33+'Income Statement'!M14-'Assumptions'!M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Accumulated other comprehensive loss</t>
         </is>
       </c>
-      <c r="E33" s="32" t="n">
+      <c r="E34" s="32" t="n">
         <v>-252584</v>
       </c>
-      <c r="F33" s="32" t="n">
+      <c r="F34" s="32" t="n">
         <v>-264256</v>
       </c>
-      <c r="G33" s="32" t="n">
+      <c r="G34" s="32" t="n">
         <v>-424441</v>
       </c>
-      <c r="H33" s="32" t="n">
+      <c r="H34" s="32" t="n">
         <v>-230690</v>
       </c>
-      <c r="I33" s="25">
-        <f>H33</f>
-        <v/>
-      </c>
-      <c r="J33" s="25">
-        <f>I33</f>
-        <v/>
-      </c>
-      <c r="K33" s="25">
-        <f>J33</f>
-        <v/>
-      </c>
-      <c r="L33" s="25">
-        <f>K33</f>
-        <v/>
-      </c>
-      <c r="M33" s="25">
-        <f>L33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="33" t="inlineStr">
-        <is>
-          <t>TOTAL SHAREHOLDERS' EQUITY</t>
-        </is>
-      </c>
-      <c r="E34" s="43" t="n">
-        <v>3148799</v>
-      </c>
-      <c r="F34" s="43" t="n">
-        <v>4232081</v>
-      </c>
-      <c r="G34" s="43" t="n">
-        <v>4324047</v>
-      </c>
-      <c r="H34" s="43" t="n">
-        <v>4961840</v>
-      </c>
-      <c r="I34" s="34">
-        <f>I31+I32+I33</f>
-        <v/>
-      </c>
-      <c r="J34" s="34">
-        <f>J31+J32+J33</f>
-        <v/>
-      </c>
-      <c r="K34" s="34">
-        <f>K31+K32+K33</f>
-        <v/>
-      </c>
-      <c r="L34" s="34">
-        <f>L31+L32+L33</f>
-        <v/>
-      </c>
-      <c r="M34" s="34">
-        <f>M31+M32+M33</f>
+      <c r="I34" s="25">
+        <f>H34</f>
+        <v/>
+      </c>
+      <c r="J34" s="25">
+        <f>I34</f>
+        <v/>
+      </c>
+      <c r="K34" s="25">
+        <f>J34</f>
+        <v/>
+      </c>
+      <c r="L34" s="25">
+        <f>K34</f>
+        <v/>
+      </c>
+      <c r="M34" s="25">
+        <f>L34</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="33" t="inlineStr">
         <is>
+          <t>TOTAL SHAREHOLDERS' EQUITY</t>
+        </is>
+      </c>
+      <c r="E35" s="43" t="n">
+        <v>3148799</v>
+      </c>
+      <c r="F35" s="43" t="n">
+        <v>4232081</v>
+      </c>
+      <c r="G35" s="43" t="n">
+        <v>4324047</v>
+      </c>
+      <c r="H35" s="43" t="n">
+        <v>4961840</v>
+      </c>
+      <c r="I35" s="34">
+        <f>I32+I33+I34</f>
+        <v/>
+      </c>
+      <c r="J35" s="34">
+        <f>J32+J33+J34</f>
+        <v/>
+      </c>
+      <c r="K35" s="34">
+        <f>K32+K33+K34</f>
+        <v/>
+      </c>
+      <c r="L35" s="34">
+        <f>L32+L33+L34</f>
+        <v/>
+      </c>
+      <c r="M35" s="34">
+        <f>M32+M33+M34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="33" t="inlineStr">
+        <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="E35" s="35">
-        <f>E28+E34</f>
-        <v/>
-      </c>
-      <c r="F35" s="35">
-        <f>F28+F34</f>
-        <v/>
-      </c>
-      <c r="G35" s="35">
-        <f>G28+G34</f>
-        <v/>
-      </c>
-      <c r="H35" s="35">
-        <f>H28+H34</f>
-        <v/>
-      </c>
-      <c r="I35" s="35">
-        <f>I28+I34</f>
-        <v/>
-      </c>
-      <c r="J35" s="35">
-        <f>J28+J34</f>
-        <v/>
-      </c>
-      <c r="K35" s="35">
-        <f>K28+K34</f>
-        <v/>
-      </c>
-      <c r="L35" s="35">
-        <f>L28+L34</f>
-        <v/>
-      </c>
-      <c r="M35" s="35">
-        <f>M28+M34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="39" t="inlineStr">
+      <c r="E36" s="35">
+        <f>E29+E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="35">
+        <f>F29+F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="35">
+        <f>G29+G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="35">
+        <f>H29+H35</f>
+        <v/>
+      </c>
+      <c r="I36" s="35">
+        <f>I29+I35</f>
+        <v/>
+      </c>
+      <c r="J36" s="35">
+        <f>J29+J35</f>
+        <v/>
+      </c>
+      <c r="K36" s="35">
+        <f>K29+K35</f>
+        <v/>
+      </c>
+      <c r="L36" s="35">
+        <f>L29+L35</f>
+        <v/>
+      </c>
+      <c r="M36" s="35">
+        <f>M29+M35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="39" t="inlineStr">
         <is>
           <t>Balance check (Assets − L&amp;E)</t>
         </is>
       </c>
-      <c r="E37" s="45">
-        <f>E15-E35</f>
-        <v/>
-      </c>
-      <c r="F37" s="45">
-        <f>F15-F35</f>
-        <v/>
-      </c>
-      <c r="G37" s="45">
-        <f>G15-G35</f>
-        <v/>
-      </c>
-      <c r="H37" s="45">
-        <f>H15-H35</f>
-        <v/>
-      </c>
-      <c r="I37" s="45">
-        <f>I15-I35</f>
-        <v/>
-      </c>
-      <c r="J37" s="45">
-        <f>J15-J35</f>
-        <v/>
-      </c>
-      <c r="K37" s="45">
-        <f>K15-K35</f>
-        <v/>
-      </c>
-      <c r="L37" s="45">
-        <f>L15-L35</f>
-        <v/>
-      </c>
-      <c r="M37" s="45">
-        <f>M15-M35</f>
+      <c r="E38" s="45">
+        <f>E16-E36</f>
+        <v/>
+      </c>
+      <c r="F38" s="45">
+        <f>F16-F36</f>
+        <v/>
+      </c>
+      <c r="G38" s="45">
+        <f>G16-G36</f>
+        <v/>
+      </c>
+      <c r="H38" s="45">
+        <f>H16-H36</f>
+        <v/>
+      </c>
+      <c r="I38" s="45">
+        <f>I16-I36</f>
+        <v/>
+      </c>
+      <c r="J38" s="45">
+        <f>J16-J36</f>
+        <v/>
+      </c>
+      <c r="K38" s="45">
+        <f>K16-K36</f>
+        <v/>
+      </c>
+      <c r="L38" s="45">
+        <f>L16-L36</f>
+        <v/>
+      </c>
+      <c r="M38" s="45">
+        <f>M16-M36</f>
         <v/>
       </c>
     </row>
@@ -4587,34 +4691,34 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId45"/>
@@ -4626,42 +4730,47 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4673,7 +4782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4951,22 +5060,22 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
+          <t xml:space="preserve">  (Incr.)/decr. in accounts receivable</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Wholesale and marketplace receivables; hold the FY25 mix.</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657 ($000). 190,657 / 11,102,600 = 1.7% of sales. Model holds 1.7%.</t>
         </is>
       </c>
       <c r="E8" s="46" t="inlineStr">
@@ -5013,12 +5122,12 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
+          <t xml:space="preserve">  (Incr.)/decr. in inventories</t>
         </is>
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>OCA 6.8% = FY25 current assets 4,262,701 − cash 1,807,202 − inventories 1,700,753, as % of revenue (not the prepaid line alone).</t>
+          <t>Inventory 33–34% of COGS; slight normalization from FY25 build as Americas demand softens and clears.</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -5028,7 +5137,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current assets" → 4,262,701 minus "Cash and cash equivalents" 1,807,202 minus "Inventories" 1,700,753 = 754,746 (6.8% of revenue)</t>
+          <t>Ctrl+F "Inventories" → 1,700,753 ÷ "Cost of goods sold" 4,818,468 = 35.3%</t>
         </is>
       </c>
       <c r="E9" s="46" t="inlineStr">
@@ -5075,22 +5184,22 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
+          <t xml:space="preserve">  (Incr.)/decr. in other current assets</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
+          <t>OCA 5.1% is current assets minus cash, AR, and inventory (prepaids / tax receivables). AR is its own line, not inside OCA.</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>LULU lease disclosures (10-K)</t>
+          <t>LULU balance sheet (10-K)</t>
         </is>
       </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
+          <t>OCA = "Total current assets" 4,262,701 − cash 1,807,202 − "Accounts receivable, net" 190,657 − "Inventories" 1,700,753 = 564,089 (5.1% of sales). AR is not inside this residual.</t>
         </is>
       </c>
       <c r="E10" s="46" t="inlineStr">
@@ -5114,45 +5223,45 @@
         </is>
       </c>
       <c r="I10" s="26">
-        <f>-('Balance Sheet'!I12-'Balance Sheet'!H12)</f>
+        <f>-('Balance Sheet'!I9-'Balance Sheet'!H9)</f>
         <v/>
       </c>
       <c r="J10" s="26">
-        <f>-('Balance Sheet'!J12-'Balance Sheet'!I12)</f>
+        <f>-('Balance Sheet'!J9-'Balance Sheet'!I9)</f>
         <v/>
       </c>
       <c r="K10" s="26">
-        <f>-('Balance Sheet'!K12-'Balance Sheet'!J12)</f>
+        <f>-('Balance Sheet'!K9-'Balance Sheet'!J9)</f>
         <v/>
       </c>
       <c r="L10" s="26">
-        <f>-('Balance Sheet'!L12-'Balance Sheet'!K12)</f>
+        <f>-('Balance Sheet'!L9-'Balance Sheet'!K9)</f>
         <v/>
       </c>
       <c r="M10" s="26">
-        <f>-('Balance Sheet'!M12-'Balance Sheet'!L12)</f>
+        <f>-('Balance Sheet'!M9-'Balance Sheet'!L9)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
+          <t xml:space="preserve">  (Incr.)/decr. in ROU assets</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
+          <t>ROU assets 14.7% of revenue; lease-intensive store model, stable vs FY25 operating lease footprint.</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>LULU balance sheet (10-K)</t>
+          <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
       <c r="D11" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
+          <t>Ctrl+F "Right-of-use lease assets" → 1,630,181 ÷ "Net revenue" 11,102,600 = 14.7%</t>
         </is>
       </c>
       <c r="E11" s="46" t="inlineStr">
@@ -5176,35 +5285,35 @@
         </is>
       </c>
       <c r="I11" s="26">
-        <f>-('Balance Sheet'!I14-'Balance Sheet'!H14)</f>
+        <f>-('Balance Sheet'!I13-'Balance Sheet'!H13)</f>
         <v/>
       </c>
       <c r="J11" s="26">
-        <f>-('Balance Sheet'!J14-'Balance Sheet'!I14)</f>
+        <f>-('Balance Sheet'!J13-'Balance Sheet'!I13)</f>
         <v/>
       </c>
       <c r="K11" s="26">
-        <f>-('Balance Sheet'!K14-'Balance Sheet'!J14)</f>
+        <f>-('Balance Sheet'!K13-'Balance Sheet'!J13)</f>
         <v/>
       </c>
       <c r="L11" s="26">
-        <f>-('Balance Sheet'!L14-'Balance Sheet'!K14)</f>
+        <f>-('Balance Sheet'!L13-'Balance Sheet'!K13)</f>
         <v/>
       </c>
       <c r="M11" s="26">
-        <f>-('Balance Sheet'!M14-'Balance Sheet'!L14)</f>
+        <f>-('Balance Sheet'!M13-'Balance Sheet'!L13)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
+          <t xml:space="preserve">  (Incr.)/decr. in other non-current assets</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
+          <t>ONCA 3.0% = FY25 total assets − CA − PPE − ROU − GW (338,947); matches earnings 'deferred taxes and other NC assets'.</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
@@ -5214,7 +5323,7 @@
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
+          <t>Ctrl+F "Total assets" 8,456,743 − current assets − "Property and equipment, net" − "Right-of-use lease assets" − goodwill/intangibles = 338,947 (3.0%)</t>
         </is>
       </c>
       <c r="E12" s="46" t="inlineStr">
@@ -5238,35 +5347,35 @@
         </is>
       </c>
       <c r="I12" s="26">
-        <f>('Balance Sheet'!I19-'Balance Sheet'!H19)</f>
+        <f>-('Balance Sheet'!I15-'Balance Sheet'!H15)</f>
         <v/>
       </c>
       <c r="J12" s="26">
-        <f>('Balance Sheet'!J19-'Balance Sheet'!I19)</f>
+        <f>-('Balance Sheet'!J15-'Balance Sheet'!I15)</f>
         <v/>
       </c>
       <c r="K12" s="26">
-        <f>('Balance Sheet'!K19-'Balance Sheet'!J19)</f>
+        <f>-('Balance Sheet'!K15-'Balance Sheet'!J15)</f>
         <v/>
       </c>
       <c r="L12" s="26">
-        <f>('Balance Sheet'!L19-'Balance Sheet'!K19)</f>
+        <f>-('Balance Sheet'!L15-'Balance Sheet'!K15)</f>
         <v/>
       </c>
       <c r="M12" s="26">
-        <f>('Balance Sheet'!M19-'Balance Sheet'!L19)</f>
+        <f>-('Balance Sheet'!M15-'Balance Sheet'!L15)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
+          <t xml:space="preserve">  Incr./(decr.) in accounts payable</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
+          <t>AP 6.8% of COGS; holds near FY25 level reflecting vendor terms and production payment cadence.</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -5276,7 +5385,7 @@
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
+          <t>Ctrl+F "Accounts payable" → 331,421 ÷ "Cost of goods sold" 4,818,468 = 6.9%</t>
         </is>
       </c>
       <c r="E13" s="46" t="inlineStr">
@@ -5323,12 +5432,12 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
+          <t xml:space="preserve">  Incr./(decr.) in accrued liabilities</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+          <t>Accrued liabilities 5.8% of revenue; stable comp, marketing, and operating accrual ratio.</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -5338,7 +5447,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+          <t>Ctrl+F "Accrued liabilities and other" → 662,982 ÷ "Net revenue" 11,102,600 = 6.0%</t>
         </is>
       </c>
       <c r="E14" s="46" t="inlineStr">
@@ -5362,139 +5471,154 @@
         </is>
       </c>
       <c r="I14" s="26">
-        <f>('Balance Sheet'!I22-'Balance Sheet'!H22)</f>
+        <f>('Balance Sheet'!I21-'Balance Sheet'!H21)</f>
         <v/>
       </c>
       <c r="J14" s="26">
-        <f>('Balance Sheet'!J22-'Balance Sheet'!I22)</f>
+        <f>('Balance Sheet'!J21-'Balance Sheet'!I21)</f>
         <v/>
       </c>
       <c r="K14" s="26">
-        <f>('Balance Sheet'!K22-'Balance Sheet'!J22)</f>
+        <f>('Balance Sheet'!K21-'Balance Sheet'!J21)</f>
         <v/>
       </c>
       <c r="L14" s="26">
-        <f>('Balance Sheet'!L22-'Balance Sheet'!K22)</f>
+        <f>('Balance Sheet'!L21-'Balance Sheet'!K21)</f>
         <v/>
       </c>
       <c r="M14" s="26">
-        <f>('Balance Sheet'!M22-'Balance Sheet'!L22)</f>
+        <f>('Balance Sheet'!M21-'Balance Sheet'!L21)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Incr./(decr.) in other current liabilities</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>OCL 5.5% = FY25 current liabilities minus AP, accrued, and current leases (residual ~594k); not the 45,954 'other' line alone.</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>LULU balance sheet (10-K)</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Total current liabilities" 1,887,548 − "Accounts payable" 331,421 − "Accrued liabilities and other" 662,982 − "Current lease liabilities" 298,724 ≈ 594,421 (5.4%)</t>
+        </is>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="26">
+        <f>('Balance Sheet'!I23-'Balance Sheet'!H23)</f>
+        <v/>
+      </c>
+      <c r="J15" s="26">
+        <f>('Balance Sheet'!J23-'Balance Sheet'!I23)</f>
+        <v/>
+      </c>
+      <c r="K15" s="26">
+        <f>('Balance Sheet'!K23-'Balance Sheet'!J23)</f>
+        <v/>
+      </c>
+      <c r="L15" s="26">
+        <f>('Balance Sheet'!L23-'Balance Sheet'!K23)</f>
+        <v/>
+      </c>
+      <c r="M15" s="26">
+        <f>('Balance Sheet'!M23-'Balance Sheet'!L23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Incr./(decr.) in operating lease liab.</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>Current lease liabilities 2.7% of revenue; short-term portion of operating lease obligations.</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>LULU lease disclosures (10-K)</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Current lease liabilities" → 298,724 ÷ "Net revenue" 11,102,600 = 2.7%</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="F16" s="46" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="46" t="inlineStr">
+      <c r="G16" s="46" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
+      <c r="H16" s="46" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I15" s="26">
-        <f>('Balance Sheet'!I21-'Balance Sheet'!H21)+('Balance Sheet'!I25-'Balance Sheet'!H25)</f>
-        <v/>
-      </c>
-      <c r="J15" s="26">
-        <f>('Balance Sheet'!J21-'Balance Sheet'!I21)+('Balance Sheet'!J25-'Balance Sheet'!I25)</f>
-        <v/>
-      </c>
-      <c r="K15" s="26">
-        <f>('Balance Sheet'!K21-'Balance Sheet'!J21)+('Balance Sheet'!K25-'Balance Sheet'!J25)</f>
-        <v/>
-      </c>
-      <c r="L15" s="26">
-        <f>('Balance Sheet'!L21-'Balance Sheet'!K21)+('Balance Sheet'!L25-'Balance Sheet'!K25)</f>
-        <v/>
-      </c>
-      <c r="M15" s="26">
-        <f>('Balance Sheet'!M21-'Balance Sheet'!L21)+('Balance Sheet'!M25-'Balance Sheet'!L25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Incr./(decr.) in deferred income taxes</t>
-        </is>
-      </c>
-      <c r="E16" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="25">
-        <f>('Balance Sheet'!I26-'Balance Sheet'!H26)</f>
-        <v/>
-      </c>
-      <c r="J16" s="25">
-        <f>('Balance Sheet'!J26-'Balance Sheet'!I26)</f>
-        <v/>
-      </c>
-      <c r="K16" s="25">
-        <f>('Balance Sheet'!K26-'Balance Sheet'!J26)</f>
-        <v/>
-      </c>
-      <c r="L16" s="25">
-        <f>('Balance Sheet'!L26-'Balance Sheet'!K26)</f>
-        <v/>
-      </c>
-      <c r="M16" s="25">
-        <f>('Balance Sheet'!M26-'Balance Sheet'!L26)</f>
+      <c r="I16" s="26">
+        <f>('Balance Sheet'!I22-'Balance Sheet'!H22)+('Balance Sheet'!I26-'Balance Sheet'!H26)</f>
+        <v/>
+      </c>
+      <c r="J16" s="26">
+        <f>('Balance Sheet'!J22-'Balance Sheet'!I22)+('Balance Sheet'!J26-'Balance Sheet'!I26)</f>
+        <v/>
+      </c>
+      <c r="K16" s="26">
+        <f>('Balance Sheet'!K22-'Balance Sheet'!J22)+('Balance Sheet'!K26-'Balance Sheet'!J26)</f>
+        <v/>
+      </c>
+      <c r="L16" s="26">
+        <f>('Balance Sheet'!L22-'Balance Sheet'!K22)+('Balance Sheet'!L26-'Balance Sheet'!K26)</f>
+        <v/>
+      </c>
+      <c r="M16" s="26">
+        <f>('Balance Sheet'!M22-'Balance Sheet'!L22)+('Balance Sheet'!M26-'Balance Sheet'!L26)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Incr./(decr.) in other non-current liab.</t>
+          <t xml:space="preserve">  Incr./(decr.) in deferred income taxes</t>
         </is>
       </c>
       <c r="E17" s="46" t="inlineStr">
@@ -5541,98 +5665,145 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Incr./(decr.) in other non-current liab.</t>
+        </is>
+      </c>
+      <c r="E18" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="25">
+        <f>('Balance Sheet'!I28-'Balance Sheet'!H28)</f>
+        <v/>
+      </c>
+      <c r="J18" s="25">
+        <f>('Balance Sheet'!J28-'Balance Sheet'!I28)</f>
+        <v/>
+      </c>
+      <c r="K18" s="25">
+        <f>('Balance Sheet'!K28-'Balance Sheet'!J28)</f>
+        <v/>
+      </c>
+      <c r="L18" s="25">
+        <f>('Balance Sheet'!L28-'Balance Sheet'!K28)</f>
+        <v/>
+      </c>
+      <c r="M18" s="25">
+        <f>('Balance Sheet'!M28-'Balance Sheet'!L28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Working capital &amp; other (reported, net)</t>
         </is>
       </c>
-      <c r="E18" s="25">
-        <f>E19-E5-E6-E7</f>
-        <v/>
-      </c>
-      <c r="F18" s="25">
-        <f>F19-F5-F6-F7</f>
-        <v/>
-      </c>
-      <c r="G18" s="25">
-        <f>G19-G5-G6-G7</f>
-        <v/>
-      </c>
-      <c r="H18" s="25">
-        <f>H19-H5-H6-H7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="E19" s="25">
+        <f>E20-E5-E6-E7</f>
+        <v/>
+      </c>
+      <c r="F19" s="25">
+        <f>F20-F5-F6-F7</f>
+        <v/>
+      </c>
+      <c r="G19" s="25">
+        <f>G20-G5-G6-G7</f>
+        <v/>
+      </c>
+      <c r="H19" s="25">
+        <f>H20-H5-H6-H7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="E19" s="43" t="n">
+      <c r="E20" s="43" t="n">
         <v>966463</v>
       </c>
-      <c r="F19" s="43" t="n">
+      <c r="F20" s="43" t="n">
         <v>2296164</v>
       </c>
-      <c r="G19" s="43" t="n">
+      <c r="G20" s="43" t="n">
         <v>2272713</v>
       </c>
-      <c r="H19" s="43" t="n">
+      <c r="H20" s="43" t="n">
         <v>1602477</v>
       </c>
-      <c r="I19" s="34">
-        <f>I5+I6+I7+SUM(I8:I17)</f>
-        <v/>
-      </c>
-      <c r="J19" s="34">
-        <f>J5+J6+J7+SUM(J8:J17)</f>
-        <v/>
-      </c>
-      <c r="K19" s="34">
-        <f>K5+K6+K7+SUM(K8:K17)</f>
-        <v/>
-      </c>
-      <c r="L19" s="34">
-        <f>L5+L6+L7+SUM(L8:L17)</f>
-        <v/>
-      </c>
-      <c r="M19" s="34">
-        <f>M5+M6+M7+SUM(M8:M17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="I20" s="34">
+        <f>I5+I6+I7+SUM(I8:I18)</f>
+        <v/>
+      </c>
+      <c r="J20" s="34">
+        <f>J5+J6+J7+SUM(J8:J18)</f>
+        <v/>
+      </c>
+      <c r="K20" s="34">
+        <f>K5+K6+K7+SUM(K8:K18)</f>
+        <v/>
+      </c>
+      <c r="L20" s="34">
+        <f>L5+L6+L7+SUM(L8:L18)</f>
+        <v/>
+      </c>
+      <c r="M20" s="34">
+        <f>M5+M6+M7+SUM(M8:M18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>INVESTING ACTIVITIES</t>
         </is>
       </c>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="18" t="n"/>
-      <c r="I21" s="18" t="n"/>
-      <c r="J21" s="18" t="n"/>
-      <c r="K21" s="18" t="n"/>
-      <c r="L21" s="18" t="n"/>
-      <c r="M21" s="18" t="n"/>
-    </row>
-    <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="18" t="n"/>
+      <c r="K22" s="18" t="n"/>
+      <c r="L22" s="18" t="n"/>
+      <c r="M22" s="18" t="n"/>
+    </row>
+    <row r="23" ht="150" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Capital expenditures</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>FY26 7.0% is $735M / $10.4B, not / FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: 7.0 / 6.0 / 5.5 / 5.0 / 5.0.</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>LULU CF statement (10-K)</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>FY25 actual (10-K)
   Ctrl+F "680,802"  →  capex $680.8M
@@ -5648,319 +5819,319 @@
   5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
-      <c r="E22" s="32" t="n">
+      <c r="E23" s="32" t="n">
         <v>-638657</v>
       </c>
-      <c r="F22" s="32" t="n">
+      <c r="F23" s="32" t="n">
         <v>-651865</v>
       </c>
-      <c r="G22" s="32" t="n">
+      <c r="G23" s="32" t="n">
         <v>-689232</v>
       </c>
-      <c r="H22" s="32" t="n">
+      <c r="H23" s="32" t="n">
         <v>-680802</v>
       </c>
-      <c r="I22" s="26">
+      <c r="I23" s="26">
         <f>-'Income Statement'!I4*'Assumptions'!I14</f>
         <v/>
       </c>
-      <c r="J22" s="26">
+      <c r="J23" s="26">
         <f>-'Income Statement'!J4*'Assumptions'!J14</f>
         <v/>
       </c>
-      <c r="K22" s="26">
+      <c r="K23" s="26">
         <f>-'Income Statement'!K4*'Assumptions'!K14</f>
         <v/>
       </c>
-      <c r="L22" s="26">
+      <c r="L23" s="26">
         <f>-'Income Statement'!L4*'Assumptions'!L14</f>
         <v/>
       </c>
-      <c r="M22" s="26">
+      <c r="M23" s="26">
         <f>-'Income Statement'!M4*'Assumptions'!M14</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>Net cash from investing activities</t>
         </is>
       </c>
-      <c r="E23" s="43" t="n">
+      <c r="E24" s="43" t="n">
         <v>-569937</v>
       </c>
-      <c r="F23" s="43" t="n">
+      <c r="F24" s="43" t="n">
         <v>-654132</v>
       </c>
-      <c r="G23" s="43" t="n">
+      <c r="G24" s="43" t="n">
         <v>-798174</v>
       </c>
-      <c r="H23" s="43" t="n">
+      <c r="H24" s="43" t="n">
         <v>-662118</v>
       </c>
-      <c r="I23" s="34">
-        <f>I22</f>
-        <v/>
-      </c>
-      <c r="J23" s="34">
-        <f>J22</f>
-        <v/>
-      </c>
-      <c r="K23" s="34">
-        <f>K22</f>
-        <v/>
-      </c>
-      <c r="L23" s="34">
-        <f>L22</f>
-        <v/>
-      </c>
-      <c r="M23" s="34">
-        <f>M22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="I24" s="34">
+        <f>I23</f>
+        <v/>
+      </c>
+      <c r="J24" s="34">
+        <f>J23</f>
+        <v/>
+      </c>
+      <c r="K24" s="34">
+        <f>K23</f>
+        <v/>
+      </c>
+      <c r="L24" s="34">
+        <f>L23</f>
+        <v/>
+      </c>
+      <c r="M24" s="34">
+        <f>M23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Projections: investing ≈ capex; excl. M&amp;A / securities)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>FINANCING ACTIVITIES</t>
         </is>
       </c>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
-      <c r="I26" s="18" t="n"/>
-      <c r="J26" s="18" t="n"/>
-      <c r="K26" s="18" t="n"/>
-      <c r="L26" s="18" t="n"/>
-      <c r="M26" s="18" t="n"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Repurchase of common stock</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>$500M annual repurchases; continued capital return at moderated pace vs FY24–25 peak buyback levels.</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>LULU CF: share repurchases (10-K)</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr</t>
         </is>
       </c>
-      <c r="E27" s="32" t="n">
+      <c r="E28" s="32" t="n">
         <v>-444001</v>
       </c>
-      <c r="F27" s="32" t="n">
+      <c r="F28" s="32" t="n">
         <v>-558652</v>
       </c>
-      <c r="G27" s="32" t="n">
+      <c r="G28" s="32" t="n">
         <v>-1636879</v>
       </c>
-      <c r="H27" s="32" t="n">
+      <c r="H28" s="32" t="n">
         <v>-1178349</v>
       </c>
-      <c r="I27" s="26">
-        <f>-'Assumptions'!I28</f>
-        <v/>
-      </c>
-      <c r="J27" s="26">
-        <f>-'Assumptions'!J28</f>
-        <v/>
-      </c>
-      <c r="K27" s="26">
-        <f>-'Assumptions'!K28</f>
-        <v/>
-      </c>
-      <c r="L27" s="26">
-        <f>-'Assumptions'!L28</f>
-        <v/>
-      </c>
-      <c r="M27" s="26">
-        <f>-'Assumptions'!M28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="33" t="inlineStr">
+      <c r="I28" s="26">
+        <f>-'Assumptions'!I29</f>
+        <v/>
+      </c>
+      <c r="J28" s="26">
+        <f>-'Assumptions'!J29</f>
+        <v/>
+      </c>
+      <c r="K28" s="26">
+        <f>-'Assumptions'!K29</f>
+        <v/>
+      </c>
+      <c r="L28" s="26">
+        <f>-'Assumptions'!L29</f>
+        <v/>
+      </c>
+      <c r="M28" s="26">
+        <f>-'Assumptions'!M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>Net cash from financing activities</t>
         </is>
       </c>
-      <c r="E28" s="43" t="n">
+      <c r="E29" s="43" t="n">
         <v>-467487</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F29" s="43" t="n">
         <v>-548828</v>
       </c>
-      <c r="G28" s="43" t="n">
+      <c r="G29" s="43" t="n">
         <v>-1652508</v>
       </c>
-      <c r="H28" s="43" t="n">
+      <c r="H29" s="43" t="n">
         <v>-1208656</v>
       </c>
-      <c r="I28" s="34">
-        <f>I27</f>
-        <v/>
-      </c>
-      <c r="J28" s="34">
-        <f>J27</f>
-        <v/>
-      </c>
-      <c r="K28" s="34">
-        <f>K27</f>
-        <v/>
-      </c>
-      <c r="L28" s="34">
-        <f>L27</f>
-        <v/>
-      </c>
-      <c r="M28" s="34">
-        <f>M27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
+      <c r="I29" s="34">
+        <f>I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="34">
+        <f>J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="34">
+        <f>K28</f>
+        <v/>
+      </c>
+      <c r="L29" s="34">
+        <f>L28</f>
+        <v/>
+      </c>
+      <c r="M29" s="34">
+        <f>M28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  (Projections: financing ≈ buybacks; SBC non-cash in equity)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="33" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="E31" s="34">
-        <f>E19+E23+E28</f>
-        <v/>
-      </c>
-      <c r="F31" s="34">
-        <f>F19+F23+F28</f>
-        <v/>
-      </c>
-      <c r="G31" s="34">
-        <f>G19+G23+G28</f>
-        <v/>
-      </c>
-      <c r="H31" s="34">
-        <f>H19+H23+H28</f>
-        <v/>
-      </c>
-      <c r="I31" s="34">
-        <f>I19+I23+I28</f>
-        <v/>
-      </c>
-      <c r="J31" s="34">
-        <f>J19+J23+J28</f>
-        <v/>
-      </c>
-      <c r="K31" s="34">
-        <f>K19+K23+K28</f>
-        <v/>
-      </c>
-      <c r="L31" s="34">
-        <f>L19+L23+L28</f>
-        <v/>
-      </c>
-      <c r="M31" s="34">
-        <f>M19+M23+M28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="E32" s="34">
+        <f>E20+E24+E29</f>
+        <v/>
+      </c>
+      <c r="F32" s="34">
+        <f>F20+F24+F29</f>
+        <v/>
+      </c>
+      <c r="G32" s="34">
+        <f>G20+G24+G29</f>
+        <v/>
+      </c>
+      <c r="H32" s="34">
+        <f>H20+H24+H29</f>
+        <v/>
+      </c>
+      <c r="I32" s="34">
+        <f>I20+I24+I29</f>
+        <v/>
+      </c>
+      <c r="J32" s="34">
+        <f>J20+J24+J29</f>
+        <v/>
+      </c>
+      <c r="K32" s="34">
+        <f>K20+K24+K29</f>
+        <v/>
+      </c>
+      <c r="L32" s="34">
+        <f>L20+L24+L29</f>
+        <v/>
+      </c>
+      <c r="M32" s="34">
+        <f>M20+M24+M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Cash, beginning of year</t>
         </is>
       </c>
-      <c r="E32" s="32" t="n">
+      <c r="E33" s="32" t="n">
         <v>1150517</v>
       </c>
-      <c r="F32" s="32" t="n">
+      <c r="F33" s="32" t="n">
         <v>1154867</v>
       </c>
-      <c r="G32" s="32" t="n">
+      <c r="G33" s="32" t="n">
         <v>2243971</v>
       </c>
-      <c r="H32" s="32" t="n">
+      <c r="H33" s="32" t="n">
         <v>1984336</v>
       </c>
-      <c r="I32" s="25">
-        <f>H33</f>
-        <v/>
-      </c>
-      <c r="J32" s="25">
-        <f>I33</f>
-        <v/>
-      </c>
-      <c r="K32" s="25">
-        <f>J33</f>
-        <v/>
-      </c>
-      <c r="L32" s="25">
-        <f>K33</f>
-        <v/>
-      </c>
-      <c r="M32" s="25">
-        <f>L33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="I33" s="25">
+        <f>H34</f>
+        <v/>
+      </c>
+      <c r="J33" s="25">
+        <f>I34</f>
+        <v/>
+      </c>
+      <c r="K33" s="25">
+        <f>J34</f>
+        <v/>
+      </c>
+      <c r="L33" s="25">
+        <f>K34</f>
+        <v/>
+      </c>
+      <c r="M33" s="25">
+        <f>L34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
         <is>
           <t>Cash, end of year</t>
         </is>
       </c>
-      <c r="E33" s="44" t="n">
+      <c r="E34" s="44" t="n">
         <v>1154867</v>
       </c>
-      <c r="F33" s="44" t="n">
+      <c r="F34" s="44" t="n">
         <v>2243971</v>
       </c>
-      <c r="G33" s="44" t="n">
+      <c r="G34" s="44" t="n">
         <v>1984336</v>
       </c>
-      <c r="H33" s="44" t="n">
+      <c r="H34" s="44" t="n">
         <v>1807202</v>
       </c>
-      <c r="I33" s="35">
-        <f>I32+I31</f>
-        <v/>
-      </c>
-      <c r="J33" s="35">
-        <f>J32+J31</f>
-        <v/>
-      </c>
-      <c r="K33" s="35">
-        <f>K32+K31</f>
-        <v/>
-      </c>
-      <c r="L33" s="35">
-        <f>L32+L31</f>
-        <v/>
-      </c>
-      <c r="M33" s="35">
-        <f>M32+M31</f>
+      <c r="I34" s="35">
+        <f>I33+I32</f>
+        <v/>
+      </c>
+      <c r="J34" s="35">
+        <f>J33+J32</f>
+        <v/>
+      </c>
+      <c r="K34" s="35">
+        <f>K33+K32</f>
+        <v/>
+      </c>
+      <c r="L34" s="35">
+        <f>L33+L32</f>
+        <v/>
+      </c>
+      <c r="M34" s="35">
+        <f>M33+M32</f>
         <v/>
       </c>
     </row>
@@ -5992,36 +6163,37 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add bottom-up revenue drivers, Firecrawl ingestion, and assumptions memo PDF
- ingest_kpis.py scrapes FY2025 10-K via Firecrawl for store counts, channel
  revenue, geo splits, comp sales, SPSF, and category mix into ingested_kpis.json
- New Revenue Drivers tab: store fleet by geo, SPSF/comp sales, DTC traffic ×
  conversion × AOV, category mix, and reconciliation to Scenarios base revenue
- LULU_Assumptions_Memo.pdf (1-page FICO-style summary) linked from Cover/DCF
- driver_kpis.py holds canonical anchors and FY26-30 red assumptions with B/C/D docs

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B22"/>
+  <dimension ref="B2:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -846,12 +846,27 @@
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Assumptions  •  Income Statement  •  Balance Sheet  •  Cash Flow</t>
+          <t>Assumptions  •  Revenue Drivers  •  Income Statement  •  Balance Sheet  •  Cash Flow</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>ASSUMPTIONS MEMO (1-page PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>LULU_Assumptions_Memo.pdf — justifications, Ctrl+F anchors, and strategic context
+Ctrl+F: Open the linked PDF for a single-page summary of all red assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Built from scratch for the GIS IR selection assignment. Units: US$ thousands unless noted.</t>
         </is>
@@ -862,6 +877,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand assumptions PDF to full guide for every model tab
Auto-generate 9-page LULU_Assumptions_Memo.pdf from data.py (102 assumptions
across WACC, Scenarios, Revenue Drivers, DCF, Comps, 3-Statement). Update
Cover links on both workbooks.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -853,15 +853,15 @@
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ASSUMPTIONS MEMO (1-page PDF)</t>
+          <t>ASSUMPTIONS GUIDE (PDF — every tab)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>LULU_Assumptions_Memo.pdf — justifications, Ctrl+F anchors, and strategic context
-Ctrl+F: Open the linked PDF for a single-page summary of all red assumptions.</t>
+          <t>LULU_Assumptions_Memo.pdf — full guide: every red assumption on WACC, Scenarios, Revenue Drivers, DCF, Comps &amp; 3-Statement
+Ctrl+F: Open for justification, clickable source links, and Ctrl+F proof for every assumption.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Ctrl+F hints for NASDAQ price and FY25 shares outstanding
Replace useless Ctrl+F "LULU" on NASDAQ with Firecrawl-verified
"closed at $100.61". Split WACC market-equity row into price (NASDAQ)
and shares (10-K: "111,380 and 116,166 issued and outstanding").
Update DCF bridge/comps share rows, verify script uses Firecrawl for
NASDAQ, and rebuild workbooks and assumptions PDF.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -2191,7 +2191,7 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
+          <t>Ctrl+F "closed at $100.61" → Last Sale (NASDAQ). Model repurchase price starts at $100.</t>
         </is>
       </c>
       <c r="I30" s="28" t="n">
@@ -2940,7 +2940,7 @@
       <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Ctrl+F "Repurchase of common stock" → ( 1,178,349 ) ($000) FY25; model (500,000)/yr
-Also: Ctrl+F "LULU" → Last Sale / Previous Close (~$100). FY26 model repurchase price starts at $100.</t>
+Also: Ctrl+F "closed at $100.61" → Last Sale (NASDAQ). Model repurchase price starts at $100.</t>
         </is>
       </c>
       <c r="E16" s="32" t="n">

</xml_diff>

<commit_message>
Restore slides 1-12 to user exact copy; confirm $500M/yr buybacks
- Replace institutional refactor with verbatim narrative text for slides 1-12
- Slide 1: Table of Contents with roadmap paragraph (not labeled bullets)
- Slide 12: single $500M buyback bullet (18.7M shares, $13.36 EPS)
- Model: Scenarios G21=500000, G158:G162=-G21 ($500M/yr fixed buybacks)
- Rebuild pitch deck and valuation spreadsheets

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_3_Statement_Model.xlsx
+++ b/LULU/LULU_3_Statement_Model.xlsx
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
+          <t>Add back $134.5M in FY26 only; already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
+          <t>Add back $134.5M in FY26 only; already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">

</xml_diff>